<commit_message>
Add SP+/PPA/talent features, totals+moneyline betting, rebuilt tracking page
</commit_message>
<xml_diff>
--- a/excel/MW_Handicapping_Tracker.xlsx
+++ b/excel/MW_Handicapping_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\deene\Mountain Dub Handicapping\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_C56C0D99AC13B70F6075011805D2AE0EA748AB8C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D81218B9-12FD-4D58-B002-03798A267726}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Read Me" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="109">
   <si>
     <t>Week</t>
   </si>
@@ -292,18 +292,6 @@
   </si>
   <si>
     <t>Running Bankroll</t>
-  </si>
-  <si>
-    <t>San José State @ Air Force</t>
-  </si>
-  <si>
-    <t>Spread</t>
-  </si>
-  <si>
-    <t>Air Force -4.5</t>
-  </si>
-  <si>
-    <t>W</t>
   </si>
   <si>
     <t>CLV note: Closing Line - Line Taken. For a favorite (negative number), a less-negative closing line than what you bet means the market moved toward you -- positive CLV. Read each row in context of which side you took.</t>
@@ -976,7 +964,7 @@
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="2" width="11" customWidth="1"/>
     <col min="3" max="3" width="20.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="4" max="4" width="18" bestFit="1" customWidth="1"/>
     <col min="5" max="6" width="16" customWidth="1"/>
     <col min="7" max="7" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="7.5703125" bestFit="1" customWidth="1"/>
@@ -2121,7 +2109,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:M45"/>
+  <dimension ref="A1:M44"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -2180,612 +2168,568 @@
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="B2" s="8">
-        <v>1</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="D2" s="8" t="s">
-        <v>86</v>
-      </c>
-      <c r="E2" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="F2" s="8">
-        <v>-4.5</v>
-      </c>
-      <c r="G2" s="8">
-        <v>-110</v>
-      </c>
-      <c r="H2" s="8">
-        <v>2</v>
-      </c>
-      <c r="I2" s="8">
-        <v>-6</v>
-      </c>
-      <c r="J2" s="6">
-        <f>I2-F2</f>
-        <v>-1.5</v>
-      </c>
-      <c r="K2" s="8" t="s">
-        <v>88</v>
+      <c r="J2" s="6" t="str">
+        <f t="shared" ref="J2:J41" si="0">IF(I2="","",I2-F2)</f>
+        <v/>
       </c>
       <c r="L2" s="6">
-        <f t="shared" ref="L2:L42" si="0">IF(K2="W",IF(G2&lt;0,H2*100/ABS(G2),H2*G2/100),IF(K2="L",-H2,0))</f>
-        <v>1.8181818181818181</v>
+        <f t="shared" ref="L2:L41" si="1">IF(K2="W",IF(G2&lt;0,H2*100/ABS(G2),H2*G2/100),IF(K2="L",-H2,0))</f>
+        <v>0</v>
       </c>
       <c r="M2" s="6">
         <f>Settings!$B$4+SUM(L$2:L2)</f>
-        <v>101.81818181818181</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="J3" s="6" t="str">
-        <f t="shared" ref="J3:J42" si="1">IF(I3="","",I3-F3)</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="L3" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M3" s="6">
         <f>Settings!$B$4+SUM(L$2:L3)</f>
-        <v>101.81818181818181</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="J4" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="L4" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M4" s="6">
         <f>Settings!$B$4+SUM(L$2:L4)</f>
-        <v>101.81818181818181</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="J5" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="L5" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M5" s="6">
         <f>Settings!$B$4+SUM(L$2:L5)</f>
-        <v>101.81818181818181</v>
+        <v>100</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="J6" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="L6" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M6" s="6">
         <f>Settings!$B$4+SUM(L$2:L6)</f>
-        <v>101.81818181818181</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="J7" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="L7" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M7" s="6">
         <f>Settings!$B$4+SUM(L$2:L7)</f>
-        <v>101.81818181818181</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="J8" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="L8" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M8" s="6">
         <f>Settings!$B$4+SUM(L$2:L8)</f>
-        <v>101.81818181818181</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="J9" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="L9" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M9" s="6">
         <f>Settings!$B$4+SUM(L$2:L9)</f>
-        <v>101.81818181818181</v>
+        <v>100</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="J10" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="L10" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M10" s="6">
         <f>Settings!$B$4+SUM(L$2:L10)</f>
-        <v>101.81818181818181</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="J11" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="L11" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M11" s="6">
         <f>Settings!$B$4+SUM(L$2:L11)</f>
-        <v>101.81818181818181</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="J12" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="L12" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M12" s="6">
         <f>Settings!$B$4+SUM(L$2:L12)</f>
-        <v>101.81818181818181</v>
+        <v>100</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="J13" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="L13" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M13" s="6">
         <f>Settings!$B$4+SUM(L$2:L13)</f>
-        <v>101.81818181818181</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="J14" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="L14" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M14" s="6">
         <f>Settings!$B$4+SUM(L$2:L14)</f>
-        <v>101.81818181818181</v>
+        <v>100</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="J15" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="L15" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M15" s="6">
         <f>Settings!$B$4+SUM(L$2:L15)</f>
-        <v>101.81818181818181</v>
+        <v>100</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="J16" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="L16" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M16" s="6">
         <f>Settings!$B$4+SUM(L$2:L16)</f>
-        <v>101.81818181818181</v>
+        <v>100</v>
       </c>
     </row>
     <row r="17" spans="10:13" x14ac:dyDescent="0.25">
       <c r="J17" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="L17" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M17" s="6">
         <f>Settings!$B$4+SUM(L$2:L17)</f>
-        <v>101.81818181818181</v>
+        <v>100</v>
       </c>
     </row>
     <row r="18" spans="10:13" x14ac:dyDescent="0.25">
       <c r="J18" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="L18" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M18" s="6">
         <f>Settings!$B$4+SUM(L$2:L18)</f>
-        <v>101.81818181818181</v>
+        <v>100</v>
       </c>
     </row>
     <row r="19" spans="10:13" x14ac:dyDescent="0.25">
       <c r="J19" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="L19" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M19" s="6">
         <f>Settings!$B$4+SUM(L$2:L19)</f>
-        <v>101.81818181818181</v>
+        <v>100</v>
       </c>
     </row>
     <row r="20" spans="10:13" x14ac:dyDescent="0.25">
       <c r="J20" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="L20" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M20" s="6">
         <f>Settings!$B$4+SUM(L$2:L20)</f>
-        <v>101.81818181818181</v>
+        <v>100</v>
       </c>
     </row>
     <row r="21" spans="10:13" x14ac:dyDescent="0.25">
       <c r="J21" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="L21" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M21" s="6">
         <f>Settings!$B$4+SUM(L$2:L21)</f>
-        <v>101.81818181818181</v>
+        <v>100</v>
       </c>
     </row>
     <row r="22" spans="10:13" x14ac:dyDescent="0.25">
       <c r="J22" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="L22" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M22" s="6">
         <f>Settings!$B$4+SUM(L$2:L22)</f>
-        <v>101.81818181818181</v>
+        <v>100</v>
       </c>
     </row>
     <row r="23" spans="10:13" x14ac:dyDescent="0.25">
       <c r="J23" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="L23" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M23" s="6">
         <f>Settings!$B$4+SUM(L$2:L23)</f>
-        <v>101.81818181818181</v>
+        <v>100</v>
       </c>
     </row>
     <row r="24" spans="10:13" x14ac:dyDescent="0.25">
       <c r="J24" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="L24" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M24" s="6">
         <f>Settings!$B$4+SUM(L$2:L24)</f>
-        <v>101.81818181818181</v>
+        <v>100</v>
       </c>
     </row>
     <row r="25" spans="10:13" x14ac:dyDescent="0.25">
       <c r="J25" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="L25" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M25" s="6">
         <f>Settings!$B$4+SUM(L$2:L25)</f>
-        <v>101.81818181818181</v>
+        <v>100</v>
       </c>
     </row>
     <row r="26" spans="10:13" x14ac:dyDescent="0.25">
       <c r="J26" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="L26" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M26" s="6">
         <f>Settings!$B$4+SUM(L$2:L26)</f>
-        <v>101.81818181818181</v>
+        <v>100</v>
       </c>
     </row>
     <row r="27" spans="10:13" x14ac:dyDescent="0.25">
       <c r="J27" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="L27" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M27" s="6">
         <f>Settings!$B$4+SUM(L$2:L27)</f>
-        <v>101.81818181818181</v>
+        <v>100</v>
       </c>
     </row>
     <row r="28" spans="10:13" x14ac:dyDescent="0.25">
       <c r="J28" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="L28" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M28" s="6">
         <f>Settings!$B$4+SUM(L$2:L28)</f>
-        <v>101.81818181818181</v>
+        <v>100</v>
       </c>
     </row>
     <row r="29" spans="10:13" x14ac:dyDescent="0.25">
       <c r="J29" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="L29" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M29" s="6">
         <f>Settings!$B$4+SUM(L$2:L29)</f>
-        <v>101.81818181818181</v>
+        <v>100</v>
       </c>
     </row>
     <row r="30" spans="10:13" x14ac:dyDescent="0.25">
       <c r="J30" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="L30" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M30" s="6">
         <f>Settings!$B$4+SUM(L$2:L30)</f>
-        <v>101.81818181818181</v>
+        <v>100</v>
       </c>
     </row>
     <row r="31" spans="10:13" x14ac:dyDescent="0.25">
       <c r="J31" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="L31" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M31" s="6">
         <f>Settings!$B$4+SUM(L$2:L31)</f>
-        <v>101.81818181818181</v>
+        <v>100</v>
       </c>
     </row>
     <row r="32" spans="10:13" x14ac:dyDescent="0.25">
       <c r="J32" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="L32" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M32" s="6">
         <f>Settings!$B$4+SUM(L$2:L32)</f>
-        <v>101.81818181818181</v>
+        <v>100</v>
       </c>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="J33" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="L33" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M33" s="6">
         <f>Settings!$B$4+SUM(L$2:L33)</f>
-        <v>101.81818181818181</v>
+        <v>100</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.25">
       <c r="J34" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="L34" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M34" s="6">
         <f>Settings!$B$4+SUM(L$2:L34)</f>
-        <v>101.81818181818181</v>
+        <v>100</v>
       </c>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="J35" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="L35" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M35" s="6">
         <f>Settings!$B$4+SUM(L$2:L35)</f>
-        <v>101.81818181818181</v>
+        <v>100</v>
       </c>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.25">
       <c r="J36" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="L36" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M36" s="6">
         <f>Settings!$B$4+SUM(L$2:L36)</f>
-        <v>101.81818181818181</v>
+        <v>100</v>
       </c>
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.25">
       <c r="J37" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="L37" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M37" s="6">
         <f>Settings!$B$4+SUM(L$2:L37)</f>
-        <v>101.81818181818181</v>
+        <v>100</v>
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.25">
       <c r="J38" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="L38" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M38" s="6">
         <f>Settings!$B$4+SUM(L$2:L38)</f>
-        <v>101.81818181818181</v>
+        <v>100</v>
       </c>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.25">
       <c r="J39" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="L39" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M39" s="6">
         <f>Settings!$B$4+SUM(L$2:L39)</f>
-        <v>101.81818181818181</v>
+        <v>100</v>
       </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.25">
       <c r="J40" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="L40" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M40" s="6">
         <f>Settings!$B$4+SUM(L$2:L40)</f>
-        <v>101.81818181818181</v>
+        <v>100</v>
       </c>
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.25">
       <c r="J41" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="L41" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="M41" s="6">
         <f>Settings!$B$4+SUM(L$2:L41)</f>
-        <v>101.81818181818181</v>
-      </c>
-    </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="J42" s="6" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="L42" s="6">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="M42" s="6">
-        <f>Settings!$B$4+SUM(L$2:L42)</f>
-        <v>101.81818181818181</v>
-      </c>
-    </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A45" s="2" t="s">
-        <v>89</v>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A44" s="2" t="s">
+        <v>85</v>
       </c>
     </row>
   </sheetData>
@@ -2811,28 +2755,28 @@
   <sheetData>
     <row r="1" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="F1" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="G1" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="H1" s="5" t="s">
         <v>93</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>97</v>
       </c>
       <c r="I1" s="5" t="s">
         <v>65</v>
@@ -2843,10 +2787,10 @@
         <v>19</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="D2" s="8">
         <v>1473</v>
@@ -2864,7 +2808,7 @@
         <v>141</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -2872,10 +2816,10 @@
         <v>28</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="D3" s="8">
         <v>1561.1</v>
@@ -2893,7 +2837,7 @@
         <v>124</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -2901,10 +2845,10 @@
         <v>31</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="D4" s="8">
         <v>1361.9</v>
@@ -2922,7 +2866,7 @@
         <v>98</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
@@ -2930,10 +2874,10 @@
         <v>33</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="D5" s="8">
         <v>1566.5</v>
@@ -2951,7 +2895,7 @@
         <v>87</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
@@ -2959,10 +2903,10 @@
         <v>21</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="D6" s="8">
         <v>1790.9</v>
@@ -2976,7 +2920,7 @@
         <v>117</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
@@ -2984,10 +2928,10 @@
         <v>25</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="D7" s="8">
         <v>1394.5</v>
@@ -3005,7 +2949,7 @@
         <v>82</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
@@ -3013,10 +2957,10 @@
         <v>23</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="D8" s="8">
         <v>1388.2</v>
@@ -3034,7 +2978,7 @@
         <v>129</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
@@ -3042,10 +2986,10 @@
         <v>35</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="D9" s="8">
         <v>1645.3</v>
@@ -3063,7 +3007,7 @@
         <v>63</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
@@ -3071,10 +3015,10 @@
         <v>42</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="D10" s="8">
         <v>1302.8</v>
@@ -3092,7 +3036,7 @@
         <v>92</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
@@ -3100,10 +3044,10 @@
         <v>29</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="D11" s="8">
         <v>1399.9</v>
@@ -3121,7 +3065,7 @@
         <v>114</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Pending Bets section to Tracking page
</commit_message>
<xml_diff>
--- a/excel/MW_Handicapping_Tracker.xlsx
+++ b/excel/MW_Handicapping_Tracker.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\deene\Mountain Dub Handicapping\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_34675B918E07B70F6075012A0DD7B51B670FD0CF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{844C6AA8-16BC-4493-9EEE-F31799BE265D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="112">
   <si>
     <t>Date</t>
   </si>
@@ -364,6 +364,15 @@
   </si>
   <si>
     <t>Full history. Home elevation ~7,220 ft — coldest, highest venue in the league.</t>
+  </si>
+  <si>
+    <t>Spread</t>
+  </si>
+  <si>
+    <t>Jacksonvillie State @ North Dakota State</t>
+  </si>
+  <si>
+    <t>North Dakota State -7</t>
   </si>
 </sst>
 </file>
@@ -1031,49 +1040,49 @@
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A2" s="8">
+      <c r="A2">
         <v>1</v>
       </c>
-      <c r="B2" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="D2" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="E2" s="8">
-        <v>-18.100000000000001</v>
-      </c>
-      <c r="F2" s="8">
-        <v>-30.5</v>
+      <c r="B2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E2">
+        <v>-38.6</v>
+      </c>
+      <c r="F2">
+        <v>-38.200000000000003</v>
       </c>
       <c r="G2" s="6">
-        <f t="shared" ref="G2:G29" si="0">F2-E2</f>
-        <v>-12.399999999999999</v>
+        <f>F2-E2</f>
+        <v>0.39999999999999858</v>
       </c>
       <c r="H2" s="6" t="str">
-        <f t="shared" ref="H2:H29" si="1">IF(G2=0,"Pick'em",IF(G2&gt;0,"Home","Away"))</f>
-        <v>Away</v>
-      </c>
-      <c r="I2" s="8">
-        <v>56.3</v>
-      </c>
-      <c r="J2" s="8">
-        <v>58.5</v>
+        <f>IF(G2=0,"Pick'em",IF(G2&gt;0,"Home","Away"))</f>
+        <v>Home</v>
+      </c>
+      <c r="I2">
+        <v>58.3</v>
+      </c>
+      <c r="J2">
+        <v>60.5</v>
       </c>
       <c r="K2" s="6">
-        <f t="shared" ref="K2:K29" si="2">I2-J2</f>
+        <f>I2-J2</f>
         <v>-2.2000000000000028</v>
       </c>
       <c r="L2" s="6" t="str">
-        <f t="shared" ref="L2:L29" si="3">IF(K2=0,"Push",IF(K2&gt;0,"Over","Under"))</f>
+        <f>IF(K2=0,"Push",IF(K2&gt;0,"Over","Under"))</f>
         <v>Under</v>
       </c>
       <c r="M2" s="6" t="str">
         <f>IF(ABS(G2)&gt;=Settings!$B$5,H2,"Pass")</f>
-        <v>Away</v>
+        <v>Pass</v>
       </c>
       <c r="N2" s="6" t="str">
         <f>IF(ABS(K2)&gt;=Settings!$B$6,L2,"Pass")</f>
@@ -1087,40 +1096,40 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="C3" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="D3" t="s">
         <v>63</v>
       </c>
       <c r="E3">
-        <v>-51.8</v>
+        <v>-21.2</v>
       </c>
       <c r="F3">
-        <v>-39.5</v>
+        <v>-7</v>
       </c>
       <c r="G3" s="6">
-        <f t="shared" si="0"/>
-        <v>12.299999999999997</v>
+        <f>F3-E3</f>
+        <v>14.2</v>
       </c>
       <c r="H3" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(G3=0,"Pick'em",IF(G3&gt;0,"Home","Away"))</f>
         <v>Home</v>
       </c>
       <c r="I3">
-        <v>60.8</v>
+        <v>53.2</v>
       </c>
       <c r="J3">
-        <v>57.5</v>
+        <v>46.2</v>
       </c>
       <c r="K3" s="6">
-        <f t="shared" si="2"/>
-        <v>3.2999999999999972</v>
+        <f>I3-J3</f>
+        <v>7</v>
       </c>
       <c r="L3" s="6" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(K3=0,"Push",IF(K3&gt;0,"Over","Under"))</f>
         <v>Over</v>
       </c>
       <c r="M3" s="6" t="str">
@@ -1140,38 +1149,38 @@
         <v>64</v>
       </c>
       <c r="C4" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="D4" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="E4">
-        <v>-38.6</v>
+        <v>-2.9</v>
       </c>
       <c r="F4">
-        <v>-38.200000000000003</v>
+        <v>-4</v>
       </c>
       <c r="G4" s="6">
-        <f t="shared" si="0"/>
-        <v>0.39999999999999858</v>
+        <f>F4-E4</f>
+        <v>-1.1000000000000001</v>
       </c>
       <c r="H4" s="6" t="str">
-        <f t="shared" si="1"/>
-        <v>Home</v>
+        <f>IF(G4=0,"Pick'em",IF(G4&gt;0,"Home","Away"))</f>
+        <v>Away</v>
       </c>
       <c r="I4">
-        <v>58.3</v>
+        <v>55.5</v>
       </c>
       <c r="J4">
-        <v>60.5</v>
+        <v>48.8</v>
       </c>
       <c r="K4" s="6">
-        <f t="shared" si="2"/>
-        <v>-2.2000000000000028</v>
+        <f>I4-J4</f>
+        <v>6.7000000000000028</v>
       </c>
       <c r="L4" s="6" t="str">
-        <f t="shared" si="3"/>
-        <v>Under</v>
+        <f>IF(K4=0,"Push",IF(K4&gt;0,"Over","Under"))</f>
+        <v>Over</v>
       </c>
       <c r="M4" s="6" t="str">
         <f>IF(ABS(G4)&gt;=Settings!$B$5,H4,"Pass")</f>
@@ -1179,7 +1188,7 @@
       </c>
       <c r="N4" s="6" t="str">
         <f>IF(ABS(K4)&gt;=Settings!$B$6,L4,"Pass")</f>
-        <v>Under</v>
+        <v>Over</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.25">
@@ -1187,49 +1196,49 @@
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>59</v>
+        <v>78</v>
       </c>
       <c r="C5" t="s">
-        <v>67</v>
+        <v>79</v>
       </c>
       <c r="D5" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="E5">
-        <v>-33</v>
+        <v>-11.9</v>
       </c>
       <c r="F5">
-        <v>-31.8</v>
+        <v>-4.5</v>
       </c>
       <c r="G5" s="6">
-        <f t="shared" si="0"/>
-        <v>1.1999999999999993</v>
+        <f>F5-E5</f>
+        <v>7.4</v>
       </c>
       <c r="H5" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(G5=0,"Pick'em",IF(G5&gt;0,"Home","Away"))</f>
         <v>Home</v>
       </c>
       <c r="I5">
-        <v>46.8</v>
+        <v>62.9</v>
       </c>
       <c r="J5">
-        <v>45.5</v>
+        <v>56.5</v>
       </c>
       <c r="K5" s="6">
-        <f t="shared" si="2"/>
-        <v>1.2999999999999972</v>
+        <f>I5-J5</f>
+        <v>6.3999999999999986</v>
       </c>
       <c r="L5" s="6" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(K5=0,"Push",IF(K5&gt;0,"Over","Under"))</f>
         <v>Over</v>
       </c>
       <c r="M5" s="6" t="str">
         <f>IF(ABS(G5)&gt;=Settings!$B$5,H5,"Pass")</f>
-        <v>Pass</v>
+        <v>Home</v>
       </c>
       <c r="N5" s="6" t="str">
         <f>IF(ABS(K5)&gt;=Settings!$B$6,L5,"Pass")</f>
-        <v>Pass</v>
+        <v>Over</v>
       </c>
       <c r="R5" s="6" t="s">
         <v>61</v>
@@ -1240,40 +1249,40 @@
         <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>64</v>
+        <v>82</v>
       </c>
       <c r="C6" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="D6" t="s">
-        <v>63</v>
+        <v>83</v>
       </c>
       <c r="E6">
-        <v>-21.2</v>
+        <v>-11.2</v>
       </c>
       <c r="F6">
-        <v>-7</v>
+        <v>-5</v>
       </c>
       <c r="G6" s="6">
-        <f t="shared" si="0"/>
-        <v>14.2</v>
+        <f>F6-E6</f>
+        <v>6.1999999999999993</v>
       </c>
       <c r="H6" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(G6=0,"Pick'em",IF(G6&gt;0,"Home","Away"))</f>
         <v>Home</v>
       </c>
       <c r="I6">
-        <v>53.2</v>
+        <v>55.2</v>
       </c>
       <c r="J6">
-        <v>46.2</v>
+        <v>53.5</v>
       </c>
       <c r="K6" s="6">
-        <f t="shared" si="2"/>
-        <v>7</v>
+        <f>I6-J6</f>
+        <v>1.7000000000000028</v>
       </c>
       <c r="L6" s="6" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(K6=0,"Push",IF(K6&gt;0,"Over","Under"))</f>
         <v>Over</v>
       </c>
       <c r="M6" s="6" t="str">
@@ -1282,60 +1291,60 @@
       </c>
       <c r="N6" s="6" t="str">
         <f>IF(ABS(K6)&gt;=Settings!$B$6,L6,"Pass")</f>
-        <v>Over</v>
+        <v>Pass</v>
       </c>
       <c r="R6" s="6" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A7">
+      <c r="A7" s="8">
         <v>1</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="C7" t="s">
-        <v>71</v>
-      </c>
-      <c r="D7" t="s">
-        <v>72</v>
-      </c>
-      <c r="E7">
-        <v>-6.4</v>
-      </c>
-      <c r="F7">
-        <v>-3.5</v>
+      <c r="C7" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="E7" s="8">
+        <v>-18.100000000000001</v>
+      </c>
+      <c r="F7" s="8">
+        <v>-30.5</v>
       </c>
       <c r="G7" s="6">
-        <f t="shared" si="0"/>
-        <v>2.9000000000000004</v>
+        <f>F7-E7</f>
+        <v>-12.399999999999999</v>
       </c>
       <c r="H7" s="6" t="str">
-        <f t="shared" si="1"/>
-        <v>Home</v>
-      </c>
-      <c r="I7">
-        <v>51.2</v>
-      </c>
-      <c r="J7">
-        <v>47.8</v>
+        <f>IF(G7=0,"Pick'em",IF(G7&gt;0,"Home","Away"))</f>
+        <v>Away</v>
+      </c>
+      <c r="I7" s="8">
+        <v>56.3</v>
+      </c>
+      <c r="J7" s="8">
+        <v>58.5</v>
       </c>
       <c r="K7" s="6">
-        <f t="shared" si="2"/>
-        <v>3.4000000000000057</v>
+        <f>I7-J7</f>
+        <v>-2.2000000000000028</v>
       </c>
       <c r="L7" s="6" t="str">
-        <f t="shared" si="3"/>
-        <v>Over</v>
+        <f>IF(K7=0,"Push",IF(K7&gt;0,"Over","Under"))</f>
+        <v>Under</v>
       </c>
       <c r="M7" s="6" t="str">
         <f>IF(ABS(G7)&gt;=Settings!$B$5,H7,"Pass")</f>
-        <v>Home</v>
+        <v>Away</v>
       </c>
       <c r="N7" s="6" t="str">
         <f>IF(ABS(K7)&gt;=Settings!$B$6,L7,"Pass")</f>
-        <v>Over</v>
+        <v>Under</v>
       </c>
       <c r="R7" s="6" t="s">
         <v>73</v>
@@ -1346,45 +1355,45 @@
         <v>1</v>
       </c>
       <c r="B8" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="C8" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="D8" t="s">
-        <v>74</v>
+        <v>63</v>
       </c>
       <c r="E8">
-        <v>-2.9</v>
+        <v>-51.8</v>
       </c>
       <c r="F8">
-        <v>-4</v>
+        <v>-39.5</v>
       </c>
       <c r="G8" s="6">
-        <f t="shared" si="0"/>
-        <v>-1.1000000000000001</v>
+        <f>F8-E8</f>
+        <v>12.299999999999997</v>
       </c>
       <c r="H8" s="6" t="str">
-        <f t="shared" si="1"/>
-        <v>Away</v>
+        <f>IF(G8=0,"Pick'em",IF(G8&gt;0,"Home","Away"))</f>
+        <v>Home</v>
       </c>
       <c r="I8">
-        <v>55.5</v>
+        <v>60.8</v>
       </c>
       <c r="J8">
-        <v>48.8</v>
+        <v>57.5</v>
       </c>
       <c r="K8" s="6">
-        <f t="shared" si="2"/>
-        <v>6.7000000000000028</v>
+        <f>I8-J8</f>
+        <v>3.2999999999999972</v>
       </c>
       <c r="L8" s="6" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(K8=0,"Push",IF(K8&gt;0,"Over","Under"))</f>
         <v>Over</v>
       </c>
       <c r="M8" s="6" t="str">
         <f>IF(ABS(G8)&gt;=Settings!$B$5,H8,"Pass")</f>
-        <v>Pass</v>
+        <v>Home</v>
       </c>
       <c r="N8" s="6" t="str">
         <f>IF(ABS(K8)&gt;=Settings!$B$6,L8,"Pass")</f>
@@ -1399,45 +1408,45 @@
         <v>1</v>
       </c>
       <c r="B9" t="s">
-        <v>76</v>
+        <v>59</v>
       </c>
       <c r="C9" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="D9" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E9">
-        <v>6.1</v>
+        <v>-33</v>
       </c>
       <c r="F9">
-        <v>2.8</v>
+        <v>-31.8</v>
       </c>
       <c r="G9" s="6">
-        <f t="shared" si="0"/>
-        <v>-3.3</v>
+        <f>F9-E9</f>
+        <v>1.1999999999999993</v>
       </c>
       <c r="H9" s="6" t="str">
-        <f t="shared" si="1"/>
-        <v>Away</v>
+        <f>IF(G9=0,"Pick'em",IF(G9&gt;0,"Home","Away"))</f>
+        <v>Home</v>
       </c>
       <c r="I9">
-        <v>59.2</v>
+        <v>46.8</v>
       </c>
       <c r="J9">
-        <v>58.5</v>
+        <v>45.5</v>
       </c>
       <c r="K9" s="6">
-        <f t="shared" si="2"/>
-        <v>0.70000000000000284</v>
+        <f>I9-J9</f>
+        <v>1.2999999999999972</v>
       </c>
       <c r="L9" s="6" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(K9=0,"Push",IF(K9&gt;0,"Over","Under"))</f>
         <v>Over</v>
       </c>
       <c r="M9" s="6" t="str">
         <f>IF(ABS(G9)&gt;=Settings!$B$5,H9,"Pass")</f>
-        <v>Away</v>
+        <v>Pass</v>
       </c>
       <c r="N9" s="6" t="str">
         <f>IF(ABS(K9)&gt;=Settings!$B$6,L9,"Pass")</f>
@@ -1452,40 +1461,40 @@
         <v>1</v>
       </c>
       <c r="B10" t="s">
-        <v>78</v>
+        <v>59</v>
       </c>
       <c r="C10" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
       <c r="D10" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="E10">
-        <v>-11.9</v>
+        <v>-6.4</v>
       </c>
       <c r="F10">
-        <v>-4.5</v>
+        <v>-3.5</v>
       </c>
       <c r="G10" s="6">
-        <f t="shared" si="0"/>
-        <v>7.4</v>
+        <f>F10-E10</f>
+        <v>2.9000000000000004</v>
       </c>
       <c r="H10" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(G10=0,"Pick'em",IF(G10&gt;0,"Home","Away"))</f>
         <v>Home</v>
       </c>
       <c r="I10">
-        <v>62.9</v>
+        <v>51.2</v>
       </c>
       <c r="J10">
-        <v>56.5</v>
+        <v>47.8</v>
       </c>
       <c r="K10" s="6">
-        <f t="shared" si="2"/>
-        <v>6.3999999999999986</v>
+        <f>I10-J10</f>
+        <v>3.4000000000000057</v>
       </c>
       <c r="L10" s="6" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(K10=0,"Push",IF(K10&gt;0,"Over","Under"))</f>
         <v>Over</v>
       </c>
       <c r="M10" s="6" t="str">
@@ -1505,45 +1514,45 @@
         <v>1</v>
       </c>
       <c r="B11" t="s">
-        <v>76</v>
+        <v>59</v>
       </c>
       <c r="C11" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="D11" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="E11">
-        <v>-17.8</v>
+        <v>-37.799999999999997</v>
       </c>
       <c r="F11">
-        <v>-11.5</v>
+        <v>-41</v>
       </c>
       <c r="G11" s="6">
-        <f t="shared" si="0"/>
-        <v>6.3000000000000007</v>
+        <f>F11-E11</f>
+        <v>-3.2000000000000028</v>
       </c>
       <c r="H11" s="6" t="str">
-        <f t="shared" si="1"/>
-        <v>Home</v>
+        <f>IF(G11=0,"Pick'em",IF(G11&gt;0,"Home","Away"))</f>
+        <v>Away</v>
       </c>
       <c r="I11">
-        <v>55.1</v>
+        <v>58.2</v>
       </c>
       <c r="J11">
-        <v>47.5</v>
+        <v>50.5</v>
       </c>
       <c r="K11" s="6">
-        <f t="shared" si="2"/>
-        <v>7.6000000000000014</v>
+        <f>I11-J11</f>
+        <v>7.7000000000000028</v>
       </c>
       <c r="L11" s="6" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(K11=0,"Push",IF(K11&gt;0,"Over","Under"))</f>
         <v>Over</v>
       </c>
       <c r="M11" s="6" t="str">
         <f>IF(ABS(G11)&gt;=Settings!$B$5,H11,"Pass")</f>
-        <v>Home</v>
+        <v>Away</v>
       </c>
       <c r="N11" s="6" t="str">
         <f>IF(ABS(K11)&gt;=Settings!$B$6,L11,"Pass")</f>
@@ -1561,42 +1570,42 @@
         <v>76</v>
       </c>
       <c r="C12" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="D12" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="E12">
-        <v>4.0999999999999996</v>
+        <v>6.1</v>
       </c>
       <c r="F12">
-        <v>2.5</v>
+        <v>2.8</v>
       </c>
       <c r="G12" s="6">
-        <f t="shared" si="0"/>
-        <v>-1.5999999999999996</v>
+        <f>F12-E12</f>
+        <v>-3.3</v>
       </c>
       <c r="H12" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(G12=0,"Pick'em",IF(G12&gt;0,"Home","Away"))</f>
         <v>Away</v>
       </c>
       <c r="I12">
-        <v>55.1</v>
+        <v>59.2</v>
       </c>
       <c r="J12">
-        <v>53.2</v>
+        <v>58.5</v>
       </c>
       <c r="K12" s="6">
-        <f t="shared" si="2"/>
-        <v>1.8999999999999986</v>
+        <f>I12-J12</f>
+        <v>0.70000000000000284</v>
       </c>
       <c r="L12" s="6" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(K12=0,"Push",IF(K12&gt;0,"Over","Under"))</f>
         <v>Over</v>
       </c>
       <c r="M12" s="6" t="str">
         <f>IF(ABS(G12)&gt;=Settings!$B$5,H12,"Pass")</f>
-        <v>Pass</v>
+        <v>Away</v>
       </c>
       <c r="N12" s="6" t="str">
         <f>IF(ABS(K12)&gt;=Settings!$B$6,L12,"Pass")</f>
@@ -1611,40 +1620,40 @@
         <v>1</v>
       </c>
       <c r="B13" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="C13" t="s">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="D13" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="E13">
-        <v>-11.2</v>
+        <v>-17.8</v>
       </c>
       <c r="F13">
-        <v>-5</v>
+        <v>-11.5</v>
       </c>
       <c r="G13" s="6">
-        <f t="shared" si="0"/>
-        <v>6.1999999999999993</v>
+        <f>F13-E13</f>
+        <v>6.3000000000000007</v>
       </c>
       <c r="H13" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(G13=0,"Pick'em",IF(G13&gt;0,"Home","Away"))</f>
         <v>Home</v>
       </c>
       <c r="I13">
-        <v>55.2</v>
+        <v>55.1</v>
       </c>
       <c r="J13">
-        <v>53.5</v>
+        <v>47.5</v>
       </c>
       <c r="K13" s="6">
-        <f t="shared" si="2"/>
-        <v>1.7000000000000028</v>
+        <f>I13-J13</f>
+        <v>7.6000000000000014</v>
       </c>
       <c r="L13" s="6" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(K13=0,"Push",IF(K13&gt;0,"Over","Under"))</f>
         <v>Over</v>
       </c>
       <c r="M13" s="6" t="str">
@@ -1653,7 +1662,7 @@
       </c>
       <c r="N13" s="6" t="str">
         <f>IF(ABS(K13)&gt;=Settings!$B$6,L13,"Pass")</f>
-        <v>Pass</v>
+        <v>Over</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.25">
@@ -1661,66 +1670,66 @@
         <v>1</v>
       </c>
       <c r="B14" t="s">
-        <v>59</v>
+        <v>76</v>
       </c>
       <c r="C14" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="D14" t="s">
-        <v>85</v>
+        <v>73</v>
       </c>
       <c r="E14">
-        <v>-37.799999999999997</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="F14">
-        <v>-41</v>
+        <v>2.5</v>
       </c>
       <c r="G14" s="6">
-        <f t="shared" si="0"/>
-        <v>-3.2000000000000028</v>
+        <f>F14-E14</f>
+        <v>-1.5999999999999996</v>
       </c>
       <c r="H14" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f>IF(G14=0,"Pick'em",IF(G14&gt;0,"Home","Away"))</f>
         <v>Away</v>
       </c>
       <c r="I14">
-        <v>58.2</v>
+        <v>55.1</v>
       </c>
       <c r="J14">
-        <v>50.5</v>
+        <v>53.2</v>
       </c>
       <c r="K14" s="6">
-        <f t="shared" si="2"/>
-        <v>7.7000000000000028</v>
+        <f>I14-J14</f>
+        <v>1.8999999999999986</v>
       </c>
       <c r="L14" s="6" t="str">
-        <f t="shared" si="3"/>
+        <f>IF(K14=0,"Push",IF(K14&gt;0,"Over","Under"))</f>
         <v>Over</v>
       </c>
       <c r="M14" s="6" t="str">
         <f>IF(ABS(G14)&gt;=Settings!$B$5,H14,"Pass")</f>
-        <v>Away</v>
+        <v>Pass</v>
       </c>
       <c r="N14" s="6" t="str">
         <f>IF(ABS(K14)&gt;=Settings!$B$6,L14,"Pass")</f>
-        <v>Over</v>
+        <v>Pass</v>
       </c>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="G15" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="G2:G29" si="0">F15-E15</f>
         <v>0</v>
       </c>
       <c r="H15" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="H2:H29" si="1">IF(G15=0,"Pick'em",IF(G15&gt;0,"Home","Away"))</f>
         <v>Pick'em</v>
       </c>
       <c r="K15" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="K2:K29" si="2">I15-J15</f>
         <v>0</v>
       </c>
       <c r="L15" s="6" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" ref="L2:L29" si="3">IF(K15=0,"Push",IF(K15&gt;0,"Over","Under"))</f>
         <v>Push</v>
       </c>
       <c r="M15" s="6" t="str">
@@ -2097,6 +2106,9 @@
       </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:N14">
+    <sortCondition ref="B2:B14"/>
+  </sortState>
   <conditionalFormatting sqref="C2:D29">
     <cfRule type="expression" dxfId="0" priority="2">
       <formula>COUNTIF($R$5:$R$12,C2)&gt;0</formula>
@@ -2114,7 +2126,7 @@
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
     <col min="2" max="2" width="6" customWidth="1"/>
-    <col min="3" max="3" width="26" customWidth="1"/>
+    <col min="3" max="3" width="37.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10" customWidth="1"/>
     <col min="5" max="5" width="18" customWidth="1"/>
     <col min="6" max="6" width="11" customWidth="1"/>
@@ -2168,6 +2180,30 @@
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D2" t="s">
+        <v>109</v>
+      </c>
+      <c r="E2" t="s">
+        <v>111</v>
+      </c>
+      <c r="F2">
+        <v>-7</v>
+      </c>
+      <c r="G2">
+        <v>-110</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
+      </c>
       <c r="J2" s="6" t="str">
         <f t="shared" ref="J2:J41" si="0">IF(I2="","",I2-F2)</f>
         <v/>

</xml_diff>

<commit_message>
Add Live Lines page and Pending Bets section
</commit_message>
<xml_diff>
--- a/excel/MW_Handicapping_Tracker.xlsx
+++ b/excel/MW_Handicapping_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\deene\Mountain Dub Handicapping\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{844C6AA8-16BC-4493-9EEE-F31799BE265D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80FC07B6-3E90-416D-9A66-52103EA66F40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Read Me" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="165" uniqueCount="114">
   <si>
     <t>Date</t>
   </si>
@@ -373,13 +373,19 @@
   </si>
   <si>
     <t>North Dakota State -7</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>Over 46.5</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -429,6 +435,12 @@
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -1059,11 +1071,11 @@
         <v>-38.200000000000003</v>
       </c>
       <c r="G2" s="6">
-        <f>F2-E2</f>
+        <f t="shared" ref="G2:G14" si="0">F2-E2</f>
         <v>0.39999999999999858</v>
       </c>
       <c r="H2" s="6" t="str">
-        <f>IF(G2=0,"Pick'em",IF(G2&gt;0,"Home","Away"))</f>
+        <f t="shared" ref="H2:H14" si="1">IF(G2=0,"Pick'em",IF(G2&gt;0,"Home","Away"))</f>
         <v>Home</v>
       </c>
       <c r="I2">
@@ -1073,11 +1085,11 @@
         <v>60.5</v>
       </c>
       <c r="K2" s="6">
-        <f>I2-J2</f>
+        <f t="shared" ref="K2:K14" si="2">I2-J2</f>
         <v>-2.2000000000000028</v>
       </c>
       <c r="L2" s="6" t="str">
-        <f>IF(K2=0,"Push",IF(K2&gt;0,"Over","Under"))</f>
+        <f t="shared" ref="L2:L14" si="3">IF(K2=0,"Push",IF(K2&gt;0,"Over","Under"))</f>
         <v>Under</v>
       </c>
       <c r="M2" s="6" t="str">
@@ -1111,11 +1123,11 @@
         <v>-7</v>
       </c>
       <c r="G3" s="6">
-        <f>F3-E3</f>
+        <f t="shared" si="0"/>
         <v>14.2</v>
       </c>
       <c r="H3" s="6" t="str">
-        <f>IF(G3=0,"Pick'em",IF(G3&gt;0,"Home","Away"))</f>
+        <f t="shared" si="1"/>
         <v>Home</v>
       </c>
       <c r="I3">
@@ -1125,11 +1137,11 @@
         <v>46.2</v>
       </c>
       <c r="K3" s="6">
-        <f>I3-J3</f>
+        <f t="shared" si="2"/>
         <v>7</v>
       </c>
       <c r="L3" s="6" t="str">
-        <f>IF(K3=0,"Push",IF(K3&gt;0,"Over","Under"))</f>
+        <f t="shared" si="3"/>
         <v>Over</v>
       </c>
       <c r="M3" s="6" t="str">
@@ -1161,11 +1173,11 @@
         <v>-4</v>
       </c>
       <c r="G4" s="6">
-        <f>F4-E4</f>
+        <f t="shared" si="0"/>
         <v>-1.1000000000000001</v>
       </c>
       <c r="H4" s="6" t="str">
-        <f>IF(G4=0,"Pick'em",IF(G4&gt;0,"Home","Away"))</f>
+        <f t="shared" si="1"/>
         <v>Away</v>
       </c>
       <c r="I4">
@@ -1175,11 +1187,11 @@
         <v>48.8</v>
       </c>
       <c r="K4" s="6">
-        <f>I4-J4</f>
+        <f t="shared" si="2"/>
         <v>6.7000000000000028</v>
       </c>
       <c r="L4" s="6" t="str">
-        <f>IF(K4=0,"Push",IF(K4&gt;0,"Over","Under"))</f>
+        <f t="shared" si="3"/>
         <v>Over</v>
       </c>
       <c r="M4" s="6" t="str">
@@ -1211,11 +1223,11 @@
         <v>-4.5</v>
       </c>
       <c r="G5" s="6">
-        <f>F5-E5</f>
+        <f t="shared" si="0"/>
         <v>7.4</v>
       </c>
       <c r="H5" s="6" t="str">
-        <f>IF(G5=0,"Pick'em",IF(G5&gt;0,"Home","Away"))</f>
+        <f t="shared" si="1"/>
         <v>Home</v>
       </c>
       <c r="I5">
@@ -1225,11 +1237,11 @@
         <v>56.5</v>
       </c>
       <c r="K5" s="6">
-        <f>I5-J5</f>
+        <f t="shared" si="2"/>
         <v>6.3999999999999986</v>
       </c>
       <c r="L5" s="6" t="str">
-        <f>IF(K5=0,"Push",IF(K5&gt;0,"Over","Under"))</f>
+        <f t="shared" si="3"/>
         <v>Over</v>
       </c>
       <c r="M5" s="6" t="str">
@@ -1264,11 +1276,11 @@
         <v>-5</v>
       </c>
       <c r="G6" s="6">
-        <f>F6-E6</f>
+        <f t="shared" si="0"/>
         <v>6.1999999999999993</v>
       </c>
       <c r="H6" s="6" t="str">
-        <f>IF(G6=0,"Pick'em",IF(G6&gt;0,"Home","Away"))</f>
+        <f t="shared" si="1"/>
         <v>Home</v>
       </c>
       <c r="I6">
@@ -1278,11 +1290,11 @@
         <v>53.5</v>
       </c>
       <c r="K6" s="6">
-        <f>I6-J6</f>
+        <f t="shared" si="2"/>
         <v>1.7000000000000028</v>
       </c>
       <c r="L6" s="6" t="str">
-        <f>IF(K6=0,"Push",IF(K6&gt;0,"Over","Under"))</f>
+        <f t="shared" si="3"/>
         <v>Over</v>
       </c>
       <c r="M6" s="6" t="str">
@@ -1317,11 +1329,11 @@
         <v>-30.5</v>
       </c>
       <c r="G7" s="6">
-        <f>F7-E7</f>
+        <f t="shared" si="0"/>
         <v>-12.399999999999999</v>
       </c>
       <c r="H7" s="6" t="str">
-        <f>IF(G7=0,"Pick'em",IF(G7&gt;0,"Home","Away"))</f>
+        <f t="shared" si="1"/>
         <v>Away</v>
       </c>
       <c r="I7" s="8">
@@ -1331,11 +1343,11 @@
         <v>58.5</v>
       </c>
       <c r="K7" s="6">
-        <f>I7-J7</f>
+        <f t="shared" si="2"/>
         <v>-2.2000000000000028</v>
       </c>
       <c r="L7" s="6" t="str">
-        <f>IF(K7=0,"Push",IF(K7&gt;0,"Over","Under"))</f>
+        <f t="shared" si="3"/>
         <v>Under</v>
       </c>
       <c r="M7" s="6" t="str">
@@ -1370,11 +1382,11 @@
         <v>-39.5</v>
       </c>
       <c r="G8" s="6">
-        <f>F8-E8</f>
+        <f t="shared" si="0"/>
         <v>12.299999999999997</v>
       </c>
       <c r="H8" s="6" t="str">
-        <f>IF(G8=0,"Pick'em",IF(G8&gt;0,"Home","Away"))</f>
+        <f t="shared" si="1"/>
         <v>Home</v>
       </c>
       <c r="I8">
@@ -1384,11 +1396,11 @@
         <v>57.5</v>
       </c>
       <c r="K8" s="6">
-        <f>I8-J8</f>
+        <f t="shared" si="2"/>
         <v>3.2999999999999972</v>
       </c>
       <c r="L8" s="6" t="str">
-        <f>IF(K8=0,"Push",IF(K8&gt;0,"Over","Under"))</f>
+        <f t="shared" si="3"/>
         <v>Over</v>
       </c>
       <c r="M8" s="6" t="str">
@@ -1423,11 +1435,11 @@
         <v>-31.8</v>
       </c>
       <c r="G9" s="6">
-        <f>F9-E9</f>
+        <f t="shared" si="0"/>
         <v>1.1999999999999993</v>
       </c>
       <c r="H9" s="6" t="str">
-        <f>IF(G9=0,"Pick'em",IF(G9&gt;0,"Home","Away"))</f>
+        <f t="shared" si="1"/>
         <v>Home</v>
       </c>
       <c r="I9">
@@ -1437,11 +1449,11 @@
         <v>45.5</v>
       </c>
       <c r="K9" s="6">
-        <f>I9-J9</f>
+        <f t="shared" si="2"/>
         <v>1.2999999999999972</v>
       </c>
       <c r="L9" s="6" t="str">
-        <f>IF(K9=0,"Push",IF(K9&gt;0,"Over","Under"))</f>
+        <f t="shared" si="3"/>
         <v>Over</v>
       </c>
       <c r="M9" s="6" t="str">
@@ -1476,11 +1488,11 @@
         <v>-3.5</v>
       </c>
       <c r="G10" s="6">
-        <f>F10-E10</f>
+        <f t="shared" si="0"/>
         <v>2.9000000000000004</v>
       </c>
       <c r="H10" s="6" t="str">
-        <f>IF(G10=0,"Pick'em",IF(G10&gt;0,"Home","Away"))</f>
+        <f t="shared" si="1"/>
         <v>Home</v>
       </c>
       <c r="I10">
@@ -1490,11 +1502,11 @@
         <v>47.8</v>
       </c>
       <c r="K10" s="6">
-        <f>I10-J10</f>
+        <f t="shared" si="2"/>
         <v>3.4000000000000057</v>
       </c>
       <c r="L10" s="6" t="str">
-        <f>IF(K10=0,"Push",IF(K10&gt;0,"Over","Under"))</f>
+        <f t="shared" si="3"/>
         <v>Over</v>
       </c>
       <c r="M10" s="6" t="str">
@@ -1529,11 +1541,11 @@
         <v>-41</v>
       </c>
       <c r="G11" s="6">
-        <f>F11-E11</f>
+        <f t="shared" si="0"/>
         <v>-3.2000000000000028</v>
       </c>
       <c r="H11" s="6" t="str">
-        <f>IF(G11=0,"Pick'em",IF(G11&gt;0,"Home","Away"))</f>
+        <f t="shared" si="1"/>
         <v>Away</v>
       </c>
       <c r="I11">
@@ -1543,11 +1555,11 @@
         <v>50.5</v>
       </c>
       <c r="K11" s="6">
-        <f>I11-J11</f>
+        <f t="shared" si="2"/>
         <v>7.7000000000000028</v>
       </c>
       <c r="L11" s="6" t="str">
-        <f>IF(K11=0,"Push",IF(K11&gt;0,"Over","Under"))</f>
+        <f t="shared" si="3"/>
         <v>Over</v>
       </c>
       <c r="M11" s="6" t="str">
@@ -1582,11 +1594,11 @@
         <v>2.8</v>
       </c>
       <c r="G12" s="6">
-        <f>F12-E12</f>
+        <f t="shared" si="0"/>
         <v>-3.3</v>
       </c>
       <c r="H12" s="6" t="str">
-        <f>IF(G12=0,"Pick'em",IF(G12&gt;0,"Home","Away"))</f>
+        <f t="shared" si="1"/>
         <v>Away</v>
       </c>
       <c r="I12">
@@ -1596,11 +1608,11 @@
         <v>58.5</v>
       </c>
       <c r="K12" s="6">
-        <f>I12-J12</f>
+        <f t="shared" si="2"/>
         <v>0.70000000000000284</v>
       </c>
       <c r="L12" s="6" t="str">
-        <f>IF(K12=0,"Push",IF(K12&gt;0,"Over","Under"))</f>
+        <f t="shared" si="3"/>
         <v>Over</v>
       </c>
       <c r="M12" s="6" t="str">
@@ -1635,11 +1647,11 @@
         <v>-11.5</v>
       </c>
       <c r="G13" s="6">
-        <f>F13-E13</f>
+        <f t="shared" si="0"/>
         <v>6.3000000000000007</v>
       </c>
       <c r="H13" s="6" t="str">
-        <f>IF(G13=0,"Pick'em",IF(G13&gt;0,"Home","Away"))</f>
+        <f t="shared" si="1"/>
         <v>Home</v>
       </c>
       <c r="I13">
@@ -1649,11 +1661,11 @@
         <v>47.5</v>
       </c>
       <c r="K13" s="6">
-        <f>I13-J13</f>
+        <f t="shared" si="2"/>
         <v>7.6000000000000014</v>
       </c>
       <c r="L13" s="6" t="str">
-        <f>IF(K13=0,"Push",IF(K13&gt;0,"Over","Under"))</f>
+        <f t="shared" si="3"/>
         <v>Over</v>
       </c>
       <c r="M13" s="6" t="str">
@@ -1685,11 +1697,11 @@
         <v>2.5</v>
       </c>
       <c r="G14" s="6">
-        <f>F14-E14</f>
+        <f t="shared" si="0"/>
         <v>-1.5999999999999996</v>
       </c>
       <c r="H14" s="6" t="str">
-        <f>IF(G14=0,"Pick'em",IF(G14&gt;0,"Home","Away"))</f>
+        <f t="shared" si="1"/>
         <v>Away</v>
       </c>
       <c r="I14">
@@ -1699,11 +1711,11 @@
         <v>53.2</v>
       </c>
       <c r="K14" s="6">
-        <f>I14-J14</f>
+        <f t="shared" si="2"/>
         <v>1.8999999999999986</v>
       </c>
       <c r="L14" s="6" t="str">
-        <f>IF(K14=0,"Push",IF(K14&gt;0,"Over","Under"))</f>
+        <f t="shared" si="3"/>
         <v>Over</v>
       </c>
       <c r="M14" s="6" t="str">
@@ -1717,19 +1729,19 @@
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="G15" s="6">
-        <f t="shared" ref="G2:G29" si="0">F15-E15</f>
+        <f t="shared" ref="G15:G29" si="4">F15-E15</f>
         <v>0</v>
       </c>
       <c r="H15" s="6" t="str">
-        <f t="shared" ref="H2:H29" si="1">IF(G15=0,"Pick'em",IF(G15&gt;0,"Home","Away"))</f>
+        <f t="shared" ref="H15:H29" si="5">IF(G15=0,"Pick'em",IF(G15&gt;0,"Home","Away"))</f>
         <v>Pick'em</v>
       </c>
       <c r="K15" s="6">
-        <f t="shared" ref="K2:K29" si="2">I15-J15</f>
+        <f t="shared" ref="K15:K29" si="6">I15-J15</f>
         <v>0</v>
       </c>
       <c r="L15" s="6" t="str">
-        <f t="shared" ref="L2:L29" si="3">IF(K15=0,"Push",IF(K15&gt;0,"Over","Under"))</f>
+        <f t="shared" ref="L15:L29" si="7">IF(K15=0,"Push",IF(K15&gt;0,"Over","Under"))</f>
         <v>Push</v>
       </c>
       <c r="M15" s="6" t="str">
@@ -1743,19 +1755,19 @@
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="G16" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="H16" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>Pick'em</v>
       </c>
       <c r="K16" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="L16" s="6" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>Push</v>
       </c>
       <c r="M16" s="6" t="str">
@@ -1769,19 +1781,19 @@
     </row>
     <row r="17" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G17" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="H17" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>Pick'em</v>
       </c>
       <c r="K17" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="L17" s="6" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>Push</v>
       </c>
       <c r="M17" s="6" t="str">
@@ -1795,19 +1807,19 @@
     </row>
     <row r="18" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G18" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="H18" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>Pick'em</v>
       </c>
       <c r="K18" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="L18" s="6" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>Push</v>
       </c>
       <c r="M18" s="6" t="str">
@@ -1821,19 +1833,19 @@
     </row>
     <row r="19" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G19" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="H19" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>Pick'em</v>
       </c>
       <c r="K19" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="L19" s="6" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>Push</v>
       </c>
       <c r="M19" s="6" t="str">
@@ -1847,19 +1859,19 @@
     </row>
     <row r="20" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G20" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="H20" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>Pick'em</v>
       </c>
       <c r="K20" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="L20" s="6" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>Push</v>
       </c>
       <c r="M20" s="6" t="str">
@@ -1873,19 +1885,19 @@
     </row>
     <row r="21" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G21" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="H21" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>Pick'em</v>
       </c>
       <c r="K21" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="L21" s="6" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>Push</v>
       </c>
       <c r="M21" s="6" t="str">
@@ -1899,19 +1911,19 @@
     </row>
     <row r="22" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G22" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="H22" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>Pick'em</v>
       </c>
       <c r="K22" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="L22" s="6" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>Push</v>
       </c>
       <c r="M22" s="6" t="str">
@@ -1925,19 +1937,19 @@
     </row>
     <row r="23" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G23" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="H23" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>Pick'em</v>
       </c>
       <c r="K23" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="L23" s="6" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>Push</v>
       </c>
       <c r="M23" s="6" t="str">
@@ -1951,19 +1963,19 @@
     </row>
     <row r="24" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G24" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="H24" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>Pick'em</v>
       </c>
       <c r="K24" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="L24" s="6" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>Push</v>
       </c>
       <c r="M24" s="6" t="str">
@@ -1977,19 +1989,19 @@
     </row>
     <row r="25" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G25" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="H25" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>Pick'em</v>
       </c>
       <c r="K25" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="L25" s="6" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>Push</v>
       </c>
       <c r="M25" s="6" t="str">
@@ -2003,19 +2015,19 @@
     </row>
     <row r="26" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G26" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="H26" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>Pick'em</v>
       </c>
       <c r="K26" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="L26" s="6" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>Push</v>
       </c>
       <c r="M26" s="6" t="str">
@@ -2029,19 +2041,19 @@
     </row>
     <row r="27" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G27" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="H27" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>Pick'em</v>
       </c>
       <c r="K27" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="L27" s="6" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>Push</v>
       </c>
       <c r="M27" s="6" t="str">
@@ -2055,19 +2067,19 @@
     </row>
     <row r="28" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G28" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="H28" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>Pick'em</v>
       </c>
       <c r="K28" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="L28" s="6" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>Push</v>
       </c>
       <c r="M28" s="6" t="str">
@@ -2081,19 +2093,19 @@
     </row>
     <row r="29" spans="7:14" x14ac:dyDescent="0.25">
       <c r="G29" s="6">
-        <f t="shared" si="0"/>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="H29" s="6" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="5"/>
         <v>Pick'em</v>
       </c>
       <c r="K29" s="6">
-        <f t="shared" si="2"/>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="L29" s="6" t="str">
-        <f t="shared" si="3"/>
+        <f t="shared" si="7"/>
         <v>Push</v>
       </c>
       <c r="M29" s="6" t="str">
@@ -2181,7 +2193,7 @@
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="B2">
         <v>1</v>
@@ -2218,6 +2230,30 @@
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>110</v>
+      </c>
+      <c r="D3" t="s">
+        <v>112</v>
+      </c>
+      <c r="E3" t="s">
+        <v>113</v>
+      </c>
+      <c r="F3">
+        <v>46.5</v>
+      </c>
+      <c r="G3">
+        <v>-110</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
+      </c>
       <c r="J3" s="6" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -2769,6 +2805,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="8" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>

</xml_diff>

<commit_message>
Add MW home-field spread fix, in-season PPA totals candidate, spread bias diagnostics
</commit_message>
<xml_diff>
--- a/excel/MW_Handicapping_Tracker.xlsx
+++ b/excel/MW_Handicapping_Tracker.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="0" activeTab="3" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Read Me" sheetId="1" state="visible" r:id="rId1"/>
@@ -73,9 +73,9 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <charset val="1"/>
       <family val="2"/>
-      <sz val="8"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -134,7 +134,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -149,16 +149,33 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="3">
     <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
-          <bgColor rgb="FFFFFF00"/>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF00B050"/>
         </patternFill>
       </fill>
     </dxf>
@@ -804,7 +821,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>-38.6</v>
+        <v>-37</v>
       </c>
       <c r="F2" t="n">
         <v>-38.2</v>
@@ -818,7 +835,7 @@
         <v/>
       </c>
       <c r="I2" t="n">
-        <v>58.3</v>
+        <v>55.1</v>
       </c>
       <c r="J2" t="n">
         <v>60.5</v>
@@ -862,7 +879,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>-21.2</v>
+        <v>-19.9</v>
       </c>
       <c r="F3" t="n">
         <v>-7</v>
@@ -876,7 +893,7 @@
         <v/>
       </c>
       <c r="I3" t="n">
-        <v>53.2</v>
+        <v>54.9</v>
       </c>
       <c r="J3" t="n">
         <v>46.2</v>
@@ -918,7 +935,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>-2.9</v>
+        <v>-2.6</v>
       </c>
       <c r="F4" t="n">
         <v>-4</v>
@@ -932,7 +949,7 @@
         <v/>
       </c>
       <c r="I4" t="n">
-        <v>55.5</v>
+        <v>53.3</v>
       </c>
       <c r="J4" t="n">
         <v>48.8</v>
@@ -974,7 +991,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>-11.9</v>
+        <v>-11.2</v>
       </c>
       <c r="F5" t="n">
         <v>-4.5</v>
@@ -988,7 +1005,7 @@
         <v/>
       </c>
       <c r="I5" t="n">
-        <v>62.9</v>
+        <v>57.7</v>
       </c>
       <c r="J5" t="n">
         <v>56.5</v>
@@ -1035,7 +1052,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>-11.2</v>
+        <v>-10.2</v>
       </c>
       <c r="F6" t="n">
         <v>-5</v>
@@ -1049,7 +1066,7 @@
         <v/>
       </c>
       <c r="I6" t="n">
-        <v>55.2</v>
+        <v>56</v>
       </c>
       <c r="J6" t="n">
         <v>53.5</v>
@@ -1077,57 +1094,57 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="n">
+      <c r="A7" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="10" t="inlineStr">
         <is>
           <t>2026-09-05</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C7" s="10" t="inlineStr">
         <is>
           <t>Duquesne</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D7" s="10" t="inlineStr">
         <is>
           <t>Air Force</t>
         </is>
       </c>
-      <c r="E7" s="8" t="n">
-        <v>-18.1</v>
-      </c>
-      <c r="F7" s="8" t="n">
+      <c r="E7" s="10" t="n">
+        <v>-16.8</v>
+      </c>
+      <c r="F7" s="10" t="n">
         <v>-30.5</v>
       </c>
-      <c r="G7" s="6">
+      <c r="G7" s="10">
         <f>F7-E7</f>
         <v/>
       </c>
-      <c r="H7" s="6">
+      <c r="H7" s="10">
         <f>IF(G7=0,"Pick'em",IF(G7&gt;0,"Home","Away"))</f>
         <v/>
       </c>
-      <c r="I7" s="8" t="n">
-        <v>56.3</v>
-      </c>
-      <c r="J7" s="8" t="n">
+      <c r="I7" s="10" t="n">
+        <v>55.2</v>
+      </c>
+      <c r="J7" s="10" t="n">
         <v>58.5</v>
       </c>
-      <c r="K7" s="6">
+      <c r="K7" s="10">
         <f>I7-J7</f>
         <v/>
       </c>
-      <c r="L7" s="6">
+      <c r="L7" s="10">
         <f>IF(K7=0,"Push",IF(K7&gt;0,"Over","Under"))</f>
         <v/>
       </c>
-      <c r="M7" s="6">
+      <c r="M7" s="10">
         <f>IF(ABS(G7)&gt;=Settings!$B$5,H7,"Pass")</f>
         <v/>
       </c>
-      <c r="N7" s="6">
+      <c r="N7" s="10">
         <f>IF(ABS(K7)&gt;=Settings!$B$6,L7,"Pass")</f>
         <v/>
       </c>
@@ -1157,7 +1174,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>-51.8</v>
+        <v>-50.5</v>
       </c>
       <c r="F8" t="n">
         <v>-39.5</v>
@@ -1171,7 +1188,7 @@
         <v/>
       </c>
       <c r="I8" t="n">
-        <v>60.8</v>
+        <v>57.6</v>
       </c>
       <c r="J8" t="n">
         <v>57.5</v>
@@ -1218,7 +1235,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>-33</v>
+        <v>-30.8</v>
       </c>
       <c r="F9" t="n">
         <v>-31.8</v>
@@ -1232,7 +1249,7 @@
         <v/>
       </c>
       <c r="I9" t="n">
-        <v>46.8</v>
+        <v>49.7</v>
       </c>
       <c r="J9" t="n">
         <v>45.5</v>
@@ -1279,7 +1296,7 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>-6.4</v>
+        <v>-5</v>
       </c>
       <c r="F10" t="n">
         <v>-3.5</v>
@@ -1340,7 +1357,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>-37.8</v>
+        <v>-35.5</v>
       </c>
       <c r="F11" t="n">
         <v>-41</v>
@@ -1354,7 +1371,7 @@
         <v/>
       </c>
       <c r="I11" t="n">
-        <v>58.2</v>
+        <v>53.3</v>
       </c>
       <c r="J11" t="n">
         <v>50.5</v>
@@ -1401,7 +1418,7 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>6.1</v>
+        <v>7.3</v>
       </c>
       <c r="F12" t="n">
         <v>2.8</v>
@@ -1415,7 +1432,7 @@
         <v/>
       </c>
       <c r="I12" t="n">
-        <v>59.2</v>
+        <v>56.7</v>
       </c>
       <c r="J12" t="n">
         <v>58.5</v>
@@ -1462,7 +1479,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>-17.8</v>
+        <v>-15.9</v>
       </c>
       <c r="F13" t="n">
         <v>-11.5</v>
@@ -1476,7 +1493,7 @@
         <v/>
       </c>
       <c r="I13" t="n">
-        <v>55.1</v>
+        <v>51.6</v>
       </c>
       <c r="J13" t="n">
         <v>47.5</v>
@@ -1518,7 +1535,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>4.1</v>
+        <v>5.3</v>
       </c>
       <c r="F14" t="n">
         <v>2.5</v>
@@ -1532,7 +1549,7 @@
         <v/>
       </c>
       <c r="I14" t="n">
-        <v>55.1</v>
+        <v>53</v>
       </c>
       <c r="J14" t="n">
         <v>53.2</v>
@@ -1555,394 +1572,124 @@
       </c>
     </row>
     <row r="15">
-      <c r="G15" s="6">
-        <f>F15-E15</f>
-        <v/>
-      </c>
-      <c r="H15" s="6">
-        <f>IF(G15=0,"Pick'em",IF(G15&gt;0,"Home","Away"))</f>
-        <v/>
-      </c>
-      <c r="K15" s="6">
-        <f>I15-J15</f>
-        <v/>
-      </c>
-      <c r="L15" s="6">
-        <f>IF(K15=0,"Push",IF(K15&gt;0,"Over","Under"))</f>
-        <v/>
-      </c>
-      <c r="M15" s="6">
-        <f>IF(ABS(G15)&gt;=Settings!$B$5,H15,"Pass")</f>
-        <v/>
-      </c>
-      <c r="N15" s="6">
-        <f>IF(ABS(K15)&gt;=Settings!$B$6,L15,"Pass")</f>
-        <v/>
-      </c>
+      <c r="G15" s="6" t="n"/>
+      <c r="H15" s="6" t="n"/>
+      <c r="K15" s="6" t="n"/>
+      <c r="L15" s="6" t="n"/>
+      <c r="M15" s="6" t="n"/>
+      <c r="N15" s="6" t="n"/>
     </row>
     <row r="16">
-      <c r="G16" s="6">
-        <f>F16-E16</f>
-        <v/>
-      </c>
-      <c r="H16" s="6">
-        <f>IF(G16=0,"Pick'em",IF(G16&gt;0,"Home","Away"))</f>
-        <v/>
-      </c>
-      <c r="K16" s="6">
-        <f>I16-J16</f>
-        <v/>
-      </c>
-      <c r="L16" s="6">
-        <f>IF(K16=0,"Push",IF(K16&gt;0,"Over","Under"))</f>
-        <v/>
-      </c>
-      <c r="M16" s="6">
-        <f>IF(ABS(G16)&gt;=Settings!$B$5,H16,"Pass")</f>
-        <v/>
-      </c>
-      <c r="N16" s="6">
-        <f>IF(ABS(K16)&gt;=Settings!$B$6,L16,"Pass")</f>
-        <v/>
-      </c>
+      <c r="G16" s="6" t="n"/>
+      <c r="H16" s="6" t="n"/>
+      <c r="K16" s="6" t="n"/>
+      <c r="L16" s="6" t="n"/>
+      <c r="M16" s="6" t="n"/>
+      <c r="N16" s="6" t="n"/>
     </row>
     <row r="17">
-      <c r="G17" s="6">
-        <f>F17-E17</f>
-        <v/>
-      </c>
-      <c r="H17" s="6">
-        <f>IF(G17=0,"Pick'em",IF(G17&gt;0,"Home","Away"))</f>
-        <v/>
-      </c>
-      <c r="K17" s="6">
-        <f>I17-J17</f>
-        <v/>
-      </c>
-      <c r="L17" s="6">
-        <f>IF(K17=0,"Push",IF(K17&gt;0,"Over","Under"))</f>
-        <v/>
-      </c>
-      <c r="M17" s="6">
-        <f>IF(ABS(G17)&gt;=Settings!$B$5,H17,"Pass")</f>
-        <v/>
-      </c>
-      <c r="N17" s="6">
-        <f>IF(ABS(K17)&gt;=Settings!$B$6,L17,"Pass")</f>
-        <v/>
-      </c>
+      <c r="G17" s="6" t="n"/>
+      <c r="H17" s="6" t="n"/>
+      <c r="K17" s="6" t="n"/>
+      <c r="L17" s="6" t="n"/>
+      <c r="M17" s="6" t="n"/>
+      <c r="N17" s="6" t="n"/>
     </row>
     <row r="18">
-      <c r="G18" s="6">
-        <f>F18-E18</f>
-        <v/>
-      </c>
-      <c r="H18" s="6">
-        <f>IF(G18=0,"Pick'em",IF(G18&gt;0,"Home","Away"))</f>
-        <v/>
-      </c>
-      <c r="K18" s="6">
-        <f>I18-J18</f>
-        <v/>
-      </c>
-      <c r="L18" s="6">
-        <f>IF(K18=0,"Push",IF(K18&gt;0,"Over","Under"))</f>
-        <v/>
-      </c>
-      <c r="M18" s="6">
-        <f>IF(ABS(G18)&gt;=Settings!$B$5,H18,"Pass")</f>
-        <v/>
-      </c>
-      <c r="N18" s="6">
-        <f>IF(ABS(K18)&gt;=Settings!$B$6,L18,"Pass")</f>
-        <v/>
-      </c>
+      <c r="G18" s="6" t="n"/>
+      <c r="H18" s="6" t="n"/>
+      <c r="K18" s="6" t="n"/>
+      <c r="L18" s="6" t="n"/>
+      <c r="M18" s="6" t="n"/>
+      <c r="N18" s="6" t="n"/>
     </row>
     <row r="19">
-      <c r="G19" s="6">
-        <f>F19-E19</f>
-        <v/>
-      </c>
-      <c r="H19" s="6">
-        <f>IF(G19=0,"Pick'em",IF(G19&gt;0,"Home","Away"))</f>
-        <v/>
-      </c>
-      <c r="K19" s="6">
-        <f>I19-J19</f>
-        <v/>
-      </c>
-      <c r="L19" s="6">
-        <f>IF(K19=0,"Push",IF(K19&gt;0,"Over","Under"))</f>
-        <v/>
-      </c>
-      <c r="M19" s="6">
-        <f>IF(ABS(G19)&gt;=Settings!$B$5,H19,"Pass")</f>
-        <v/>
-      </c>
-      <c r="N19" s="6">
-        <f>IF(ABS(K19)&gt;=Settings!$B$6,L19,"Pass")</f>
-        <v/>
-      </c>
+      <c r="G19" s="6" t="n"/>
+      <c r="H19" s="6" t="n"/>
+      <c r="K19" s="6" t="n"/>
+      <c r="L19" s="6" t="n"/>
+      <c r="M19" s="6" t="n"/>
+      <c r="N19" s="6" t="n"/>
     </row>
     <row r="20">
-      <c r="G20" s="6">
-        <f>F20-E20</f>
-        <v/>
-      </c>
-      <c r="H20" s="6">
-        <f>IF(G20=0,"Pick'em",IF(G20&gt;0,"Home","Away"))</f>
-        <v/>
-      </c>
-      <c r="K20" s="6">
-        <f>I20-J20</f>
-        <v/>
-      </c>
-      <c r="L20" s="6">
-        <f>IF(K20=0,"Push",IF(K20&gt;0,"Over","Under"))</f>
-        <v/>
-      </c>
-      <c r="M20" s="6">
-        <f>IF(ABS(G20)&gt;=Settings!$B$5,H20,"Pass")</f>
-        <v/>
-      </c>
-      <c r="N20" s="6">
-        <f>IF(ABS(K20)&gt;=Settings!$B$6,L20,"Pass")</f>
-        <v/>
-      </c>
+      <c r="G20" s="6" t="n"/>
+      <c r="H20" s="6" t="n"/>
+      <c r="K20" s="6" t="n"/>
+      <c r="L20" s="6" t="n"/>
+      <c r="M20" s="6" t="n"/>
+      <c r="N20" s="6" t="n"/>
     </row>
     <row r="21">
-      <c r="G21" s="6">
-        <f>F21-E21</f>
-        <v/>
-      </c>
-      <c r="H21" s="6">
-        <f>IF(G21=0,"Pick'em",IF(G21&gt;0,"Home","Away"))</f>
-        <v/>
-      </c>
-      <c r="K21" s="6">
-        <f>I21-J21</f>
-        <v/>
-      </c>
-      <c r="L21" s="6">
-        <f>IF(K21=0,"Push",IF(K21&gt;0,"Over","Under"))</f>
-        <v/>
-      </c>
-      <c r="M21" s="6">
-        <f>IF(ABS(G21)&gt;=Settings!$B$5,H21,"Pass")</f>
-        <v/>
-      </c>
-      <c r="N21" s="6">
-        <f>IF(ABS(K21)&gt;=Settings!$B$6,L21,"Pass")</f>
-        <v/>
-      </c>
+      <c r="G21" s="6" t="n"/>
+      <c r="H21" s="6" t="n"/>
+      <c r="K21" s="6" t="n"/>
+      <c r="L21" s="6" t="n"/>
+      <c r="M21" s="6" t="n"/>
+      <c r="N21" s="6" t="n"/>
     </row>
     <row r="22">
-      <c r="G22" s="6">
-        <f>F22-E22</f>
-        <v/>
-      </c>
-      <c r="H22" s="6">
-        <f>IF(G22=0,"Pick'em",IF(G22&gt;0,"Home","Away"))</f>
-        <v/>
-      </c>
-      <c r="K22" s="6">
-        <f>I22-J22</f>
-        <v/>
-      </c>
-      <c r="L22" s="6">
-        <f>IF(K22=0,"Push",IF(K22&gt;0,"Over","Under"))</f>
-        <v/>
-      </c>
-      <c r="M22" s="6">
-        <f>IF(ABS(G22)&gt;=Settings!$B$5,H22,"Pass")</f>
-        <v/>
-      </c>
-      <c r="N22" s="6">
-        <f>IF(ABS(K22)&gt;=Settings!$B$6,L22,"Pass")</f>
-        <v/>
-      </c>
+      <c r="G22" s="6" t="n"/>
+      <c r="H22" s="6" t="n"/>
+      <c r="K22" s="6" t="n"/>
+      <c r="L22" s="6" t="n"/>
+      <c r="M22" s="6" t="n"/>
+      <c r="N22" s="6" t="n"/>
     </row>
     <row r="23">
-      <c r="G23" s="6">
-        <f>F23-E23</f>
-        <v/>
-      </c>
-      <c r="H23" s="6">
-        <f>IF(G23=0,"Pick'em",IF(G23&gt;0,"Home","Away"))</f>
-        <v/>
-      </c>
-      <c r="K23" s="6">
-        <f>I23-J23</f>
-        <v/>
-      </c>
-      <c r="L23" s="6">
-        <f>IF(K23=0,"Push",IF(K23&gt;0,"Over","Under"))</f>
-        <v/>
-      </c>
-      <c r="M23" s="6">
-        <f>IF(ABS(G23)&gt;=Settings!$B$5,H23,"Pass")</f>
-        <v/>
-      </c>
-      <c r="N23" s="6">
-        <f>IF(ABS(K23)&gt;=Settings!$B$6,L23,"Pass")</f>
-        <v/>
-      </c>
+      <c r="G23" s="6" t="n"/>
+      <c r="H23" s="6" t="n"/>
+      <c r="K23" s="6" t="n"/>
+      <c r="L23" s="6" t="n"/>
+      <c r="M23" s="6" t="n"/>
+      <c r="N23" s="6" t="n"/>
     </row>
     <row r="24">
-      <c r="G24" s="6">
-        <f>F24-E24</f>
-        <v/>
-      </c>
-      <c r="H24" s="6">
-        <f>IF(G24=0,"Pick'em",IF(G24&gt;0,"Home","Away"))</f>
-        <v/>
-      </c>
-      <c r="K24" s="6">
-        <f>I24-J24</f>
-        <v/>
-      </c>
-      <c r="L24" s="6">
-        <f>IF(K24=0,"Push",IF(K24&gt;0,"Over","Under"))</f>
-        <v/>
-      </c>
-      <c r="M24" s="6">
-        <f>IF(ABS(G24)&gt;=Settings!$B$5,H24,"Pass")</f>
-        <v/>
-      </c>
-      <c r="N24" s="6">
-        <f>IF(ABS(K24)&gt;=Settings!$B$6,L24,"Pass")</f>
-        <v/>
-      </c>
+      <c r="G24" s="6" t="n"/>
+      <c r="H24" s="6" t="n"/>
+      <c r="K24" s="6" t="n"/>
+      <c r="L24" s="6" t="n"/>
+      <c r="M24" s="6" t="n"/>
+      <c r="N24" s="6" t="n"/>
     </row>
     <row r="25">
-      <c r="G25" s="6">
-        <f>F25-E25</f>
-        <v/>
-      </c>
-      <c r="H25" s="6">
-        <f>IF(G25=0,"Pick'em",IF(G25&gt;0,"Home","Away"))</f>
-        <v/>
-      </c>
-      <c r="K25" s="6">
-        <f>I25-J25</f>
-        <v/>
-      </c>
-      <c r="L25" s="6">
-        <f>IF(K25=0,"Push",IF(K25&gt;0,"Over","Under"))</f>
-        <v/>
-      </c>
-      <c r="M25" s="6">
-        <f>IF(ABS(G25)&gt;=Settings!$B$5,H25,"Pass")</f>
-        <v/>
-      </c>
-      <c r="N25" s="6">
-        <f>IF(ABS(K25)&gt;=Settings!$B$6,L25,"Pass")</f>
-        <v/>
-      </c>
+      <c r="G25" s="6" t="n"/>
+      <c r="H25" s="6" t="n"/>
+      <c r="K25" s="6" t="n"/>
+      <c r="L25" s="6" t="n"/>
+      <c r="M25" s="6" t="n"/>
+      <c r="N25" s="6" t="n"/>
     </row>
     <row r="26">
-      <c r="G26" s="6">
-        <f>F26-E26</f>
-        <v/>
-      </c>
-      <c r="H26" s="6">
-        <f>IF(G26=0,"Pick'em",IF(G26&gt;0,"Home","Away"))</f>
-        <v/>
-      </c>
-      <c r="K26" s="6">
-        <f>I26-J26</f>
-        <v/>
-      </c>
-      <c r="L26" s="6">
-        <f>IF(K26=0,"Push",IF(K26&gt;0,"Over","Under"))</f>
-        <v/>
-      </c>
-      <c r="M26" s="6">
-        <f>IF(ABS(G26)&gt;=Settings!$B$5,H26,"Pass")</f>
-        <v/>
-      </c>
-      <c r="N26" s="6">
-        <f>IF(ABS(K26)&gt;=Settings!$B$6,L26,"Pass")</f>
-        <v/>
-      </c>
+      <c r="G26" s="6" t="n"/>
+      <c r="H26" s="6" t="n"/>
+      <c r="K26" s="6" t="n"/>
+      <c r="L26" s="6" t="n"/>
+      <c r="M26" s="6" t="n"/>
+      <c r="N26" s="6" t="n"/>
     </row>
     <row r="27">
-      <c r="G27" s="6">
-        <f>F27-E27</f>
-        <v/>
-      </c>
-      <c r="H27" s="6">
-        <f>IF(G27=0,"Pick'em",IF(G27&gt;0,"Home","Away"))</f>
-        <v/>
-      </c>
-      <c r="K27" s="6">
-        <f>I27-J27</f>
-        <v/>
-      </c>
-      <c r="L27" s="6">
-        <f>IF(K27=0,"Push",IF(K27&gt;0,"Over","Under"))</f>
-        <v/>
-      </c>
-      <c r="M27" s="6">
-        <f>IF(ABS(G27)&gt;=Settings!$B$5,H27,"Pass")</f>
-        <v/>
-      </c>
-      <c r="N27" s="6">
-        <f>IF(ABS(K27)&gt;=Settings!$B$6,L27,"Pass")</f>
-        <v/>
-      </c>
+      <c r="G27" s="6" t="n"/>
+      <c r="H27" s="6" t="n"/>
+      <c r="K27" s="6" t="n"/>
+      <c r="L27" s="6" t="n"/>
+      <c r="M27" s="6" t="n"/>
+      <c r="N27" s="6" t="n"/>
     </row>
     <row r="28">
-      <c r="G28" s="6">
-        <f>F28-E28</f>
-        <v/>
-      </c>
-      <c r="H28" s="6">
-        <f>IF(G28=0,"Pick'em",IF(G28&gt;0,"Home","Away"))</f>
-        <v/>
-      </c>
-      <c r="K28" s="6">
-        <f>I28-J28</f>
-        <v/>
-      </c>
-      <c r="L28" s="6">
-        <f>IF(K28=0,"Push",IF(K28&gt;0,"Over","Under"))</f>
-        <v/>
-      </c>
-      <c r="M28" s="6">
-        <f>IF(ABS(G28)&gt;=Settings!$B$5,H28,"Pass")</f>
-        <v/>
-      </c>
-      <c r="N28" s="6">
-        <f>IF(ABS(K28)&gt;=Settings!$B$6,L28,"Pass")</f>
-        <v/>
-      </c>
+      <c r="G28" s="6" t="n"/>
+      <c r="H28" s="6" t="n"/>
+      <c r="K28" s="6" t="n"/>
+      <c r="L28" s="6" t="n"/>
+      <c r="M28" s="6" t="n"/>
+      <c r="N28" s="6" t="n"/>
     </row>
     <row r="29">
-      <c r="G29" s="6">
-        <f>F29-E29</f>
-        <v/>
-      </c>
-      <c r="H29" s="6">
-        <f>IF(G29=0,"Pick'em",IF(G29&gt;0,"Home","Away"))</f>
-        <v/>
-      </c>
-      <c r="K29" s="6">
-        <f>I29-J29</f>
-        <v/>
-      </c>
-      <c r="L29" s="6">
-        <f>IF(K29=0,"Push",IF(K29&gt;0,"Over","Under"))</f>
-        <v/>
-      </c>
-      <c r="M29" s="6">
-        <f>IF(ABS(G29)&gt;=Settings!$B$5,H29,"Pass")</f>
-        <v/>
-      </c>
-      <c r="N29" s="6">
-        <f>IF(ABS(K29)&gt;=Settings!$B$6,L29,"Pass")</f>
-        <v/>
-      </c>
+      <c r="G29" s="6" t="n"/>
+      <c r="H29" s="6" t="n"/>
+      <c r="K29" s="6" t="n"/>
+      <c r="L29" s="6" t="n"/>
+      <c r="M29" s="6" t="n"/>
+      <c r="N29" s="6" t="n"/>
     </row>
     <row r="30"/>
     <row r="31"/>
@@ -1958,9 +1705,19 @@
     <row r="41"/>
     <row r="42"/>
   </sheetData>
-  <conditionalFormatting sqref="C2:D29">
+  <conditionalFormatting sqref="C2:C500">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>AND(OR($G2&lt;=-7,$G2&gt;=7),$H2="Away")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D2:D500">
     <cfRule type="expression" priority="2" dxfId="0">
-      <formula>COUNTIF($R$5:$R$12,C2)&gt;0</formula>
+      <formula>AND(OR($G2&lt;=-7,$G2&gt;=7),$H2="Home")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E2:F500">
+    <cfRule type="expression" priority="3" dxfId="0">
+      <formula>OR($G2&lt;=-7,$G2&gt;=7)</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1981,7 +1738,7 @@
     <col width="6" customWidth="1" min="2" max="2"/>
     <col width="37.42578125" bestFit="1" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="22.28515625" bestFit="1" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="9"/>
@@ -2091,10 +1848,7 @@
       <c r="H2" t="n">
         <v>1</v>
       </c>
-      <c r="J2" s="6">
-        <f>IF(I2="","",I2-F2)</f>
-        <v/>
-      </c>
+      <c r="J2" s="6" t="n"/>
       <c r="L2" s="6">
         <f>IF(K2="W",IF(G2&lt;0,H2*100/ABS(G2),H2*G2/100),IF(K2="L",-H2,0))</f>
         <v/>
@@ -2120,22 +1874,19 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Total</t>
+          <t>Moneyline</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Over 46.5</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>46.5</v>
+          <t>North Dakota State -265</t>
+        </is>
       </c>
       <c r="G3" t="n">
-        <v>-110</v>
+        <v>-265</v>
       </c>
       <c r="H3" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J3" s="6">
         <f>IF(I3="","",I3-F3)</f>
@@ -2151,8 +1902,37 @@
       </c>
     </row>
     <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-29</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Memphis @ UNLV</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>UNLV -184</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>-184</v>
+      </c>
+      <c r="H4" t="n">
+        <v>5</v>
+      </c>
       <c r="J4" s="6">
-        <f>IF(I4="","",I4-F4)</f>
+        <f>IF(I4="","",I4-F5)</f>
         <v/>
       </c>
       <c r="L4" s="6">
@@ -2165,8 +1945,9 @@
       </c>
     </row>
     <row r="5">
+      <c r="A5" s="8" t="n"/>
       <c r="J5" s="6">
-        <f>IF(I5="","",I5-F5)</f>
+        <f>IF(I5="","",I5-#REF!)</f>
         <v/>
       </c>
       <c r="L5" s="6">
@@ -2705,8 +2486,8 @@
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="37" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="7.140625" bestFit="1" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="7"/>
@@ -2764,33 +2545,29 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Air Force</t>
+          <t>North Dakota State</t>
         </is>
       </c>
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>Mountain West</t>
+          <t>FCS (Missouri Valley Football Conference)</t>
         </is>
       </c>
       <c r="C2" s="6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="D2" s="8" t="n">
-        <v>1473</v>
+        <v>1790.9</v>
       </c>
       <c r="E2" s="8" t="n">
-        <v>-3.2</v>
-      </c>
-      <c r="F2" s="8" t="n">
-        <v>0.286935598221958</v>
-      </c>
-      <c r="G2" s="8" t="n">
-        <v>0.4016443170135715</v>
-      </c>
+        <v>-1.8</v>
+      </c>
+      <c r="F2" s="8" t="n"/>
+      <c r="G2" s="8" t="n"/>
       <c r="H2" s="8" t="n">
-        <v>141</v>
+        <v>117</v>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
@@ -2801,7 +2578,7 @@
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>Hawai'i</t>
+          <t>UNLV</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
@@ -2815,19 +2592,19 @@
         </is>
       </c>
       <c r="D3" s="8" t="n">
-        <v>1561.1</v>
+        <v>1645.3</v>
       </c>
       <c r="E3" s="8" t="n">
-        <v>-2.6</v>
+        <v>3.6</v>
       </c>
       <c r="F3" s="8" t="n">
-        <v>0.1674201707393385</v>
+        <v>0.2978672891337787</v>
       </c>
       <c r="G3" s="8" t="n">
-        <v>0.163302527678112</v>
+        <v>927</v>
       </c>
       <c r="H3" s="8" t="n">
-        <v>124</v>
+        <v>63</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
@@ -2838,7 +2615,7 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Nevada</t>
+          <t>New Mexico</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -2852,19 +2629,19 @@
         </is>
       </c>
       <c r="D4" s="8" t="n">
-        <v>1361.9</v>
+        <v>1566.5</v>
       </c>
       <c r="E4" s="8" t="n">
-        <v>-11.7</v>
+        <v>0</v>
       </c>
       <c r="F4" s="8" t="n">
-        <v>0.03365966628322248</v>
+        <v>0.1604555999630125</v>
       </c>
       <c r="G4" s="8" t="n">
-        <v>0.187141422349949</v>
+        <v>850</v>
       </c>
       <c r="H4" s="8" t="n">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
@@ -2875,7 +2652,7 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>New Mexico</t>
+          <t>Hawai'i</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
@@ -2889,19 +2666,19 @@
         </is>
       </c>
       <c r="D5" s="8" t="n">
-        <v>1566.5</v>
+        <v>1561.1</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>0</v>
+        <v>-2.6</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>0.1604555999630125</v>
+        <v>0.1674201707393385</v>
       </c>
       <c r="G5" s="8" t="n">
-        <v>0.1048040165888917</v>
+        <v>916</v>
       </c>
       <c r="H5" s="8" t="n">
-        <v>87</v>
+        <v>124</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
@@ -2912,29 +2689,33 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>North Dakota State</t>
+          <t>Air Force</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>FCS (Missouri Valley Football Conference)</t>
+          <t>Mountain West</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="D6" s="8" t="n">
-        <v>1790.9</v>
+        <v>1473</v>
       </c>
       <c r="E6" s="8" t="n">
-        <v>-1.8</v>
-      </c>
-      <c r="F6" s="8" t="n"/>
-      <c r="G6" s="8" t="n"/>
+        <v>-3.2</v>
+      </c>
+      <c r="F6" s="8" t="n">
+        <v>0.286935598221958</v>
+      </c>
+      <c r="G6" s="8" t="n">
+        <v>823</v>
+      </c>
       <c r="H6" s="8" t="n">
-        <v>117</v>
+        <v>141</v>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
@@ -2945,33 +2726,33 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>Northern Illinois</t>
+          <t>Wyoming</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>MAC</t>
+          <t>Mountain West</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="D7" s="8" t="n">
-        <v>1394.5</v>
+        <v>1399.9</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>-17.2</v>
+        <v>-10.8</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>0.04689237303920656</v>
+        <v>0.04868411996031556</v>
       </c>
       <c r="G7" s="8" t="n">
-        <v>0.1861273080394991</v>
+        <v>811</v>
       </c>
       <c r="H7" s="8" t="n">
-        <v>82</v>
+        <v>114</v>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
@@ -2982,33 +2763,33 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>San José State</t>
+          <t>Northern Illinois</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Mountain West</t>
+          <t>MAC</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="D8" s="8" t="n">
-        <v>1388.2</v>
+        <v>1394.5</v>
       </c>
       <c r="E8" s="8" t="n">
-        <v>-15.7</v>
+        <v>-17.2</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>0.1717992412693814</v>
+        <v>0.04689237303920656</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>0.2035861313923595</v>
+        <v>746</v>
       </c>
       <c r="H8" s="8" t="n">
-        <v>129</v>
+        <v>82</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
@@ -3019,7 +2800,7 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>UNLV</t>
+          <t>San José State</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
@@ -3033,19 +2814,19 @@
         </is>
       </c>
       <c r="D9" s="8" t="n">
-        <v>1645.3</v>
+        <v>1388.2</v>
       </c>
       <c r="E9" s="8" t="n">
-        <v>3.6</v>
+        <v>-15.7</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>0.2978672891337787</v>
+        <v>0.1717992412693814</v>
       </c>
       <c r="G9" s="8" t="n">
-        <v>0.2101010006427078</v>
+        <v>814</v>
       </c>
       <c r="H9" s="8" t="n">
-        <v>63</v>
+        <v>129</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
@@ -3056,33 +2837,33 @@
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>UTEP</t>
+          <t>Nevada</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Conference USA</t>
+          <t>Mountain West</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>N</t>
         </is>
       </c>
       <c r="D10" s="8" t="n">
-        <v>1302.8</v>
+        <v>1361.9</v>
       </c>
       <c r="E10" s="8" t="n">
-        <v>-19.3</v>
+        <v>-11.7</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>0.0127842137907675</v>
+        <v>0.03365966628322248</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>0.1007763319294122</v>
+        <v>728</v>
       </c>
       <c r="H10" s="8" t="n">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
@@ -3093,33 +2874,33 @@
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>Wyoming</t>
+          <t>UTEP</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Mountain West</t>
+          <t>Conference USA</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="D11" s="8" t="n">
-        <v>1399.9</v>
+        <v>1302.8</v>
       </c>
       <c r="E11" s="8" t="n">
-        <v>-10.8</v>
+        <v>-19.3</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>0.04868411996031556</v>
+        <v>0.0127842137907675</v>
       </c>
       <c r="G11" s="8" t="n">
-        <v>0.06891172319885128</v>
+        <v>789</v>
       </c>
       <c r="H11" s="8" t="n">
-        <v>114</v>
+        <v>92</v>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Stop committing the compiled DuckDB file -- fully rebuildable from data/raw/
</commit_message>
<xml_diff>
--- a/excel/MW_Handicapping_Tracker.xlsx
+++ b/excel/MW_Handicapping_Tracker.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Weekly Slate" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Bet Log" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Team Profiles" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Model Comparison" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1" iterateDelta="0.0001"/>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -77,8 +78,36 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00666666"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -97,8 +126,23 @@
         <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4EC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -130,11 +174,25 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -150,6 +208,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -821,7 +888,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>-31.7</v>
+        <v>-32.2</v>
       </c>
       <c r="F2" t="n">
         <v>-37.2</v>
@@ -879,7 +946,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>-16.3</v>
+        <v>-16.4</v>
       </c>
       <c r="F3" t="n">
         <v>-6.8</v>
@@ -935,7 +1002,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>-5</v>
+        <v>-4.3</v>
       </c>
       <c r="F4" t="n">
         <v>-4.8</v>
@@ -991,7 +1058,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>-10.6</v>
+        <v>-9.9</v>
       </c>
       <c r="F5" t="n">
         <v>-4.8</v>
@@ -1052,7 +1119,7 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>-11.9</v>
+        <v>-12.8</v>
       </c>
       <c r="F6" t="n">
         <v>-3</v>
@@ -1113,7 +1180,7 @@
         </is>
       </c>
       <c r="E7" s="10" t="n">
-        <v>-16.8</v>
+        <v>-22</v>
       </c>
       <c r="F7" s="10" t="n">
         <v>-28.5</v>
@@ -1174,7 +1241,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>-46.4</v>
+        <v>-49.9</v>
       </c>
       <c r="F8" t="n">
         <v>-39.5</v>
@@ -1235,7 +1302,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>-30.8</v>
+        <v>-30.4</v>
       </c>
       <c r="F9" t="n">
         <v>-31.2</v>
@@ -1296,7 +1363,7 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>-5</v>
+        <v>-5.2</v>
       </c>
       <c r="F10" t="n">
         <v>-3</v>
@@ -1357,7 +1424,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>-35.5</v>
+        <v>-33.9</v>
       </c>
       <c r="F11" t="n">
         <v>-41.5</v>
@@ -1418,7 +1485,7 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>6.1</v>
+        <v>6.5</v>
       </c>
       <c r="F12" t="n">
         <v>3</v>
@@ -1479,7 +1546,7 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>-15.9</v>
+        <v>-17.2</v>
       </c>
       <c r="F13" t="n">
         <v>-10</v>
@@ -1535,7 +1602,7 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>5.3</v>
+        <v>5</v>
       </c>
       <c r="F14" t="n">
         <v>2.5</v>
@@ -3031,4 +3098,742 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>Ridge vs. XGBoost -- Model Comparison</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>Informational only. Ridge is still the live model everywhere else in this workbook and on the website -- XGBoost is a candidate being evaluated here, not a replacement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>All-Time (every season in the backtest)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>Games Graded</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="inlineStr">
+        <is>
+          <t>Bets Made</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="inlineStr">
+        <is>
+          <t>Wins</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="inlineStr">
+        <is>
+          <t>Losses</t>
+        </is>
+      </c>
+      <c r="F5" s="14" t="inlineStr">
+        <is>
+          <t>Pushes</t>
+        </is>
+      </c>
+      <c r="G5" s="14" t="inlineStr">
+        <is>
+          <t>ATS Win %</t>
+        </is>
+      </c>
+      <c r="H5" s="14" t="inlineStr">
+        <is>
+          <t>ROI (flat stake)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>Ridge (live model) -- all FBS</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="n">
+        <v>8441</v>
+      </c>
+      <c r="C6" s="15" t="n">
+        <v>6578</v>
+      </c>
+      <c r="D6" s="15" t="n">
+        <v>3264</v>
+      </c>
+      <c r="E6" s="15" t="n">
+        <v>3314</v>
+      </c>
+      <c r="F6" s="15" t="n">
+        <v>59</v>
+      </c>
+      <c r="G6" s="15" t="inlineStr">
+        <is>
+          <t>49.6%</t>
+        </is>
+      </c>
+      <c r="H6" s="15" t="inlineStr">
+        <is>
+          <t>-5.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="15" t="inlineStr">
+        <is>
+          <t>Ridge (live model) -- MW-involved</t>
+        </is>
+      </c>
+      <c r="B7" s="15" t="n">
+        <v>960</v>
+      </c>
+      <c r="C7" s="15" t="n">
+        <v>756</v>
+      </c>
+      <c r="D7" s="15" t="n">
+        <v>377</v>
+      </c>
+      <c r="E7" s="15" t="n">
+        <v>379</v>
+      </c>
+      <c r="F7" s="15" t="n">
+        <v>12</v>
+      </c>
+      <c r="G7" s="15" t="inlineStr">
+        <is>
+          <t>49.9%</t>
+        </is>
+      </c>
+      <c r="H7" s="15" t="inlineStr">
+        <is>
+          <t>-4.8%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="15" t="inlineStr">
+        <is>
+          <t>XGBoost (candidate) -- all FBS</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="n">
+        <v>8441</v>
+      </c>
+      <c r="C8" s="15" t="n">
+        <v>6519</v>
+      </c>
+      <c r="D8" s="15" t="n">
+        <v>3260</v>
+      </c>
+      <c r="E8" s="15" t="n">
+        <v>3259</v>
+      </c>
+      <c r="F8" s="15" t="n">
+        <v>59</v>
+      </c>
+      <c r="G8" s="15" t="inlineStr">
+        <is>
+          <t>50.0%</t>
+        </is>
+      </c>
+      <c r="H8" s="15" t="inlineStr">
+        <is>
+          <t>-4.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="15" t="inlineStr">
+        <is>
+          <t>XGBoost (candidate) -- MW-involved</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="n">
+        <v>960</v>
+      </c>
+      <c r="C9" s="15" t="n">
+        <v>742</v>
+      </c>
+      <c r="D9" s="15" t="n">
+        <v>384</v>
+      </c>
+      <c r="E9" s="15" t="n">
+        <v>358</v>
+      </c>
+      <c r="F9" s="15" t="n">
+        <v>11</v>
+      </c>
+      <c r="G9" s="15" t="inlineStr">
+        <is>
+          <t>51.7%</t>
+        </is>
+      </c>
+      <c r="H9" s="15" t="inlineStr">
+        <is>
+          <t>-1.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>2026 Season Only</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>Games Graded</t>
+        </is>
+      </c>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>Bets Made</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="inlineStr">
+        <is>
+          <t>Wins</t>
+        </is>
+      </c>
+      <c r="E12" s="14" t="inlineStr">
+        <is>
+          <t>Losses</t>
+        </is>
+      </c>
+      <c r="F12" s="14" t="inlineStr">
+        <is>
+          <t>Pushes</t>
+        </is>
+      </c>
+      <c r="G12" s="14" t="inlineStr">
+        <is>
+          <t>ATS Win %</t>
+        </is>
+      </c>
+      <c r="H12" s="14" t="inlineStr">
+        <is>
+          <t>ROI (flat stake)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>Ridge (live model) -- all FBS</t>
+        </is>
+      </c>
+      <c r="B13" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="C13" s="15" t="n">
+        <v>7</v>
+      </c>
+      <c r="D13" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="F13" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="15" t="inlineStr">
+        <is>
+          <t>42.9%</t>
+        </is>
+      </c>
+      <c r="H13" s="15" t="inlineStr">
+        <is>
+          <t>-18.2%</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>Ridge (live model) -- MW-involved</t>
+        </is>
+      </c>
+      <c r="B14" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="C14" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D14" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="E14" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="15" t="inlineStr">
+        <is>
+          <t>66.7%</t>
+        </is>
+      </c>
+      <c r="H14" s="15" t="inlineStr">
+        <is>
+          <t>+27.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>XGBoost (candidate) -- all FBS</t>
+        </is>
+      </c>
+      <c r="B15" s="15" t="n">
+        <v>8</v>
+      </c>
+      <c r="C15" s="15" t="n">
+        <v>6</v>
+      </c>
+      <c r="D15" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="E15" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="F15" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="15" t="inlineStr">
+        <is>
+          <t>50.0%</t>
+        </is>
+      </c>
+      <c r="H15" s="15" t="inlineStr">
+        <is>
+          <t>-4.5%</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="15" t="inlineStr">
+        <is>
+          <t>XGBoost (candidate) -- MW-involved</t>
+        </is>
+      </c>
+      <c r="B16" s="15" t="n">
+        <v>4</v>
+      </c>
+      <c r="C16" s="15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D16" s="15" t="n">
+        <v>2</v>
+      </c>
+      <c r="E16" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="15" t="inlineStr">
+        <is>
+          <t>66.7%</t>
+        </is>
+      </c>
+      <c r="H16" s="15" t="inlineStr">
+        <is>
+          <t>+27.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>Ridge and XGBoost agree on which side to lean in 81.1% of all graded games.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>2026 Mountain West Games -- Game by Game</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t>Week</t>
+        </is>
+      </c>
+      <c r="B21" s="14" t="inlineStr">
+        <is>
+          <t>Matchup</t>
+        </is>
+      </c>
+      <c r="C21" s="14" t="inlineStr">
+        <is>
+          <t>Vegas Spread (Home)</t>
+        </is>
+      </c>
+      <c r="D21" s="14" t="inlineStr">
+        <is>
+          <t>Actual Margin (Home)</t>
+        </is>
+      </c>
+      <c r="E21" s="14" t="inlineStr">
+        <is>
+          <t>Ridge Line</t>
+        </is>
+      </c>
+      <c r="F21" s="14" t="inlineStr">
+        <is>
+          <t>Ridge Edge</t>
+        </is>
+      </c>
+      <c r="G21" s="14" t="inlineStr">
+        <is>
+          <t>Ridge Lean</t>
+        </is>
+      </c>
+      <c r="H21" s="14" t="inlineStr">
+        <is>
+          <t>Ridge Result</t>
+        </is>
+      </c>
+      <c r="I21" s="14" t="inlineStr">
+        <is>
+          <t>XGBoost Line</t>
+        </is>
+      </c>
+      <c r="J21" s="14" t="inlineStr">
+        <is>
+          <t>XGBoost Edge</t>
+        </is>
+      </c>
+      <c r="K21" s="14" t="inlineStr">
+        <is>
+          <t>XGBoost Lean</t>
+        </is>
+      </c>
+      <c r="L21" s="14" t="inlineStr">
+        <is>
+          <t>XGBoost Result</t>
+        </is>
+      </c>
+      <c r="M21" s="14" t="inlineStr">
+        <is>
+          <t>Models Agree?</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="B22" s="15" t="inlineStr">
+        <is>
+          <t>Jacksonville State @ North Dakota State</t>
+        </is>
+      </c>
+      <c r="C22" s="15" t="inlineStr">
+        <is>
+          <t>-6.8</t>
+        </is>
+      </c>
+      <c r="D22" s="15" t="inlineStr">
+        <is>
+          <t>+26.0</t>
+        </is>
+      </c>
+      <c r="E22" s="15" t="inlineStr">
+        <is>
+          <t>-16.3</t>
+        </is>
+      </c>
+      <c r="F22" s="15" t="inlineStr">
+        <is>
+          <t>+9.6</t>
+        </is>
+      </c>
+      <c r="G22" s="15" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="H22" s="16" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="I22" s="15" t="inlineStr">
+        <is>
+          <t>-15.3</t>
+        </is>
+      </c>
+      <c r="J22" s="15" t="inlineStr">
+        <is>
+          <t>+8.6</t>
+        </is>
+      </c>
+      <c r="K22" s="15" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="L22" s="16" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="M22" s="15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="B23" s="15" t="inlineStr">
+        <is>
+          <t>Hawai'i @ Stanford</t>
+        </is>
+      </c>
+      <c r="C23" s="15" t="inlineStr">
+        <is>
+          <t>-4.8</t>
+        </is>
+      </c>
+      <c r="D23" s="15" t="inlineStr">
+        <is>
+          <t>+10.0</t>
+        </is>
+      </c>
+      <c r="E23" s="15" t="inlineStr">
+        <is>
+          <t>-4.2</t>
+        </is>
+      </c>
+      <c r="F23" s="15" t="inlineStr">
+        <is>
+          <t>-0.5</t>
+        </is>
+      </c>
+      <c r="G23" s="15" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="H23" s="15" t="inlineStr">
+        <is>
+          <t>Lean only</t>
+        </is>
+      </c>
+      <c r="I23" s="15" t="inlineStr">
+        <is>
+          <t>-0.7</t>
+        </is>
+      </c>
+      <c r="J23" s="15" t="inlineStr">
+        <is>
+          <t>-4.1</t>
+        </is>
+      </c>
+      <c r="K23" s="15" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="L23" s="17" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="M23" s="15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="B24" s="15" t="inlineStr">
+        <is>
+          <t>Memphis @ UNLV</t>
+        </is>
+      </c>
+      <c r="C24" s="15" t="inlineStr">
+        <is>
+          <t>-4.8</t>
+        </is>
+      </c>
+      <c r="D24" s="15" t="inlineStr">
+        <is>
+          <t>-6.0</t>
+        </is>
+      </c>
+      <c r="E24" s="15" t="inlineStr">
+        <is>
+          <t>-9.8</t>
+        </is>
+      </c>
+      <c r="F24" s="15" t="inlineStr">
+        <is>
+          <t>+5.1</t>
+        </is>
+      </c>
+      <c r="G24" s="15" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="H24" s="17" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="I24" s="15" t="inlineStr">
+        <is>
+          <t>-6.5</t>
+        </is>
+      </c>
+      <c r="J24" s="15" t="inlineStr">
+        <is>
+          <t>+1.8</t>
+        </is>
+      </c>
+      <c r="K24" s="15" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="L24" s="15" t="inlineStr">
+        <is>
+          <t>Lean only</t>
+        </is>
+      </c>
+      <c r="M24" s="15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="B25" s="15" t="inlineStr">
+        <is>
+          <t>San José State @ USC</t>
+        </is>
+      </c>
+      <c r="C25" s="15" t="inlineStr">
+        <is>
+          <t>-37.2</t>
+        </is>
+      </c>
+      <c r="D25" s="15" t="inlineStr">
+        <is>
+          <t>+16.0</t>
+        </is>
+      </c>
+      <c r="E25" s="15" t="inlineStr">
+        <is>
+          <t>-32.1</t>
+        </is>
+      </c>
+      <c r="F25" s="15" t="inlineStr">
+        <is>
+          <t>-5.1</t>
+        </is>
+      </c>
+      <c r="G25" s="15" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="H25" s="16" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="I25" s="15" t="inlineStr">
+        <is>
+          <t>-32.9</t>
+        </is>
+      </c>
+      <c r="J25" s="15" t="inlineStr">
+        <is>
+          <t>-4.4</t>
+        </is>
+      </c>
+      <c r="K25" s="15" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="L25" s="16" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="M25" s="15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Pull weekend results, update site
</commit_message>
<xml_diff>
--- a/excel/MW_Handicapping_Tracker.xlsx
+++ b/excel/MW_Handicapping_Tracker.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="0" activeTab="5" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Read Me" sheetId="1" state="visible" r:id="rId1"/>
@@ -80,30 +80,35 @@
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <b val="1"/>
       <sz val="14"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <i val="1"/>
-      <color rgb="00666666"/>
+      <color rgb="FF666666"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="001F3864"/>
+      <color rgb="FF1F3864"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="00000000"/>
+      <family val="2"/>
+      <color rgb="FF000000"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -128,17 +133,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F3864"/>
+        <fgColor rgb="FF1F3864"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E2EFDA"/>
+        <fgColor rgb="FFE2EFDA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCE4EC"/>
+        <fgColor rgb="FFFCE4EC"/>
       </patternFill>
     </fill>
   </fills>
@@ -176,17 +181,18 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="FFCCCCCC"/>
       </left>
       <right style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="FFCCCCCC"/>
       </right>
       <top style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="FFCCCCCC"/>
       </top>
       <bottom style="thin">
-        <color rgb="00CCCCCC"/>
+        <color rgb="FFCCCCCC"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -3109,22 +3115,18 @@
   <dimension ref="A1:M25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="136" bestFit="1" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="3" max="4"/>
+    <col width="12" customWidth="1" min="5" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="8" max="10"/>
     <col width="11" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="18" customHeight="1">
       <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Ridge vs. XGBoost -- Model Comparison</t>
@@ -3145,7 +3147,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="25.5" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
         <is>
           <t>Model</t>
@@ -3322,7 +3324,7 @@
         </is>
       </c>
     </row>
-    <row r="12">
+    <row r="12" ht="25.5" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
         <is>
           <t>Model</t>
@@ -3506,7 +3508,7 @@
         </is>
       </c>
     </row>
-    <row r="21">
+    <row r="21" ht="25.5" customHeight="1">
       <c r="A21" s="14" t="inlineStr">
         <is>
           <t>Week</t>

</xml_diff>

<commit_message>
Update predictions CSV and tracker from latest pipeline run
</commit_message>
<xml_diff>
--- a/excel/MW_Handicapping_Tracker.xlsx
+++ b/excel/MW_Handicapping_Tracker.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\deene\Mountain Dub Handicapping\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C260CAF-5799-48DD-805B-C61E2172065A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_EF4F49679EBFFEBBC78155D7FE90A1BC0643DDDE" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Read Me" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="197">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="397" uniqueCount="245">
   <si>
     <t>Ridge vs. XGBoost -- Model Comparison</t>
   </si>
@@ -127,13 +127,196 @@
     <t>Ridge and XGBoost agree on which side to lean in 81.1% of all graded games.</t>
   </si>
   <si>
+    <t>Upcoming Games -- Ridge vs. XGBoost (Not Yet Graded)</t>
+  </si>
+  <si>
+    <t>Week</t>
+  </si>
+  <si>
+    <t>Matchup</t>
+  </si>
+  <si>
+    <t>Market Line (Home)</t>
+  </si>
+  <si>
+    <t>Ridge Line</t>
+  </si>
+  <si>
+    <t>XGBoost Line</t>
+  </si>
+  <si>
+    <t>Ridge Lean</t>
+  </si>
+  <si>
+    <t>XGBoost Lean</t>
+  </si>
+  <si>
+    <t>Models Agree?</t>
+  </si>
+  <si>
+    <t>San José State @ USC</t>
+  </si>
+  <si>
+    <t>-37.2</t>
+  </si>
+  <si>
+    <t>-32.2</t>
+  </si>
+  <si>
+    <t>-31.0</t>
+  </si>
+  <si>
+    <t>Away</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Jacksonville State @ North Dakota State</t>
+  </si>
+  <si>
+    <t>-6.8</t>
+  </si>
+  <si>
+    <t>-16.4</t>
+  </si>
+  <si>
+    <t>-16.7</t>
+  </si>
+  <si>
+    <t>Home</t>
+  </si>
+  <si>
+    <t>Hawai'i @ Stanford</t>
+  </si>
+  <si>
+    <t>-4.8</t>
+  </si>
+  <si>
+    <t>-4.3</t>
+  </si>
+  <si>
+    <t>-1.8</t>
+  </si>
+  <si>
+    <t>Memphis @ UNLV</t>
+  </si>
+  <si>
+    <t>-9.9</t>
+  </si>
+  <si>
+    <t>-5.7</t>
+  </si>
+  <si>
+    <t>San José State @ Eastern Michigan</t>
+  </si>
+  <si>
+    <t>-3.0</t>
+  </si>
+  <si>
+    <t>-12.8</t>
+  </si>
+  <si>
+    <t>-11.3</t>
+  </si>
+  <si>
+    <t>UTEP @ Oklahoma</t>
+  </si>
+  <si>
+    <t>-41.5</t>
+  </si>
+  <si>
+    <t>-33.9</t>
+  </si>
+  <si>
+    <t>-33.5</t>
+  </si>
+  <si>
+    <t>Duquesne @ Air Force</t>
+  </si>
+  <si>
+    <t>-28.5</t>
+  </si>
+  <si>
+    <t>-22.0</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Fordham @ North Dakota State</t>
+  </si>
+  <si>
+    <t>-39.5</t>
+  </si>
+  <si>
+    <t>-49.9</t>
+  </si>
+  <si>
+    <t>-36.7</t>
+  </si>
+  <si>
+    <t>Northern Illinois @ Iowa</t>
+  </si>
+  <si>
+    <t>-31.2</t>
+  </si>
+  <si>
+    <t>-30.4</t>
+  </si>
+  <si>
+    <t>-27.0</t>
+  </si>
+  <si>
+    <t>Wyoming @ Colorado State</t>
+  </si>
+  <si>
+    <t>-5.2</t>
+  </si>
+  <si>
+    <t>-1.6</t>
+  </si>
+  <si>
+    <t>Central Michigan @ New Mexico</t>
+  </si>
+  <si>
+    <t>-10.0</t>
+  </si>
+  <si>
+    <t>-17.2</t>
+  </si>
+  <si>
+    <t>-10.7</t>
+  </si>
+  <si>
+    <t>UNLV @ Hawai'i</t>
+  </si>
+  <si>
+    <t>+3.0</t>
+  </si>
+  <si>
+    <t>+6.5</t>
+  </si>
+  <si>
+    <t>+0.1</t>
+  </si>
+  <si>
+    <t>Western Kentucky @ Nevada</t>
+  </si>
+  <si>
+    <t>+2.5</t>
+  </si>
+  <si>
+    <t>+5.0</t>
+  </si>
+  <si>
+    <t>+10.7</t>
+  </si>
+  <si>
     <t>2026 Mountain West Games -- Game by Game</t>
   </si>
   <si>
-    <t>Week</t>
-  </si>
-  <si>
-    <t>Matchup</t>
+    <t>Final Score</t>
   </si>
   <si>
     <t>Vegas Spread (Home)</t>
@@ -142,37 +325,19 @@
     <t>Actual Margin (Home)</t>
   </si>
   <si>
-    <t>Ridge Line</t>
-  </si>
-  <si>
     <t>Ridge Edge</t>
   </si>
   <si>
-    <t>Ridge Lean</t>
-  </si>
-  <si>
     <t>Ridge Result</t>
   </si>
   <si>
-    <t>XGBoost Line</t>
-  </si>
-  <si>
     <t>XGBoost Edge</t>
   </si>
   <si>
-    <t>XGBoost Lean</t>
-  </si>
-  <si>
     <t>XGBoost Result</t>
   </si>
   <si>
-    <t>Models Agree?</t>
-  </si>
-  <si>
-    <t>Jacksonville State @ North Dakota State</t>
-  </si>
-  <si>
-    <t>-6.8</t>
+    <t>7-33</t>
   </si>
   <si>
     <t>+26.0</t>
@@ -184,9 +349,6 @@
     <t>+9.6</t>
   </si>
   <si>
-    <t>Home</t>
-  </si>
-  <si>
     <t>Win</t>
   </si>
   <si>
@@ -196,13 +358,7 @@
     <t>+8.6</t>
   </si>
   <si>
-    <t>Yes</t>
-  </si>
-  <si>
-    <t>Hawai'i @ Stanford</t>
-  </si>
-  <si>
-    <t>-4.8</t>
+    <t>27-37</t>
   </si>
   <si>
     <t>+10.0</t>
@@ -214,9 +370,6 @@
     <t>-0.5</t>
   </si>
   <si>
-    <t>Away</t>
-  </si>
-  <si>
     <t>Lean only</t>
   </si>
   <si>
@@ -229,7 +382,7 @@
     <t>Loss</t>
   </si>
   <si>
-    <t>Memphis @ UNLV</t>
+    <t>27-21</t>
   </si>
   <si>
     <t>-6.0</t>
@@ -247,10 +400,7 @@
     <t>+1.8</t>
   </si>
   <si>
-    <t>San José State @ USC</t>
-  </si>
-  <si>
-    <t>-37.2</t>
+    <t>26-42</t>
   </si>
   <si>
     <t>+16.0</t>
@@ -370,9 +520,6 @@
     <t>Model Line (Home)</t>
   </si>
   <si>
-    <t>Market Line (Home)</t>
-  </si>
-  <si>
     <t>Spread Edge (pts)</t>
   </si>
   <si>
@@ -538,15 +685,15 @@
     <t>L</t>
   </si>
   <si>
+    <t>Jacksonville State @ North Dakota State,Memphis @ UNLV</t>
+  </si>
+  <si>
     <t>ML Parlay</t>
   </si>
   <si>
     <t>North Dakota State / UNLV</t>
   </si>
   <si>
-    <t>San José State @ Eastern Michigan</t>
-  </si>
-  <si>
     <t>Eastern Michigan -3.5</t>
   </si>
   <si>
@@ -626,9 +773,6 @@
   </si>
   <si>
     <t>Full history. Home elevation ~7,220 ft — coldest, highest venue in the league.</t>
-  </si>
-  <si>
-    <t>Jacksonville State @ North Dakota State,Memphis @ UNLV</t>
   </si>
 </sst>
 </file>
@@ -1127,111 +1271,111 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:A22"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="110" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" ht="18" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" s="3"/>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A8" s="3"/>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A9" s="4" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A13" s="3"/>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A14" s="4" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A18" s="3" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A20" s="3"/>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
-        <v>93</v>
+        <v>143</v>
       </c>
     </row>
   </sheetData>
@@ -1243,71 +1387,71 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="70" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="5" t="s">
-        <v>95</v>
+        <v>145</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>96</v>
+        <v>146</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" s="6" t="s">
-        <v>98</v>
+        <v>148</v>
       </c>
       <c r="B4" s="7">
         <v>100</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="s">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="B5" s="7">
         <v>2</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" s="6" t="s">
-        <v>102</v>
+        <v>152</v>
       </c>
       <c r="B6" s="7">
         <v>2</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="s">
-        <v>104</v>
+        <v>154</v>
       </c>
       <c r="B7" s="7">
         <v>-110</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>105</v>
+        <v>155</v>
       </c>
     </row>
   </sheetData>
@@ -1319,89 +1463,89 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:R29"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
     <col min="2" max="2" width="11" customWidth="1"/>
-    <col min="3" max="3" width="20.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.54296875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="18" bestFit="1" customWidth="1"/>
     <col min="5" max="6" width="16" customWidth="1"/>
-    <col min="7" max="7" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.54296875" bestFit="1" customWidth="1"/>
     <col min="9" max="10" width="11" customWidth="1"/>
     <col min="11" max="11" width="12" customWidth="1"/>
-    <col min="12" max="12" width="5.5703125" bestFit="1" customWidth="1"/>
-    <col min="13" max="14" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="5.54296875" bestFit="1" customWidth="1"/>
+    <col min="13" max="14" width="14.26953125" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="30" customWidth="1"/>
     <col min="16" max="16" width="16" customWidth="1"/>
     <col min="18" max="18" width="17" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
         <v>30</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>106</v>
+        <v>156</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>107</v>
+        <v>157</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>108</v>
+        <v>158</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>109</v>
+        <v>159</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>110</v>
+        <v>32</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>111</v>
+        <v>160</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>112</v>
+        <v>161</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>113</v>
+        <v>162</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>114</v>
+        <v>163</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>115</v>
+        <v>164</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>116</v>
+        <v>165</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>117</v>
+        <v>166</v>
       </c>
       <c r="N1" s="5" t="s">
-        <v>118</v>
+        <v>167</v>
       </c>
       <c r="O1" s="5" t="s">
-        <v>119</v>
+        <v>168</v>
       </c>
       <c r="P1" s="5" t="s">
-        <v>120</v>
+        <v>169</v>
       </c>
       <c r="R1" s="9" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>122</v>
+        <v>171</v>
       </c>
       <c r="C2" t="s">
-        <v>123</v>
+        <v>172</v>
       </c>
       <c r="D2" t="s">
-        <v>124</v>
+        <v>173</v>
       </c>
       <c r="E2">
         <v>-32.200000000000003</v>
@@ -1442,18 +1586,18 @@
       <c r="O2" s="8"/>
       <c r="P2" s="8"/>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>122</v>
+        <v>171</v>
       </c>
       <c r="C3" t="s">
-        <v>125</v>
+        <v>174</v>
       </c>
       <c r="D3" t="s">
-        <v>126</v>
+        <v>175</v>
       </c>
       <c r="E3">
         <v>-16.399999999999999</v>
@@ -1492,18 +1636,18 @@
         <v>Over</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>1</v>
       </c>
       <c r="B4" t="s">
-        <v>122</v>
+        <v>171</v>
       </c>
       <c r="C4" t="s">
-        <v>127</v>
+        <v>176</v>
       </c>
       <c r="D4" t="s">
-        <v>128</v>
+        <v>177</v>
       </c>
       <c r="E4">
         <v>-4.3</v>
@@ -1542,18 +1686,18 @@
         <v>Over</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>1</v>
       </c>
       <c r="B5" t="s">
-        <v>129</v>
+        <v>178</v>
       </c>
       <c r="C5" t="s">
-        <v>130</v>
+        <v>179</v>
       </c>
       <c r="D5" t="s">
-        <v>131</v>
+        <v>180</v>
       </c>
       <c r="E5">
         <v>-9.9</v>
@@ -1592,21 +1736,21 @@
         <v>Pass</v>
       </c>
       <c r="R5" s="6" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>1</v>
       </c>
       <c r="B6" t="s">
-        <v>133</v>
+        <v>182</v>
       </c>
       <c r="C6" t="s">
-        <v>123</v>
+        <v>172</v>
       </c>
       <c r="D6" t="s">
-        <v>134</v>
+        <v>183</v>
       </c>
       <c r="E6">
         <v>-12.8</v>
@@ -1645,21 +1789,21 @@
         <v>Pass</v>
       </c>
       <c r="R6" s="6" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A7" s="10">
         <v>1</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>135</v>
+        <v>184</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>136</v>
+        <v>185</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>132</v>
+        <v>181</v>
       </c>
       <c r="E7" s="10">
         <v>-22</v>
@@ -1698,21 +1842,21 @@
         <v>Under</v>
       </c>
       <c r="R7" s="6" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>1</v>
       </c>
       <c r="B8" t="s">
-        <v>135</v>
+        <v>184</v>
       </c>
       <c r="C8" t="s">
-        <v>138</v>
+        <v>187</v>
       </c>
       <c r="D8" t="s">
-        <v>126</v>
+        <v>175</v>
       </c>
       <c r="E8">
         <v>-49.9</v>
@@ -1751,21 +1895,21 @@
         <v>Pass</v>
       </c>
       <c r="R8" s="6" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>1</v>
       </c>
       <c r="B9" t="s">
-        <v>135</v>
+        <v>184</v>
       </c>
       <c r="C9" t="s">
-        <v>140</v>
+        <v>189</v>
       </c>
       <c r="D9" t="s">
-        <v>141</v>
+        <v>190</v>
       </c>
       <c r="E9">
         <v>-30.4</v>
@@ -1804,21 +1948,21 @@
         <v>Over</v>
       </c>
       <c r="R9" s="6" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>1</v>
       </c>
       <c r="B10" t="s">
-        <v>135</v>
+        <v>184</v>
       </c>
       <c r="C10" t="s">
-        <v>142</v>
+        <v>191</v>
       </c>
       <c r="D10" t="s">
-        <v>143</v>
+        <v>192</v>
       </c>
       <c r="E10">
         <v>-5.2</v>
@@ -1857,21 +2001,21 @@
         <v>Over</v>
       </c>
       <c r="R10" s="6" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>1</v>
       </c>
       <c r="B11" t="s">
-        <v>135</v>
+        <v>184</v>
       </c>
       <c r="C11" t="s">
-        <v>144</v>
+        <v>193</v>
       </c>
       <c r="D11" t="s">
-        <v>145</v>
+        <v>194</v>
       </c>
       <c r="E11">
         <v>-33.9</v>
@@ -1910,21 +2054,21 @@
         <v>Pass</v>
       </c>
       <c r="R11" s="6" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>1</v>
       </c>
       <c r="B12" t="s">
-        <v>146</v>
+        <v>195</v>
       </c>
       <c r="C12" t="s">
-        <v>131</v>
+        <v>180</v>
       </c>
       <c r="D12" t="s">
-        <v>127</v>
+        <v>176</v>
       </c>
       <c r="E12">
         <v>6.5</v>
@@ -1963,21 +2107,21 @@
         <v>Pass</v>
       </c>
       <c r="R12" s="6" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>1</v>
       </c>
       <c r="B13" t="s">
-        <v>146</v>
+        <v>195</v>
       </c>
       <c r="C13" t="s">
-        <v>147</v>
+        <v>196</v>
       </c>
       <c r="D13" t="s">
-        <v>139</v>
+        <v>188</v>
       </c>
       <c r="E13">
         <v>-17.2</v>
@@ -2016,18 +2160,18 @@
         <v>Over</v>
       </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>1</v>
       </c>
       <c r="B14" t="s">
-        <v>146</v>
+        <v>195</v>
       </c>
       <c r="C14" t="s">
-        <v>148</v>
+        <v>197</v>
       </c>
       <c r="D14" t="s">
-        <v>137</v>
+        <v>186</v>
       </c>
       <c r="E14">
         <v>5</v>
@@ -2066,7 +2210,7 @@
         <v>Pass</v>
       </c>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.35">
       <c r="G15" s="6"/>
       <c r="H15" s="6"/>
       <c r="K15" s="6"/>
@@ -2074,7 +2218,7 @@
       <c r="M15" s="6"/>
       <c r="N15" s="6"/>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.35">
       <c r="G16" s="6"/>
       <c r="H16" s="6"/>
       <c r="K16" s="6"/>
@@ -2082,7 +2226,7 @@
       <c r="M16" s="6"/>
       <c r="N16" s="6"/>
     </row>
-    <row r="17" spans="7:14" x14ac:dyDescent="0.25">
+    <row r="17" spans="7:14" x14ac:dyDescent="0.35">
       <c r="G17" s="6"/>
       <c r="H17" s="6"/>
       <c r="K17" s="6"/>
@@ -2090,7 +2234,7 @@
       <c r="M17" s="6"/>
       <c r="N17" s="6"/>
     </row>
-    <row r="18" spans="7:14" x14ac:dyDescent="0.25">
+    <row r="18" spans="7:14" x14ac:dyDescent="0.35">
       <c r="G18" s="6"/>
       <c r="H18" s="6"/>
       <c r="K18" s="6"/>
@@ -2098,7 +2242,7 @@
       <c r="M18" s="6"/>
       <c r="N18" s="6"/>
     </row>
-    <row r="19" spans="7:14" x14ac:dyDescent="0.25">
+    <row r="19" spans="7:14" x14ac:dyDescent="0.35">
       <c r="G19" s="6"/>
       <c r="H19" s="6"/>
       <c r="K19" s="6"/>
@@ -2106,7 +2250,7 @@
       <c r="M19" s="6"/>
       <c r="N19" s="6"/>
     </row>
-    <row r="20" spans="7:14" x14ac:dyDescent="0.25">
+    <row r="20" spans="7:14" x14ac:dyDescent="0.35">
       <c r="G20" s="6"/>
       <c r="H20" s="6"/>
       <c r="K20" s="6"/>
@@ -2114,7 +2258,7 @@
       <c r="M20" s="6"/>
       <c r="N20" s="6"/>
     </row>
-    <row r="21" spans="7:14" x14ac:dyDescent="0.25">
+    <row r="21" spans="7:14" x14ac:dyDescent="0.35">
       <c r="G21" s="6"/>
       <c r="H21" s="6"/>
       <c r="K21" s="6"/>
@@ -2122,7 +2266,7 @@
       <c r="M21" s="6"/>
       <c r="N21" s="6"/>
     </row>
-    <row r="22" spans="7:14" x14ac:dyDescent="0.25">
+    <row r="22" spans="7:14" x14ac:dyDescent="0.35">
       <c r="G22" s="6"/>
       <c r="H22" s="6"/>
       <c r="K22" s="6"/>
@@ -2130,7 +2274,7 @@
       <c r="M22" s="6"/>
       <c r="N22" s="6"/>
     </row>
-    <row r="23" spans="7:14" x14ac:dyDescent="0.25">
+    <row r="23" spans="7:14" x14ac:dyDescent="0.35">
       <c r="G23" s="6"/>
       <c r="H23" s="6"/>
       <c r="K23" s="6"/>
@@ -2138,7 +2282,7 @@
       <c r="M23" s="6"/>
       <c r="N23" s="6"/>
     </row>
-    <row r="24" spans="7:14" x14ac:dyDescent="0.25">
+    <row r="24" spans="7:14" x14ac:dyDescent="0.35">
       <c r="G24" s="6"/>
       <c r="H24" s="6"/>
       <c r="K24" s="6"/>
@@ -2146,7 +2290,7 @@
       <c r="M24" s="6"/>
       <c r="N24" s="6"/>
     </row>
-    <row r="25" spans="7:14" x14ac:dyDescent="0.25">
+    <row r="25" spans="7:14" x14ac:dyDescent="0.35">
       <c r="G25" s="6"/>
       <c r="H25" s="6"/>
       <c r="K25" s="6"/>
@@ -2154,7 +2298,7 @@
       <c r="M25" s="6"/>
       <c r="N25" s="6"/>
     </row>
-    <row r="26" spans="7:14" x14ac:dyDescent="0.25">
+    <row r="26" spans="7:14" x14ac:dyDescent="0.35">
       <c r="G26" s="6"/>
       <c r="H26" s="6"/>
       <c r="K26" s="6"/>
@@ -2162,7 +2306,7 @@
       <c r="M26" s="6"/>
       <c r="N26" s="6"/>
     </row>
-    <row r="27" spans="7:14" x14ac:dyDescent="0.25">
+    <row r="27" spans="7:14" x14ac:dyDescent="0.35">
       <c r="G27" s="6"/>
       <c r="H27" s="6"/>
       <c r="K27" s="6"/>
@@ -2170,7 +2314,7 @@
       <c r="M27" s="6"/>
       <c r="N27" s="6"/>
     </row>
-    <row r="28" spans="7:14" x14ac:dyDescent="0.25">
+    <row r="28" spans="7:14" x14ac:dyDescent="0.35">
       <c r="G28" s="6"/>
       <c r="H28" s="6"/>
       <c r="K28" s="6"/>
@@ -2178,7 +2322,7 @@
       <c r="M28" s="6"/>
       <c r="N28" s="6"/>
     </row>
-    <row r="29" spans="7:14" x14ac:dyDescent="0.25">
+    <row r="29" spans="7:14" x14ac:dyDescent="0.35">
       <c r="G29" s="6"/>
       <c r="H29" s="6"/>
       <c r="K29" s="6"/>
@@ -2210,13 +2354,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:M44"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
     <col min="2" max="2" width="6" customWidth="1"/>
-    <col min="3" max="3" width="37.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="37.453125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10" customWidth="1"/>
-    <col min="5" max="5" width="22.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.26953125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="11" customWidth="1"/>
     <col min="7" max="7" width="14" customWidth="1"/>
     <col min="8" max="9" width="12" customWidth="1"/>
@@ -2226,9 +2370,9 @@
     <col min="13" max="13" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
-        <v>106</v>
+        <v>156</v>
       </c>
       <c r="B1" s="5" t="s">
         <v>30</v>
@@ -2237,51 +2381,51 @@
         <v>31</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>149</v>
+        <v>198</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>150</v>
+        <v>199</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>151</v>
+        <v>200</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>152</v>
+        <v>201</v>
       </c>
       <c r="H1" s="5" t="s">
-        <v>153</v>
+        <v>202</v>
       </c>
       <c r="I1" s="5" t="s">
-        <v>154</v>
+        <v>203</v>
       </c>
       <c r="J1" s="5" t="s">
-        <v>155</v>
+        <v>204</v>
       </c>
       <c r="K1" s="5" t="s">
-        <v>156</v>
+        <v>205</v>
       </c>
       <c r="L1" s="5" t="s">
-        <v>157</v>
+        <v>206</v>
       </c>
       <c r="M1" s="5" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>122</v>
+        <v>171</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D2" t="s">
-        <v>159</v>
+        <v>208</v>
       </c>
       <c r="E2" t="s">
-        <v>160</v>
+        <v>209</v>
       </c>
       <c r="F2">
         <v>-7.5</v>
@@ -2300,7 +2444,7 @@
         <v>0.5</v>
       </c>
       <c r="K2" t="s">
-        <v>161</v>
+        <v>210</v>
       </c>
       <c r="L2" s="6">
         <f t="shared" ref="L2:L41" si="0">IF(K2="W",IF(G2&lt;0,H2*100/ABS(G2),H2*G2/100),IF(K2="L",-H2,0))</f>
@@ -2311,21 +2455,21 @@
         <v>101</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>122</v>
+        <v>171</v>
       </c>
       <c r="B3">
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D3" t="s">
-        <v>162</v>
+        <v>211</v>
       </c>
       <c r="E3" t="s">
-        <v>163</v>
+        <v>212</v>
       </c>
       <c r="G3">
         <v>-285</v>
@@ -2338,7 +2482,7 @@
         <v/>
       </c>
       <c r="K3" t="s">
-        <v>161</v>
+        <v>210</v>
       </c>
       <c r="L3" s="6">
         <f t="shared" si="0"/>
@@ -2349,21 +2493,21 @@
         <v>102.75438596491227</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>122</v>
+        <v>171</v>
       </c>
       <c r="B4">
         <v>1</v>
       </c>
       <c r="C4" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="D4" t="s">
-        <v>162</v>
+        <v>211</v>
       </c>
       <c r="E4" t="s">
-        <v>164</v>
+        <v>213</v>
       </c>
       <c r="G4">
         <v>-178</v>
@@ -2376,7 +2520,7 @@
         <v/>
       </c>
       <c r="K4" t="s">
-        <v>165</v>
+        <v>214</v>
       </c>
       <c r="L4" s="6">
         <f t="shared" si="0"/>
@@ -2387,21 +2531,21 @@
         <v>97.754385964912274</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>122</v>
+        <v>171</v>
       </c>
       <c r="B5">
         <v>1</v>
       </c>
       <c r="C5" t="s">
-        <v>196</v>
+        <v>215</v>
       </c>
       <c r="D5" t="s">
-        <v>166</v>
+        <v>216</v>
       </c>
       <c r="E5" t="s">
-        <v>167</v>
+        <v>217</v>
       </c>
       <c r="G5">
         <v>110</v>
@@ -2414,7 +2558,7 @@
         <v/>
       </c>
       <c r="K5" t="s">
-        <v>165</v>
+        <v>214</v>
       </c>
       <c r="L5" s="6">
         <f t="shared" si="0"/>
@@ -2425,21 +2569,21 @@
         <v>94.754385964912274</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>133</v>
+        <v>182</v>
       </c>
       <c r="B6">
         <v>1</v>
       </c>
       <c r="C6" t="s">
-        <v>168</v>
+        <v>56</v>
       </c>
       <c r="D6" t="s">
-        <v>159</v>
+        <v>208</v>
       </c>
       <c r="E6" t="s">
-        <v>169</v>
+        <v>218</v>
       </c>
       <c r="F6">
         <v>-3.5</v>
@@ -2463,21 +2607,21 @@
         <v>94.754385964912274</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" s="10" t="s">
-        <v>135</v>
+        <v>184</v>
       </c>
       <c r="B7">
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>170</v>
+        <v>219</v>
       </c>
       <c r="D7" t="s">
-        <v>166</v>
+        <v>216</v>
       </c>
       <c r="E7" t="s">
-        <v>171</v>
+        <v>220</v>
       </c>
       <c r="G7">
         <v>149</v>
@@ -2498,7 +2642,7 @@
         <v>94.754385964912274</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="J8" s="6" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2512,7 +2656,7 @@
         <v>94.754385964912274</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="J9" s="6" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2526,7 +2670,7 @@
         <v>94.754385964912274</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="J10" s="6" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2540,7 +2684,7 @@
         <v>94.754385964912274</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="J11" s="6" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2554,7 +2698,7 @@
         <v>94.754385964912274</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="J12" s="6" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2568,7 +2712,7 @@
         <v>94.754385964912274</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="J13" s="6" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2582,7 +2726,7 @@
         <v>94.754385964912274</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
       <c r="J14" s="6" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2596,7 +2740,7 @@
         <v>94.754385964912274</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
       <c r="J15" s="6" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2610,7 +2754,7 @@
         <v>94.754385964912274</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
       <c r="J16" s="6" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2624,7 +2768,7 @@
         <v>94.754385964912274</v>
       </c>
     </row>
-    <row r="17" spans="10:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="10:13" x14ac:dyDescent="0.35">
       <c r="J17" s="6" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2638,7 +2782,7 @@
         <v>94.754385964912274</v>
       </c>
     </row>
-    <row r="18" spans="10:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="10:13" x14ac:dyDescent="0.35">
       <c r="J18" s="6" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2652,7 +2796,7 @@
         <v>94.754385964912274</v>
       </c>
     </row>
-    <row r="19" spans="10:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="10:13" x14ac:dyDescent="0.35">
       <c r="J19" s="6" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2666,7 +2810,7 @@
         <v>94.754385964912274</v>
       </c>
     </row>
-    <row r="20" spans="10:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="10:13" x14ac:dyDescent="0.35">
       <c r="J20" s="6" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2680,7 +2824,7 @@
         <v>94.754385964912274</v>
       </c>
     </row>
-    <row r="21" spans="10:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="10:13" x14ac:dyDescent="0.35">
       <c r="J21" s="6" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2694,7 +2838,7 @@
         <v>94.754385964912274</v>
       </c>
     </row>
-    <row r="22" spans="10:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="10:13" x14ac:dyDescent="0.35">
       <c r="J22" s="6" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2708,7 +2852,7 @@
         <v>94.754385964912274</v>
       </c>
     </row>
-    <row r="23" spans="10:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="10:13" x14ac:dyDescent="0.35">
       <c r="J23" s="6" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2722,7 +2866,7 @@
         <v>94.754385964912274</v>
       </c>
     </row>
-    <row r="24" spans="10:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="10:13" x14ac:dyDescent="0.35">
       <c r="J24" s="6" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2736,7 +2880,7 @@
         <v>94.754385964912274</v>
       </c>
     </row>
-    <row r="25" spans="10:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="10:13" x14ac:dyDescent="0.35">
       <c r="J25" s="6" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2750,7 +2894,7 @@
         <v>94.754385964912274</v>
       </c>
     </row>
-    <row r="26" spans="10:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="10:13" x14ac:dyDescent="0.35">
       <c r="J26" s="6" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2764,7 +2908,7 @@
         <v>94.754385964912274</v>
       </c>
     </row>
-    <row r="27" spans="10:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="10:13" x14ac:dyDescent="0.35">
       <c r="J27" s="6" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2778,7 +2922,7 @@
         <v>94.754385964912274</v>
       </c>
     </row>
-    <row r="28" spans="10:13" x14ac:dyDescent="0.25">
+    <row r="28" spans="10:13" x14ac:dyDescent="0.35">
       <c r="J28" s="6" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2792,7 +2936,7 @@
         <v>94.754385964912274</v>
       </c>
     </row>
-    <row r="29" spans="10:13" x14ac:dyDescent="0.25">
+    <row r="29" spans="10:13" x14ac:dyDescent="0.35">
       <c r="J29" s="6" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2806,7 +2950,7 @@
         <v>94.754385964912274</v>
       </c>
     </row>
-    <row r="30" spans="10:13" x14ac:dyDescent="0.25">
+    <row r="30" spans="10:13" x14ac:dyDescent="0.35">
       <c r="J30" s="6" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2820,7 +2964,7 @@
         <v>94.754385964912274</v>
       </c>
     </row>
-    <row r="31" spans="10:13" x14ac:dyDescent="0.25">
+    <row r="31" spans="10:13" x14ac:dyDescent="0.35">
       <c r="J31" s="6" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2834,7 +2978,7 @@
         <v>94.754385964912274</v>
       </c>
     </row>
-    <row r="32" spans="10:13" x14ac:dyDescent="0.25">
+    <row r="32" spans="10:13" x14ac:dyDescent="0.35">
       <c r="J32" s="6" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2848,7 +2992,7 @@
         <v>94.754385964912274</v>
       </c>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.35">
       <c r="J33" s="6" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2862,7 +3006,7 @@
         <v>94.754385964912274</v>
       </c>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.35">
       <c r="J34" s="6" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2876,7 +3020,7 @@
         <v>94.754385964912274</v>
       </c>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.35">
       <c r="J35" s="6" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2890,7 +3034,7 @@
         <v>94.754385964912274</v>
       </c>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.35">
       <c r="J36" s="6" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2904,7 +3048,7 @@
         <v>94.754385964912274</v>
       </c>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.35">
       <c r="J37" s="6" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2918,7 +3062,7 @@
         <v>94.754385964912274</v>
       </c>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.35">
       <c r="J38" s="6" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2932,7 +3076,7 @@
         <v>94.754385964912274</v>
       </c>
     </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.35">
       <c r="J39" s="6" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2946,7 +3090,7 @@
         <v>94.754385964912274</v>
       </c>
     </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.35">
       <c r="J40" s="6" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2960,7 +3104,7 @@
         <v>94.754385964912274</v>
       </c>
     </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:13" x14ac:dyDescent="0.35">
       <c r="J41" s="6" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -2974,9 +3118,9 @@
         <v>94.754385964912274</v>
       </c>
     </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A44" s="2" t="s">
-        <v>172</v>
+        <v>221</v>
       </c>
     </row>
   </sheetData>
@@ -2988,11 +3132,11 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:I11"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="37" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.1796875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="17" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
     <col min="6" max="7" width="10" customWidth="1"/>
@@ -3000,44 +3144,44 @@
     <col min="9" max="9" width="60" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
-        <v>173</v>
+        <v>222</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>174</v>
+        <v>223</v>
       </c>
       <c r="C1" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>226</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A2" s="6" t="s">
         <v>175</v>
       </c>
-      <c r="D1" s="5" t="s">
-        <v>176</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>177</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>178</v>
-      </c>
-      <c r="G1" s="5" t="s">
-        <v>179</v>
-      </c>
-      <c r="H1" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="I1" s="5" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
-        <v>126</v>
-      </c>
       <c r="B2" s="6" t="s">
-        <v>181</v>
+        <v>230</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>182</v>
+        <v>231</v>
       </c>
       <c r="D2" s="8">
         <v>1731.3</v>
@@ -3055,18 +3199,18 @@
         <v>117</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" s="6" t="s">
-        <v>131</v>
+        <v>180</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>184</v>
+        <v>233</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>185</v>
+        <v>234</v>
       </c>
       <c r="D3" s="8">
         <v>1585.5</v>
@@ -3084,18 +3228,18 @@
         <v>63</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" s="6" t="s">
-        <v>139</v>
+        <v>188</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>184</v>
+        <v>233</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>185</v>
+        <v>234</v>
       </c>
       <c r="D4" s="8">
         <v>1566.5</v>
@@ -3113,18 +3257,18 @@
         <v>87</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" s="6" t="s">
-        <v>127</v>
+        <v>176</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>184</v>
+        <v>233</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>185</v>
+        <v>234</v>
       </c>
       <c r="D5" s="8">
         <v>1519.4</v>
@@ -3142,18 +3286,18 @@
         <v>124</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" s="6" t="s">
-        <v>132</v>
+        <v>181</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>184</v>
+        <v>233</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>185</v>
+        <v>234</v>
       </c>
       <c r="D6" s="8">
         <v>1473</v>
@@ -3171,18 +3315,18 @@
         <v>141</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" s="6" t="s">
-        <v>142</v>
+        <v>191</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>184</v>
+        <v>233</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>185</v>
+        <v>234</v>
       </c>
       <c r="D7" s="8">
         <v>1399.9</v>
@@ -3200,18 +3344,18 @@
         <v>114</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" s="6" t="s">
-        <v>140</v>
+        <v>189</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>191</v>
+        <v>240</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>182</v>
+        <v>231</v>
       </c>
       <c r="D8" s="8">
         <v>1394.5</v>
@@ -3229,18 +3373,18 @@
         <v>82</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" s="6" t="s">
-        <v>123</v>
+        <v>172</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>184</v>
+        <v>233</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>185</v>
+        <v>234</v>
       </c>
       <c r="D9" s="8">
         <v>1408.4</v>
@@ -3258,18 +3402,18 @@
         <v>129</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" s="6" t="s">
-        <v>137</v>
+        <v>186</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>184</v>
+        <v>233</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>185</v>
+        <v>234</v>
       </c>
       <c r="D10" s="8">
         <v>1361.9</v>
@@ -3287,18 +3431,18 @@
         <v>98</v>
       </c>
       <c r="I10" s="2" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A11" s="6" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="6" t="s">
-        <v>144</v>
-      </c>
       <c r="B11" s="6" t="s">
-        <v>194</v>
+        <v>243</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>182</v>
+        <v>231</v>
       </c>
       <c r="D11" s="8">
         <v>1302.8</v>
@@ -3316,7 +3460,7 @@
         <v>92</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>195</v>
+        <v>244</v>
       </c>
     </row>
   </sheetData>
@@ -3327,36 +3471,37 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:M25"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:N42"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="136" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="26" customWidth="1"/>
-    <col min="3" max="4" width="18" customWidth="1"/>
-    <col min="5" max="6" width="12" customWidth="1"/>
-    <col min="7" max="7" width="11" customWidth="1"/>
-    <col min="8" max="10" width="12" customWidth="1"/>
-    <col min="11" max="11" width="11" customWidth="1"/>
-    <col min="12" max="12" width="12" customWidth="1"/>
-    <col min="13" max="13" width="13" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="5" width="18" customWidth="1"/>
+    <col min="6" max="7" width="12" customWidth="1"/>
+    <col min="8" max="8" width="11" customWidth="1"/>
+    <col min="9" max="11" width="12" customWidth="1"/>
+    <col min="12" max="12" width="11" customWidth="1"/>
+    <col min="13" max="13" width="12" customWidth="1"/>
+    <col min="14" max="14" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="18" x14ac:dyDescent="0.4">
       <c r="A1" s="11" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="12" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" s="13" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" ht="26" x14ac:dyDescent="0.35">
       <c r="A5" s="14" t="s">
         <v>3</v>
       </c>
@@ -3382,7 +3527,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="15" t="s">
         <v>11</v>
       </c>
@@ -3408,7 +3553,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" s="15" t="s">
         <v>14</v>
       </c>
@@ -3434,7 +3579,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" s="15" t="s">
         <v>17</v>
       </c>
@@ -3442,10 +3587,10 @@
         <v>8441</v>
       </c>
       <c r="C8" s="15">
-        <v>6519</v>
+        <v>6518</v>
       </c>
       <c r="D8" s="15">
-        <v>3260</v>
+        <v>3259</v>
       </c>
       <c r="E8" s="15">
         <v>3259</v>
@@ -3460,7 +3605,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="15" t="s">
         <v>20</v>
       </c>
@@ -3486,12 +3631,12 @@
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" s="13" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" ht="26" x14ac:dyDescent="0.35">
       <c r="A12" s="14" t="s">
         <v>3</v>
       </c>
@@ -3517,7 +3662,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" s="15" t="s">
         <v>11</v>
       </c>
@@ -3543,7 +3688,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" s="15" t="s">
         <v>14</v>
       </c>
@@ -3569,7 +3714,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" s="15" t="s">
         <v>17</v>
       </c>
@@ -3595,7 +3740,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" s="15" t="s">
         <v>20</v>
       </c>
@@ -3621,17 +3766,17 @@
         <v>27</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" s="12" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20" s="13" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="21" spans="1:13" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" ht="26" x14ac:dyDescent="0.35">
       <c r="A21" s="14" t="s">
         <v>30</v>
       </c>
@@ -3656,184 +3801,568 @@
       <c r="H21" s="14" t="s">
         <v>37</v>
       </c>
-      <c r="I21" s="14" t="s">
-        <v>38</v>
-      </c>
-      <c r="J21" s="14" t="s">
-        <v>39</v>
-      </c>
-      <c r="K21" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="L21" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="M21" s="14" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22" s="15">
         <v>1</v>
       </c>
       <c r="B22" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="C22" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="D22" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="E22" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="F22" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="G22" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="H22" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="C22" s="15" t="s">
-        <v>44</v>
-      </c>
-      <c r="D22" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="E22" s="15" t="s">
-        <v>46</v>
-      </c>
-      <c r="F22" s="15" t="s">
-        <v>47</v>
-      </c>
-      <c r="G22" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="H22" s="16" t="s">
-        <v>49</v>
-      </c>
-      <c r="I22" s="15" t="s">
-        <v>50</v>
-      </c>
-      <c r="J22" s="15" t="s">
-        <v>51</v>
-      </c>
-      <c r="K22" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="L22" s="16" t="s">
-        <v>49</v>
-      </c>
-      <c r="M22" s="15" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" s="15">
         <v>1</v>
       </c>
       <c r="B23" s="15" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="C23" s="15" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="E23" s="15" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="F23" s="15" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="G23" s="15" t="s">
-        <v>58</v>
+        <v>48</v>
       </c>
       <c r="H23" s="15" t="s">
-        <v>59</v>
-      </c>
-      <c r="I23" s="15" t="s">
-        <v>60</v>
-      </c>
-      <c r="J23" s="15" t="s">
-        <v>61</v>
-      </c>
-      <c r="K23" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="L23" s="17" t="s">
-        <v>62</v>
-      </c>
-      <c r="M23" s="15" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" s="15">
         <v>1</v>
       </c>
       <c r="B24" s="15" t="s">
-        <v>63</v>
+        <v>49</v>
       </c>
       <c r="C24" s="15" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="D24" s="15" t="s">
-        <v>64</v>
+        <v>51</v>
       </c>
       <c r="E24" s="15" t="s">
-        <v>65</v>
+        <v>52</v>
       </c>
       <c r="F24" s="15" t="s">
-        <v>66</v>
+        <v>42</v>
       </c>
       <c r="G24" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="H24" s="17" t="s">
-        <v>62</v>
-      </c>
-      <c r="I24" s="15" t="s">
-        <v>67</v>
-      </c>
-      <c r="J24" s="15" t="s">
-        <v>68</v>
-      </c>
-      <c r="K24" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="L24" s="15" t="s">
-        <v>59</v>
-      </c>
-      <c r="M24" s="15" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+        <v>42</v>
+      </c>
+      <c r="H24" s="15" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25" s="15">
         <v>1</v>
       </c>
       <c r="B25" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="C25" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="D25" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="E25" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="F25" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="G25" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="H25" s="15" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A26" s="15">
+        <v>1</v>
+      </c>
+      <c r="B26" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="C26" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="D26" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="E26" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="F26" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="G26" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="H26" s="15" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A27" s="15">
+        <v>1</v>
+      </c>
+      <c r="B27" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="C27" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="D27" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="E27" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="F27" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="G27" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="H27" s="15" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A28" s="15">
+        <v>1</v>
+      </c>
+      <c r="B28" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="C28" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="D28" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="E28" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="F28" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="G28" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="H28" s="15" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A29" s="15">
+        <v>1</v>
+      </c>
+      <c r="B29" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="C29" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="C25" s="15" t="s">
+      <c r="D29" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="D25" s="15" t="s">
+      <c r="E29" s="15" t="s">
         <v>71</v>
       </c>
-      <c r="E25" s="15" t="s">
+      <c r="F29" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="G29" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="H29" s="15" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A30" s="15">
+        <v>1</v>
+      </c>
+      <c r="B30" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="F25" s="15" t="s">
+      <c r="C30" s="15" t="s">
         <v>73</v>
       </c>
-      <c r="G25" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="H25" s="16" t="s">
+      <c r="D30" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="E30" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="F30" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="G30" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="H30" s="15" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A31" s="15">
+        <v>1</v>
+      </c>
+      <c r="B31" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="C31" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="D31" s="15" t="s">
+        <v>77</v>
+      </c>
+      <c r="E31" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="F31" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="G31" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="H31" s="15" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A32" s="15">
+        <v>1</v>
+      </c>
+      <c r="B32" s="15" t="s">
+        <v>79</v>
+      </c>
+      <c r="C32" s="15" t="s">
+        <v>80</v>
+      </c>
+      <c r="D32" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="E32" s="15" t="s">
+        <v>82</v>
+      </c>
+      <c r="F32" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="G32" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="H32" s="15" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A33" s="15">
+        <v>1</v>
+      </c>
+      <c r="B33" s="15" t="s">
+        <v>83</v>
+      </c>
+      <c r="C33" s="15" t="s">
+        <v>84</v>
+      </c>
+      <c r="D33" s="15" t="s">
+        <v>85</v>
+      </c>
+      <c r="E33" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="F33" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="G33" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="H33" s="15" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A34" s="15">
+        <v>1</v>
+      </c>
+      <c r="B34" s="15" t="s">
+        <v>87</v>
+      </c>
+      <c r="C34" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="D34" s="15" t="s">
+        <v>89</v>
+      </c>
+      <c r="E34" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="F34" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="G34" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="H34" s="15" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A37" s="13" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" ht="26" x14ac:dyDescent="0.35">
+      <c r="A38" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B38" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="C38" s="14" t="s">
+        <v>92</v>
+      </c>
+      <c r="D38" s="14" t="s">
+        <v>93</v>
+      </c>
+      <c r="E38" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="F38" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="G38" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="H38" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="I38" s="14" t="s">
+        <v>96</v>
+      </c>
+      <c r="J38" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="K38" s="14" t="s">
+        <v>97</v>
+      </c>
+      <c r="L38" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="M38" s="14" t="s">
+        <v>98</v>
+      </c>
+      <c r="N38" s="14" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A39" s="15">
+        <v>1</v>
+      </c>
+      <c r="B39" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="C39" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="D39" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="E39" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="F39" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="G39" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="H39" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="I39" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="J39" s="15" t="s">
+        <v>104</v>
+      </c>
+      <c r="K39" s="15" t="s">
+        <v>105</v>
+      </c>
+      <c r="L39" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="M39" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="N39" s="15" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A40" s="15">
+        <v>1</v>
+      </c>
+      <c r="B40" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="I25" s="15" t="s">
-        <v>74</v>
-      </c>
-      <c r="J25" s="15" t="s">
-        <v>75</v>
-      </c>
-      <c r="K25" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="L25" s="16" t="s">
-        <v>49</v>
-      </c>
-      <c r="M25" s="15" t="s">
-        <v>52</v>
+      <c r="C40" s="15" t="s">
+        <v>106</v>
+      </c>
+      <c r="D40" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="E40" s="15" t="s">
+        <v>107</v>
+      </c>
+      <c r="F40" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="G40" s="15" t="s">
+        <v>109</v>
+      </c>
+      <c r="H40" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="I40" s="15" t="s">
+        <v>110</v>
+      </c>
+      <c r="J40" s="15" t="s">
+        <v>111</v>
+      </c>
+      <c r="K40" s="15" t="s">
+        <v>112</v>
+      </c>
+      <c r="L40" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="M40" s="17" t="s">
+        <v>113</v>
+      </c>
+      <c r="N40" s="15" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="41" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A41" s="15">
+        <v>1</v>
+      </c>
+      <c r="B41" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="C41" s="15" t="s">
+        <v>114</v>
+      </c>
+      <c r="D41" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="E41" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="F41" s="15" t="s">
+        <v>116</v>
+      </c>
+      <c r="G41" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="H41" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="I41" s="17" t="s">
+        <v>113</v>
+      </c>
+      <c r="J41" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="K41" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="L41" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="M41" s="15" t="s">
+        <v>110</v>
+      </c>
+      <c r="N41" s="15" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="42" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A42" s="15">
+        <v>1</v>
+      </c>
+      <c r="B42" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="C42" s="15" t="s">
+        <v>120</v>
+      </c>
+      <c r="D42" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="E42" s="15" t="s">
+        <v>121</v>
+      </c>
+      <c r="F42" s="15" t="s">
+        <v>122</v>
+      </c>
+      <c r="G42" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="H42" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="I42" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="J42" s="15" t="s">
+        <v>124</v>
+      </c>
+      <c r="K42" s="15" t="s">
+        <v>125</v>
+      </c>
+      <c r="L42" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="M42" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="N42" s="15" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Bet Log entries
</commit_message>
<xml_diff>
--- a/excel/MW_Handicapping_Tracker.xlsx
+++ b/excel/MW_Handicapping_Tracker.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="1" activeTab="5" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="1" activeTab="3" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Read Me" sheetId="1" state="visible" r:id="rId1"/>
@@ -2123,6 +2123,11 @@
         <f>IF(I6="","",I6-F6)</f>
         <v/>
       </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
       <c r="L6" s="6">
         <f>IF(K6="W",IF(G6&lt;0,H6*100/ABS(G6),H6*G6/100),IF(K6="L",-H6,0))</f>
         <v/>
@@ -2166,6 +2171,11 @@
         <f>IF(I7="","",I7-F7)</f>
         <v/>
       </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
       <c r="L7" s="6">
         <f>IF(K7="W",IF(G7&lt;0,H7*100/ABS(G7),H7*G7/100),IF(K7="L",-H7,0))</f>
         <v/>
@@ -2176,10 +2186,50 @@
       </c>
     </row>
     <row r="8">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Wyoming @  Colorado State</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Spread</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Colorado State</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>-2.5</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-110</v>
+      </c>
+      <c r="H8" t="n">
+        <v>2</v>
+      </c>
+      <c r="I8" t="n">
+        <v>-3</v>
+      </c>
       <c r="J8" s="6">
         <f>IF(I8="","",I8-F8)</f>
         <v/>
       </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
       <c r="L8" s="6">
         <f>IF(K8="W",IF(G8&lt;0,H8*100/ABS(G8),H8*G8/100),IF(K8="L",-H8,0))</f>
         <v/>
@@ -2190,10 +2240,44 @@
       </c>
     </row>
     <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Wyoming @  Colorado State</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Moneyline</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Colorado State</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>-145</v>
+      </c>
+      <c r="H9" t="n">
+        <v>2</v>
+      </c>
       <c r="J9" s="6">
         <f>IF(I9="","",I9-F9)</f>
         <v/>
       </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
       <c r="L9" s="6">
         <f>IF(K9="W",IF(G9&lt;0,H9*100/ABS(G9),H9*G9/100),IF(K9="L",-H9,0))</f>
         <v/>
@@ -2204,10 +2288,50 @@
       </c>
     </row>
     <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-05</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Central Michigan @ New Mexico</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Spread</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>New Mexico</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>-12.5</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-110</v>
+      </c>
+      <c r="H10" t="n">
+        <v>5</v>
+      </c>
+      <c r="I10" t="n">
+        <v>-10</v>
+      </c>
       <c r="J10" s="6">
         <f>IF(I10="","",I10-F10)</f>
         <v/>
       </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
       <c r="L10" s="6">
         <f>IF(K10="W",IF(G10&lt;0,H10*100/ABS(G10),H10*G10/100),IF(K10="L",-H10,0))</f>
         <v/>
@@ -2218,6 +2342,7 @@
       </c>
     </row>
     <row r="11">
+      <c r="A11" s="10" t="n"/>
       <c r="J11" s="6">
         <f>IF(I11="","",I11-F11)</f>
         <v/>

</xml_diff>

<commit_message>
Refresh Dub Beta Model comparison with latest games
</commit_message>
<xml_diff>
--- a/excel/MW_Handicapping_Tracker.xlsx
+++ b/excel/MW_Handicapping_Tracker.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="1" activeTab="3" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="1" activeTab="5" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Read Me" sheetId="1" state="visible" r:id="rId1"/>
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="14">
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -111,8 +111,36 @@
       <color rgb="FF000000"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00666666"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -146,8 +174,23 @@
         <fgColor rgb="FFFCE4EC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4EC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -194,11 +237,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -223,6 +280,15 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -768,7 +834,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R42"/>
+  <dimension ref="A1:R29"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1764,19 +1830,6 @@
       <c r="M29" s="6" t="n"/>
       <c r="N29" s="6" t="n"/>
     </row>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
   </sheetData>
   <conditionalFormatting sqref="C2:C500">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -3237,14 +3290,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q43"/>
+  <dimension ref="A1:Q52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="5"/>
-    <col width="12" customWidth="1" min="6" max="7"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="16" customWidth="1" min="10" max="10"/>
@@ -3253,1561 +3308,2327 @@
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="13" customWidth="1" min="14" max="14"/>
     <col width="15" customWidth="1" min="15" max="15"/>
-    <col width="17" customWidth="1" min="16" max="17"/>
+    <col width="17" customWidth="1" min="16" max="16"/>
+    <col width="17" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18" customHeight="1">
-      <c r="A1" s="11" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="18" t="inlineStr">
         <is>
           <t>Ridge vs. XGBoost -- Model Comparison</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="19" t="inlineStr">
         <is>
           <t>Informational only. Ridge is still the live model everywhere else in this workbook and on the website -- XGBoost is a candidate being evaluated here, not a replacement.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="20" t="inlineStr">
         <is>
           <t>All-Time (every season in the backtest)</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="25.5" customHeight="1">
-      <c r="A5" s="14" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="21" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="B5" s="14" t="inlineStr">
+      <c r="B5" s="21" t="inlineStr">
         <is>
           <t>Games Graded</t>
         </is>
       </c>
-      <c r="C5" s="14" t="inlineStr">
+      <c r="C5" s="21" t="inlineStr">
         <is>
           <t>Bets Made</t>
         </is>
       </c>
-      <c r="D5" s="14" t="inlineStr">
+      <c r="D5" s="21" t="inlineStr">
         <is>
           <t>Wins</t>
         </is>
       </c>
-      <c r="E5" s="14" t="inlineStr">
+      <c r="E5" s="21" t="inlineStr">
         <is>
           <t>Losses</t>
         </is>
       </c>
-      <c r="F5" s="14" t="inlineStr">
+      <c r="F5" s="21" t="inlineStr">
         <is>
           <t>Pushes</t>
         </is>
       </c>
-      <c r="G5" s="14" t="inlineStr">
+      <c r="G5" s="21" t="inlineStr">
         <is>
           <t>ATS Win %</t>
         </is>
       </c>
-      <c r="H5" s="14" t="inlineStr">
+      <c r="H5" s="21" t="inlineStr">
         <is>
           <t>ROI (flat stake)</t>
         </is>
       </c>
-      <c r="I5" s="14" t="inlineStr">
+      <c r="I5" s="21" t="inlineStr">
         <is>
           <t>Tighter Than Other (CLV)</t>
         </is>
       </c>
-      <c r="J5" s="14" t="inlineStr">
+      <c r="J5" s="21" t="inlineStr">
         <is>
           <t>CLV Pts (cum.)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="15" t="inlineStr">
+      <c r="A6" s="22" t="inlineStr">
         <is>
           <t>Ridge (live model) -- all FBS</t>
         </is>
       </c>
-      <c r="B6" s="15" t="n">
-        <v>8441</v>
-      </c>
-      <c r="C6" s="15" t="n">
-        <v>6578</v>
-      </c>
-      <c r="D6" s="15" t="n">
-        <v>3264</v>
-      </c>
-      <c r="E6" s="15" t="n">
-        <v>3314</v>
-      </c>
-      <c r="F6" s="15" t="n">
+      <c r="B6" s="22" t="n">
+        <v>8528</v>
+      </c>
+      <c r="C6" s="22" t="n">
+        <v>6627</v>
+      </c>
+      <c r="D6" s="22" t="n">
+        <v>3296</v>
+      </c>
+      <c r="E6" s="22" t="n">
+        <v>3331</v>
+      </c>
+      <c r="F6" s="22" t="n">
+        <v>54</v>
+      </c>
+      <c r="G6" s="22" t="inlineStr">
+        <is>
+          <t>49.7%</t>
+        </is>
+      </c>
+      <c r="H6" s="22" t="inlineStr">
+        <is>
+          <t>-5.1%</t>
+        </is>
+      </c>
+      <c r="I6" s="22" t="inlineStr">
+        <is>
+          <t>4043/8528 (47%)</t>
+        </is>
+      </c>
+      <c r="J6" s="22" t="inlineStr">
+        <is>
+          <t>+5661.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="22" t="inlineStr">
+        <is>
+          <t>Ridge (live model) -- MW-involved</t>
+        </is>
+      </c>
+      <c r="B7" s="22" t="n">
+        <v>969</v>
+      </c>
+      <c r="C7" s="22" t="n">
+        <v>768</v>
+      </c>
+      <c r="D7" s="22" t="n">
+        <v>379</v>
+      </c>
+      <c r="E7" s="22" t="n">
+        <v>389</v>
+      </c>
+      <c r="F7" s="22" t="n">
+        <v>8</v>
+      </c>
+      <c r="G7" s="22" t="inlineStr">
+        <is>
+          <t>49.4%</t>
+        </is>
+      </c>
+      <c r="H7" s="22" t="inlineStr">
+        <is>
+          <t>-5.8%</t>
+        </is>
+      </c>
+      <c r="I7" s="22" t="inlineStr">
+        <is>
+          <t>457/969 (47%)</t>
+        </is>
+      </c>
+      <c r="J7" s="22" t="inlineStr">
+        <is>
+          <t>+600.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="22" t="inlineStr">
+        <is>
+          <t>XGBoost (candidate) -- all FBS</t>
+        </is>
+      </c>
+      <c r="B8" s="22" t="n">
+        <v>8528</v>
+      </c>
+      <c r="C8" s="22" t="n">
+        <v>6561</v>
+      </c>
+      <c r="D8" s="22" t="n">
+        <v>3312</v>
+      </c>
+      <c r="E8" s="22" t="n">
+        <v>3249</v>
+      </c>
+      <c r="F8" s="22" t="n">
         <v>59</v>
       </c>
-      <c r="G6" s="15" t="inlineStr">
-        <is>
-          <t>49.6%</t>
-        </is>
-      </c>
-      <c r="H6" s="15" t="inlineStr">
-        <is>
-          <t>-5.3%</t>
-        </is>
-      </c>
-      <c r="I6" s="15" t="inlineStr">
-        <is>
-          <t>4073/8441 (48%)</t>
-        </is>
-      </c>
-      <c r="J6" s="15" t="inlineStr">
-        <is>
-          <t>+1605.3</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="15" t="inlineStr">
+      <c r="G8" s="22" t="inlineStr">
+        <is>
+          <t>50.5%</t>
+        </is>
+      </c>
+      <c r="H8" s="22" t="inlineStr">
+        <is>
+          <t>-3.6%</t>
+        </is>
+      </c>
+      <c r="I8" s="22" t="inlineStr">
+        <is>
+          <t>4485/8528 (53%)</t>
+        </is>
+      </c>
+      <c r="J8" s="22" t="inlineStr">
+        <is>
+          <t>+741.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="22" t="inlineStr">
+        <is>
+          <t>XGBoost (candidate) -- MW-involved</t>
+        </is>
+      </c>
+      <c r="B9" s="22" t="n">
+        <v>969</v>
+      </c>
+      <c r="C9" s="22" t="n">
+        <v>729</v>
+      </c>
+      <c r="D9" s="22" t="n">
+        <v>375</v>
+      </c>
+      <c r="E9" s="22" t="n">
+        <v>354</v>
+      </c>
+      <c r="F9" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="G9" s="22" t="inlineStr">
+        <is>
+          <t>51.4%</t>
+        </is>
+      </c>
+      <c r="H9" s="22" t="inlineStr">
+        <is>
+          <t>-1.8%</t>
+        </is>
+      </c>
+      <c r="I9" s="22" t="inlineStr">
+        <is>
+          <t>512/969 (53%)</t>
+        </is>
+      </c>
+      <c r="J9" s="22" t="inlineStr">
+        <is>
+          <t>+895.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="20" t="inlineStr">
+        <is>
+          <t>2026 Season Only</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="21" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B12" s="21" t="inlineStr">
+        <is>
+          <t>Games Graded</t>
+        </is>
+      </c>
+      <c r="C12" s="21" t="inlineStr">
+        <is>
+          <t>Bets Made</t>
+        </is>
+      </c>
+      <c r="D12" s="21" t="inlineStr">
+        <is>
+          <t>Wins</t>
+        </is>
+      </c>
+      <c r="E12" s="21" t="inlineStr">
+        <is>
+          <t>Losses</t>
+        </is>
+      </c>
+      <c r="F12" s="21" t="inlineStr">
+        <is>
+          <t>Pushes</t>
+        </is>
+      </c>
+      <c r="G12" s="21" t="inlineStr">
+        <is>
+          <t>ATS Win %</t>
+        </is>
+      </c>
+      <c r="H12" s="21" t="inlineStr">
+        <is>
+          <t>ROI (flat stake)</t>
+        </is>
+      </c>
+      <c r="I12" s="21" t="inlineStr">
+        <is>
+          <t>Tighter Than Other (CLV)</t>
+        </is>
+      </c>
+      <c r="J12" s="21" t="inlineStr">
+        <is>
+          <t>CLV Pts (cum.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="22" t="inlineStr">
+        <is>
+          <t>Ridge (live model) -- all FBS</t>
+        </is>
+      </c>
+      <c r="B13" s="22" t="n">
+        <v>95</v>
+      </c>
+      <c r="C13" s="22" t="n">
+        <v>84</v>
+      </c>
+      <c r="D13" s="22" t="n">
+        <v>33</v>
+      </c>
+      <c r="E13" s="22" t="n">
+        <v>51</v>
+      </c>
+      <c r="F13" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="22" t="inlineStr">
+        <is>
+          <t>39.3%</t>
+        </is>
+      </c>
+      <c r="H13" s="22" t="inlineStr">
+        <is>
+          <t>-25.0%</t>
+        </is>
+      </c>
+      <c r="I13" s="22" t="inlineStr">
+        <is>
+          <t>42/95 (44%)</t>
+        </is>
+      </c>
+      <c r="J13" s="22" t="inlineStr">
+        <is>
+          <t>-433.7</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="22" t="inlineStr">
         <is>
           <t>Ridge (live model) -- MW-involved</t>
         </is>
       </c>
-      <c r="B7" s="15" t="n">
-        <v>960</v>
-      </c>
-      <c r="C7" s="15" t="n">
-        <v>756</v>
-      </c>
-      <c r="D7" s="15" t="n">
-        <v>377</v>
-      </c>
-      <c r="E7" s="15" t="n">
-        <v>379</v>
-      </c>
-      <c r="F7" s="15" t="n">
-        <v>12</v>
-      </c>
-      <c r="G7" s="15" t="inlineStr">
-        <is>
-          <t>49.9%</t>
-        </is>
-      </c>
-      <c r="H7" s="15" t="inlineStr">
-        <is>
-          <t>-4.8%</t>
-        </is>
-      </c>
-      <c r="I7" s="15" t="inlineStr">
-        <is>
-          <t>464/960 (48%)</t>
-        </is>
-      </c>
-      <c r="J7" s="15" t="inlineStr">
-        <is>
-          <t>+377.9</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="15" t="inlineStr">
+      <c r="B14" s="22" t="n">
+        <v>13</v>
+      </c>
+      <c r="C14" s="22" t="n">
+        <v>11</v>
+      </c>
+      <c r="D14" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="E14" s="22" t="n">
+        <v>7</v>
+      </c>
+      <c r="F14" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="22" t="inlineStr">
+        <is>
+          <t>36.4%</t>
+        </is>
+      </c>
+      <c r="H14" s="22" t="inlineStr">
+        <is>
+          <t>-30.6%</t>
+        </is>
+      </c>
+      <c r="I14" s="22" t="inlineStr">
+        <is>
+          <t>6/13 (46%)</t>
+        </is>
+      </c>
+      <c r="J14" s="22" t="inlineStr">
+        <is>
+          <t>+11.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="22" t="inlineStr">
         <is>
           <t>XGBoost (candidate) -- all FBS</t>
         </is>
       </c>
-      <c r="B8" s="15" t="n">
-        <v>8441</v>
-      </c>
-      <c r="C8" s="15" t="n">
-        <v>6518</v>
-      </c>
-      <c r="D8" s="15" t="n">
-        <v>3259</v>
-      </c>
-      <c r="E8" s="15" t="n">
-        <v>3259</v>
-      </c>
-      <c r="F8" s="15" t="n">
-        <v>59</v>
-      </c>
-      <c r="G8" s="15" t="inlineStr">
-        <is>
-          <t>50.0%</t>
-        </is>
-      </c>
-      <c r="H8" s="15" t="inlineStr">
-        <is>
-          <t>-4.5%</t>
-        </is>
-      </c>
-      <c r="I8" s="15" t="inlineStr">
-        <is>
-          <t>4368/8441 (52%)</t>
-        </is>
-      </c>
-      <c r="J8" s="15" t="inlineStr">
-        <is>
-          <t>+191.6</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="15" t="inlineStr">
+      <c r="B15" s="22" t="n">
+        <v>95</v>
+      </c>
+      <c r="C15" s="22" t="n">
+        <v>78</v>
+      </c>
+      <c r="D15" s="22" t="n">
+        <v>31</v>
+      </c>
+      <c r="E15" s="22" t="n">
+        <v>47</v>
+      </c>
+      <c r="F15" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="22" t="inlineStr">
+        <is>
+          <t>39.7%</t>
+        </is>
+      </c>
+      <c r="H15" s="22" t="inlineStr">
+        <is>
+          <t>-24.1%</t>
+        </is>
+      </c>
+      <c r="I15" s="22" t="inlineStr">
+        <is>
+          <t>53/95 (56%)</t>
+        </is>
+      </c>
+      <c r="J15" s="22" t="inlineStr">
+        <is>
+          <t>-162.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="22" t="inlineStr">
         <is>
           <t>XGBoost (candidate) -- MW-involved</t>
         </is>
       </c>
-      <c r="B9" s="15" t="n">
-        <v>960</v>
-      </c>
-      <c r="C9" s="15" t="n">
-        <v>742</v>
-      </c>
-      <c r="D9" s="15" t="n">
-        <v>384</v>
-      </c>
-      <c r="E9" s="15" t="n">
-        <v>358</v>
-      </c>
-      <c r="F9" s="15" t="n">
-        <v>11</v>
-      </c>
-      <c r="G9" s="15" t="inlineStr">
-        <is>
-          <t>51.7%</t>
-        </is>
-      </c>
-      <c r="H9" s="15" t="inlineStr">
-        <is>
-          <t>-1.2%</t>
-        </is>
-      </c>
-      <c r="I9" s="15" t="inlineStr">
-        <is>
-          <t>496/960 (52%)</t>
-        </is>
-      </c>
-      <c r="J9" s="15" t="inlineStr">
-        <is>
-          <t>+764.5</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="13" t="inlineStr">
-        <is>
-          <t>2026 Season Only</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="25.5" customHeight="1">
-      <c r="A12" s="14" t="inlineStr">
-        <is>
-          <t>Model</t>
-        </is>
-      </c>
-      <c r="B12" s="14" t="inlineStr">
-        <is>
-          <t>Games Graded</t>
-        </is>
-      </c>
-      <c r="C12" s="14" t="inlineStr">
-        <is>
-          <t>Bets Made</t>
-        </is>
-      </c>
-      <c r="D12" s="14" t="inlineStr">
-        <is>
-          <t>Wins</t>
-        </is>
-      </c>
-      <c r="E12" s="14" t="inlineStr">
-        <is>
-          <t>Losses</t>
-        </is>
-      </c>
-      <c r="F12" s="14" t="inlineStr">
-        <is>
-          <t>Pushes</t>
-        </is>
-      </c>
-      <c r="G12" s="14" t="inlineStr">
-        <is>
-          <t>ATS Win %</t>
-        </is>
-      </c>
-      <c r="H12" s="14" t="inlineStr">
-        <is>
-          <t>ROI (flat stake)</t>
-        </is>
-      </c>
-      <c r="I12" s="14" t="inlineStr">
-        <is>
-          <t>Tighter Than Other (CLV)</t>
-        </is>
-      </c>
-      <c r="J12" s="14" t="inlineStr">
-        <is>
-          <t>CLV Pts (cum.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="15" t="inlineStr">
-        <is>
-          <t>Ridge (live model) -- all FBS</t>
-        </is>
-      </c>
-      <c r="B13" s="15" t="n">
-        <v>8</v>
-      </c>
-      <c r="C13" s="15" t="n">
+      <c r="B16" s="22" t="n">
+        <v>13</v>
+      </c>
+      <c r="C16" s="22" t="n">
+        <v>9</v>
+      </c>
+      <c r="D16" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="E16" s="22" t="n">
         <v>7</v>
       </c>
-      <c r="D13" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="E13" s="15" t="n">
-        <v>4</v>
-      </c>
-      <c r="F13" s="15" t="n">
+      <c r="F16" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="G13" s="15" t="inlineStr">
-        <is>
-          <t>42.9%</t>
-        </is>
-      </c>
-      <c r="H13" s="15" t="inlineStr">
-        <is>
-          <t>-18.2%</t>
-        </is>
-      </c>
-      <c r="I13" s="15" t="inlineStr">
-        <is>
-          <t>2/8 (25%)</t>
-        </is>
-      </c>
-      <c r="J13" s="15" t="inlineStr">
+      <c r="G16" s="22" t="inlineStr">
+        <is>
+          <t>22.2%</t>
+        </is>
+      </c>
+      <c r="H16" s="22" t="inlineStr">
+        <is>
+          <t>-57.6%</t>
+        </is>
+      </c>
+      <c r="I16" s="22" t="inlineStr">
+        <is>
+          <t>7/13 (54%)</t>
+        </is>
+      </c>
+      <c r="J16" s="22" t="inlineStr">
+        <is>
+          <t>-13.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="19" t="inlineStr">
+        <is>
+          <t>Ridge and XGBoost agree on which side to lean in 76.9% of all graded games.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="20" t="inlineStr">
+        <is>
+          <t>Upcoming Games -- Ridge vs. XGBoost (Not Yet Graded)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="21" t="inlineStr">
+        <is>
+          <t>Week</t>
+        </is>
+      </c>
+      <c r="B21" s="21" t="inlineStr">
+        <is>
+          <t>Matchup</t>
+        </is>
+      </c>
+      <c r="C21" s="21" t="inlineStr">
+        <is>
+          <t>Market Line (Home)</t>
+        </is>
+      </c>
+      <c r="D21" s="21" t="inlineStr">
+        <is>
+          <t>Ridge Line</t>
+        </is>
+      </c>
+      <c r="E21" s="21" t="inlineStr">
+        <is>
+          <t>XGBoost Line</t>
+        </is>
+      </c>
+      <c r="F21" s="21" t="inlineStr">
+        <is>
+          <t>Ridge Lean</t>
+        </is>
+      </c>
+      <c r="G21" s="21" t="inlineStr">
+        <is>
+          <t>XGBoost Lean</t>
+        </is>
+      </c>
+      <c r="H21" s="21" t="inlineStr">
+        <is>
+          <t>Models Agree?</t>
+        </is>
+      </c>
+      <c r="I21" s="21" t="inlineStr">
+        <is>
+          <t>Tighter (Live)*</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="B22" s="22" t="inlineStr">
+        <is>
+          <t>San José State @ USC</t>
+        </is>
+      </c>
+      <c r="C22" s="22" t="inlineStr">
+        <is>
+          <t>-37.2</t>
+        </is>
+      </c>
+      <c r="D22" s="22" t="inlineStr">
+        <is>
+          <t>-34.9</t>
+        </is>
+      </c>
+      <c r="E22" s="22" t="inlineStr">
+        <is>
+          <t>-32.3</t>
+        </is>
+      </c>
+      <c r="F22" s="22" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="G22" s="22" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="H22" s="22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I22" s="23" t="inlineStr">
+        <is>
+          <t>Ridge</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="B23" s="22" t="inlineStr">
+        <is>
+          <t>Jacksonville State @ North Dakota State</t>
+        </is>
+      </c>
+      <c r="C23" s="22" t="inlineStr">
+        <is>
+          <t>-6.8</t>
+        </is>
+      </c>
+      <c r="D23" s="22" t="inlineStr">
+        <is>
+          <t>-18.9</t>
+        </is>
+      </c>
+      <c r="E23" s="22" t="inlineStr">
+        <is>
+          <t>-16.3</t>
+        </is>
+      </c>
+      <c r="F23" s="22" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="G23" s="22" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="H23" s="22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I23" s="23" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="B24" s="22" t="inlineStr">
+        <is>
+          <t>Hawai'i @ Stanford</t>
+        </is>
+      </c>
+      <c r="C24" s="22" t="inlineStr">
+        <is>
+          <t>-4.8</t>
+        </is>
+      </c>
+      <c r="D24" s="22" t="inlineStr">
+        <is>
+          <t>-1.8</t>
+        </is>
+      </c>
+      <c r="E24" s="22" t="inlineStr">
+        <is>
+          <t>-0.3</t>
+        </is>
+      </c>
+      <c r="F24" s="22" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="G24" s="22" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="H24" s="22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I24" s="23" t="inlineStr">
+        <is>
+          <t>Ridge</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="B25" s="22" t="inlineStr">
+        <is>
+          <t>Memphis @ UNLV</t>
+        </is>
+      </c>
+      <c r="C25" s="22" t="inlineStr">
+        <is>
+          <t>-4.8</t>
+        </is>
+      </c>
+      <c r="D25" s="22" t="inlineStr">
+        <is>
+          <t>-11.3</t>
+        </is>
+      </c>
+      <c r="E25" s="22" t="inlineStr">
+        <is>
+          <t>-6.7</t>
+        </is>
+      </c>
+      <c r="F25" s="22" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="G25" s="22" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="H25" s="22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I25" s="23" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="B26" s="22" t="inlineStr">
+        <is>
+          <t>San José State @ Eastern Michigan</t>
+        </is>
+      </c>
+      <c r="C26" s="22" t="inlineStr">
+        <is>
+          <t>-1.5</t>
+        </is>
+      </c>
+      <c r="D26" s="22" t="inlineStr">
+        <is>
+          <t>-16.0</t>
+        </is>
+      </c>
+      <c r="E26" s="22" t="inlineStr">
+        <is>
+          <t>-9.9</t>
+        </is>
+      </c>
+      <c r="F26" s="22" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="G26" s="22" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="H26" s="22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I26" s="23" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="B27" s="22" t="inlineStr">
+        <is>
+          <t>UTEP @ Oklahoma</t>
+        </is>
+      </c>
+      <c r="C27" s="22" t="inlineStr">
+        <is>
+          <t>-40.8</t>
+        </is>
+      </c>
+      <c r="D27" s="22" t="inlineStr">
+        <is>
+          <t>-35.0</t>
+        </is>
+      </c>
+      <c r="E27" s="22" t="inlineStr">
+        <is>
+          <t>-33.6</t>
+        </is>
+      </c>
+      <c r="F27" s="22" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="G27" s="22" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="H27" s="22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I27" s="23" t="inlineStr">
+        <is>
+          <t>Ridge</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="B28" s="22" t="inlineStr">
+        <is>
+          <t>Duquesne @ Air Force</t>
+        </is>
+      </c>
+      <c r="C28" s="22" t="inlineStr">
+        <is>
+          <t>-30.0</t>
+        </is>
+      </c>
+      <c r="D28" s="22" t="inlineStr">
+        <is>
+          <t>-17.3</t>
+        </is>
+      </c>
+      <c r="E28" s="22" t="inlineStr">
+        <is>
+          <t>-29.5</t>
+        </is>
+      </c>
+      <c r="F28" s="22" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="G28" s="22" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="H28" s="22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I28" s="23" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="B29" s="22" t="inlineStr">
+        <is>
+          <t>Fordham @ North Dakota State</t>
+        </is>
+      </c>
+      <c r="C29" s="22" t="inlineStr">
+        <is>
+          <t>-41.5</t>
+        </is>
+      </c>
+      <c r="D29" s="22" t="inlineStr">
+        <is>
+          <t>-39.8</t>
+        </is>
+      </c>
+      <c r="E29" s="22" t="inlineStr">
+        <is>
+          <t>-32.6</t>
+        </is>
+      </c>
+      <c r="F29" s="22" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="G29" s="22" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="H29" s="22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I29" s="23" t="inlineStr">
+        <is>
+          <t>Ridge</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="B30" s="22" t="inlineStr">
+        <is>
+          <t>Northern Illinois @ Iowa</t>
+        </is>
+      </c>
+      <c r="C30" s="22" t="inlineStr">
+        <is>
+          <t>-31.8</t>
+        </is>
+      </c>
+      <c r="D30" s="22" t="inlineStr">
+        <is>
+          <t>-28.7</t>
+        </is>
+      </c>
+      <c r="E30" s="22" t="inlineStr">
+        <is>
+          <t>-25.6</t>
+        </is>
+      </c>
+      <c r="F30" s="22" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="G30" s="22" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="H30" s="22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I30" s="23" t="inlineStr">
+        <is>
+          <t>Ridge</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="B31" s="22" t="inlineStr">
+        <is>
+          <t>Wyoming @ Colorado State</t>
+        </is>
+      </c>
+      <c r="C31" s="22" t="inlineStr">
+        <is>
+          <t>-2.8</t>
+        </is>
+      </c>
+      <c r="D31" s="22" t="inlineStr">
+        <is>
+          <t>-8.3</t>
+        </is>
+      </c>
+      <c r="E31" s="22" t="inlineStr">
+        <is>
+          <t>-3.9</t>
+        </is>
+      </c>
+      <c r="F31" s="22" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="G31" s="22" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="H31" s="22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I31" s="23" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="B32" s="22" t="inlineStr">
+        <is>
+          <t>Central Michigan @ New Mexico</t>
+        </is>
+      </c>
+      <c r="C32" s="22" t="inlineStr">
+        <is>
+          <t>-11.2</t>
+        </is>
+      </c>
+      <c r="D32" s="22" t="inlineStr">
+        <is>
+          <t>-18.2</t>
+        </is>
+      </c>
+      <c r="E32" s="22" t="inlineStr">
+        <is>
+          <t>-12.2</t>
+        </is>
+      </c>
+      <c r="F32" s="22" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="G32" s="22" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="H32" s="22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I32" s="23" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="B33" s="22" t="inlineStr">
+        <is>
+          <t>UNLV @ Hawai'i</t>
+        </is>
+      </c>
+      <c r="C33" s="22" t="inlineStr">
+        <is>
+          <t>+2.8</t>
+        </is>
+      </c>
+      <c r="D33" s="22" t="inlineStr">
+        <is>
+          <t>+3.5</t>
+        </is>
+      </c>
+      <c r="E33" s="22" t="inlineStr">
+        <is>
+          <t>-1.1</t>
+        </is>
+      </c>
+      <c r="F33" s="22" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="G33" s="22" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="H33" s="22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I33" s="23" t="inlineStr">
+        <is>
+          <t>Ridge</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="B34" s="22" t="inlineStr">
+        <is>
+          <t>Western Kentucky @ Nevada</t>
+        </is>
+      </c>
+      <c r="C34" s="22" t="inlineStr">
+        <is>
+          <t>+0.2</t>
+        </is>
+      </c>
+      <c r="D34" s="22" t="inlineStr">
+        <is>
+          <t>+2.6</t>
+        </is>
+      </c>
+      <c r="E34" s="22" t="inlineStr">
+        <is>
+          <t>+4.4</t>
+        </is>
+      </c>
+      <c r="F34" s="22" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="G34" s="22" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="H34" s="22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I34" s="23" t="inlineStr">
+        <is>
+          <t>Ridge</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="19" t="inlineStr">
+        <is>
+          <t>* Tighter (Live) compares each model's line to TODAY's still-moving market line, not a final closing line -- it will keep changing until kickoff. See the graded Game-by-Game table below for the real, closing-line version of this comparison.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="20" t="inlineStr">
+        <is>
+          <t>2026 Mountain West Games -- Game by Game</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="21" t="inlineStr">
+        <is>
+          <t>Week</t>
+        </is>
+      </c>
+      <c r="B39" s="21" t="inlineStr">
+        <is>
+          <t>Matchup</t>
+        </is>
+      </c>
+      <c r="C39" s="21" t="inlineStr">
+        <is>
+          <t>Final Score</t>
+        </is>
+      </c>
+      <c r="D39" s="21" t="inlineStr">
+        <is>
+          <t>Vegas Spread (Home)</t>
+        </is>
+      </c>
+      <c r="E39" s="21" t="inlineStr">
+        <is>
+          <t>Actual Margin (Home)</t>
+        </is>
+      </c>
+      <c r="F39" s="21" t="inlineStr">
+        <is>
+          <t>Ridge Line</t>
+        </is>
+      </c>
+      <c r="G39" s="21" t="inlineStr">
+        <is>
+          <t>Ridge Edge</t>
+        </is>
+      </c>
+      <c r="H39" s="21" t="inlineStr">
+        <is>
+          <t>Ridge Lean</t>
+        </is>
+      </c>
+      <c r="I39" s="21" t="inlineStr">
+        <is>
+          <t>Ridge Result</t>
+        </is>
+      </c>
+      <c r="J39" s="21" t="inlineStr">
+        <is>
+          <t>XGBoost Line</t>
+        </is>
+      </c>
+      <c r="K39" s="21" t="inlineStr">
+        <is>
+          <t>XGBoost Edge</t>
+        </is>
+      </c>
+      <c r="L39" s="21" t="inlineStr">
+        <is>
+          <t>XGBoost Lean</t>
+        </is>
+      </c>
+      <c r="M39" s="21" t="inlineStr">
+        <is>
+          <t>XGBoost Result</t>
+        </is>
+      </c>
+      <c r="N39" s="21" t="inlineStr">
+        <is>
+          <t>Models Agree?</t>
+        </is>
+      </c>
+      <c r="O39" s="21" t="inlineStr">
+        <is>
+          <t>Tighter CLV Line</t>
+        </is>
+      </c>
+      <c r="P39" s="21" t="inlineStr">
+        <is>
+          <t>Ridge CLV Pts (Cum.)</t>
+        </is>
+      </c>
+      <c r="Q39" s="21" t="inlineStr">
+        <is>
+          <t>XGBoost CLV Pts (Cum.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="B40" s="22" t="inlineStr">
+        <is>
+          <t>Duquesne @ Air Force</t>
+        </is>
+      </c>
+      <c r="C40" s="22" t="inlineStr">
+        <is>
+          <t>0-34</t>
+        </is>
+      </c>
+      <c r="D40" s="22" t="inlineStr">
+        <is>
+          <t>-30.0</t>
+        </is>
+      </c>
+      <c r="E40" s="22" t="inlineStr">
+        <is>
+          <t>+34.0</t>
+        </is>
+      </c>
+      <c r="F40" s="22" t="inlineStr">
+        <is>
+          <t>-17.0</t>
+        </is>
+      </c>
+      <c r="G40" s="22" t="inlineStr">
+        <is>
+          <t>-13.0</t>
+        </is>
+      </c>
+      <c r="H40" s="22" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="I40" s="24" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="J40" s="22" t="inlineStr">
+        <is>
+          <t>-28.3</t>
+        </is>
+      </c>
+      <c r="K40" s="22" t="inlineStr">
+        <is>
+          <t>-1.7</t>
+        </is>
+      </c>
+      <c r="L40" s="22" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="M40" s="22" t="inlineStr">
+        <is>
+          <t>Lean only</t>
+        </is>
+      </c>
+      <c r="N40" s="22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O40" s="23" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="P40" s="22" t="inlineStr">
+        <is>
+          <t>-13.0</t>
+        </is>
+      </c>
+      <c r="Q40" s="22" t="inlineStr">
+        <is>
+          <t>-1.7</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="B41" s="22" t="inlineStr">
+        <is>
+          <t>Wyoming @ Colorado State</t>
+        </is>
+      </c>
+      <c r="C41" s="22" t="inlineStr">
+        <is>
+          <t>13-35</t>
+        </is>
+      </c>
+      <c r="D41" s="22" t="inlineStr">
+        <is>
+          <t>-2.8</t>
+        </is>
+      </c>
+      <c r="E41" s="22" t="inlineStr">
+        <is>
+          <t>+22.0</t>
+        </is>
+      </c>
+      <c r="F41" s="22" t="inlineStr">
+        <is>
+          <t>-7.8</t>
+        </is>
+      </c>
+      <c r="G41" s="22" t="inlineStr">
+        <is>
+          <t>+5.1</t>
+        </is>
+      </c>
+      <c r="H41" s="22" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="I41" s="23" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="J41" s="22" t="inlineStr">
         <is>
           <t>-2.5</t>
         </is>
       </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="15" t="inlineStr">
-        <is>
-          <t>Ridge (live model) -- MW-involved</t>
-        </is>
-      </c>
-      <c r="B14" s="15" t="n">
-        <v>4</v>
-      </c>
-      <c r="C14" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="D14" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="E14" s="15" t="n">
+      <c r="K41" s="22" t="inlineStr">
+        <is>
+          <t>-0.2</t>
+        </is>
+      </c>
+      <c r="L41" s="22" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="M41" s="22" t="inlineStr">
+        <is>
+          <t>Lean only</t>
+        </is>
+      </c>
+      <c r="N41" s="22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O41" s="23" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="P41" s="22" t="inlineStr">
+        <is>
+          <t>-7.9</t>
+        </is>
+      </c>
+      <c r="Q41" s="22" t="inlineStr">
+        <is>
+          <t>-1.9</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="22" t="n">
         <v>1</v>
       </c>
-      <c r="F14" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" s="15" t="inlineStr">
-        <is>
-          <t>66.7%</t>
-        </is>
-      </c>
-      <c r="H14" s="15" t="inlineStr">
-        <is>
-          <t>+27.3%</t>
-        </is>
-      </c>
-      <c r="I14" s="15" t="inlineStr">
-        <is>
-          <t>1/4 (25%)</t>
-        </is>
-      </c>
-      <c r="J14" s="15" t="inlineStr">
+      <c r="B42" s="22" t="inlineStr">
+        <is>
+          <t>San José State @ Eastern Michigan</t>
+        </is>
+      </c>
+      <c r="C42" s="22" t="inlineStr">
+        <is>
+          <t>27-21</t>
+        </is>
+      </c>
+      <c r="D42" s="22" t="inlineStr">
+        <is>
+          <t>-1.5</t>
+        </is>
+      </c>
+      <c r="E42" s="22" t="inlineStr">
+        <is>
+          <t>-6.0</t>
+        </is>
+      </c>
+      <c r="F42" s="22" t="inlineStr">
+        <is>
+          <t>-15.8</t>
+        </is>
+      </c>
+      <c r="G42" s="22" t="inlineStr">
+        <is>
+          <t>+14.3</t>
+        </is>
+      </c>
+      <c r="H42" s="22" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="I42" s="24" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="J42" s="22" t="inlineStr">
+        <is>
+          <t>-10.5</t>
+        </is>
+      </c>
+      <c r="K42" s="22" t="inlineStr">
         <is>
           <t>+9.0</t>
         </is>
       </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="15" t="inlineStr">
-        <is>
-          <t>XGBoost (candidate) -- all FBS</t>
-        </is>
-      </c>
-      <c r="B15" s="15" t="n">
-        <v>8</v>
-      </c>
-      <c r="C15" s="15" t="n">
-        <v>6</v>
-      </c>
-      <c r="D15" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="E15" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="F15" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" s="15" t="inlineStr">
-        <is>
-          <t>50.0%</t>
-        </is>
-      </c>
-      <c r="H15" s="15" t="inlineStr">
-        <is>
-          <t>-4.5%</t>
-        </is>
-      </c>
-      <c r="I15" s="15" t="inlineStr">
-        <is>
-          <t>6/8 (75%)</t>
-        </is>
-      </c>
-      <c r="J15" s="15" t="inlineStr">
-        <is>
-          <t>-6.3</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="15" t="inlineStr">
-        <is>
-          <t>XGBoost (candidate) -- MW-involved</t>
-        </is>
-      </c>
-      <c r="B16" s="15" t="n">
-        <v>4</v>
-      </c>
-      <c r="C16" s="15" t="n">
-        <v>3</v>
-      </c>
-      <c r="D16" s="15" t="n">
-        <v>2</v>
-      </c>
-      <c r="E16" s="15" t="n">
+      <c r="L42" s="22" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="M42" s="24" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="N42" s="22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O42" s="23" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="P42" s="22" t="inlineStr">
+        <is>
+          <t>+6.4</t>
+        </is>
+      </c>
+      <c r="Q42" s="22" t="inlineStr">
+        <is>
+          <t>+7.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="22" t="n">
         <v>1</v>
       </c>
-      <c r="F16" s="15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" s="15" t="inlineStr">
-        <is>
-          <t>66.7%</t>
-        </is>
-      </c>
-      <c r="H16" s="15" t="inlineStr">
-        <is>
-          <t>+27.3%</t>
-        </is>
-      </c>
-      <c r="I16" s="15" t="inlineStr">
-        <is>
-          <t>3/4 (75%)</t>
-        </is>
-      </c>
-      <c r="J16" s="15" t="inlineStr">
-        <is>
-          <t>+1.9</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="12" t="inlineStr">
-        <is>
-          <t>Ridge and XGBoost agree on which side to lean in 81.1% of all graded games.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="13" t="inlineStr">
-        <is>
-          <t>Upcoming Games -- Ridge vs. XGBoost (Not Yet Graded)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="25.5" customHeight="1">
-      <c r="A21" s="14" t="inlineStr">
-        <is>
-          <t>Week</t>
-        </is>
-      </c>
-      <c r="B21" s="14" t="inlineStr">
-        <is>
-          <t>Matchup</t>
-        </is>
-      </c>
-      <c r="C21" s="14" t="inlineStr">
-        <is>
-          <t>Market Line (Home)</t>
-        </is>
-      </c>
-      <c r="D21" s="14" t="inlineStr">
-        <is>
-          <t>Ridge Line</t>
-        </is>
-      </c>
-      <c r="E21" s="14" t="inlineStr">
-        <is>
-          <t>XGBoost Line</t>
-        </is>
-      </c>
-      <c r="F21" s="14" t="inlineStr">
-        <is>
-          <t>Ridge Lean</t>
-        </is>
-      </c>
-      <c r="G21" s="14" t="inlineStr">
-        <is>
-          <t>XGBoost Lean</t>
-        </is>
-      </c>
-      <c r="H21" s="14" t="inlineStr">
-        <is>
-          <t>Models Agree?</t>
-        </is>
-      </c>
-      <c r="I21" s="14" t="inlineStr">
-        <is>
-          <t>Tighter (Live)*</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="15" t="n">
+      <c r="B43" s="22" t="inlineStr">
+        <is>
+          <t>UNLV @ Hawai'i</t>
+        </is>
+      </c>
+      <c r="C43" s="22" t="inlineStr">
+        <is>
+          <t>21-6</t>
+        </is>
+      </c>
+      <c r="D43" s="22" t="inlineStr">
+        <is>
+          <t>+2.8</t>
+        </is>
+      </c>
+      <c r="E43" s="22" t="inlineStr">
+        <is>
+          <t>-15.0</t>
+        </is>
+      </c>
+      <c r="F43" s="22" t="inlineStr">
+        <is>
+          <t>+2.9</t>
+        </is>
+      </c>
+      <c r="G43" s="22" t="inlineStr">
+        <is>
+          <t>-0.1</t>
+        </is>
+      </c>
+      <c r="H43" s="22" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="I43" s="22" t="inlineStr">
+        <is>
+          <t>Lean only</t>
+        </is>
+      </c>
+      <c r="J43" s="22" t="inlineStr">
+        <is>
+          <t>-1.8</t>
+        </is>
+      </c>
+      <c r="K43" s="22" t="inlineStr">
+        <is>
+          <t>+4.6</t>
+        </is>
+      </c>
+      <c r="L43" s="22" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="M43" s="24" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="N43" s="22" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="O43" s="23" t="inlineStr">
+        <is>
+          <t>Ridge</t>
+        </is>
+      </c>
+      <c r="P43" s="22" t="inlineStr">
+        <is>
+          <t>+6.2</t>
+        </is>
+      </c>
+      <c r="Q43" s="22" t="inlineStr">
+        <is>
+          <t>+11.8</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="22" t="n">
         <v>1</v>
       </c>
-      <c r="B22" s="15" t="inlineStr">
+      <c r="B44" s="22" t="inlineStr">
+        <is>
+          <t>Northern Illinois @ Iowa</t>
+        </is>
+      </c>
+      <c r="C44" s="22" t="inlineStr">
+        <is>
+          <t>0-40</t>
+        </is>
+      </c>
+      <c r="D44" s="22" t="inlineStr">
+        <is>
+          <t>-31.8</t>
+        </is>
+      </c>
+      <c r="E44" s="22" t="inlineStr">
+        <is>
+          <t>+40.0</t>
+        </is>
+      </c>
+      <c r="F44" s="22" t="inlineStr">
+        <is>
+          <t>-28.3</t>
+        </is>
+      </c>
+      <c r="G44" s="22" t="inlineStr">
+        <is>
+          <t>-3.5</t>
+        </is>
+      </c>
+      <c r="H44" s="22" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="I44" s="24" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="J44" s="22" t="inlineStr">
+        <is>
+          <t>-25.4</t>
+        </is>
+      </c>
+      <c r="K44" s="22" t="inlineStr">
+        <is>
+          <t>-6.4</t>
+        </is>
+      </c>
+      <c r="L44" s="22" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="M44" s="24" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="N44" s="22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O44" s="23" t="inlineStr">
+        <is>
+          <t>Ridge</t>
+        </is>
+      </c>
+      <c r="P44" s="22" t="inlineStr">
+        <is>
+          <t>+2.8</t>
+        </is>
+      </c>
+      <c r="Q44" s="22" t="inlineStr">
+        <is>
+          <t>+5.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="B45" s="22" t="inlineStr">
+        <is>
+          <t>Western Kentucky @ Nevada</t>
+        </is>
+      </c>
+      <c r="C45" s="22" t="inlineStr">
+        <is>
+          <t>14-49</t>
+        </is>
+      </c>
+      <c r="D45" s="22" t="inlineStr">
+        <is>
+          <t>+0.2</t>
+        </is>
+      </c>
+      <c r="E45" s="22" t="inlineStr">
+        <is>
+          <t>+35.0</t>
+        </is>
+      </c>
+      <c r="F45" s="22" t="inlineStr">
+        <is>
+          <t>+3.3</t>
+        </is>
+      </c>
+      <c r="G45" s="22" t="inlineStr">
+        <is>
+          <t>-3.0</t>
+        </is>
+      </c>
+      <c r="H45" s="22" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="I45" s="24" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="J45" s="22" t="inlineStr">
+        <is>
+          <t>+7.3</t>
+        </is>
+      </c>
+      <c r="K45" s="22" t="inlineStr">
+        <is>
+          <t>-7.1</t>
+        </is>
+      </c>
+      <c r="L45" s="22" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="M45" s="24" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="N45" s="22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O45" s="23" t="inlineStr">
+        <is>
+          <t>Ridge</t>
+        </is>
+      </c>
+      <c r="P45" s="22" t="inlineStr">
+        <is>
+          <t>-0.3</t>
+        </is>
+      </c>
+      <c r="Q45" s="22" t="inlineStr">
+        <is>
+          <t>-1.7</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="B46" s="22" t="inlineStr">
+        <is>
+          <t>Central Michigan @ New Mexico</t>
+        </is>
+      </c>
+      <c r="C46" s="22" t="inlineStr">
+        <is>
+          <t>7-38</t>
+        </is>
+      </c>
+      <c r="D46" s="22" t="inlineStr">
+        <is>
+          <t>-11.2</t>
+        </is>
+      </c>
+      <c r="E46" s="22" t="inlineStr">
+        <is>
+          <t>+31.0</t>
+        </is>
+      </c>
+      <c r="F46" s="22" t="inlineStr">
+        <is>
+          <t>-17.5</t>
+        </is>
+      </c>
+      <c r="G46" s="22" t="inlineStr">
+        <is>
+          <t>+6.2</t>
+        </is>
+      </c>
+      <c r="H46" s="22" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="I46" s="23" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="J46" s="22" t="inlineStr">
+        <is>
+          <t>-11.6</t>
+        </is>
+      </c>
+      <c r="K46" s="22" t="inlineStr">
+        <is>
+          <t>+0.3</t>
+        </is>
+      </c>
+      <c r="L46" s="22" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="M46" s="22" t="inlineStr">
+        <is>
+          <t>Lean only</t>
+        </is>
+      </c>
+      <c r="N46" s="22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O46" s="23" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="P46" s="22" t="inlineStr">
+        <is>
+          <t>+5.9</t>
+        </is>
+      </c>
+      <c r="Q46" s="22" t="inlineStr">
+        <is>
+          <t>-1.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="B47" s="22" t="inlineStr">
+        <is>
+          <t>Jacksonville State @ North Dakota State</t>
+        </is>
+      </c>
+      <c r="C47" s="22" t="inlineStr">
+        <is>
+          <t>7-33</t>
+        </is>
+      </c>
+      <c r="D47" s="22" t="inlineStr">
+        <is>
+          <t>-6.8</t>
+        </is>
+      </c>
+      <c r="E47" s="22" t="inlineStr">
+        <is>
+          <t>+26.0</t>
+        </is>
+      </c>
+      <c r="F47" s="22" t="inlineStr">
+        <is>
+          <t>-18.4</t>
+        </is>
+      </c>
+      <c r="G47" s="22" t="inlineStr">
+        <is>
+          <t>+11.6</t>
+        </is>
+      </c>
+      <c r="H47" s="22" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="I47" s="23" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="J47" s="22" t="inlineStr">
+        <is>
+          <t>-14.4</t>
+        </is>
+      </c>
+      <c r="K47" s="22" t="inlineStr">
+        <is>
+          <t>+7.7</t>
+        </is>
+      </c>
+      <c r="L47" s="22" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="M47" s="23" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="N47" s="22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O47" s="23" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="P47" s="22" t="inlineStr">
+        <is>
+          <t>+17.6</t>
+        </is>
+      </c>
+      <c r="Q47" s="22" t="inlineStr">
+        <is>
+          <t>+6.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="B48" s="22" t="inlineStr">
+        <is>
+          <t>Fordham @ North Dakota State</t>
+        </is>
+      </c>
+      <c r="C48" s="22" t="inlineStr">
+        <is>
+          <t>0-38</t>
+        </is>
+      </c>
+      <c r="D48" s="22" t="inlineStr">
+        <is>
+          <t>-41.5</t>
+        </is>
+      </c>
+      <c r="E48" s="22" t="inlineStr">
+        <is>
+          <t>+38.0</t>
+        </is>
+      </c>
+      <c r="F48" s="22" t="inlineStr">
+        <is>
+          <t>-40.9</t>
+        </is>
+      </c>
+      <c r="G48" s="22" t="inlineStr">
+        <is>
+          <t>-0.6</t>
+        </is>
+      </c>
+      <c r="H48" s="22" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="I48" s="22" t="inlineStr">
+        <is>
+          <t>Lean only</t>
+        </is>
+      </c>
+      <c r="J48" s="22" t="inlineStr">
+        <is>
+          <t>-35.0</t>
+        </is>
+      </c>
+      <c r="K48" s="22" t="inlineStr">
+        <is>
+          <t>-6.5</t>
+        </is>
+      </c>
+      <c r="L48" s="22" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="M48" s="23" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="N48" s="22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O48" s="23" t="inlineStr">
+        <is>
+          <t>Ridge</t>
+        </is>
+      </c>
+      <c r="P48" s="22" t="inlineStr">
+        <is>
+          <t>+16.9</t>
+        </is>
+      </c>
+      <c r="Q48" s="22" t="inlineStr">
+        <is>
+          <t>-0.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="B49" s="22" t="inlineStr">
+        <is>
+          <t>UTEP @ Oklahoma</t>
+        </is>
+      </c>
+      <c r="C49" s="22" t="inlineStr">
+        <is>
+          <t>0-51</t>
+        </is>
+      </c>
+      <c r="D49" s="22" t="inlineStr">
+        <is>
+          <t>-40.8</t>
+        </is>
+      </c>
+      <c r="E49" s="22" t="inlineStr">
+        <is>
+          <t>+51.0</t>
+        </is>
+      </c>
+      <c r="F49" s="22" t="inlineStr">
+        <is>
+          <t>-34.8</t>
+        </is>
+      </c>
+      <c r="G49" s="22" t="inlineStr">
+        <is>
+          <t>-5.9</t>
+        </is>
+      </c>
+      <c r="H49" s="22" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="I49" s="24" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="J49" s="22" t="inlineStr">
+        <is>
+          <t>-32.8</t>
+        </is>
+      </c>
+      <c r="K49" s="22" t="inlineStr">
+        <is>
+          <t>-8.0</t>
+        </is>
+      </c>
+      <c r="L49" s="22" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="M49" s="24" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="N49" s="22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O49" s="23" t="inlineStr">
+        <is>
+          <t>Ridge</t>
+        </is>
+      </c>
+      <c r="P49" s="22" t="inlineStr">
+        <is>
+          <t>+11.0</t>
+        </is>
+      </c>
+      <c r="Q49" s="22" t="inlineStr">
+        <is>
+          <t>-8.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="B50" s="22" t="inlineStr">
+        <is>
+          <t>Hawai'i @ Stanford</t>
+        </is>
+      </c>
+      <c r="C50" s="22" t="inlineStr">
+        <is>
+          <t>27-37</t>
+        </is>
+      </c>
+      <c r="D50" s="22" t="inlineStr">
+        <is>
+          <t>-4.8</t>
+        </is>
+      </c>
+      <c r="E50" s="22" t="inlineStr">
+        <is>
+          <t>+10.0</t>
+        </is>
+      </c>
+      <c r="F50" s="22" t="inlineStr">
+        <is>
+          <t>-1.5</t>
+        </is>
+      </c>
+      <c r="G50" s="22" t="inlineStr">
+        <is>
+          <t>-3.3</t>
+        </is>
+      </c>
+      <c r="H50" s="22" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="I50" s="24" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="J50" s="22" t="inlineStr">
+        <is>
+          <t>+1.1</t>
+        </is>
+      </c>
+      <c r="K50" s="22" t="inlineStr">
+        <is>
+          <t>-5.8</t>
+        </is>
+      </c>
+      <c r="L50" s="22" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="M50" s="24" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="N50" s="22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O50" s="23" t="inlineStr">
+        <is>
+          <t>Ridge</t>
+        </is>
+      </c>
+      <c r="P50" s="22" t="inlineStr">
+        <is>
+          <t>+7.7</t>
+        </is>
+      </c>
+      <c r="Q50" s="22" t="inlineStr">
+        <is>
+          <t>-14.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="B51" s="22" t="inlineStr">
+        <is>
+          <t>Memphis @ UNLV</t>
+        </is>
+      </c>
+      <c r="C51" s="22" t="inlineStr">
+        <is>
+          <t>27-21</t>
+        </is>
+      </c>
+      <c r="D51" s="22" t="inlineStr">
+        <is>
+          <t>-4.8</t>
+        </is>
+      </c>
+      <c r="E51" s="22" t="inlineStr">
+        <is>
+          <t>-6.0</t>
+        </is>
+      </c>
+      <c r="F51" s="22" t="inlineStr">
+        <is>
+          <t>-10.9</t>
+        </is>
+      </c>
+      <c r="G51" s="22" t="inlineStr">
+        <is>
+          <t>+6.2</t>
+        </is>
+      </c>
+      <c r="H51" s="22" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="I51" s="24" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="J51" s="22" t="inlineStr">
+        <is>
+          <t>-7.4</t>
+        </is>
+      </c>
+      <c r="K51" s="22" t="inlineStr">
+        <is>
+          <t>+2.6</t>
+        </is>
+      </c>
+      <c r="L51" s="22" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="M51" s="24" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="N51" s="22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="O51" s="23" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="P51" s="22" t="inlineStr">
+        <is>
+          <t>+13.9</t>
+        </is>
+      </c>
+      <c r="Q51" s="22" t="inlineStr">
+        <is>
+          <t>-11.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="B52" s="22" t="inlineStr">
         <is>
           <t>San José State @ USC</t>
         </is>
       </c>
-      <c r="C22" s="15" t="inlineStr">
+      <c r="C52" s="22" t="inlineStr">
+        <is>
+          <t>26-42</t>
+        </is>
+      </c>
+      <c r="D52" s="22" t="inlineStr">
         <is>
           <t>-37.2</t>
         </is>
       </c>
-      <c r="D22" s="15" t="inlineStr">
-        <is>
-          <t>-32.2</t>
-        </is>
-      </c>
-      <c r="E22" s="15" t="inlineStr">
-        <is>
-          <t>-31.0</t>
-        </is>
-      </c>
-      <c r="F22" s="15" t="inlineStr">
+      <c r="E52" s="22" t="inlineStr">
+        <is>
+          <t>+16.0</t>
+        </is>
+      </c>
+      <c r="F52" s="22" t="inlineStr">
+        <is>
+          <t>-34.6</t>
+        </is>
+      </c>
+      <c r="G52" s="22" t="inlineStr">
+        <is>
+          <t>-2.7</t>
+        </is>
+      </c>
+      <c r="H52" s="22" t="inlineStr">
         <is>
           <t>Away</t>
         </is>
       </c>
-      <c r="G22" s="15" t="inlineStr">
+      <c r="I52" s="23" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="J52" s="22" t="inlineStr">
+        <is>
+          <t>-35.3</t>
+        </is>
+      </c>
+      <c r="K52" s="22" t="inlineStr">
+        <is>
+          <t>-2.0</t>
+        </is>
+      </c>
+      <c r="L52" s="22" t="inlineStr">
         <is>
           <t>Away</t>
         </is>
       </c>
-      <c r="H22" s="15" t="inlineStr">
+      <c r="M52" s="22" t="inlineStr">
+        <is>
+          <t>Lean only</t>
+        </is>
+      </c>
+      <c r="N52" s="22" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="I22" s="16" t="inlineStr">
-        <is>
-          <t>Ridge</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="B23" s="15" t="inlineStr">
-        <is>
-          <t>Jacksonville State @ North Dakota State</t>
-        </is>
-      </c>
-      <c r="C23" s="15" t="inlineStr">
-        <is>
-          <t>-6.8</t>
-        </is>
-      </c>
-      <c r="D23" s="15" t="inlineStr">
-        <is>
-          <t>-16.4</t>
-        </is>
-      </c>
-      <c r="E23" s="15" t="inlineStr">
-        <is>
-          <t>-16.7</t>
-        </is>
-      </c>
-      <c r="F23" s="15" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="G23" s="15" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="H23" s="15" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I23" s="16" t="inlineStr">
-        <is>
-          <t>Ridge</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="B24" s="15" t="inlineStr">
-        <is>
-          <t>Hawai'i @ Stanford</t>
-        </is>
-      </c>
-      <c r="C24" s="15" t="inlineStr">
-        <is>
-          <t>-4.8</t>
-        </is>
-      </c>
-      <c r="D24" s="15" t="inlineStr">
-        <is>
-          <t>-4.3</t>
-        </is>
-      </c>
-      <c r="E24" s="15" t="inlineStr">
-        <is>
-          <t>-1.8</t>
-        </is>
-      </c>
-      <c r="F24" s="15" t="inlineStr">
-        <is>
-          <t>Away</t>
-        </is>
-      </c>
-      <c r="G24" s="15" t="inlineStr">
-        <is>
-          <t>Away</t>
-        </is>
-      </c>
-      <c r="H24" s="15" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I24" s="16" t="inlineStr">
-        <is>
-          <t>Ridge</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="B25" s="15" t="inlineStr">
-        <is>
-          <t>Memphis @ UNLV</t>
-        </is>
-      </c>
-      <c r="C25" s="15" t="inlineStr">
-        <is>
-          <t>-4.8</t>
-        </is>
-      </c>
-      <c r="D25" s="15" t="inlineStr">
-        <is>
-          <t>-9.9</t>
-        </is>
-      </c>
-      <c r="E25" s="15" t="inlineStr">
-        <is>
-          <t>-5.7</t>
-        </is>
-      </c>
-      <c r="F25" s="15" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="G25" s="15" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="H25" s="15" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I25" s="16" t="inlineStr">
+      <c r="O52" s="23" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="B26" s="15" t="inlineStr">
-        <is>
-          <t>San José State @ Eastern Michigan</t>
-        </is>
-      </c>
-      <c r="C26" s="15" t="inlineStr">
-        <is>
-          <t>-3.0</t>
-        </is>
-      </c>
-      <c r="D26" s="15" t="inlineStr">
-        <is>
-          <t>-12.8</t>
-        </is>
-      </c>
-      <c r="E26" s="15" t="inlineStr">
-        <is>
-          <t>-11.3</t>
-        </is>
-      </c>
-      <c r="F26" s="15" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="G26" s="15" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="H26" s="15" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I26" s="16" t="inlineStr">
-        <is>
-          <t>XGBoost</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="B27" s="15" t="inlineStr">
-        <is>
-          <t>UTEP @ Oklahoma</t>
-        </is>
-      </c>
-      <c r="C27" s="15" t="inlineStr">
-        <is>
-          <t>-41.5</t>
-        </is>
-      </c>
-      <c r="D27" s="15" t="inlineStr">
-        <is>
-          <t>-33.9</t>
-        </is>
-      </c>
-      <c r="E27" s="15" t="inlineStr">
-        <is>
-          <t>-33.5</t>
-        </is>
-      </c>
-      <c r="F27" s="15" t="inlineStr">
-        <is>
-          <t>Away</t>
-        </is>
-      </c>
-      <c r="G27" s="15" t="inlineStr">
-        <is>
-          <t>Away</t>
-        </is>
-      </c>
-      <c r="H27" s="15" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I27" s="16" t="inlineStr">
-        <is>
-          <t>Ridge</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="B28" s="15" t="inlineStr">
-        <is>
-          <t>Duquesne @ Air Force</t>
-        </is>
-      </c>
-      <c r="C28" s="15" t="inlineStr">
-        <is>
-          <t>-28.5</t>
-        </is>
-      </c>
-      <c r="D28" s="15" t="inlineStr">
-        <is>
-          <t>-22.0</t>
-        </is>
-      </c>
-      <c r="E28" s="15" t="inlineStr">
-        <is>
-          <t>-33.5</t>
-        </is>
-      </c>
-      <c r="F28" s="15" t="inlineStr">
-        <is>
-          <t>Away</t>
-        </is>
-      </c>
-      <c r="G28" s="15" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="H28" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I28" s="16" t="inlineStr">
-        <is>
-          <t>XGBoost</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="B29" s="15" t="inlineStr">
-        <is>
-          <t>Fordham @ North Dakota State</t>
-        </is>
-      </c>
-      <c r="C29" s="15" t="inlineStr">
-        <is>
-          <t>-39.5</t>
-        </is>
-      </c>
-      <c r="D29" s="15" t="inlineStr">
-        <is>
-          <t>-49.9</t>
-        </is>
-      </c>
-      <c r="E29" s="15" t="inlineStr">
-        <is>
-          <t>-36.7</t>
-        </is>
-      </c>
-      <c r="F29" s="15" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="G29" s="15" t="inlineStr">
-        <is>
-          <t>Away</t>
-        </is>
-      </c>
-      <c r="H29" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I29" s="16" t="inlineStr">
-        <is>
-          <t>XGBoost</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="B30" s="15" t="inlineStr">
-        <is>
-          <t>Northern Illinois @ Iowa</t>
-        </is>
-      </c>
-      <c r="C30" s="15" t="inlineStr">
-        <is>
-          <t>-31.2</t>
-        </is>
-      </c>
-      <c r="D30" s="15" t="inlineStr">
-        <is>
-          <t>-30.4</t>
-        </is>
-      </c>
-      <c r="E30" s="15" t="inlineStr">
-        <is>
-          <t>-27.0</t>
-        </is>
-      </c>
-      <c r="F30" s="15" t="inlineStr">
-        <is>
-          <t>Away</t>
-        </is>
-      </c>
-      <c r="G30" s="15" t="inlineStr">
-        <is>
-          <t>Away</t>
-        </is>
-      </c>
-      <c r="H30" s="15" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I30" s="16" t="inlineStr">
-        <is>
-          <t>Ridge</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="B31" s="15" t="inlineStr">
-        <is>
-          <t>Wyoming @ Colorado State</t>
-        </is>
-      </c>
-      <c r="C31" s="15" t="inlineStr">
-        <is>
-          <t>-3.0</t>
-        </is>
-      </c>
-      <c r="D31" s="15" t="inlineStr">
-        <is>
-          <t>-5.2</t>
-        </is>
-      </c>
-      <c r="E31" s="15" t="inlineStr">
-        <is>
-          <t>-1.6</t>
-        </is>
-      </c>
-      <c r="F31" s="15" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="G31" s="15" t="inlineStr">
-        <is>
-          <t>Away</t>
-        </is>
-      </c>
-      <c r="H31" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I31" s="16" t="inlineStr">
-        <is>
-          <t>XGBoost</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="B32" s="15" t="inlineStr">
-        <is>
-          <t>Central Michigan @ New Mexico</t>
-        </is>
-      </c>
-      <c r="C32" s="15" t="inlineStr">
-        <is>
-          <t>-10.0</t>
-        </is>
-      </c>
-      <c r="D32" s="15" t="inlineStr">
-        <is>
-          <t>-17.2</t>
-        </is>
-      </c>
-      <c r="E32" s="15" t="inlineStr">
-        <is>
-          <t>-10.7</t>
-        </is>
-      </c>
-      <c r="F32" s="15" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="G32" s="15" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="H32" s="15" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I32" s="16" t="inlineStr">
-        <is>
-          <t>XGBoost</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="B33" s="15" t="inlineStr">
-        <is>
-          <t>UNLV @ Hawai'i</t>
-        </is>
-      </c>
-      <c r="C33" s="15" t="inlineStr">
-        <is>
-          <t>+3.0</t>
-        </is>
-      </c>
-      <c r="D33" s="15" t="inlineStr">
-        <is>
-          <t>+6.5</t>
-        </is>
-      </c>
-      <c r="E33" s="15" t="inlineStr">
-        <is>
-          <t>+0.1</t>
-        </is>
-      </c>
-      <c r="F33" s="15" t="inlineStr">
-        <is>
-          <t>Away</t>
-        </is>
-      </c>
-      <c r="G33" s="15" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="H33" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="I33" s="16" t="inlineStr">
-        <is>
-          <t>XGBoost</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="B34" s="15" t="inlineStr">
-        <is>
-          <t>Western Kentucky @ Nevada</t>
-        </is>
-      </c>
-      <c r="C34" s="15" t="inlineStr">
-        <is>
-          <t>+2.5</t>
-        </is>
-      </c>
-      <c r="D34" s="15" t="inlineStr">
-        <is>
-          <t>+5.0</t>
-        </is>
-      </c>
-      <c r="E34" s="15" t="inlineStr">
-        <is>
-          <t>+10.7</t>
-        </is>
-      </c>
-      <c r="F34" s="15" t="inlineStr">
-        <is>
-          <t>Away</t>
-        </is>
-      </c>
-      <c r="G34" s="15" t="inlineStr">
-        <is>
-          <t>Away</t>
-        </is>
-      </c>
-      <c r="H34" s="15" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="I34" s="16" t="inlineStr">
-        <is>
-          <t>Ridge</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="12" t="inlineStr">
-        <is>
-          <t>* Tighter (Live) compares each model's line to TODAY's still-moving market line, not a final closing line -- it will keep changing until kickoff. See the graded Game-by-Game table below for the real, closing-line version of this comparison.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="13" t="inlineStr">
-        <is>
-          <t>2026 Mountain West Games -- Game by Game</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="25.5" customHeight="1">
-      <c r="A39" s="14" t="inlineStr">
-        <is>
-          <t>Week</t>
-        </is>
-      </c>
-      <c r="B39" s="14" t="inlineStr">
-        <is>
-          <t>Matchup</t>
-        </is>
-      </c>
-      <c r="C39" s="14" t="inlineStr">
-        <is>
-          <t>Final Score</t>
-        </is>
-      </c>
-      <c r="D39" s="14" t="inlineStr">
-        <is>
-          <t>Vegas Spread (Home)</t>
-        </is>
-      </c>
-      <c r="E39" s="14" t="inlineStr">
-        <is>
-          <t>Actual Margin (Home)</t>
-        </is>
-      </c>
-      <c r="F39" s="14" t="inlineStr">
-        <is>
-          <t>Ridge Line</t>
-        </is>
-      </c>
-      <c r="G39" s="14" t="inlineStr">
-        <is>
-          <t>Ridge Edge</t>
-        </is>
-      </c>
-      <c r="H39" s="14" t="inlineStr">
-        <is>
-          <t>Ridge Lean</t>
-        </is>
-      </c>
-      <c r="I39" s="14" t="inlineStr">
-        <is>
-          <t>Ridge Result</t>
-        </is>
-      </c>
-      <c r="J39" s="14" t="inlineStr">
-        <is>
-          <t>XGBoost Line</t>
-        </is>
-      </c>
-      <c r="K39" s="14" t="inlineStr">
-        <is>
-          <t>XGBoost Edge</t>
-        </is>
-      </c>
-      <c r="L39" s="14" t="inlineStr">
-        <is>
-          <t>XGBoost Lean</t>
-        </is>
-      </c>
-      <c r="M39" s="14" t="inlineStr">
-        <is>
-          <t>XGBoost Result</t>
-        </is>
-      </c>
-      <c r="N39" s="14" t="inlineStr">
-        <is>
-          <t>Models Agree?</t>
-        </is>
-      </c>
-      <c r="O39" s="14" t="inlineStr">
-        <is>
-          <t>Tighter CLV Line</t>
-        </is>
-      </c>
-      <c r="P39" s="14" t="inlineStr">
-        <is>
-          <t>Ridge CLV Pts (Cum.)</t>
-        </is>
-      </c>
-      <c r="Q39" s="14" t="inlineStr">
-        <is>
-          <t>XGBoost CLV Pts (Cum.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="B40" s="15" t="inlineStr">
-        <is>
-          <t>Jacksonville State @ North Dakota State</t>
-        </is>
-      </c>
-      <c r="C40" s="15" t="inlineStr">
-        <is>
-          <t>7-33</t>
-        </is>
-      </c>
-      <c r="D40" s="15" t="inlineStr">
-        <is>
-          <t>-6.8</t>
-        </is>
-      </c>
-      <c r="E40" s="15" t="inlineStr">
-        <is>
-          <t>+26.0</t>
-        </is>
-      </c>
-      <c r="F40" s="15" t="inlineStr">
-        <is>
-          <t>-16.3</t>
-        </is>
-      </c>
-      <c r="G40" s="15" t="inlineStr">
-        <is>
-          <t>+9.6</t>
-        </is>
-      </c>
-      <c r="H40" s="15" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="I40" s="16" t="inlineStr">
-        <is>
-          <t>Win</t>
-        </is>
-      </c>
-      <c r="J40" s="15" t="inlineStr">
-        <is>
-          <t>-15.3</t>
-        </is>
-      </c>
-      <c r="K40" s="15" t="inlineStr">
-        <is>
-          <t>+8.6</t>
-        </is>
-      </c>
-      <c r="L40" s="15" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="M40" s="16" t="inlineStr">
-        <is>
-          <t>Win</t>
-        </is>
-      </c>
-      <c r="N40" s="15" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O40" s="16" t="inlineStr">
-        <is>
-          <t>XGBoost</t>
-        </is>
-      </c>
-      <c r="P40" s="15" t="inlineStr">
-        <is>
-          <t>+9.6</t>
-        </is>
-      </c>
-      <c r="Q40" s="15" t="inlineStr">
-        <is>
-          <t>+8.6</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="B41" s="15" t="inlineStr">
-        <is>
-          <t>Hawai'i @ Stanford</t>
-        </is>
-      </c>
-      <c r="C41" s="15" t="inlineStr">
-        <is>
-          <t>27-37</t>
-        </is>
-      </c>
-      <c r="D41" s="15" t="inlineStr">
-        <is>
-          <t>-4.8</t>
-        </is>
-      </c>
-      <c r="E41" s="15" t="inlineStr">
-        <is>
-          <t>+10.0</t>
-        </is>
-      </c>
-      <c r="F41" s="15" t="inlineStr">
-        <is>
-          <t>-4.2</t>
-        </is>
-      </c>
-      <c r="G41" s="15" t="inlineStr">
-        <is>
-          <t>-0.5</t>
-        </is>
-      </c>
-      <c r="H41" s="15" t="inlineStr">
-        <is>
-          <t>Away</t>
-        </is>
-      </c>
-      <c r="I41" s="15" t="inlineStr">
-        <is>
-          <t>Lean only</t>
-        </is>
-      </c>
-      <c r="J41" s="15" t="inlineStr">
-        <is>
-          <t>-0.7</t>
-        </is>
-      </c>
-      <c r="K41" s="15" t="inlineStr">
-        <is>
-          <t>-4.1</t>
-        </is>
-      </c>
-      <c r="L41" s="15" t="inlineStr">
-        <is>
-          <t>Away</t>
-        </is>
-      </c>
-      <c r="M41" s="17" t="inlineStr">
-        <is>
-          <t>Loss</t>
-        </is>
-      </c>
-      <c r="N41" s="15" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O41" s="16" t="inlineStr">
-        <is>
-          <t>Ridge</t>
-        </is>
-      </c>
-      <c r="P41" s="15" t="inlineStr">
-        <is>
-          <t>+9.0</t>
-        </is>
-      </c>
-      <c r="Q41" s="15" t="inlineStr">
-        <is>
-          <t>+4.5</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="B42" s="15" t="inlineStr">
-        <is>
-          <t>Memphis @ UNLV</t>
-        </is>
-      </c>
-      <c r="C42" s="15" t="inlineStr">
-        <is>
-          <t>27-21</t>
-        </is>
-      </c>
-      <c r="D42" s="15" t="inlineStr">
-        <is>
-          <t>-4.8</t>
-        </is>
-      </c>
-      <c r="E42" s="15" t="inlineStr">
-        <is>
-          <t>-6.0</t>
-        </is>
-      </c>
-      <c r="F42" s="15" t="inlineStr">
-        <is>
-          <t>-9.8</t>
-        </is>
-      </c>
-      <c r="G42" s="15" t="inlineStr">
-        <is>
-          <t>+5.1</t>
-        </is>
-      </c>
-      <c r="H42" s="15" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="I42" s="17" t="inlineStr">
-        <is>
-          <t>Loss</t>
-        </is>
-      </c>
-      <c r="J42" s="15" t="inlineStr">
-        <is>
-          <t>-6.5</t>
-        </is>
-      </c>
-      <c r="K42" s="15" t="inlineStr">
-        <is>
-          <t>+1.8</t>
-        </is>
-      </c>
-      <c r="L42" s="15" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="M42" s="15" t="inlineStr">
-        <is>
-          <t>Lean only</t>
-        </is>
-      </c>
-      <c r="N42" s="15" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O42" s="16" t="inlineStr">
-        <is>
-          <t>XGBoost</t>
-        </is>
-      </c>
-      <c r="P42" s="15" t="inlineStr">
-        <is>
-          <t>+14.1</t>
-        </is>
-      </c>
-      <c r="Q42" s="15" t="inlineStr">
-        <is>
-          <t>+6.3</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="B43" s="15" t="inlineStr">
-        <is>
-          <t>San José State @ USC</t>
-        </is>
-      </c>
-      <c r="C43" s="15" t="inlineStr">
-        <is>
-          <t>26-42</t>
-        </is>
-      </c>
-      <c r="D43" s="15" t="inlineStr">
-        <is>
-          <t>-37.2</t>
-        </is>
-      </c>
-      <c r="E43" s="15" t="inlineStr">
-        <is>
-          <t>+16.0</t>
-        </is>
-      </c>
-      <c r="F43" s="15" t="inlineStr">
-        <is>
-          <t>-32.1</t>
-        </is>
-      </c>
-      <c r="G43" s="15" t="inlineStr">
-        <is>
-          <t>-5.1</t>
-        </is>
-      </c>
-      <c r="H43" s="15" t="inlineStr">
-        <is>
-          <t>Away</t>
-        </is>
-      </c>
-      <c r="I43" s="16" t="inlineStr">
-        <is>
-          <t>Win</t>
-        </is>
-      </c>
-      <c r="J43" s="15" t="inlineStr">
-        <is>
-          <t>-32.9</t>
-        </is>
-      </c>
-      <c r="K43" s="15" t="inlineStr">
-        <is>
-          <t>-4.4</t>
-        </is>
-      </c>
-      <c r="L43" s="15" t="inlineStr">
-        <is>
-          <t>Away</t>
-        </is>
-      </c>
-      <c r="M43" s="16" t="inlineStr">
-        <is>
-          <t>Win</t>
-        </is>
-      </c>
-      <c r="N43" s="15" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="O43" s="16" t="inlineStr">
-        <is>
-          <t>XGBoost</t>
-        </is>
-      </c>
-      <c r="P43" s="15" t="inlineStr">
-        <is>
-          <t>+9.0</t>
-        </is>
-      </c>
-      <c r="Q43" s="15" t="inlineStr">
-        <is>
-          <t>+1.9</t>
+      <c r="P52" s="22" t="inlineStr">
+        <is>
+          <t>+11.2</t>
+        </is>
+      </c>
+      <c r="Q52" s="22" t="inlineStr">
+        <is>
+          <t>-13.3</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update either data or bets
</commit_message>
<xml_diff>
--- a/excel/MW_Handicapping_Tracker.xlsx
+++ b/excel/MW_Handicapping_Tracker.xlsx
@@ -255,7 +255,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -280,6 +280,7 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -834,7 +835,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R29"/>
+  <dimension ref="A1:R42"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1830,6 +1831,19 @@
       <c r="M29" s="6" t="n"/>
       <c r="N29" s="6" t="n"/>
     </row>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42"/>
   </sheetData>
   <conditionalFormatting sqref="C2:C500">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -1962,7 +1976,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>North Dakota State -7.5</t>
+          <t>North Dakota State</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -1986,11 +2000,11 @@
           <t>W</t>
         </is>
       </c>
-      <c r="L2" s="6">
+      <c r="L2" s="18">
         <f>IF(K2="W",IF(G2&lt;0,H2*100/ABS(G2),H2*G2/100),IF(K2="L",-H2,0))</f>
         <v/>
       </c>
-      <c r="M2" s="6">
+      <c r="M2" s="18">
         <f>Settings!$B$4+SUM(L$2:L2)</f>
         <v/>
       </c>
@@ -2016,7 +2030,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>North Dakota State -285</t>
+          <t>North Dakota State</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -2034,11 +2048,11 @@
           <t>W</t>
         </is>
       </c>
-      <c r="L3" s="6">
+      <c r="L3" s="18">
         <f>IF(K3="W",IF(G3&lt;0,H3*100/ABS(G3),H3*G3/100),IF(K3="L",-H3,0))</f>
         <v/>
       </c>
-      <c r="M3" s="6">
+      <c r="M3" s="18">
         <f>Settings!$B$4+SUM(L$2:L3)</f>
         <v/>
       </c>
@@ -2064,7 +2078,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>UNLV -178</t>
+          <t>UNLV</t>
         </is>
       </c>
       <c r="G4" t="n">
@@ -2082,11 +2096,11 @@
           <t>L</t>
         </is>
       </c>
-      <c r="L4" s="6">
+      <c r="L4" s="18">
         <f>IF(K4="W",IF(G4&lt;0,H4*100/ABS(G4),H4*G4/100),IF(K4="L",-H4,0))</f>
         <v/>
       </c>
-      <c r="M4" s="6">
+      <c r="M4" s="18">
         <f>Settings!$B$4+SUM(L$2:L4)</f>
         <v/>
       </c>
@@ -2130,11 +2144,11 @@
           <t>L</t>
         </is>
       </c>
-      <c r="L5" s="6">
+      <c r="L5" s="18">
         <f>IF(K5="W",IF(G5&lt;0,H5*100/ABS(G5),H5*G5/100),IF(K5="L",-H5,0))</f>
         <v/>
       </c>
-      <c r="M5" s="6">
+      <c r="M5" s="18">
         <f>Settings!$B$4+SUM(L$2:L5)</f>
         <v/>
       </c>
@@ -2160,7 +2174,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Eastern Michigan -3.5</t>
+          <t>Eastern Michigan</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -2181,11 +2195,11 @@
           <t>L</t>
         </is>
       </c>
-      <c r="L6" s="6">
+      <c r="L6" s="18">
         <f>IF(K6="W",IF(G6&lt;0,H6*100/ABS(G6),H6*G6/100),IF(K6="L",-H6,0))</f>
         <v/>
       </c>
-      <c r="M6" s="6">
+      <c r="M6" s="18">
         <f>Settings!$B$4+SUM(L$2:L6)</f>
         <v/>
       </c>
@@ -2229,11 +2243,11 @@
           <t>L</t>
         </is>
       </c>
-      <c r="L7" s="6">
+      <c r="L7" s="18">
         <f>IF(K7="W",IF(G7&lt;0,H7*100/ABS(G7),H7*G7/100),IF(K7="L",-H7,0))</f>
         <v/>
       </c>
-      <c r="M7" s="6">
+      <c r="M7" s="18">
         <f>Settings!$B$4+SUM(L$2:L7)</f>
         <v/>
       </c>
@@ -2283,11 +2297,11 @@
           <t>W</t>
         </is>
       </c>
-      <c r="L8" s="6">
+      <c r="L8" s="18">
         <f>IF(K8="W",IF(G8&lt;0,H8*100/ABS(G8),H8*G8/100),IF(K8="L",-H8,0))</f>
         <v/>
       </c>
-      <c r="M8" s="6">
+      <c r="M8" s="18">
         <f>Settings!$B$4+SUM(L$2:L8)</f>
         <v/>
       </c>
@@ -2331,11 +2345,11 @@
           <t>W</t>
         </is>
       </c>
-      <c r="L9" s="6">
+      <c r="L9" s="18">
         <f>IF(K9="W",IF(G9&lt;0,H9*100/ABS(G9),H9*G9/100),IF(K9="L",-H9,0))</f>
         <v/>
       </c>
-      <c r="M9" s="6">
+      <c r="M9" s="18">
         <f>Settings!$B$4+SUM(L$2:L9)</f>
         <v/>
       </c>
@@ -2385,11 +2399,11 @@
           <t>W</t>
         </is>
       </c>
-      <c r="L10" s="6">
+      <c r="L10" s="18">
         <f>IF(K10="W",IF(G10&lt;0,H10*100/ABS(G10),H10*G10/100),IF(K10="L",-H10,0))</f>
         <v/>
       </c>
-      <c r="M10" s="6">
+      <c r="M10" s="18">
         <f>Settings!$B$4+SUM(L$2:L10)</f>
         <v/>
       </c>
@@ -2400,11 +2414,11 @@
         <f>IF(I11="","",I11-F11)</f>
         <v/>
       </c>
-      <c r="L11" s="6">
+      <c r="L11" s="18">
         <f>IF(K11="W",IF(G11&lt;0,H11*100/ABS(G11),H11*G11/100),IF(K11="L",-H11,0))</f>
         <v/>
       </c>
-      <c r="M11" s="6">
+      <c r="M11" s="18">
         <f>Settings!$B$4+SUM(L$2:L11)</f>
         <v/>
       </c>
@@ -2414,11 +2428,11 @@
         <f>IF(I12="","",I12-F12)</f>
         <v/>
       </c>
-      <c r="L12" s="6">
+      <c r="L12" s="18">
         <f>IF(K12="W",IF(G12&lt;0,H12*100/ABS(G12),H12*G12/100),IF(K12="L",-H12,0))</f>
         <v/>
       </c>
-      <c r="M12" s="6">
+      <c r="M12" s="18">
         <f>Settings!$B$4+SUM(L$2:L12)</f>
         <v/>
       </c>
@@ -2428,11 +2442,11 @@
         <f>IF(I13="","",I13-F13)</f>
         <v/>
       </c>
-      <c r="L13" s="6">
+      <c r="L13" s="18">
         <f>IF(K13="W",IF(G13&lt;0,H13*100/ABS(G13),H13*G13/100),IF(K13="L",-H13,0))</f>
         <v/>
       </c>
-      <c r="M13" s="6">
+      <c r="M13" s="18">
         <f>Settings!$B$4+SUM(L$2:L13)</f>
         <v/>
       </c>
@@ -2442,11 +2456,11 @@
         <f>IF(I14="","",I14-F14)</f>
         <v/>
       </c>
-      <c r="L14" s="6">
+      <c r="L14" s="18">
         <f>IF(K14="W",IF(G14&lt;0,H14*100/ABS(G14),H14*G14/100),IF(K14="L",-H14,0))</f>
         <v/>
       </c>
-      <c r="M14" s="6">
+      <c r="M14" s="18">
         <f>Settings!$B$4+SUM(L$2:L14)</f>
         <v/>
       </c>
@@ -2456,11 +2470,11 @@
         <f>IF(I15="","",I15-F15)</f>
         <v/>
       </c>
-      <c r="L15" s="6">
+      <c r="L15" s="18">
         <f>IF(K15="W",IF(G15&lt;0,H15*100/ABS(G15),H15*G15/100),IF(K15="L",-H15,0))</f>
         <v/>
       </c>
-      <c r="M15" s="6">
+      <c r="M15" s="18">
         <f>Settings!$B$4+SUM(L$2:L15)</f>
         <v/>
       </c>
@@ -2470,11 +2484,11 @@
         <f>IF(I16="","",I16-F16)</f>
         <v/>
       </c>
-      <c r="L16" s="6">
+      <c r="L16" s="18">
         <f>IF(K16="W",IF(G16&lt;0,H16*100/ABS(G16),H16*G16/100),IF(K16="L",-H16,0))</f>
         <v/>
       </c>
-      <c r="M16" s="6">
+      <c r="M16" s="18">
         <f>Settings!$B$4+SUM(L$2:L16)</f>
         <v/>
       </c>
@@ -2484,11 +2498,11 @@
         <f>IF(I17="","",I17-F17)</f>
         <v/>
       </c>
-      <c r="L17" s="6">
+      <c r="L17" s="18">
         <f>IF(K17="W",IF(G17&lt;0,H17*100/ABS(G17),H17*G17/100),IF(K17="L",-H17,0))</f>
         <v/>
       </c>
-      <c r="M17" s="6">
+      <c r="M17" s="18">
         <f>Settings!$B$4+SUM(L$2:L17)</f>
         <v/>
       </c>
@@ -2498,11 +2512,11 @@
         <f>IF(I18="","",I18-F18)</f>
         <v/>
       </c>
-      <c r="L18" s="6">
+      <c r="L18" s="18">
         <f>IF(K18="W",IF(G18&lt;0,H18*100/ABS(G18),H18*G18/100),IF(K18="L",-H18,0))</f>
         <v/>
       </c>
-      <c r="M18" s="6">
+      <c r="M18" s="18">
         <f>Settings!$B$4+SUM(L$2:L18)</f>
         <v/>
       </c>
@@ -2512,11 +2526,11 @@
         <f>IF(I19="","",I19-F19)</f>
         <v/>
       </c>
-      <c r="L19" s="6">
+      <c r="L19" s="18">
         <f>IF(K19="W",IF(G19&lt;0,H19*100/ABS(G19),H19*G19/100),IF(K19="L",-H19,0))</f>
         <v/>
       </c>
-      <c r="M19" s="6">
+      <c r="M19" s="18">
         <f>Settings!$B$4+SUM(L$2:L19)</f>
         <v/>
       </c>
@@ -2526,11 +2540,11 @@
         <f>IF(I20="","",I20-F20)</f>
         <v/>
       </c>
-      <c r="L20" s="6">
+      <c r="L20" s="18">
         <f>IF(K20="W",IF(G20&lt;0,H20*100/ABS(G20),H20*G20/100),IF(K20="L",-H20,0))</f>
         <v/>
       </c>
-      <c r="M20" s="6">
+      <c r="M20" s="18">
         <f>Settings!$B$4+SUM(L$2:L20)</f>
         <v/>
       </c>
@@ -2540,11 +2554,11 @@
         <f>IF(I21="","",I21-F21)</f>
         <v/>
       </c>
-      <c r="L21" s="6">
+      <c r="L21" s="18">
         <f>IF(K21="W",IF(G21&lt;0,H21*100/ABS(G21),H21*G21/100),IF(K21="L",-H21,0))</f>
         <v/>
       </c>
-      <c r="M21" s="6">
+      <c r="M21" s="18">
         <f>Settings!$B$4+SUM(L$2:L21)</f>
         <v/>
       </c>
@@ -2554,11 +2568,11 @@
         <f>IF(I22="","",I22-F22)</f>
         <v/>
       </c>
-      <c r="L22" s="6">
+      <c r="L22" s="18">
         <f>IF(K22="W",IF(G22&lt;0,H22*100/ABS(G22),H22*G22/100),IF(K22="L",-H22,0))</f>
         <v/>
       </c>
-      <c r="M22" s="6">
+      <c r="M22" s="18">
         <f>Settings!$B$4+SUM(L$2:L22)</f>
         <v/>
       </c>
@@ -2568,11 +2582,11 @@
         <f>IF(I23="","",I23-F23)</f>
         <v/>
       </c>
-      <c r="L23" s="6">
+      <c r="L23" s="18">
         <f>IF(K23="W",IF(G23&lt;0,H23*100/ABS(G23),H23*G23/100),IF(K23="L",-H23,0))</f>
         <v/>
       </c>
-      <c r="M23" s="6">
+      <c r="M23" s="18">
         <f>Settings!$B$4+SUM(L$2:L23)</f>
         <v/>
       </c>
@@ -2582,11 +2596,11 @@
         <f>IF(I24="","",I24-F24)</f>
         <v/>
       </c>
-      <c r="L24" s="6">
+      <c r="L24" s="18">
         <f>IF(K24="W",IF(G24&lt;0,H24*100/ABS(G24),H24*G24/100),IF(K24="L",-H24,0))</f>
         <v/>
       </c>
-      <c r="M24" s="6">
+      <c r="M24" s="18">
         <f>Settings!$B$4+SUM(L$2:L24)</f>
         <v/>
       </c>
@@ -2596,11 +2610,11 @@
         <f>IF(I25="","",I25-F25)</f>
         <v/>
       </c>
-      <c r="L25" s="6">
+      <c r="L25" s="18">
         <f>IF(K25="W",IF(G25&lt;0,H25*100/ABS(G25),H25*G25/100),IF(K25="L",-H25,0))</f>
         <v/>
       </c>
-      <c r="M25" s="6">
+      <c r="M25" s="18">
         <f>Settings!$B$4+SUM(L$2:L25)</f>
         <v/>
       </c>
@@ -2610,11 +2624,11 @@
         <f>IF(I26="","",I26-F26)</f>
         <v/>
       </c>
-      <c r="L26" s="6">
+      <c r="L26" s="18">
         <f>IF(K26="W",IF(G26&lt;0,H26*100/ABS(G26),H26*G26/100),IF(K26="L",-H26,0))</f>
         <v/>
       </c>
-      <c r="M26" s="6">
+      <c r="M26" s="18">
         <f>Settings!$B$4+SUM(L$2:L26)</f>
         <v/>
       </c>
@@ -2624,11 +2638,11 @@
         <f>IF(I27="","",I27-F27)</f>
         <v/>
       </c>
-      <c r="L27" s="6">
+      <c r="L27" s="18">
         <f>IF(K27="W",IF(G27&lt;0,H27*100/ABS(G27),H27*G27/100),IF(K27="L",-H27,0))</f>
         <v/>
       </c>
-      <c r="M27" s="6">
+      <c r="M27" s="18">
         <f>Settings!$B$4+SUM(L$2:L27)</f>
         <v/>
       </c>
@@ -2638,11 +2652,11 @@
         <f>IF(I28="","",I28-F28)</f>
         <v/>
       </c>
-      <c r="L28" s="6">
+      <c r="L28" s="18">
         <f>IF(K28="W",IF(G28&lt;0,H28*100/ABS(G28),H28*G28/100),IF(K28="L",-H28,0))</f>
         <v/>
       </c>
-      <c r="M28" s="6">
+      <c r="M28" s="18">
         <f>Settings!$B$4+SUM(L$2:L28)</f>
         <v/>
       </c>
@@ -2652,11 +2666,11 @@
         <f>IF(I29="","",I29-F29)</f>
         <v/>
       </c>
-      <c r="L29" s="6">
+      <c r="L29" s="18">
         <f>IF(K29="W",IF(G29&lt;0,H29*100/ABS(G29),H29*G29/100),IF(K29="L",-H29,0))</f>
         <v/>
       </c>
-      <c r="M29" s="6">
+      <c r="M29" s="18">
         <f>Settings!$B$4+SUM(L$2:L29)</f>
         <v/>
       </c>
@@ -2666,11 +2680,11 @@
         <f>IF(I30="","",I30-F30)</f>
         <v/>
       </c>
-      <c r="L30" s="6">
+      <c r="L30" s="18">
         <f>IF(K30="W",IF(G30&lt;0,H30*100/ABS(G30),H30*G30/100),IF(K30="L",-H30,0))</f>
         <v/>
       </c>
-      <c r="M30" s="6">
+      <c r="M30" s="18">
         <f>Settings!$B$4+SUM(L$2:L30)</f>
         <v/>
       </c>
@@ -2680,11 +2694,11 @@
         <f>IF(I31="","",I31-F31)</f>
         <v/>
       </c>
-      <c r="L31" s="6">
+      <c r="L31" s="18">
         <f>IF(K31="W",IF(G31&lt;0,H31*100/ABS(G31),H31*G31/100),IF(K31="L",-H31,0))</f>
         <v/>
       </c>
-      <c r="M31" s="6">
+      <c r="M31" s="18">
         <f>Settings!$B$4+SUM(L$2:L31)</f>
         <v/>
       </c>
@@ -2694,11 +2708,11 @@
         <f>IF(I32="","",I32-F32)</f>
         <v/>
       </c>
-      <c r="L32" s="6">
+      <c r="L32" s="18">
         <f>IF(K32="W",IF(G32&lt;0,H32*100/ABS(G32),H32*G32/100),IF(K32="L",-H32,0))</f>
         <v/>
       </c>
-      <c r="M32" s="6">
+      <c r="M32" s="18">
         <f>Settings!$B$4+SUM(L$2:L32)</f>
         <v/>
       </c>
@@ -2708,11 +2722,11 @@
         <f>IF(I33="","",I33-F33)</f>
         <v/>
       </c>
-      <c r="L33" s="6">
+      <c r="L33" s="18">
         <f>IF(K33="W",IF(G33&lt;0,H33*100/ABS(G33),H33*G33/100),IF(K33="L",-H33,0))</f>
         <v/>
       </c>
-      <c r="M33" s="6">
+      <c r="M33" s="18">
         <f>Settings!$B$4+SUM(L$2:L33)</f>
         <v/>
       </c>
@@ -2722,11 +2736,11 @@
         <f>IF(I34="","",I34-F34)</f>
         <v/>
       </c>
-      <c r="L34" s="6">
+      <c r="L34" s="18">
         <f>IF(K34="W",IF(G34&lt;0,H34*100/ABS(G34),H34*G34/100),IF(K34="L",-H34,0))</f>
         <v/>
       </c>
-      <c r="M34" s="6">
+      <c r="M34" s="18">
         <f>Settings!$B$4+SUM(L$2:L34)</f>
         <v/>
       </c>
@@ -2736,11 +2750,11 @@
         <f>IF(I35="","",I35-F35)</f>
         <v/>
       </c>
-      <c r="L35" s="6">
+      <c r="L35" s="18">
         <f>IF(K35="W",IF(G35&lt;0,H35*100/ABS(G35),H35*G35/100),IF(K35="L",-H35,0))</f>
         <v/>
       </c>
-      <c r="M35" s="6">
+      <c r="M35" s="18">
         <f>Settings!$B$4+SUM(L$2:L35)</f>
         <v/>
       </c>
@@ -2750,11 +2764,11 @@
         <f>IF(I36="","",I36-F36)</f>
         <v/>
       </c>
-      <c r="L36" s="6">
+      <c r="L36" s="18">
         <f>IF(K36="W",IF(G36&lt;0,H36*100/ABS(G36),H36*G36/100),IF(K36="L",-H36,0))</f>
         <v/>
       </c>
-      <c r="M36" s="6">
+      <c r="M36" s="18">
         <f>Settings!$B$4+SUM(L$2:L36)</f>
         <v/>
       </c>
@@ -2764,11 +2778,11 @@
         <f>IF(I37="","",I37-F37)</f>
         <v/>
       </c>
-      <c r="L37" s="6">
+      <c r="L37" s="18">
         <f>IF(K37="W",IF(G37&lt;0,H37*100/ABS(G37),H37*G37/100),IF(K37="L",-H37,0))</f>
         <v/>
       </c>
-      <c r="M37" s="6">
+      <c r="M37" s="18">
         <f>Settings!$B$4+SUM(L$2:L37)</f>
         <v/>
       </c>
@@ -2778,11 +2792,11 @@
         <f>IF(I38="","",I38-F38)</f>
         <v/>
       </c>
-      <c r="L38" s="6">
+      <c r="L38" s="18">
         <f>IF(K38="W",IF(G38&lt;0,H38*100/ABS(G38),H38*G38/100),IF(K38="L",-H38,0))</f>
         <v/>
       </c>
-      <c r="M38" s="6">
+      <c r="M38" s="18">
         <f>Settings!$B$4+SUM(L$2:L38)</f>
         <v/>
       </c>
@@ -2792,11 +2806,11 @@
         <f>IF(I39="","",I39-F39)</f>
         <v/>
       </c>
-      <c r="L39" s="6">
+      <c r="L39" s="18">
         <f>IF(K39="W",IF(G39&lt;0,H39*100/ABS(G39),H39*G39/100),IF(K39="L",-H39,0))</f>
         <v/>
       </c>
-      <c r="M39" s="6">
+      <c r="M39" s="18">
         <f>Settings!$B$4+SUM(L$2:L39)</f>
         <v/>
       </c>
@@ -2806,11 +2820,11 @@
         <f>IF(I40="","",I40-F40)</f>
         <v/>
       </c>
-      <c r="L40" s="6">
+      <c r="L40" s="18">
         <f>IF(K40="W",IF(G40&lt;0,H40*100/ABS(G40),H40*G40/100),IF(K40="L",-H40,0))</f>
         <v/>
       </c>
-      <c r="M40" s="6">
+      <c r="M40" s="18">
         <f>Settings!$B$4+SUM(L$2:L40)</f>
         <v/>
       </c>
@@ -2820,11 +2834,11 @@
         <f>IF(I41="","",I41-F41)</f>
         <v/>
       </c>
-      <c r="L41" s="6">
+      <c r="L41" s="18">
         <f>IF(K41="W",IF(G41&lt;0,H41*100/ABS(G41),H41*G41/100),IF(K41="L",-H41,0))</f>
         <v/>
       </c>
-      <c r="M41" s="6">
+      <c r="M41" s="18">
         <f>Settings!$B$4+SUM(L$2:L41)</f>
         <v/>
       </c>
@@ -3313,2320 +3327,2320 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="18" t="inlineStr">
+      <c r="A1" s="19" t="inlineStr">
         <is>
           <t>Ridge vs. XGBoost -- Model Comparison</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="19" t="inlineStr">
+      <c r="A2" s="20" t="inlineStr">
         <is>
           <t>Informational only. Ridge is still the live model everywhere else in this workbook and on the website -- XGBoost is a candidate being evaluated here, not a replacement.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="20" t="inlineStr">
+      <c r="A4" s="21" t="inlineStr">
         <is>
           <t>All-Time (every season in the backtest)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="21" t="inlineStr">
+      <c r="A5" s="22" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="B5" s="21" t="inlineStr">
+      <c r="B5" s="22" t="inlineStr">
         <is>
           <t>Games Graded</t>
         </is>
       </c>
-      <c r="C5" s="21" t="inlineStr">
+      <c r="C5" s="22" t="inlineStr">
         <is>
           <t>Bets Made</t>
         </is>
       </c>
-      <c r="D5" s="21" t="inlineStr">
+      <c r="D5" s="22" t="inlineStr">
         <is>
           <t>Wins</t>
         </is>
       </c>
-      <c r="E5" s="21" t="inlineStr">
+      <c r="E5" s="22" t="inlineStr">
         <is>
           <t>Losses</t>
         </is>
       </c>
-      <c r="F5" s="21" t="inlineStr">
+      <c r="F5" s="22" t="inlineStr">
         <is>
           <t>Pushes</t>
         </is>
       </c>
-      <c r="G5" s="21" t="inlineStr">
+      <c r="G5" s="22" t="inlineStr">
         <is>
           <t>ATS Win %</t>
         </is>
       </c>
-      <c r="H5" s="21" t="inlineStr">
+      <c r="H5" s="22" t="inlineStr">
         <is>
           <t>ROI (flat stake)</t>
         </is>
       </c>
-      <c r="I5" s="21" t="inlineStr">
+      <c r="I5" s="22" t="inlineStr">
         <is>
           <t>Tighter Than Other (CLV)</t>
         </is>
       </c>
-      <c r="J5" s="21" t="inlineStr">
+      <c r="J5" s="22" t="inlineStr">
         <is>
           <t>CLV Pts (cum.)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="22" t="inlineStr">
+      <c r="A6" s="23" t="inlineStr">
         <is>
           <t>Ridge (live model) -- all FBS</t>
         </is>
       </c>
-      <c r="B6" s="22" t="n">
+      <c r="B6" s="23" t="n">
         <v>8528</v>
       </c>
-      <c r="C6" s="22" t="n">
+      <c r="C6" s="23" t="n">
         <v>6627</v>
       </c>
-      <c r="D6" s="22" t="n">
+      <c r="D6" s="23" t="n">
         <v>3296</v>
       </c>
-      <c r="E6" s="22" t="n">
+      <c r="E6" s="23" t="n">
         <v>3331</v>
       </c>
-      <c r="F6" s="22" t="n">
+      <c r="F6" s="23" t="n">
         <v>54</v>
       </c>
-      <c r="G6" s="22" t="inlineStr">
+      <c r="G6" s="23" t="inlineStr">
         <is>
           <t>49.7%</t>
         </is>
       </c>
-      <c r="H6" s="22" t="inlineStr">
+      <c r="H6" s="23" t="inlineStr">
         <is>
           <t>-5.1%</t>
         </is>
       </c>
-      <c r="I6" s="22" t="inlineStr">
+      <c r="I6" s="23" t="inlineStr">
         <is>
           <t>4043/8528 (47%)</t>
         </is>
       </c>
-      <c r="J6" s="22" t="inlineStr">
+      <c r="J6" s="23" t="inlineStr">
         <is>
           <t>+5661.3</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="22" t="inlineStr">
+      <c r="A7" s="23" t="inlineStr">
         <is>
           <t>Ridge (live model) -- MW-involved</t>
         </is>
       </c>
-      <c r="B7" s="22" t="n">
+      <c r="B7" s="23" t="n">
         <v>969</v>
       </c>
-      <c r="C7" s="22" t="n">
+      <c r="C7" s="23" t="n">
         <v>768</v>
       </c>
-      <c r="D7" s="22" t="n">
+      <c r="D7" s="23" t="n">
         <v>379</v>
       </c>
-      <c r="E7" s="22" t="n">
+      <c r="E7" s="23" t="n">
         <v>389</v>
       </c>
-      <c r="F7" s="22" t="n">
+      <c r="F7" s="23" t="n">
         <v>8</v>
       </c>
-      <c r="G7" s="22" t="inlineStr">
+      <c r="G7" s="23" t="inlineStr">
         <is>
           <t>49.4%</t>
         </is>
       </c>
-      <c r="H7" s="22" t="inlineStr">
+      <c r="H7" s="23" t="inlineStr">
         <is>
           <t>-5.8%</t>
         </is>
       </c>
-      <c r="I7" s="22" t="inlineStr">
+      <c r="I7" s="23" t="inlineStr">
         <is>
           <t>457/969 (47%)</t>
         </is>
       </c>
-      <c r="J7" s="22" t="inlineStr">
+      <c r="J7" s="23" t="inlineStr">
         <is>
           <t>+600.8</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="22" t="inlineStr">
+      <c r="A8" s="23" t="inlineStr">
         <is>
           <t>XGBoost (candidate) -- all FBS</t>
         </is>
       </c>
-      <c r="B8" s="22" t="n">
+      <c r="B8" s="23" t="n">
         <v>8528</v>
       </c>
-      <c r="C8" s="22" t="n">
+      <c r="C8" s="23" t="n">
         <v>6561</v>
       </c>
-      <c r="D8" s="22" t="n">
+      <c r="D8" s="23" t="n">
         <v>3312</v>
       </c>
-      <c r="E8" s="22" t="n">
+      <c r="E8" s="23" t="n">
         <v>3249</v>
       </c>
-      <c r="F8" s="22" t="n">
+      <c r="F8" s="23" t="n">
         <v>59</v>
       </c>
-      <c r="G8" s="22" t="inlineStr">
+      <c r="G8" s="23" t="inlineStr">
         <is>
           <t>50.5%</t>
         </is>
       </c>
-      <c r="H8" s="22" t="inlineStr">
+      <c r="H8" s="23" t="inlineStr">
         <is>
           <t>-3.6%</t>
         </is>
       </c>
-      <c r="I8" s="22" t="inlineStr">
+      <c r="I8" s="23" t="inlineStr">
         <is>
           <t>4485/8528 (53%)</t>
         </is>
       </c>
-      <c r="J8" s="22" t="inlineStr">
+      <c r="J8" s="23" t="inlineStr">
         <is>
           <t>+741.2</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="22" t="inlineStr">
+      <c r="A9" s="23" t="inlineStr">
         <is>
           <t>XGBoost (candidate) -- MW-involved</t>
         </is>
       </c>
-      <c r="B9" s="22" t="n">
+      <c r="B9" s="23" t="n">
         <v>969</v>
       </c>
-      <c r="C9" s="22" t="n">
+      <c r="C9" s="23" t="n">
         <v>729</v>
       </c>
-      <c r="D9" s="22" t="n">
+      <c r="D9" s="23" t="n">
         <v>375</v>
       </c>
-      <c r="E9" s="22" t="n">
+      <c r="E9" s="23" t="n">
         <v>354</v>
       </c>
-      <c r="F9" s="22" t="n">
+      <c r="F9" s="23" t="n">
         <v>10</v>
       </c>
-      <c r="G9" s="22" t="inlineStr">
+      <c r="G9" s="23" t="inlineStr">
         <is>
           <t>51.4%</t>
         </is>
       </c>
-      <c r="H9" s="22" t="inlineStr">
+      <c r="H9" s="23" t="inlineStr">
         <is>
           <t>-1.8%</t>
         </is>
       </c>
-      <c r="I9" s="22" t="inlineStr">
+      <c r="I9" s="23" t="inlineStr">
         <is>
           <t>512/969 (53%)</t>
         </is>
       </c>
-      <c r="J9" s="22" t="inlineStr">
+      <c r="J9" s="23" t="inlineStr">
         <is>
           <t>+895.0</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="20" t="inlineStr">
+      <c r="A11" s="21" t="inlineStr">
         <is>
           <t>2026 Season Only</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="21" t="inlineStr">
+      <c r="A12" s="22" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="B12" s="21" t="inlineStr">
+      <c r="B12" s="22" t="inlineStr">
         <is>
           <t>Games Graded</t>
         </is>
       </c>
-      <c r="C12" s="21" t="inlineStr">
+      <c r="C12" s="22" t="inlineStr">
         <is>
           <t>Bets Made</t>
         </is>
       </c>
-      <c r="D12" s="21" t="inlineStr">
+      <c r="D12" s="22" t="inlineStr">
         <is>
           <t>Wins</t>
         </is>
       </c>
-      <c r="E12" s="21" t="inlineStr">
+      <c r="E12" s="22" t="inlineStr">
         <is>
           <t>Losses</t>
         </is>
       </c>
-      <c r="F12" s="21" t="inlineStr">
+      <c r="F12" s="22" t="inlineStr">
         <is>
           <t>Pushes</t>
         </is>
       </c>
-      <c r="G12" s="21" t="inlineStr">
+      <c r="G12" s="22" t="inlineStr">
         <is>
           <t>ATS Win %</t>
         </is>
       </c>
-      <c r="H12" s="21" t="inlineStr">
+      <c r="H12" s="22" t="inlineStr">
         <is>
           <t>ROI (flat stake)</t>
         </is>
       </c>
-      <c r="I12" s="21" t="inlineStr">
+      <c r="I12" s="22" t="inlineStr">
         <is>
           <t>Tighter Than Other (CLV)</t>
         </is>
       </c>
-      <c r="J12" s="21" t="inlineStr">
+      <c r="J12" s="22" t="inlineStr">
         <is>
           <t>CLV Pts (cum.)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="22" t="inlineStr">
+      <c r="A13" s="23" t="inlineStr">
         <is>
           <t>Ridge (live model) -- all FBS</t>
         </is>
       </c>
-      <c r="B13" s="22" t="n">
+      <c r="B13" s="23" t="n">
         <v>95</v>
       </c>
-      <c r="C13" s="22" t="n">
+      <c r="C13" s="23" t="n">
         <v>84</v>
       </c>
-      <c r="D13" s="22" t="n">
+      <c r="D13" s="23" t="n">
         <v>33</v>
       </c>
-      <c r="E13" s="22" t="n">
+      <c r="E13" s="23" t="n">
         <v>51</v>
       </c>
-      <c r="F13" s="22" t="n">
+      <c r="F13" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="G13" s="22" t="inlineStr">
+      <c r="G13" s="23" t="inlineStr">
         <is>
           <t>39.3%</t>
         </is>
       </c>
-      <c r="H13" s="22" t="inlineStr">
+      <c r="H13" s="23" t="inlineStr">
         <is>
           <t>-25.0%</t>
         </is>
       </c>
-      <c r="I13" s="22" t="inlineStr">
+      <c r="I13" s="23" t="inlineStr">
         <is>
           <t>42/95 (44%)</t>
         </is>
       </c>
-      <c r="J13" s="22" t="inlineStr">
+      <c r="J13" s="23" t="inlineStr">
         <is>
           <t>-433.7</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="22" t="inlineStr">
+      <c r="A14" s="23" t="inlineStr">
         <is>
           <t>Ridge (live model) -- MW-involved</t>
         </is>
       </c>
-      <c r="B14" s="22" t="n">
+      <c r="B14" s="23" t="n">
         <v>13</v>
       </c>
-      <c r="C14" s="22" t="n">
+      <c r="C14" s="23" t="n">
         <v>11</v>
       </c>
-      <c r="D14" s="22" t="n">
+      <c r="D14" s="23" t="n">
         <v>4</v>
       </c>
-      <c r="E14" s="22" t="n">
+      <c r="E14" s="23" t="n">
         <v>7</v>
       </c>
-      <c r="F14" s="22" t="n">
+      <c r="F14" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="G14" s="22" t="inlineStr">
+      <c r="G14" s="23" t="inlineStr">
         <is>
           <t>36.4%</t>
         </is>
       </c>
-      <c r="H14" s="22" t="inlineStr">
+      <c r="H14" s="23" t="inlineStr">
         <is>
           <t>-30.6%</t>
         </is>
       </c>
-      <c r="I14" s="22" t="inlineStr">
+      <c r="I14" s="23" t="inlineStr">
         <is>
           <t>6/13 (46%)</t>
         </is>
       </c>
-      <c r="J14" s="22" t="inlineStr">
+      <c r="J14" s="23" t="inlineStr">
         <is>
           <t>+11.2</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="22" t="inlineStr">
+      <c r="A15" s="23" t="inlineStr">
         <is>
           <t>XGBoost (candidate) -- all FBS</t>
         </is>
       </c>
-      <c r="B15" s="22" t="n">
+      <c r="B15" s="23" t="n">
         <v>95</v>
       </c>
-      <c r="C15" s="22" t="n">
+      <c r="C15" s="23" t="n">
         <v>78</v>
       </c>
-      <c r="D15" s="22" t="n">
+      <c r="D15" s="23" t="n">
         <v>31</v>
       </c>
-      <c r="E15" s="22" t="n">
+      <c r="E15" s="23" t="n">
         <v>47</v>
       </c>
-      <c r="F15" s="22" t="n">
+      <c r="F15" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="G15" s="22" t="inlineStr">
+      <c r="G15" s="23" t="inlineStr">
         <is>
           <t>39.7%</t>
         </is>
       </c>
-      <c r="H15" s="22" t="inlineStr">
+      <c r="H15" s="23" t="inlineStr">
         <is>
           <t>-24.1%</t>
         </is>
       </c>
-      <c r="I15" s="22" t="inlineStr">
+      <c r="I15" s="23" t="inlineStr">
         <is>
           <t>53/95 (56%)</t>
         </is>
       </c>
-      <c r="J15" s="22" t="inlineStr">
+      <c r="J15" s="23" t="inlineStr">
         <is>
           <t>-162.4</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="22" t="inlineStr">
+      <c r="A16" s="23" t="inlineStr">
         <is>
           <t>XGBoost (candidate) -- MW-involved</t>
         </is>
       </c>
-      <c r="B16" s="22" t="n">
+      <c r="B16" s="23" t="n">
         <v>13</v>
       </c>
-      <c r="C16" s="22" t="n">
+      <c r="C16" s="23" t="n">
         <v>9</v>
       </c>
-      <c r="D16" s="22" t="n">
+      <c r="D16" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="E16" s="22" t="n">
+      <c r="E16" s="23" t="n">
         <v>7</v>
       </c>
-      <c r="F16" s="22" t="n">
+      <c r="F16" s="23" t="n">
         <v>0</v>
       </c>
-      <c r="G16" s="22" t="inlineStr">
+      <c r="G16" s="23" t="inlineStr">
         <is>
           <t>22.2%</t>
         </is>
       </c>
-      <c r="H16" s="22" t="inlineStr">
+      <c r="H16" s="23" t="inlineStr">
         <is>
           <t>-57.6%</t>
         </is>
       </c>
-      <c r="I16" s="22" t="inlineStr">
+      <c r="I16" s="23" t="inlineStr">
         <is>
           <t>7/13 (54%)</t>
         </is>
       </c>
-      <c r="J16" s="22" t="inlineStr">
+      <c r="J16" s="23" t="inlineStr">
         <is>
           <t>-13.3</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="19" t="inlineStr">
+      <c r="A18" s="20" t="inlineStr">
         <is>
           <t>Ridge and XGBoost agree on which side to lean in 76.9% of all graded games.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="20" t="inlineStr">
+      <c r="A20" s="21" t="inlineStr">
         <is>
           <t>Upcoming Games -- Ridge vs. XGBoost (Not Yet Graded)</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="21" t="inlineStr">
+      <c r="A21" s="22" t="inlineStr">
         <is>
           <t>Week</t>
         </is>
       </c>
-      <c r="B21" s="21" t="inlineStr">
+      <c r="B21" s="22" t="inlineStr">
         <is>
           <t>Matchup</t>
         </is>
       </c>
-      <c r="C21" s="21" t="inlineStr">
+      <c r="C21" s="22" t="inlineStr">
         <is>
           <t>Market Line (Home)</t>
         </is>
       </c>
-      <c r="D21" s="21" t="inlineStr">
+      <c r="D21" s="22" t="inlineStr">
         <is>
           <t>Ridge Line</t>
         </is>
       </c>
-      <c r="E21" s="21" t="inlineStr">
+      <c r="E21" s="22" t="inlineStr">
         <is>
           <t>XGBoost Line</t>
         </is>
       </c>
-      <c r="F21" s="21" t="inlineStr">
+      <c r="F21" s="22" t="inlineStr">
         <is>
           <t>Ridge Lean</t>
         </is>
       </c>
-      <c r="G21" s="21" t="inlineStr">
+      <c r="G21" s="22" t="inlineStr">
         <is>
           <t>XGBoost Lean</t>
         </is>
       </c>
-      <c r="H21" s="21" t="inlineStr">
+      <c r="H21" s="22" t="inlineStr">
         <is>
           <t>Models Agree?</t>
         </is>
       </c>
-      <c r="I21" s="21" t="inlineStr">
+      <c r="I21" s="22" t="inlineStr">
         <is>
           <t>Tighter (Live)*</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="22" t="n">
+      <c r="A22" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="B22" s="22" t="inlineStr">
+      <c r="B22" s="23" t="inlineStr">
         <is>
           <t>San José State @ USC</t>
         </is>
       </c>
-      <c r="C22" s="22" t="inlineStr">
+      <c r="C22" s="23" t="inlineStr">
         <is>
           <t>-37.2</t>
         </is>
       </c>
-      <c r="D22" s="22" t="inlineStr">
+      <c r="D22" s="23" t="inlineStr">
         <is>
           <t>-34.9</t>
         </is>
       </c>
-      <c r="E22" s="22" t="inlineStr">
+      <c r="E22" s="23" t="inlineStr">
         <is>
           <t>-32.3</t>
         </is>
       </c>
-      <c r="F22" s="22" t="inlineStr">
+      <c r="F22" s="23" t="inlineStr">
         <is>
           <t>Away</t>
         </is>
       </c>
-      <c r="G22" s="22" t="inlineStr">
+      <c r="G22" s="23" t="inlineStr">
         <is>
           <t>Away</t>
         </is>
       </c>
-      <c r="H22" s="22" t="inlineStr">
+      <c r="H22" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="I22" s="23" t="inlineStr">
+      <c r="I22" s="24" t="inlineStr">
         <is>
           <t>Ridge</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="22" t="n">
+      <c r="A23" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="B23" s="22" t="inlineStr">
+      <c r="B23" s="23" t="inlineStr">
         <is>
           <t>Jacksonville State @ North Dakota State</t>
         </is>
       </c>
-      <c r="C23" s="22" t="inlineStr">
+      <c r="C23" s="23" t="inlineStr">
         <is>
           <t>-6.8</t>
         </is>
       </c>
-      <c r="D23" s="22" t="inlineStr">
+      <c r="D23" s="23" t="inlineStr">
         <is>
           <t>-18.9</t>
         </is>
       </c>
-      <c r="E23" s="22" t="inlineStr">
+      <c r="E23" s="23" t="inlineStr">
         <is>
           <t>-16.3</t>
         </is>
       </c>
-      <c r="F23" s="22" t="inlineStr">
+      <c r="F23" s="23" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="G23" s="22" t="inlineStr">
+      <c r="G23" s="23" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="H23" s="22" t="inlineStr">
+      <c r="H23" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="I23" s="23" t="inlineStr">
+      <c r="I23" s="24" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="22" t="n">
+      <c r="A24" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="B24" s="22" t="inlineStr">
+      <c r="B24" s="23" t="inlineStr">
         <is>
           <t>Hawai'i @ Stanford</t>
         </is>
       </c>
-      <c r="C24" s="22" t="inlineStr">
+      <c r="C24" s="23" t="inlineStr">
         <is>
           <t>-4.8</t>
         </is>
       </c>
-      <c r="D24" s="22" t="inlineStr">
+      <c r="D24" s="23" t="inlineStr">
         <is>
           <t>-1.8</t>
         </is>
       </c>
-      <c r="E24" s="22" t="inlineStr">
+      <c r="E24" s="23" t="inlineStr">
         <is>
           <t>-0.3</t>
         </is>
       </c>
-      <c r="F24" s="22" t="inlineStr">
+      <c r="F24" s="23" t="inlineStr">
         <is>
           <t>Away</t>
         </is>
       </c>
-      <c r="G24" s="22" t="inlineStr">
+      <c r="G24" s="23" t="inlineStr">
         <is>
           <t>Away</t>
         </is>
       </c>
-      <c r="H24" s="22" t="inlineStr">
+      <c r="H24" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="I24" s="23" t="inlineStr">
+      <c r="I24" s="24" t="inlineStr">
         <is>
           <t>Ridge</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="22" t="n">
+      <c r="A25" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="B25" s="22" t="inlineStr">
+      <c r="B25" s="23" t="inlineStr">
         <is>
           <t>Memphis @ UNLV</t>
         </is>
       </c>
-      <c r="C25" s="22" t="inlineStr">
+      <c r="C25" s="23" t="inlineStr">
         <is>
           <t>-4.8</t>
         </is>
       </c>
-      <c r="D25" s="22" t="inlineStr">
+      <c r="D25" s="23" t="inlineStr">
         <is>
           <t>-11.3</t>
         </is>
       </c>
-      <c r="E25" s="22" t="inlineStr">
+      <c r="E25" s="23" t="inlineStr">
         <is>
           <t>-6.7</t>
         </is>
       </c>
-      <c r="F25" s="22" t="inlineStr">
+      <c r="F25" s="23" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="G25" s="22" t="inlineStr">
+      <c r="G25" s="23" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="H25" s="22" t="inlineStr">
+      <c r="H25" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="I25" s="23" t="inlineStr">
+      <c r="I25" s="24" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="22" t="n">
+      <c r="A26" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="B26" s="22" t="inlineStr">
+      <c r="B26" s="23" t="inlineStr">
         <is>
           <t>San José State @ Eastern Michigan</t>
         </is>
       </c>
-      <c r="C26" s="22" t="inlineStr">
+      <c r="C26" s="23" t="inlineStr">
         <is>
           <t>-1.5</t>
         </is>
       </c>
-      <c r="D26" s="22" t="inlineStr">
+      <c r="D26" s="23" t="inlineStr">
         <is>
           <t>-16.0</t>
         </is>
       </c>
-      <c r="E26" s="22" t="inlineStr">
+      <c r="E26" s="23" t="inlineStr">
         <is>
           <t>-9.9</t>
         </is>
       </c>
-      <c r="F26" s="22" t="inlineStr">
+      <c r="F26" s="23" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="G26" s="22" t="inlineStr">
+      <c r="G26" s="23" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="H26" s="22" t="inlineStr">
+      <c r="H26" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="I26" s="23" t="inlineStr">
+      <c r="I26" s="24" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="22" t="n">
+      <c r="A27" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="B27" s="22" t="inlineStr">
+      <c r="B27" s="23" t="inlineStr">
         <is>
           <t>UTEP @ Oklahoma</t>
         </is>
       </c>
-      <c r="C27" s="22" t="inlineStr">
+      <c r="C27" s="23" t="inlineStr">
         <is>
           <t>-40.8</t>
         </is>
       </c>
-      <c r="D27" s="22" t="inlineStr">
+      <c r="D27" s="23" t="inlineStr">
         <is>
           <t>-35.0</t>
         </is>
       </c>
-      <c r="E27" s="22" t="inlineStr">
+      <c r="E27" s="23" t="inlineStr">
         <is>
           <t>-33.6</t>
         </is>
       </c>
-      <c r="F27" s="22" t="inlineStr">
+      <c r="F27" s="23" t="inlineStr">
         <is>
           <t>Away</t>
         </is>
       </c>
-      <c r="G27" s="22" t="inlineStr">
+      <c r="G27" s="23" t="inlineStr">
         <is>
           <t>Away</t>
         </is>
       </c>
-      <c r="H27" s="22" t="inlineStr">
+      <c r="H27" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="I27" s="23" t="inlineStr">
+      <c r="I27" s="24" t="inlineStr">
         <is>
           <t>Ridge</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="22" t="n">
+      <c r="A28" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="B28" s="22" t="inlineStr">
+      <c r="B28" s="23" t="inlineStr">
         <is>
           <t>Duquesne @ Air Force</t>
         </is>
       </c>
-      <c r="C28" s="22" t="inlineStr">
+      <c r="C28" s="23" t="inlineStr">
         <is>
           <t>-30.0</t>
         </is>
       </c>
-      <c r="D28" s="22" t="inlineStr">
+      <c r="D28" s="23" t="inlineStr">
         <is>
           <t>-17.3</t>
         </is>
       </c>
-      <c r="E28" s="22" t="inlineStr">
+      <c r="E28" s="23" t="inlineStr">
         <is>
           <t>-29.5</t>
         </is>
       </c>
-      <c r="F28" s="22" t="inlineStr">
+      <c r="F28" s="23" t="inlineStr">
         <is>
           <t>Away</t>
         </is>
       </c>
-      <c r="G28" s="22" t="inlineStr">
+      <c r="G28" s="23" t="inlineStr">
         <is>
           <t>Away</t>
         </is>
       </c>
-      <c r="H28" s="22" t="inlineStr">
+      <c r="H28" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="I28" s="23" t="inlineStr">
+      <c r="I28" s="24" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="22" t="n">
+      <c r="A29" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="B29" s="22" t="inlineStr">
+      <c r="B29" s="23" t="inlineStr">
         <is>
           <t>Fordham @ North Dakota State</t>
         </is>
       </c>
-      <c r="C29" s="22" t="inlineStr">
+      <c r="C29" s="23" t="inlineStr">
         <is>
           <t>-41.5</t>
         </is>
       </c>
-      <c r="D29" s="22" t="inlineStr">
+      <c r="D29" s="23" t="inlineStr">
         <is>
           <t>-39.8</t>
         </is>
       </c>
-      <c r="E29" s="22" t="inlineStr">
+      <c r="E29" s="23" t="inlineStr">
         <is>
           <t>-32.6</t>
         </is>
       </c>
-      <c r="F29" s="22" t="inlineStr">
+      <c r="F29" s="23" t="inlineStr">
         <is>
           <t>Away</t>
         </is>
       </c>
-      <c r="G29" s="22" t="inlineStr">
+      <c r="G29" s="23" t="inlineStr">
         <is>
           <t>Away</t>
         </is>
       </c>
-      <c r="H29" s="22" t="inlineStr">
+      <c r="H29" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="I29" s="23" t="inlineStr">
+      <c r="I29" s="24" t="inlineStr">
         <is>
           <t>Ridge</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="22" t="n">
+      <c r="A30" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="B30" s="22" t="inlineStr">
+      <c r="B30" s="23" t="inlineStr">
         <is>
           <t>Northern Illinois @ Iowa</t>
         </is>
       </c>
-      <c r="C30" s="22" t="inlineStr">
+      <c r="C30" s="23" t="inlineStr">
         <is>
           <t>-31.8</t>
         </is>
       </c>
-      <c r="D30" s="22" t="inlineStr">
+      <c r="D30" s="23" t="inlineStr">
         <is>
           <t>-28.7</t>
         </is>
       </c>
-      <c r="E30" s="22" t="inlineStr">
+      <c r="E30" s="23" t="inlineStr">
         <is>
           <t>-25.6</t>
         </is>
       </c>
-      <c r="F30" s="22" t="inlineStr">
+      <c r="F30" s="23" t="inlineStr">
         <is>
           <t>Away</t>
         </is>
       </c>
-      <c r="G30" s="22" t="inlineStr">
+      <c r="G30" s="23" t="inlineStr">
         <is>
           <t>Away</t>
         </is>
       </c>
-      <c r="H30" s="22" t="inlineStr">
+      <c r="H30" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="I30" s="23" t="inlineStr">
+      <c r="I30" s="24" t="inlineStr">
         <is>
           <t>Ridge</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="22" t="n">
+      <c r="A31" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="B31" s="22" t="inlineStr">
+      <c r="B31" s="23" t="inlineStr">
         <is>
           <t>Wyoming @ Colorado State</t>
         </is>
       </c>
-      <c r="C31" s="22" t="inlineStr">
+      <c r="C31" s="23" t="inlineStr">
         <is>
           <t>-2.8</t>
         </is>
       </c>
-      <c r="D31" s="22" t="inlineStr">
+      <c r="D31" s="23" t="inlineStr">
         <is>
           <t>-8.3</t>
         </is>
       </c>
-      <c r="E31" s="22" t="inlineStr">
+      <c r="E31" s="23" t="inlineStr">
         <is>
           <t>-3.9</t>
         </is>
       </c>
-      <c r="F31" s="22" t="inlineStr">
+      <c r="F31" s="23" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="G31" s="22" t="inlineStr">
+      <c r="G31" s="23" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="H31" s="22" t="inlineStr">
+      <c r="H31" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="I31" s="23" t="inlineStr">
+      <c r="I31" s="24" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="22" t="n">
+      <c r="A32" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="B32" s="22" t="inlineStr">
+      <c r="B32" s="23" t="inlineStr">
         <is>
           <t>Central Michigan @ New Mexico</t>
         </is>
       </c>
-      <c r="C32" s="22" t="inlineStr">
+      <c r="C32" s="23" t="inlineStr">
         <is>
           <t>-11.2</t>
         </is>
       </c>
-      <c r="D32" s="22" t="inlineStr">
+      <c r="D32" s="23" t="inlineStr">
         <is>
           <t>-18.2</t>
         </is>
       </c>
-      <c r="E32" s="22" t="inlineStr">
+      <c r="E32" s="23" t="inlineStr">
         <is>
           <t>-12.2</t>
         </is>
       </c>
-      <c r="F32" s="22" t="inlineStr">
+      <c r="F32" s="23" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="G32" s="22" t="inlineStr">
+      <c r="G32" s="23" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="H32" s="22" t="inlineStr">
+      <c r="H32" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="I32" s="23" t="inlineStr">
+      <c r="I32" s="24" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="22" t="n">
+      <c r="A33" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="B33" s="22" t="inlineStr">
+      <c r="B33" s="23" t="inlineStr">
         <is>
           <t>UNLV @ Hawai'i</t>
         </is>
       </c>
-      <c r="C33" s="22" t="inlineStr">
+      <c r="C33" s="23" t="inlineStr">
         <is>
           <t>+2.8</t>
         </is>
       </c>
-      <c r="D33" s="22" t="inlineStr">
+      <c r="D33" s="23" t="inlineStr">
         <is>
           <t>+3.5</t>
         </is>
       </c>
-      <c r="E33" s="22" t="inlineStr">
+      <c r="E33" s="23" t="inlineStr">
         <is>
           <t>-1.1</t>
         </is>
       </c>
-      <c r="F33" s="22" t="inlineStr">
+      <c r="F33" s="23" t="inlineStr">
         <is>
           <t>Away</t>
         </is>
       </c>
-      <c r="G33" s="22" t="inlineStr">
+      <c r="G33" s="23" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="H33" s="22" t="inlineStr">
+      <c r="H33" s="23" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="I33" s="23" t="inlineStr">
+      <c r="I33" s="24" t="inlineStr">
         <is>
           <t>Ridge</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="22" t="n">
+      <c r="A34" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="B34" s="22" t="inlineStr">
+      <c r="B34" s="23" t="inlineStr">
         <is>
           <t>Western Kentucky @ Nevada</t>
         </is>
       </c>
-      <c r="C34" s="22" t="inlineStr">
+      <c r="C34" s="23" t="inlineStr">
         <is>
           <t>+0.2</t>
         </is>
       </c>
-      <c r="D34" s="22" t="inlineStr">
+      <c r="D34" s="23" t="inlineStr">
         <is>
           <t>+2.6</t>
         </is>
       </c>
-      <c r="E34" s="22" t="inlineStr">
+      <c r="E34" s="23" t="inlineStr">
         <is>
           <t>+4.4</t>
         </is>
       </c>
-      <c r="F34" s="22" t="inlineStr">
+      <c r="F34" s="23" t="inlineStr">
         <is>
           <t>Away</t>
         </is>
       </c>
-      <c r="G34" s="22" t="inlineStr">
+      <c r="G34" s="23" t="inlineStr">
         <is>
           <t>Away</t>
         </is>
       </c>
-      <c r="H34" s="22" t="inlineStr">
+      <c r="H34" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="I34" s="23" t="inlineStr">
+      <c r="I34" s="24" t="inlineStr">
         <is>
           <t>Ridge</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="19" t="inlineStr">
+      <c r="A35" s="20" t="inlineStr">
         <is>
           <t>* Tighter (Live) compares each model's line to TODAY's still-moving market line, not a final closing line -- it will keep changing until kickoff. See the graded Game-by-Game table below for the real, closing-line version of this comparison.</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="20" t="inlineStr">
+      <c r="A38" s="21" t="inlineStr">
         <is>
           <t>2026 Mountain West Games -- Game by Game</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="21" t="inlineStr">
+      <c r="A39" s="22" t="inlineStr">
         <is>
           <t>Week</t>
         </is>
       </c>
-      <c r="B39" s="21" t="inlineStr">
+      <c r="B39" s="22" t="inlineStr">
         <is>
           <t>Matchup</t>
         </is>
       </c>
-      <c r="C39" s="21" t="inlineStr">
+      <c r="C39" s="22" t="inlineStr">
         <is>
           <t>Final Score</t>
         </is>
       </c>
-      <c r="D39" s="21" t="inlineStr">
+      <c r="D39" s="22" t="inlineStr">
         <is>
           <t>Vegas Spread (Home)</t>
         </is>
       </c>
-      <c r="E39" s="21" t="inlineStr">
+      <c r="E39" s="22" t="inlineStr">
         <is>
           <t>Actual Margin (Home)</t>
         </is>
       </c>
-      <c r="F39" s="21" t="inlineStr">
+      <c r="F39" s="22" t="inlineStr">
         <is>
           <t>Ridge Line</t>
         </is>
       </c>
-      <c r="G39" s="21" t="inlineStr">
+      <c r="G39" s="22" t="inlineStr">
         <is>
           <t>Ridge Edge</t>
         </is>
       </c>
-      <c r="H39" s="21" t="inlineStr">
+      <c r="H39" s="22" t="inlineStr">
         <is>
           <t>Ridge Lean</t>
         </is>
       </c>
-      <c r="I39" s="21" t="inlineStr">
+      <c r="I39" s="22" t="inlineStr">
         <is>
           <t>Ridge Result</t>
         </is>
       </c>
-      <c r="J39" s="21" t="inlineStr">
+      <c r="J39" s="22" t="inlineStr">
         <is>
           <t>XGBoost Line</t>
         </is>
       </c>
-      <c r="K39" s="21" t="inlineStr">
+      <c r="K39" s="22" t="inlineStr">
         <is>
           <t>XGBoost Edge</t>
         </is>
       </c>
-      <c r="L39" s="21" t="inlineStr">
+      <c r="L39" s="22" t="inlineStr">
         <is>
           <t>XGBoost Lean</t>
         </is>
       </c>
-      <c r="M39" s="21" t="inlineStr">
+      <c r="M39" s="22" t="inlineStr">
         <is>
           <t>XGBoost Result</t>
         </is>
       </c>
-      <c r="N39" s="21" t="inlineStr">
+      <c r="N39" s="22" t="inlineStr">
         <is>
           <t>Models Agree?</t>
         </is>
       </c>
-      <c r="O39" s="21" t="inlineStr">
+      <c r="O39" s="22" t="inlineStr">
         <is>
           <t>Tighter CLV Line</t>
         </is>
       </c>
-      <c r="P39" s="21" t="inlineStr">
+      <c r="P39" s="22" t="inlineStr">
         <is>
           <t>Ridge CLV Pts (Cum.)</t>
         </is>
       </c>
-      <c r="Q39" s="21" t="inlineStr">
+      <c r="Q39" s="22" t="inlineStr">
         <is>
           <t>XGBoost CLV Pts (Cum.)</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="22" t="n">
+      <c r="A40" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="B40" s="22" t="inlineStr">
+      <c r="B40" s="23" t="inlineStr">
         <is>
           <t>Duquesne @ Air Force</t>
         </is>
       </c>
-      <c r="C40" s="22" t="inlineStr">
+      <c r="C40" s="23" t="inlineStr">
         <is>
           <t>0-34</t>
         </is>
       </c>
-      <c r="D40" s="22" t="inlineStr">
+      <c r="D40" s="23" t="inlineStr">
         <is>
           <t>-30.0</t>
         </is>
       </c>
-      <c r="E40" s="22" t="inlineStr">
+      <c r="E40" s="23" t="inlineStr">
         <is>
           <t>+34.0</t>
         </is>
       </c>
-      <c r="F40" s="22" t="inlineStr">
+      <c r="F40" s="23" t="inlineStr">
         <is>
           <t>-17.0</t>
         </is>
       </c>
-      <c r="G40" s="22" t="inlineStr">
+      <c r="G40" s="23" t="inlineStr">
         <is>
           <t>-13.0</t>
         </is>
       </c>
-      <c r="H40" s="22" t="inlineStr">
+      <c r="H40" s="23" t="inlineStr">
         <is>
           <t>Away</t>
         </is>
       </c>
-      <c r="I40" s="24" t="inlineStr">
+      <c r="I40" s="25" t="inlineStr">
         <is>
           <t>Loss</t>
         </is>
       </c>
-      <c r="J40" s="22" t="inlineStr">
+      <c r="J40" s="23" t="inlineStr">
         <is>
           <t>-28.3</t>
         </is>
       </c>
-      <c r="K40" s="22" t="inlineStr">
+      <c r="K40" s="23" t="inlineStr">
         <is>
           <t>-1.7</t>
         </is>
       </c>
-      <c r="L40" s="22" t="inlineStr">
+      <c r="L40" s="23" t="inlineStr">
         <is>
           <t>Away</t>
         </is>
       </c>
-      <c r="M40" s="22" t="inlineStr">
+      <c r="M40" s="23" t="inlineStr">
         <is>
           <t>Lean only</t>
         </is>
       </c>
-      <c r="N40" s="22" t="inlineStr">
+      <c r="N40" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O40" s="23" t="inlineStr">
+      <c r="O40" s="24" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="P40" s="22" t="inlineStr">
+      <c r="P40" s="23" t="inlineStr">
         <is>
           <t>-13.0</t>
         </is>
       </c>
-      <c r="Q40" s="22" t="inlineStr">
+      <c r="Q40" s="23" t="inlineStr">
         <is>
           <t>-1.7</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="22" t="n">
+      <c r="A41" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="B41" s="22" t="inlineStr">
+      <c r="B41" s="23" t="inlineStr">
         <is>
           <t>Wyoming @ Colorado State</t>
         </is>
       </c>
-      <c r="C41" s="22" t="inlineStr">
+      <c r="C41" s="23" t="inlineStr">
         <is>
           <t>13-35</t>
         </is>
       </c>
-      <c r="D41" s="22" t="inlineStr">
+      <c r="D41" s="23" t="inlineStr">
         <is>
           <t>-2.8</t>
         </is>
       </c>
-      <c r="E41" s="22" t="inlineStr">
+      <c r="E41" s="23" t="inlineStr">
         <is>
           <t>+22.0</t>
         </is>
       </c>
-      <c r="F41" s="22" t="inlineStr">
+      <c r="F41" s="23" t="inlineStr">
         <is>
           <t>-7.8</t>
         </is>
       </c>
-      <c r="G41" s="22" t="inlineStr">
+      <c r="G41" s="23" t="inlineStr">
         <is>
           <t>+5.1</t>
         </is>
       </c>
-      <c r="H41" s="22" t="inlineStr">
+      <c r="H41" s="23" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="I41" s="23" t="inlineStr">
+      <c r="I41" s="24" t="inlineStr">
         <is>
           <t>Win</t>
         </is>
       </c>
-      <c r="J41" s="22" t="inlineStr">
+      <c r="J41" s="23" t="inlineStr">
         <is>
           <t>-2.5</t>
         </is>
       </c>
-      <c r="K41" s="22" t="inlineStr">
+      <c r="K41" s="23" t="inlineStr">
         <is>
           <t>-0.2</t>
         </is>
       </c>
-      <c r="L41" s="22" t="inlineStr">
+      <c r="L41" s="23" t="inlineStr">
         <is>
           <t>Away</t>
         </is>
       </c>
-      <c r="M41" s="22" t="inlineStr">
+      <c r="M41" s="23" t="inlineStr">
         <is>
           <t>Lean only</t>
         </is>
       </c>
-      <c r="N41" s="22" t="inlineStr">
+      <c r="N41" s="23" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="O41" s="23" t="inlineStr">
+      <c r="O41" s="24" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="P41" s="22" t="inlineStr">
+      <c r="P41" s="23" t="inlineStr">
         <is>
           <t>-7.9</t>
         </is>
       </c>
-      <c r="Q41" s="22" t="inlineStr">
+      <c r="Q41" s="23" t="inlineStr">
         <is>
           <t>-1.9</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="22" t="n">
+      <c r="A42" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="B42" s="22" t="inlineStr">
+      <c r="B42" s="23" t="inlineStr">
         <is>
           <t>San José State @ Eastern Michigan</t>
         </is>
       </c>
-      <c r="C42" s="22" t="inlineStr">
+      <c r="C42" s="23" t="inlineStr">
         <is>
           <t>27-21</t>
         </is>
       </c>
-      <c r="D42" s="22" t="inlineStr">
+      <c r="D42" s="23" t="inlineStr">
         <is>
           <t>-1.5</t>
         </is>
       </c>
-      <c r="E42" s="22" t="inlineStr">
+      <c r="E42" s="23" t="inlineStr">
         <is>
           <t>-6.0</t>
         </is>
       </c>
-      <c r="F42" s="22" t="inlineStr">
+      <c r="F42" s="23" t="inlineStr">
         <is>
           <t>-15.8</t>
         </is>
       </c>
-      <c r="G42" s="22" t="inlineStr">
+      <c r="G42" s="23" t="inlineStr">
         <is>
           <t>+14.3</t>
         </is>
       </c>
-      <c r="H42" s="22" t="inlineStr">
+      <c r="H42" s="23" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="I42" s="24" t="inlineStr">
+      <c r="I42" s="25" t="inlineStr">
         <is>
           <t>Loss</t>
         </is>
       </c>
-      <c r="J42" s="22" t="inlineStr">
+      <c r="J42" s="23" t="inlineStr">
         <is>
           <t>-10.5</t>
         </is>
       </c>
-      <c r="K42" s="22" t="inlineStr">
+      <c r="K42" s="23" t="inlineStr">
         <is>
           <t>+9.0</t>
         </is>
       </c>
-      <c r="L42" s="22" t="inlineStr">
+      <c r="L42" s="23" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="M42" s="24" t="inlineStr">
+      <c r="M42" s="25" t="inlineStr">
         <is>
           <t>Loss</t>
         </is>
       </c>
-      <c r="N42" s="22" t="inlineStr">
+      <c r="N42" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O42" s="23" t="inlineStr">
+      <c r="O42" s="24" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="P42" s="22" t="inlineStr">
+      <c r="P42" s="23" t="inlineStr">
         <is>
           <t>+6.4</t>
         </is>
       </c>
-      <c r="Q42" s="22" t="inlineStr">
+      <c r="Q42" s="23" t="inlineStr">
         <is>
           <t>+7.2</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="22" t="n">
+      <c r="A43" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="B43" s="22" t="inlineStr">
+      <c r="B43" s="23" t="inlineStr">
         <is>
           <t>UNLV @ Hawai'i</t>
         </is>
       </c>
-      <c r="C43" s="22" t="inlineStr">
+      <c r="C43" s="23" t="inlineStr">
         <is>
           <t>21-6</t>
         </is>
       </c>
-      <c r="D43" s="22" t="inlineStr">
+      <c r="D43" s="23" t="inlineStr">
         <is>
           <t>+2.8</t>
         </is>
       </c>
-      <c r="E43" s="22" t="inlineStr">
+      <c r="E43" s="23" t="inlineStr">
         <is>
           <t>-15.0</t>
         </is>
       </c>
-      <c r="F43" s="22" t="inlineStr">
+      <c r="F43" s="23" t="inlineStr">
         <is>
           <t>+2.9</t>
         </is>
       </c>
-      <c r="G43" s="22" t="inlineStr">
+      <c r="G43" s="23" t="inlineStr">
         <is>
           <t>-0.1</t>
         </is>
       </c>
-      <c r="H43" s="22" t="inlineStr">
+      <c r="H43" s="23" t="inlineStr">
         <is>
           <t>Away</t>
         </is>
       </c>
-      <c r="I43" s="22" t="inlineStr">
+      <c r="I43" s="23" t="inlineStr">
         <is>
           <t>Lean only</t>
         </is>
       </c>
-      <c r="J43" s="22" t="inlineStr">
+      <c r="J43" s="23" t="inlineStr">
         <is>
           <t>-1.8</t>
         </is>
       </c>
-      <c r="K43" s="22" t="inlineStr">
+      <c r="K43" s="23" t="inlineStr">
         <is>
           <t>+4.6</t>
         </is>
       </c>
-      <c r="L43" s="22" t="inlineStr">
+      <c r="L43" s="23" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="M43" s="24" t="inlineStr">
+      <c r="M43" s="25" t="inlineStr">
         <is>
           <t>Loss</t>
         </is>
       </c>
-      <c r="N43" s="22" t="inlineStr">
+      <c r="N43" s="23" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="O43" s="23" t="inlineStr">
+      <c r="O43" s="24" t="inlineStr">
         <is>
           <t>Ridge</t>
         </is>
       </c>
-      <c r="P43" s="22" t="inlineStr">
+      <c r="P43" s="23" t="inlineStr">
         <is>
           <t>+6.2</t>
         </is>
       </c>
-      <c r="Q43" s="22" t="inlineStr">
+      <c r="Q43" s="23" t="inlineStr">
         <is>
           <t>+11.8</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="22" t="n">
+      <c r="A44" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="B44" s="22" t="inlineStr">
+      <c r="B44" s="23" t="inlineStr">
         <is>
           <t>Northern Illinois @ Iowa</t>
         </is>
       </c>
-      <c r="C44" s="22" t="inlineStr">
+      <c r="C44" s="23" t="inlineStr">
         <is>
           <t>0-40</t>
         </is>
       </c>
-      <c r="D44" s="22" t="inlineStr">
+      <c r="D44" s="23" t="inlineStr">
         <is>
           <t>-31.8</t>
         </is>
       </c>
-      <c r="E44" s="22" t="inlineStr">
+      <c r="E44" s="23" t="inlineStr">
         <is>
           <t>+40.0</t>
         </is>
       </c>
-      <c r="F44" s="22" t="inlineStr">
+      <c r="F44" s="23" t="inlineStr">
         <is>
           <t>-28.3</t>
         </is>
       </c>
-      <c r="G44" s="22" t="inlineStr">
+      <c r="G44" s="23" t="inlineStr">
         <is>
           <t>-3.5</t>
         </is>
       </c>
-      <c r="H44" s="22" t="inlineStr">
+      <c r="H44" s="23" t="inlineStr">
         <is>
           <t>Away</t>
         </is>
       </c>
-      <c r="I44" s="24" t="inlineStr">
+      <c r="I44" s="25" t="inlineStr">
         <is>
           <t>Loss</t>
         </is>
       </c>
-      <c r="J44" s="22" t="inlineStr">
+      <c r="J44" s="23" t="inlineStr">
         <is>
           <t>-25.4</t>
         </is>
       </c>
-      <c r="K44" s="22" t="inlineStr">
+      <c r="K44" s="23" t="inlineStr">
         <is>
           <t>-6.4</t>
         </is>
       </c>
-      <c r="L44" s="22" t="inlineStr">
+      <c r="L44" s="23" t="inlineStr">
         <is>
           <t>Away</t>
         </is>
       </c>
-      <c r="M44" s="24" t="inlineStr">
+      <c r="M44" s="25" t="inlineStr">
         <is>
           <t>Loss</t>
         </is>
       </c>
-      <c r="N44" s="22" t="inlineStr">
+      <c r="N44" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O44" s="23" t="inlineStr">
+      <c r="O44" s="24" t="inlineStr">
         <is>
           <t>Ridge</t>
         </is>
       </c>
-      <c r="P44" s="22" t="inlineStr">
+      <c r="P44" s="23" t="inlineStr">
         <is>
           <t>+2.8</t>
         </is>
       </c>
-      <c r="Q44" s="22" t="inlineStr">
+      <c r="Q44" s="23" t="inlineStr">
         <is>
           <t>+5.4</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="22" t="n">
+      <c r="A45" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="B45" s="22" t="inlineStr">
+      <c r="B45" s="23" t="inlineStr">
         <is>
           <t>Western Kentucky @ Nevada</t>
         </is>
       </c>
-      <c r="C45" s="22" t="inlineStr">
+      <c r="C45" s="23" t="inlineStr">
         <is>
           <t>14-49</t>
         </is>
       </c>
-      <c r="D45" s="22" t="inlineStr">
+      <c r="D45" s="23" t="inlineStr">
         <is>
           <t>+0.2</t>
         </is>
       </c>
-      <c r="E45" s="22" t="inlineStr">
+      <c r="E45" s="23" t="inlineStr">
         <is>
           <t>+35.0</t>
         </is>
       </c>
-      <c r="F45" s="22" t="inlineStr">
+      <c r="F45" s="23" t="inlineStr">
         <is>
           <t>+3.3</t>
         </is>
       </c>
-      <c r="G45" s="22" t="inlineStr">
+      <c r="G45" s="23" t="inlineStr">
         <is>
           <t>-3.0</t>
         </is>
       </c>
-      <c r="H45" s="22" t="inlineStr">
+      <c r="H45" s="23" t="inlineStr">
         <is>
           <t>Away</t>
         </is>
       </c>
-      <c r="I45" s="24" t="inlineStr">
+      <c r="I45" s="25" t="inlineStr">
         <is>
           <t>Loss</t>
         </is>
       </c>
-      <c r="J45" s="22" t="inlineStr">
+      <c r="J45" s="23" t="inlineStr">
         <is>
           <t>+7.3</t>
         </is>
       </c>
-      <c r="K45" s="22" t="inlineStr">
+      <c r="K45" s="23" t="inlineStr">
         <is>
           <t>-7.1</t>
         </is>
       </c>
-      <c r="L45" s="22" t="inlineStr">
+      <c r="L45" s="23" t="inlineStr">
         <is>
           <t>Away</t>
         </is>
       </c>
-      <c r="M45" s="24" t="inlineStr">
+      <c r="M45" s="25" t="inlineStr">
         <is>
           <t>Loss</t>
         </is>
       </c>
-      <c r="N45" s="22" t="inlineStr">
+      <c r="N45" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O45" s="23" t="inlineStr">
+      <c r="O45" s="24" t="inlineStr">
         <is>
           <t>Ridge</t>
         </is>
       </c>
-      <c r="P45" s="22" t="inlineStr">
+      <c r="P45" s="23" t="inlineStr">
         <is>
           <t>-0.3</t>
         </is>
       </c>
-      <c r="Q45" s="22" t="inlineStr">
+      <c r="Q45" s="23" t="inlineStr">
         <is>
           <t>-1.7</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="22" t="n">
+      <c r="A46" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="B46" s="22" t="inlineStr">
+      <c r="B46" s="23" t="inlineStr">
         <is>
           <t>Central Michigan @ New Mexico</t>
         </is>
       </c>
-      <c r="C46" s="22" t="inlineStr">
+      <c r="C46" s="23" t="inlineStr">
         <is>
           <t>7-38</t>
         </is>
       </c>
-      <c r="D46" s="22" t="inlineStr">
+      <c r="D46" s="23" t="inlineStr">
         <is>
           <t>-11.2</t>
         </is>
       </c>
-      <c r="E46" s="22" t="inlineStr">
+      <c r="E46" s="23" t="inlineStr">
         <is>
           <t>+31.0</t>
         </is>
       </c>
-      <c r="F46" s="22" t="inlineStr">
+      <c r="F46" s="23" t="inlineStr">
         <is>
           <t>-17.5</t>
         </is>
       </c>
-      <c r="G46" s="22" t="inlineStr">
+      <c r="G46" s="23" t="inlineStr">
         <is>
           <t>+6.2</t>
         </is>
       </c>
-      <c r="H46" s="22" t="inlineStr">
+      <c r="H46" s="23" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="I46" s="23" t="inlineStr">
+      <c r="I46" s="24" t="inlineStr">
         <is>
           <t>Win</t>
         </is>
       </c>
-      <c r="J46" s="22" t="inlineStr">
+      <c r="J46" s="23" t="inlineStr">
         <is>
           <t>-11.6</t>
         </is>
       </c>
-      <c r="K46" s="22" t="inlineStr">
+      <c r="K46" s="23" t="inlineStr">
         <is>
           <t>+0.3</t>
         </is>
       </c>
-      <c r="L46" s="22" t="inlineStr">
+      <c r="L46" s="23" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="M46" s="22" t="inlineStr">
+      <c r="M46" s="23" t="inlineStr">
         <is>
           <t>Lean only</t>
         </is>
       </c>
-      <c r="N46" s="22" t="inlineStr">
+      <c r="N46" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O46" s="23" t="inlineStr">
+      <c r="O46" s="24" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="P46" s="22" t="inlineStr">
+      <c r="P46" s="23" t="inlineStr">
         <is>
           <t>+5.9</t>
         </is>
       </c>
-      <c r="Q46" s="22" t="inlineStr">
+      <c r="Q46" s="23" t="inlineStr">
         <is>
           <t>-1.4</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="22" t="n">
+      <c r="A47" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="B47" s="22" t="inlineStr">
+      <c r="B47" s="23" t="inlineStr">
         <is>
           <t>Jacksonville State @ North Dakota State</t>
         </is>
       </c>
-      <c r="C47" s="22" t="inlineStr">
+      <c r="C47" s="23" t="inlineStr">
         <is>
           <t>7-33</t>
         </is>
       </c>
-      <c r="D47" s="22" t="inlineStr">
+      <c r="D47" s="23" t="inlineStr">
         <is>
           <t>-6.8</t>
         </is>
       </c>
-      <c r="E47" s="22" t="inlineStr">
+      <c r="E47" s="23" t="inlineStr">
         <is>
           <t>+26.0</t>
         </is>
       </c>
-      <c r="F47" s="22" t="inlineStr">
+      <c r="F47" s="23" t="inlineStr">
         <is>
           <t>-18.4</t>
         </is>
       </c>
-      <c r="G47" s="22" t="inlineStr">
+      <c r="G47" s="23" t="inlineStr">
         <is>
           <t>+11.6</t>
         </is>
       </c>
-      <c r="H47" s="22" t="inlineStr">
+      <c r="H47" s="23" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="I47" s="23" t="inlineStr">
+      <c r="I47" s="24" t="inlineStr">
         <is>
           <t>Win</t>
         </is>
       </c>
-      <c r="J47" s="22" t="inlineStr">
+      <c r="J47" s="23" t="inlineStr">
         <is>
           <t>-14.4</t>
         </is>
       </c>
-      <c r="K47" s="22" t="inlineStr">
+      <c r="K47" s="23" t="inlineStr">
         <is>
           <t>+7.7</t>
         </is>
       </c>
-      <c r="L47" s="22" t="inlineStr">
+      <c r="L47" s="23" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="M47" s="23" t="inlineStr">
+      <c r="M47" s="24" t="inlineStr">
         <is>
           <t>Win</t>
         </is>
       </c>
-      <c r="N47" s="22" t="inlineStr">
+      <c r="N47" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O47" s="23" t="inlineStr">
+      <c r="O47" s="24" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="P47" s="22" t="inlineStr">
+      <c r="P47" s="23" t="inlineStr">
         <is>
           <t>+17.6</t>
         </is>
       </c>
-      <c r="Q47" s="22" t="inlineStr">
+      <c r="Q47" s="23" t="inlineStr">
         <is>
           <t>+6.3</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="22" t="n">
+      <c r="A48" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="B48" s="22" t="inlineStr">
+      <c r="B48" s="23" t="inlineStr">
         <is>
           <t>Fordham @ North Dakota State</t>
         </is>
       </c>
-      <c r="C48" s="22" t="inlineStr">
+      <c r="C48" s="23" t="inlineStr">
         <is>
           <t>0-38</t>
         </is>
       </c>
-      <c r="D48" s="22" t="inlineStr">
+      <c r="D48" s="23" t="inlineStr">
         <is>
           <t>-41.5</t>
         </is>
       </c>
-      <c r="E48" s="22" t="inlineStr">
+      <c r="E48" s="23" t="inlineStr">
         <is>
           <t>+38.0</t>
         </is>
       </c>
-      <c r="F48" s="22" t="inlineStr">
+      <c r="F48" s="23" t="inlineStr">
         <is>
           <t>-40.9</t>
         </is>
       </c>
-      <c r="G48" s="22" t="inlineStr">
+      <c r="G48" s="23" t="inlineStr">
         <is>
           <t>-0.6</t>
         </is>
       </c>
-      <c r="H48" s="22" t="inlineStr">
+      <c r="H48" s="23" t="inlineStr">
         <is>
           <t>Away</t>
         </is>
       </c>
-      <c r="I48" s="22" t="inlineStr">
+      <c r="I48" s="23" t="inlineStr">
         <is>
           <t>Lean only</t>
         </is>
       </c>
-      <c r="J48" s="22" t="inlineStr">
+      <c r="J48" s="23" t="inlineStr">
         <is>
           <t>-35.0</t>
         </is>
       </c>
-      <c r="K48" s="22" t="inlineStr">
+      <c r="K48" s="23" t="inlineStr">
         <is>
           <t>-6.5</t>
         </is>
       </c>
-      <c r="L48" s="22" t="inlineStr">
+      <c r="L48" s="23" t="inlineStr">
         <is>
           <t>Away</t>
         </is>
       </c>
-      <c r="M48" s="23" t="inlineStr">
+      <c r="M48" s="24" t="inlineStr">
         <is>
           <t>Win</t>
         </is>
       </c>
-      <c r="N48" s="22" t="inlineStr">
+      <c r="N48" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O48" s="23" t="inlineStr">
+      <c r="O48" s="24" t="inlineStr">
         <is>
           <t>Ridge</t>
         </is>
       </c>
-      <c r="P48" s="22" t="inlineStr">
+      <c r="P48" s="23" t="inlineStr">
         <is>
           <t>+16.9</t>
         </is>
       </c>
-      <c r="Q48" s="22" t="inlineStr">
+      <c r="Q48" s="23" t="inlineStr">
         <is>
           <t>-0.2</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="22" t="n">
+      <c r="A49" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="B49" s="22" t="inlineStr">
+      <c r="B49" s="23" t="inlineStr">
         <is>
           <t>UTEP @ Oklahoma</t>
         </is>
       </c>
-      <c r="C49" s="22" t="inlineStr">
+      <c r="C49" s="23" t="inlineStr">
         <is>
           <t>0-51</t>
         </is>
       </c>
-      <c r="D49" s="22" t="inlineStr">
+      <c r="D49" s="23" t="inlineStr">
         <is>
           <t>-40.8</t>
         </is>
       </c>
-      <c r="E49" s="22" t="inlineStr">
+      <c r="E49" s="23" t="inlineStr">
         <is>
           <t>+51.0</t>
         </is>
       </c>
-      <c r="F49" s="22" t="inlineStr">
+      <c r="F49" s="23" t="inlineStr">
         <is>
           <t>-34.8</t>
         </is>
       </c>
-      <c r="G49" s="22" t="inlineStr">
+      <c r="G49" s="23" t="inlineStr">
         <is>
           <t>-5.9</t>
         </is>
       </c>
-      <c r="H49" s="22" t="inlineStr">
+      <c r="H49" s="23" t="inlineStr">
         <is>
           <t>Away</t>
         </is>
       </c>
-      <c r="I49" s="24" t="inlineStr">
+      <c r="I49" s="25" t="inlineStr">
         <is>
           <t>Loss</t>
         </is>
       </c>
-      <c r="J49" s="22" t="inlineStr">
+      <c r="J49" s="23" t="inlineStr">
         <is>
           <t>-32.8</t>
         </is>
       </c>
-      <c r="K49" s="22" t="inlineStr">
+      <c r="K49" s="23" t="inlineStr">
         <is>
           <t>-8.0</t>
         </is>
       </c>
-      <c r="L49" s="22" t="inlineStr">
+      <c r="L49" s="23" t="inlineStr">
         <is>
           <t>Away</t>
         </is>
       </c>
-      <c r="M49" s="24" t="inlineStr">
+      <c r="M49" s="25" t="inlineStr">
         <is>
           <t>Loss</t>
         </is>
       </c>
-      <c r="N49" s="22" t="inlineStr">
+      <c r="N49" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O49" s="23" t="inlineStr">
+      <c r="O49" s="24" t="inlineStr">
         <is>
           <t>Ridge</t>
         </is>
       </c>
-      <c r="P49" s="22" t="inlineStr">
+      <c r="P49" s="23" t="inlineStr">
         <is>
           <t>+11.0</t>
         </is>
       </c>
-      <c r="Q49" s="22" t="inlineStr">
+      <c r="Q49" s="23" t="inlineStr">
         <is>
           <t>-8.2</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="22" t="n">
+      <c r="A50" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="B50" s="22" t="inlineStr">
+      <c r="B50" s="23" t="inlineStr">
         <is>
           <t>Hawai'i @ Stanford</t>
         </is>
       </c>
-      <c r="C50" s="22" t="inlineStr">
+      <c r="C50" s="23" t="inlineStr">
         <is>
           <t>27-37</t>
         </is>
       </c>
-      <c r="D50" s="22" t="inlineStr">
+      <c r="D50" s="23" t="inlineStr">
         <is>
           <t>-4.8</t>
         </is>
       </c>
-      <c r="E50" s="22" t="inlineStr">
+      <c r="E50" s="23" t="inlineStr">
         <is>
           <t>+10.0</t>
         </is>
       </c>
-      <c r="F50" s="22" t="inlineStr">
+      <c r="F50" s="23" t="inlineStr">
         <is>
           <t>-1.5</t>
         </is>
       </c>
-      <c r="G50" s="22" t="inlineStr">
+      <c r="G50" s="23" t="inlineStr">
         <is>
           <t>-3.3</t>
         </is>
       </c>
-      <c r="H50" s="22" t="inlineStr">
+      <c r="H50" s="23" t="inlineStr">
         <is>
           <t>Away</t>
         </is>
       </c>
-      <c r="I50" s="24" t="inlineStr">
+      <c r="I50" s="25" t="inlineStr">
         <is>
           <t>Loss</t>
         </is>
       </c>
-      <c r="J50" s="22" t="inlineStr">
+      <c r="J50" s="23" t="inlineStr">
         <is>
           <t>+1.1</t>
         </is>
       </c>
-      <c r="K50" s="22" t="inlineStr">
+      <c r="K50" s="23" t="inlineStr">
         <is>
           <t>-5.8</t>
         </is>
       </c>
-      <c r="L50" s="22" t="inlineStr">
+      <c r="L50" s="23" t="inlineStr">
         <is>
           <t>Away</t>
         </is>
       </c>
-      <c r="M50" s="24" t="inlineStr">
+      <c r="M50" s="25" t="inlineStr">
         <is>
           <t>Loss</t>
         </is>
       </c>
-      <c r="N50" s="22" t="inlineStr">
+      <c r="N50" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O50" s="23" t="inlineStr">
+      <c r="O50" s="24" t="inlineStr">
         <is>
           <t>Ridge</t>
         </is>
       </c>
-      <c r="P50" s="22" t="inlineStr">
+      <c r="P50" s="23" t="inlineStr">
         <is>
           <t>+7.7</t>
         </is>
       </c>
-      <c r="Q50" s="22" t="inlineStr">
+      <c r="Q50" s="23" t="inlineStr">
         <is>
           <t>-14.0</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="22" t="n">
+      <c r="A51" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="B51" s="22" t="inlineStr">
+      <c r="B51" s="23" t="inlineStr">
         <is>
           <t>Memphis @ UNLV</t>
         </is>
       </c>
-      <c r="C51" s="22" t="inlineStr">
+      <c r="C51" s="23" t="inlineStr">
         <is>
           <t>27-21</t>
         </is>
       </c>
-      <c r="D51" s="22" t="inlineStr">
+      <c r="D51" s="23" t="inlineStr">
         <is>
           <t>-4.8</t>
         </is>
       </c>
-      <c r="E51" s="22" t="inlineStr">
+      <c r="E51" s="23" t="inlineStr">
         <is>
           <t>-6.0</t>
         </is>
       </c>
-      <c r="F51" s="22" t="inlineStr">
+      <c r="F51" s="23" t="inlineStr">
         <is>
           <t>-10.9</t>
         </is>
       </c>
-      <c r="G51" s="22" t="inlineStr">
+      <c r="G51" s="23" t="inlineStr">
         <is>
           <t>+6.2</t>
         </is>
       </c>
-      <c r="H51" s="22" t="inlineStr">
+      <c r="H51" s="23" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="I51" s="24" t="inlineStr">
+      <c r="I51" s="25" t="inlineStr">
         <is>
           <t>Loss</t>
         </is>
       </c>
-      <c r="J51" s="22" t="inlineStr">
+      <c r="J51" s="23" t="inlineStr">
         <is>
           <t>-7.4</t>
         </is>
       </c>
-      <c r="K51" s="22" t="inlineStr">
+      <c r="K51" s="23" t="inlineStr">
         <is>
           <t>+2.6</t>
         </is>
       </c>
-      <c r="L51" s="22" t="inlineStr">
+      <c r="L51" s="23" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="M51" s="24" t="inlineStr">
+      <c r="M51" s="25" t="inlineStr">
         <is>
           <t>Loss</t>
         </is>
       </c>
-      <c r="N51" s="22" t="inlineStr">
+      <c r="N51" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O51" s="23" t="inlineStr">
+      <c r="O51" s="24" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="P51" s="22" t="inlineStr">
+      <c r="P51" s="23" t="inlineStr">
         <is>
           <t>+13.9</t>
         </is>
       </c>
-      <c r="Q51" s="22" t="inlineStr">
+      <c r="Q51" s="23" t="inlineStr">
         <is>
           <t>-11.4</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="22" t="n">
+      <c r="A52" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="B52" s="22" t="inlineStr">
+      <c r="B52" s="23" t="inlineStr">
         <is>
           <t>San José State @ USC</t>
         </is>
       </c>
-      <c r="C52" s="22" t="inlineStr">
+      <c r="C52" s="23" t="inlineStr">
         <is>
           <t>26-42</t>
         </is>
       </c>
-      <c r="D52" s="22" t="inlineStr">
+      <c r="D52" s="23" t="inlineStr">
         <is>
           <t>-37.2</t>
         </is>
       </c>
-      <c r="E52" s="22" t="inlineStr">
+      <c r="E52" s="23" t="inlineStr">
         <is>
           <t>+16.0</t>
         </is>
       </c>
-      <c r="F52" s="22" t="inlineStr">
+      <c r="F52" s="23" t="inlineStr">
         <is>
           <t>-34.6</t>
         </is>
       </c>
-      <c r="G52" s="22" t="inlineStr">
+      <c r="G52" s="23" t="inlineStr">
         <is>
           <t>-2.7</t>
         </is>
       </c>
-      <c r="H52" s="22" t="inlineStr">
+      <c r="H52" s="23" t="inlineStr">
         <is>
           <t>Away</t>
         </is>
       </c>
-      <c r="I52" s="23" t="inlineStr">
+      <c r="I52" s="24" t="inlineStr">
         <is>
           <t>Win</t>
         </is>
       </c>
-      <c r="J52" s="22" t="inlineStr">
+      <c r="J52" s="23" t="inlineStr">
         <is>
           <t>-35.3</t>
         </is>
       </c>
-      <c r="K52" s="22" t="inlineStr">
+      <c r="K52" s="23" t="inlineStr">
         <is>
           <t>-2.0</t>
         </is>
       </c>
-      <c r="L52" s="22" t="inlineStr">
+      <c r="L52" s="23" t="inlineStr">
         <is>
           <t>Away</t>
         </is>
       </c>
-      <c r="M52" s="22" t="inlineStr">
+      <c r="M52" s="23" t="inlineStr">
         <is>
           <t>Lean only</t>
         </is>
       </c>
-      <c r="N52" s="22" t="inlineStr">
+      <c r="N52" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="O52" s="23" t="inlineStr">
+      <c r="O52" s="24" t="inlineStr">
         <is>
           <t>XGBoost</t>
         </is>
       </c>
-      <c r="P52" s="22" t="inlineStr">
+      <c r="P52" s="23" t="inlineStr">
         <is>
           <t>+11.2</t>
         </is>
       </c>
-      <c r="Q52" s="22" t="inlineStr">
+      <c r="Q52" s="23" t="inlineStr">
         <is>
           <t>-13.3</t>
         </is>

</xml_diff>

<commit_message>
Add Dub Gamma Model: data pull, replay engine, Excel, and site
</commit_message>
<xml_diff>
--- a/excel/MW_Handicapping_Tracker.xlsx
+++ b/excel/MW_Handicapping_Tracker.xlsx
@@ -835,7 +835,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R42"/>
+  <dimension ref="A1:R29"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1089,7 +1089,7 @@
         <v/>
       </c>
       <c r="I4" t="n">
-        <v>51.4</v>
+        <v>51.3</v>
       </c>
       <c r="J4" t="n">
         <v>48.5</v>
@@ -1497,7 +1497,7 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>-35</v>
+        <v>-34.9</v>
       </c>
       <c r="F11" t="n">
         <v>-40.8</v>
@@ -1633,7 +1633,7 @@
         <v/>
       </c>
       <c r="I13" t="n">
-        <v>50.6</v>
+        <v>50.5</v>
       </c>
       <c r="J13" t="n">
         <v>47.2</v>
@@ -1831,19 +1831,6 @@
       <c r="M29" s="6" t="n"/>
       <c r="N29" s="6" t="n"/>
     </row>
-    <row r="30"/>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
-    <row r="39"/>
-    <row r="40"/>
-    <row r="41"/>
-    <row r="42"/>
   </sheetData>
   <conditionalFormatting sqref="C2:C500">
     <cfRule type="expression" priority="1" dxfId="0">
@@ -3406,13 +3393,13 @@
         </is>
       </c>
       <c r="B6" s="23" t="n">
-        <v>8528</v>
+        <v>8529</v>
       </c>
       <c r="C6" s="23" t="n">
-        <v>6627</v>
+        <v>6628</v>
       </c>
       <c r="D6" s="23" t="n">
-        <v>3296</v>
+        <v>3297</v>
       </c>
       <c r="E6" s="23" t="n">
         <v>3331</v>
@@ -3427,17 +3414,17 @@
       </c>
       <c r="H6" s="23" t="inlineStr">
         <is>
-          <t>-5.1%</t>
+          <t>-5.0%</t>
         </is>
       </c>
       <c r="I6" s="23" t="inlineStr">
         <is>
-          <t>4043/8528 (47%)</t>
+          <t>4043/8529 (47%)</t>
         </is>
       </c>
       <c r="J6" s="23" t="inlineStr">
         <is>
-          <t>+5661.3</t>
+          <t>+5655.9</t>
         </is>
       </c>
     </row>
@@ -3474,7 +3461,7 @@
       </c>
       <c r="I7" s="23" t="inlineStr">
         <is>
-          <t>457/969 (47%)</t>
+          <t>455/969 (47%)</t>
         </is>
       </c>
       <c r="J7" s="23" t="inlineStr">
@@ -3490,16 +3477,16 @@
         </is>
       </c>
       <c r="B8" s="23" t="n">
-        <v>8528</v>
+        <v>8529</v>
       </c>
       <c r="C8" s="23" t="n">
-        <v>6561</v>
+        <v>6564</v>
       </c>
       <c r="D8" s="23" t="n">
-        <v>3312</v>
+        <v>3317</v>
       </c>
       <c r="E8" s="23" t="n">
-        <v>3249</v>
+        <v>3247</v>
       </c>
       <c r="F8" s="23" t="n">
         <v>59</v>
@@ -3511,17 +3498,17 @@
       </c>
       <c r="H8" s="23" t="inlineStr">
         <is>
-          <t>-3.6%</t>
+          <t>-3.5%</t>
         </is>
       </c>
       <c r="I8" s="23" t="inlineStr">
         <is>
-          <t>4485/8528 (53%)</t>
+          <t>4486/8529 (53%)</t>
         </is>
       </c>
       <c r="J8" s="23" t="inlineStr">
         <is>
-          <t>+741.2</t>
+          <t>+737.9</t>
         </is>
       </c>
     </row>
@@ -3535,10 +3522,10 @@
         <v>969</v>
       </c>
       <c r="C9" s="23" t="n">
-        <v>729</v>
+        <v>730</v>
       </c>
       <c r="D9" s="23" t="n">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="E9" s="23" t="n">
         <v>354</v>
@@ -3548,22 +3535,22 @@
       </c>
       <c r="G9" s="23" t="inlineStr">
         <is>
-          <t>51.4%</t>
+          <t>51.5%</t>
         </is>
       </c>
       <c r="H9" s="23" t="inlineStr">
         <is>
-          <t>-1.8%</t>
+          <t>-1.7%</t>
         </is>
       </c>
       <c r="I9" s="23" t="inlineStr">
         <is>
-          <t>512/969 (53%)</t>
+          <t>514/969 (53%)</t>
         </is>
       </c>
       <c r="J9" s="23" t="inlineStr">
         <is>
-          <t>+895.0</t>
+          <t>+895.9</t>
         </is>
       </c>
     </row>
@@ -3633,13 +3620,13 @@
         </is>
       </c>
       <c r="B13" s="23" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C13" s="23" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D13" s="23" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E13" s="23" t="n">
         <v>51</v>
@@ -3649,22 +3636,22 @@
       </c>
       <c r="G13" s="23" t="inlineStr">
         <is>
-          <t>39.3%</t>
+          <t>40.0%</t>
         </is>
       </c>
       <c r="H13" s="23" t="inlineStr">
         <is>
-          <t>-25.0%</t>
+          <t>-23.6%</t>
         </is>
       </c>
       <c r="I13" s="23" t="inlineStr">
         <is>
-          <t>42/95 (44%)</t>
+          <t>43/96 (45%)</t>
         </is>
       </c>
       <c r="J13" s="23" t="inlineStr">
         <is>
-          <t>-433.7</t>
+          <t>-439.0</t>
         </is>
       </c>
     </row>
@@ -3717,13 +3704,13 @@
         </is>
       </c>
       <c r="B15" s="23" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C15" s="23" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D15" s="23" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E15" s="23" t="n">
         <v>47</v>
@@ -3733,22 +3720,22 @@
       </c>
       <c r="G15" s="23" t="inlineStr">
         <is>
-          <t>39.7%</t>
+          <t>40.5%</t>
         </is>
       </c>
       <c r="H15" s="23" t="inlineStr">
         <is>
-          <t>-24.1%</t>
+          <t>-22.7%</t>
         </is>
       </c>
       <c r="I15" s="23" t="inlineStr">
         <is>
-          <t>53/95 (56%)</t>
+          <t>53/96 (55%)</t>
         </is>
       </c>
       <c r="J15" s="23" t="inlineStr">
         <is>
-          <t>-162.4</t>
+          <t>-172.9</t>
         </is>
       </c>
     </row>
@@ -3797,7 +3784,7 @@
     <row r="18">
       <c r="A18" s="20" t="inlineStr">
         <is>
-          <t>Ridge and XGBoost agree on which side to lean in 76.9% of all graded games.</t>
+          <t>Ridge and XGBoost agree on which side to lean in 77.0% of all graded games.</t>
         </is>
       </c>
     </row>
@@ -3876,7 +3863,7 @@
       </c>
       <c r="E22" s="23" t="inlineStr">
         <is>
-          <t>-32.3</t>
+          <t>-32.4</t>
         </is>
       </c>
       <c r="F22" s="23" t="inlineStr">
@@ -3921,7 +3908,7 @@
       </c>
       <c r="E23" s="23" t="inlineStr">
         <is>
-          <t>-16.3</t>
+          <t>-16.0</t>
         </is>
       </c>
       <c r="F23" s="23" t="inlineStr">
@@ -3966,7 +3953,7 @@
       </c>
       <c r="E24" s="23" t="inlineStr">
         <is>
-          <t>-0.3</t>
+          <t>-0.5</t>
         </is>
       </c>
       <c r="F24" s="23" t="inlineStr">
@@ -4011,7 +3998,7 @@
       </c>
       <c r="E25" s="23" t="inlineStr">
         <is>
-          <t>-6.7</t>
+          <t>-7.0</t>
         </is>
       </c>
       <c r="F25" s="23" t="inlineStr">
@@ -4056,7 +4043,7 @@
       </c>
       <c r="E26" s="23" t="inlineStr">
         <is>
-          <t>-9.9</t>
+          <t>-9.6</t>
         </is>
       </c>
       <c r="F26" s="23" t="inlineStr">
@@ -4096,12 +4083,12 @@
       </c>
       <c r="D27" s="23" t="inlineStr">
         <is>
-          <t>-35.0</t>
+          <t>-34.9</t>
         </is>
       </c>
       <c r="E27" s="23" t="inlineStr">
         <is>
-          <t>-33.6</t>
+          <t>-33.4</t>
         </is>
       </c>
       <c r="F27" s="23" t="inlineStr">
@@ -4146,7 +4133,7 @@
       </c>
       <c r="E28" s="23" t="inlineStr">
         <is>
-          <t>-29.5</t>
+          <t>-29.2</t>
         </is>
       </c>
       <c r="F28" s="23" t="inlineStr">
@@ -4236,7 +4223,7 @@
       </c>
       <c r="E30" s="23" t="inlineStr">
         <is>
-          <t>-25.6</t>
+          <t>-24.6</t>
         </is>
       </c>
       <c r="F30" s="23" t="inlineStr">
@@ -4281,7 +4268,7 @@
       </c>
       <c r="E31" s="23" t="inlineStr">
         <is>
-          <t>-3.9</t>
+          <t>-4.3</t>
         </is>
       </c>
       <c r="F31" s="23" t="inlineStr">
@@ -4311,42 +4298,42 @@
       </c>
       <c r="B32" s="23" t="inlineStr">
         <is>
-          <t>Central Michigan @ New Mexico</t>
+          <t>UNLV @ Hawai'i</t>
         </is>
       </c>
       <c r="C32" s="23" t="inlineStr">
         <is>
-          <t>-11.2</t>
+          <t>+2.8</t>
         </is>
       </c>
       <c r="D32" s="23" t="inlineStr">
         <is>
-          <t>-18.2</t>
+          <t>+3.5</t>
         </is>
       </c>
       <c r="E32" s="23" t="inlineStr">
         <is>
-          <t>-12.2</t>
+          <t>-0.8</t>
         </is>
       </c>
       <c r="F32" s="23" t="inlineStr">
         <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="G32" s="23" t="inlineStr">
+        <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="G32" s="23" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
       <c r="H32" s="23" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="I32" s="24" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>Ridge</t>
         </is>
       </c>
     </row>
@@ -4356,27 +4343,27 @@
       </c>
       <c r="B33" s="23" t="inlineStr">
         <is>
-          <t>UNLV @ Hawai'i</t>
+          <t>Central Michigan @ New Mexico</t>
         </is>
       </c>
       <c r="C33" s="23" t="inlineStr">
         <is>
-          <t>+2.8</t>
+          <t>-11.2</t>
         </is>
       </c>
       <c r="D33" s="23" t="inlineStr">
         <is>
-          <t>+3.5</t>
+          <t>-18.2</t>
         </is>
       </c>
       <c r="E33" s="23" t="inlineStr">
         <is>
-          <t>-1.1</t>
+          <t>-12.9</t>
         </is>
       </c>
       <c r="F33" s="23" t="inlineStr">
         <is>
-          <t>Away</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="G33" s="23" t="inlineStr">
@@ -4386,12 +4373,12 @@
       </c>
       <c r="H33" s="23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="I33" s="24" t="inlineStr">
         <is>
-          <t>Ridge</t>
+          <t>XGBoost</t>
         </is>
       </c>
     </row>
@@ -4416,7 +4403,7 @@
       </c>
       <c r="E34" s="23" t="inlineStr">
         <is>
-          <t>+4.4</t>
+          <t>+3.9</t>
         </is>
       </c>
       <c r="F34" s="23" t="inlineStr">

</xml_diff>

<commit_message>
Update Gamma Model data and grading
</commit_message>
<xml_diff>
--- a/excel/MW_Handicapping_Tracker.xlsx
+++ b/excel/MW_Handicapping_Tracker.xlsx
@@ -5428,7 +5428,7 @@
       </c>
       <c r="K6" s="37" t="inlineStr">
         <is>
-          <t>4047/8529 (47%)</t>
+          <t>4045/8529 (47%)</t>
         </is>
       </c>
       <c r="L6" s="37" t="inlineStr">
@@ -5500,10 +5500,10 @@
         <v>8458</v>
       </c>
       <c r="D8" s="37" t="n">
-        <v>4270</v>
+        <v>4269</v>
       </c>
       <c r="E8" s="37" t="n">
-        <v>4188</v>
+        <v>4189</v>
       </c>
       <c r="F8" s="37" t="n">
         <v>69</v>
@@ -5519,21 +5519,21 @@
         </is>
       </c>
       <c r="I8" s="37" t="n">
-        <v>6620</v>
+        <v>6623</v>
       </c>
       <c r="J8" s="37" t="inlineStr">
         <is>
-          <t>50.6%</t>
+          <t>50.5%</t>
         </is>
       </c>
       <c r="K8" s="37" t="inlineStr">
         <is>
-          <t>4482/8529 (53%)</t>
+          <t>4484/8529 (53%)</t>
         </is>
       </c>
       <c r="L8" s="37" t="inlineStr">
         <is>
-          <t>+738.6</t>
+          <t>+736.6</t>
         </is>
       </c>
     </row>
@@ -5583,7 +5583,7 @@
       </c>
       <c r="L9" s="37" t="inlineStr">
         <is>
-          <t>+896.4</t>
+          <t>+895.5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh game data, week 2 predictions, and Weekly Slate
</commit_message>
<xml_diff>
--- a/excel/MW_Handicapping_Tracker.xlsx
+++ b/excel/MW_Handicapping_Tracker.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="0" activeTab="5" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" firstSheet="0" activeTab="3" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Read Me" sheetId="1" state="visible" r:id="rId1"/>
@@ -965,7 +965,7 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>-34.9</v>
+        <v>-34.8</v>
       </c>
       <c r="F2" t="n">
         <v>-37.2</v>
@@ -1079,7 +1079,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>-1.8</v>
+        <v>-1.9</v>
       </c>
       <c r="F4" t="n">
         <v>-4.8</v>
@@ -1093,7 +1093,7 @@
         <v/>
       </c>
       <c r="I4" t="n">
-        <v>51.3</v>
+        <v>51.4</v>
       </c>
       <c r="J4" t="n">
         <v>48.5</v>
@@ -1210,7 +1210,7 @@
         <v/>
       </c>
       <c r="I6" t="n">
-        <v>54.3</v>
+        <v>54.2</v>
       </c>
       <c r="J6" t="n">
         <v>54.8</v>
@@ -1637,7 +1637,7 @@
         <v/>
       </c>
       <c r="I13" t="n">
-        <v>50.5</v>
+        <v>50.6</v>
       </c>
       <c r="J13" t="n">
         <v>47.2</v>
@@ -3407,10 +3407,10 @@
         <v>-1.8</v>
       </c>
       <c r="F2" s="9" t="n">
-        <v>0.23890241574583</v>
+        <v>0.2389024157458295</v>
       </c>
       <c r="G2" s="9" t="n">
-        <v>-0.313104117746208</v>
+        <v>-0.3131041177462083</v>
       </c>
       <c r="H2" s="9" t="n">
         <v>117</v>
@@ -3444,10 +3444,10 @@
         <v>3.6</v>
       </c>
       <c r="F3" s="9" t="n">
-        <v>0.120026137832497</v>
+        <v>0.1200261378324967</v>
       </c>
       <c r="G3" s="9" t="n">
-        <v>0.0892851354528907</v>
+        <v>0.08928513545289066</v>
       </c>
       <c r="H3" s="9" t="n">
         <v>63</v>
@@ -3481,10 +3481,10 @@
         <v>0</v>
       </c>
       <c r="F4" s="9" t="n">
-        <v>0.218710771609836</v>
+        <v>0.2187107716098359</v>
       </c>
       <c r="G4" s="9" t="n">
-        <v>-0.0521819579954482</v>
+        <v>-0.05218195799544816</v>
       </c>
       <c r="H4" s="9" t="n">
         <v>87</v>
@@ -3555,10 +3555,10 @@
         <v>-3.2</v>
       </c>
       <c r="F6" s="9" t="n">
-        <v>0.398894580108972</v>
+        <v>0.3988945801089721</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>-0.248118563368299</v>
+        <v>-0.2481185633682991</v>
       </c>
       <c r="H6" s="9" t="n">
         <v>141</v>
@@ -3592,10 +3592,10 @@
         <v>-10.8</v>
       </c>
       <c r="F7" s="9" t="n">
-        <v>-0.0251076991146115</v>
+        <v>-0.02510769911461149</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>0.301241820375048</v>
+        <v>0.3012418203750481</v>
       </c>
       <c r="H7" s="9" t="n">
         <v>114</v>
@@ -3629,10 +3629,10 @@
         <v>-17.2</v>
       </c>
       <c r="F8" s="9" t="n">
-        <v>-0.331732073650518</v>
+        <v>-0.3317320736505183</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>0.0613173930418566</v>
+        <v>0.06131739304185656</v>
       </c>
       <c r="H8" s="9" t="n">
         <v>82</v>
@@ -3666,10 +3666,10 @@
         <v>-15.7</v>
       </c>
       <c r="F9" s="9" t="n">
-        <v>0.165445410812368</v>
+        <v>0.1654454108123683</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>0.192612782957952</v>
+        <v>0.1926127829579521</v>
       </c>
       <c r="H9" s="9" t="n">
         <v>129</v>
@@ -3706,7 +3706,7 @@
         <v>0.556278847672138</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>0.06562288621201059</v>
+        <v>0.06562288621201061</v>
       </c>
       <c r="H10" s="9" t="n">
         <v>98</v>
@@ -3740,10 +3740,10 @@
         <v>-19.3</v>
       </c>
       <c r="F11" s="9" t="n">
-        <v>-0.251351409758154</v>
+        <v>-0.2513514097581536</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>0.387190583531566</v>
+        <v>0.3871905835315659</v>
       </c>
       <c r="H11" s="9" t="n">
         <v>92</v>

</xml_diff>

<commit_message>
Week 2 matchups and predictions
</commit_message>
<xml_diff>
--- a/excel/MW_Handicapping_Tracker.xlsx
+++ b/excel/MW_Handicapping_Tracker.xlsx
@@ -947,28 +947,28 @@
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>San José State</t>
+          <t>UNLV</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>USC</t>
+          <t>North Texas</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>-34.8</v>
+        <v>-3.9</v>
       </c>
       <c r="F2" t="n">
-        <v>-37.2</v>
+        <v>3.8</v>
       </c>
       <c r="G2" s="6">
         <f>F2-E2</f>
@@ -979,10 +979,10 @@
         <v/>
       </c>
       <c r="I2" t="n">
-        <v>53.3</v>
+        <v>58.2</v>
       </c>
       <c r="J2" t="n">
-        <v>61</v>
+        <v>57.2</v>
       </c>
       <c r="K2" s="6">
         <f>I2-J2</f>
@@ -1005,28 +1005,25 @@
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Jacksonville State</t>
+          <t>Northern Colorado</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>North Dakota State</t>
+          <t>Wyoming</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>-18.9</v>
-      </c>
-      <c r="F3" t="n">
-        <v>-6.8</v>
+        <v>-17.1</v>
       </c>
       <c r="G3" s="6">
         <f>F3-E3</f>
@@ -1037,10 +1034,7 @@
         <v/>
       </c>
       <c r="I3" t="n">
-        <v>52.9</v>
-      </c>
-      <c r="J3" t="n">
-        <v>46.5</v>
+        <v>55.2</v>
       </c>
       <c r="K3" s="6">
         <f>I3-J3</f>
@@ -1061,28 +1055,25 @@
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Hawai'i</t>
+          <t>Mercyhurst</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Stanford</t>
+          <t>New Mexico</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>-1.9</v>
-      </c>
-      <c r="F4" t="n">
-        <v>-4.8</v>
+        <v>-17.1</v>
       </c>
       <c r="G4" s="6">
         <f>F4-E4</f>
@@ -1093,10 +1084,7 @@
         <v/>
       </c>
       <c r="I4" t="n">
-        <v>51.4</v>
-      </c>
-      <c r="J4" t="n">
-        <v>48.5</v>
+        <v>54.1</v>
       </c>
       <c r="K4" s="6">
         <f>I4-J4</f>
@@ -1117,28 +1105,25 @@
     </row>
     <row r="5" ht="14.25" customHeight="1">
       <c r="A5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Memphis</t>
+          <t>Illinois State</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>UNLV</t>
+          <t>Northern Illinois</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>-11.3</v>
-      </c>
-      <c r="F5" t="n">
-        <v>-4.8</v>
+        <v>-16</v>
       </c>
       <c r="G5" s="6">
         <f>F5-E5</f>
@@ -1149,10 +1134,7 @@
         <v/>
       </c>
       <c r="I5" t="n">
-        <v>55.5</v>
-      </c>
-      <c r="J5" t="n">
-        <v>55.5</v>
+        <v>54.9</v>
       </c>
       <c r="K5" s="6">
         <f>I5-J5</f>
@@ -1178,28 +1160,25 @@
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>San José State</t>
+          <t>Texas Southern</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Eastern Michigan</t>
+          <t>UTEP</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>-16</v>
-      </c>
-      <c r="F6" t="n">
-        <v>-1.5</v>
+        <v>-16.1</v>
       </c>
       <c r="G6" s="6">
         <f>F6-E6</f>
@@ -1210,10 +1189,7 @@
         <v/>
       </c>
       <c r="I6" t="n">
-        <v>54.2</v>
-      </c>
-      <c r="J6" t="n">
-        <v>54.8</v>
+        <v>55.2</v>
       </c>
       <c r="K6" s="6">
         <f>I6-J6</f>
@@ -1239,29 +1215,27 @@
     </row>
     <row r="7" ht="14.25" customHeight="1">
       <c r="A7" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B7" s="10" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
         <is>
-          <t>Duquesne</t>
+          <t>Cal Poly</t>
         </is>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>Air Force</t>
+          <t>San José State</t>
         </is>
       </c>
       <c r="E7" s="10" t="n">
-        <v>-17.3</v>
-      </c>
-      <c r="F7" s="10" t="n">
-        <v>-30</v>
-      </c>
+        <v>-21</v>
+      </c>
+      <c r="F7" s="10" t="n"/>
       <c r="G7" s="10">
         <f>F7-E7</f>
         <v/>
@@ -1271,11 +1245,9 @@
         <v/>
       </c>
       <c r="I7" s="10" t="n">
-        <v>53</v>
-      </c>
-      <c r="J7" s="10" t="n">
-        <v>56.5</v>
-      </c>
+        <v>55.2</v>
+      </c>
+      <c r="J7" s="10" t="n"/>
       <c r="K7" s="10">
         <f>I7-J7</f>
         <v/>
@@ -1300,28 +1272,28 @@
     </row>
     <row r="8" ht="14.25" customHeight="1">
       <c r="A8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Fordham</t>
+          <t>North Dakota State</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>North Dakota State</t>
+          <t>Air Force</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>-39.8</v>
+        <v>16.9</v>
       </c>
       <c r="F8" t="n">
-        <v>-41.5</v>
+        <v>3</v>
       </c>
       <c r="G8" s="6">
         <f>F8-E8</f>
@@ -1332,10 +1304,10 @@
         <v/>
       </c>
       <c r="I8" t="n">
-        <v>55.2</v>
+        <v>53.3</v>
       </c>
       <c r="J8" t="n">
-        <v>54.2</v>
+        <v>47.2</v>
       </c>
       <c r="K8" s="6">
         <f>I8-J8</f>
@@ -1361,28 +1333,25 @@
     </row>
     <row r="9" ht="14.25" customHeight="1">
       <c r="A9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Northern Illinois</t>
+          <t>Montana State</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Iowa</t>
+          <t>Nevada</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>-28.7</v>
-      </c>
-      <c r="F9" t="n">
-        <v>-31.8</v>
+        <v>-17.2</v>
       </c>
       <c r="G9" s="6">
         <f>F9-E9</f>
@@ -1393,10 +1362,7 @@
         <v/>
       </c>
       <c r="I9" t="n">
-        <v>47.7</v>
-      </c>
-      <c r="J9" t="n">
-        <v>44.5</v>
+        <v>55.3</v>
       </c>
       <c r="K9" s="6">
         <f>I9-J9</f>
@@ -1422,28 +1388,28 @@
     </row>
     <row r="10" ht="14.25" customHeight="1">
       <c r="A10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Wyoming</t>
+          <t>New Mexico State</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Colorado State</t>
+          <t>Hawai'i</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>-8.300000000000001</v>
+        <v>-14.2</v>
       </c>
       <c r="F10" t="n">
-        <v>-2.8</v>
+        <v>-9.800000000000001</v>
       </c>
       <c r="G10" s="6">
         <f>F10-E10</f>
@@ -1454,10 +1420,10 @@
         <v/>
       </c>
       <c r="I10" t="n">
-        <v>49.3</v>
+        <v>55.6</v>
       </c>
       <c r="J10" t="n">
-        <v>46</v>
+        <v>50.5</v>
       </c>
       <c r="K10" s="6">
         <f>I10-J10</f>
@@ -1482,30 +1448,6 @@
       </c>
     </row>
     <row r="11" ht="14.25" customHeight="1">
-      <c r="A11" t="n">
-        <v>1</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>2026-09-05</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>UTEP</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Oklahoma</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>-34.9</v>
-      </c>
-      <c r="F11" t="n">
-        <v>-40.8</v>
-      </c>
       <c r="G11" s="6">
         <f>F11-E11</f>
         <v/>
@@ -1514,12 +1456,6 @@
         <f>IF(G11=0,"Pick'em",IF(G11&gt;0,"Home","Away"))</f>
         <v/>
       </c>
-      <c r="I11" t="n">
-        <v>52.4</v>
-      </c>
-      <c r="J11" t="n">
-        <v>51.2</v>
-      </c>
       <c r="K11" s="6">
         <f>I11-J11</f>
         <v/>
@@ -1543,30 +1479,6 @@
       </c>
     </row>
     <row r="12" ht="14.25" customHeight="1">
-      <c r="A12" t="n">
-        <v>1</v>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>2026-09-06</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>UNLV</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Hawai'i</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="F12" t="n">
-        <v>2.8</v>
-      </c>
       <c r="G12" s="6">
         <f>F12-E12</f>
         <v/>
@@ -1575,12 +1487,6 @@
         <f>IF(G12=0,"Pick'em",IF(G12&gt;0,"Home","Away"))</f>
         <v/>
       </c>
-      <c r="I12" t="n">
-        <v>54.4</v>
-      </c>
-      <c r="J12" t="n">
-        <v>55.5</v>
-      </c>
       <c r="K12" s="6">
         <f>I12-J12</f>
         <v/>
@@ -1604,30 +1510,6 @@
       </c>
     </row>
     <row r="13" ht="14.25" customHeight="1">
-      <c r="A13" t="n">
-        <v>1</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>2026-09-06</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Central Michigan</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>New Mexico</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>-18.2</v>
-      </c>
-      <c r="F13" t="n">
-        <v>-11.2</v>
-      </c>
       <c r="G13" s="6">
         <f>F13-E13</f>
         <v/>
@@ -1636,12 +1518,6 @@
         <f>IF(G13=0,"Pick'em",IF(G13&gt;0,"Home","Away"))</f>
         <v/>
       </c>
-      <c r="I13" t="n">
-        <v>50.6</v>
-      </c>
-      <c r="J13" t="n">
-        <v>47.2</v>
-      </c>
       <c r="K13" s="6">
         <f>I13-J13</f>
         <v/>
@@ -1660,30 +1536,6 @@
       </c>
     </row>
     <row r="14" ht="14.25" customHeight="1">
-      <c r="A14" t="n">
-        <v>1</v>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>2026-09-06</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Western Kentucky</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>Nevada</t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="F14" t="n">
-        <v>0.2</v>
-      </c>
       <c r="G14" s="6">
         <f>F14-E14</f>
         <v/>
@@ -1691,12 +1543,6 @@
       <c r="H14" s="6">
         <f>IF(G14=0,"Pick'em",IF(G14&gt;0,"Home","Away"))</f>
         <v/>
-      </c>
-      <c r="I14" t="n">
-        <v>51.7</v>
-      </c>
-      <c r="J14" t="n">
-        <v>51.5</v>
       </c>
       <c r="K14" s="6">
         <f>I14-J14</f>
@@ -3766,7 +3612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W56"/>
+  <dimension ref="A1:W52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -4619,361 +4465,361 @@
     </row>
     <row r="26">
       <c r="A26" s="23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B26" s="23" t="inlineStr">
         <is>
-          <t>San José State @ USC</t>
+          <t>UNLV @ North Texas</t>
         </is>
       </c>
       <c r="C26" s="23" t="inlineStr">
         <is>
-          <t>-37.2</t>
+          <t>+3.8</t>
         </is>
       </c>
       <c r="D26" s="23" t="inlineStr">
         <is>
-          <t>-34.8</t>
+          <t>-3.9</t>
         </is>
       </c>
       <c r="E26" s="23" t="inlineStr">
         <is>
-          <t>-31.8</t>
+          <t>+2.6</t>
         </is>
       </c>
       <c r="F26" s="23" t="inlineStr">
         <is>
-          <t>-16.1</t>
+          <t>-5.3</t>
         </is>
       </c>
       <c r="G26" s="23" t="inlineStr">
         <is>
-          <t>Away</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="H26" s="23" t="inlineStr">
         <is>
-          <t>Away</t>
+          <t>Away (auto)</t>
         </is>
       </c>
       <c r="I26" s="23" t="inlineStr">
         <is>
-          <t>Away</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="J26" s="23" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="K26" s="24" t="inlineStr">
         <is>
-          <t>Ridge</t>
+          <t>XGBoost</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B27" s="23" t="inlineStr">
         <is>
-          <t>Jacksonville State @ North Dakota State</t>
+          <t>Northern Colorado @ Wyoming</t>
         </is>
       </c>
       <c r="C27" s="23" t="inlineStr">
         <is>
-          <t>-6.8</t>
+          <t>--</t>
         </is>
       </c>
       <c r="D27" s="23" t="inlineStr">
         <is>
-          <t>-18.9</t>
+          <t>-17.1</t>
         </is>
       </c>
       <c r="E27" s="23" t="inlineStr">
         <is>
-          <t>-16.3</t>
+          <t>-21.5</t>
         </is>
       </c>
       <c r="F27" s="23" t="inlineStr">
         <is>
-          <t>-25.5</t>
+          <t>+11.3</t>
         </is>
       </c>
       <c r="G27" s="23" t="inlineStr">
         <is>
-          <t>Home</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="H27" s="23" t="inlineStr">
         <is>
-          <t>Home</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="I27" s="23" t="inlineStr">
         <is>
-          <t>Home</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="J27" s="23" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K27" s="24" t="inlineStr">
-        <is>
-          <t>XGBoost</t>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="K27" s="23" t="inlineStr">
+        <is>
+          <t>n/a</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B28" s="23" t="inlineStr">
         <is>
-          <t>Hawai'i @ Stanford</t>
+          <t>Mercyhurst @ New Mexico</t>
         </is>
       </c>
       <c r="C28" s="23" t="inlineStr">
         <is>
-          <t>-4.8</t>
+          <t>--</t>
         </is>
       </c>
       <c r="D28" s="23" t="inlineStr">
         <is>
-          <t>-1.9</t>
+          <t>-17.1</t>
         </is>
       </c>
       <c r="E28" s="23" t="inlineStr">
         <is>
-          <t>+0.2</t>
+          <t>-27.1</t>
         </is>
       </c>
       <c r="F28" s="23" t="inlineStr">
         <is>
-          <t>-11.2</t>
+          <t>-6.7</t>
         </is>
       </c>
       <c r="G28" s="23" t="inlineStr">
         <is>
-          <t>Away</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="H28" s="23" t="inlineStr">
         <is>
-          <t>Away</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="I28" s="23" t="inlineStr">
         <is>
-          <t>Home</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="J28" s="23" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K28" s="24" t="inlineStr">
-        <is>
-          <t>Ridge</t>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="K28" s="23" t="inlineStr">
+        <is>
+          <t>n/a</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B29" s="23" t="inlineStr">
         <is>
-          <t>Memphis @ UNLV</t>
+          <t>Illinois State @ Northern Illinois</t>
         </is>
       </c>
       <c r="C29" s="23" t="inlineStr">
         <is>
-          <t>-4.8</t>
+          <t>--</t>
         </is>
       </c>
       <c r="D29" s="23" t="inlineStr">
         <is>
-          <t>-11.3</t>
+          <t>-16.0</t>
         </is>
       </c>
       <c r="E29" s="23" t="inlineStr">
         <is>
-          <t>-6.9</t>
+          <t>-17.9</t>
         </is>
       </c>
       <c r="F29" s="23" t="inlineStr">
         <is>
-          <t>+1.6</t>
+          <t>+15.6</t>
         </is>
       </c>
       <c r="G29" s="23" t="inlineStr">
         <is>
-          <t>Home</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="H29" s="23" t="inlineStr">
         <is>
-          <t>Home</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="I29" s="23" t="inlineStr">
         <is>
-          <t>Away</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="J29" s="23" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K29" s="24" t="inlineStr">
-        <is>
-          <t>XGBoost</t>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="K29" s="23" t="inlineStr">
+        <is>
+          <t>n/a</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B30" s="23" t="inlineStr">
         <is>
-          <t>San José State @ Eastern Michigan</t>
+          <t>Texas Southern @ UTEP</t>
         </is>
       </c>
       <c r="C30" s="23" t="inlineStr">
         <is>
-          <t>-1.5</t>
+          <t>--</t>
         </is>
       </c>
       <c r="D30" s="23" t="inlineStr">
         <is>
-          <t>-16.0</t>
+          <t>-16.1</t>
         </is>
       </c>
       <c r="E30" s="23" t="inlineStr">
         <is>
-          <t>-10.4</t>
+          <t>-21.4</t>
         </is>
       </c>
       <c r="F30" s="23" t="inlineStr">
         <is>
-          <t>+0.5</t>
+          <t>+19.1</t>
         </is>
       </c>
       <c r="G30" s="23" t="inlineStr">
         <is>
-          <t>Home</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="H30" s="23" t="inlineStr">
         <is>
-          <t>Home</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="I30" s="23" t="inlineStr">
         <is>
-          <t>Away</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="J30" s="23" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K30" s="24" t="inlineStr">
-        <is>
-          <t>Gamma</t>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="K30" s="23" t="inlineStr">
+        <is>
+          <t>n/a</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B31" s="23" t="inlineStr">
         <is>
-          <t>UTEP @ Oklahoma</t>
+          <t>Cal Poly @ San José State</t>
         </is>
       </c>
       <c r="C31" s="23" t="inlineStr">
         <is>
-          <t>-40.8</t>
+          <t>--</t>
         </is>
       </c>
       <c r="D31" s="23" t="inlineStr">
         <is>
-          <t>-34.9</t>
+          <t>-21.0</t>
         </is>
       </c>
       <c r="E31" s="23" t="inlineStr">
         <is>
-          <t>-33.5</t>
+          <t>-30.0</t>
         </is>
       </c>
       <c r="F31" s="23" t="inlineStr">
         <is>
-          <t>-44.4</t>
+          <t>+8.1</t>
         </is>
       </c>
       <c r="G31" s="23" t="inlineStr">
         <is>
-          <t>Away</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="H31" s="23" t="inlineStr">
         <is>
-          <t>Away</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="I31" s="23" t="inlineStr">
         <is>
-          <t>Home</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="J31" s="23" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K31" s="24" t="inlineStr">
-        <is>
-          <t>Gamma</t>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="K31" s="23" t="inlineStr">
+        <is>
+          <t>n/a</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B32" s="23" t="inlineStr">
         <is>
-          <t>Duquesne @ Air Force</t>
+          <t>North Dakota State @ Air Force</t>
         </is>
       </c>
       <c r="C32" s="23" t="inlineStr">
         <is>
-          <t>-30.0</t>
+          <t>+3.0</t>
         </is>
       </c>
       <c r="D32" s="23" t="inlineStr">
         <is>
-          <t>-17.3</t>
+          <t>+16.9</t>
         </is>
       </c>
       <c r="E32" s="23" t="inlineStr">
         <is>
-          <t>-29.9</t>
+          <t>+15.3</t>
         </is>
       </c>
       <c r="F32" s="23" t="inlineStr">
         <is>
-          <t>+2.3</t>
+          <t>+17.9</t>
         </is>
       </c>
       <c r="G32" s="23" t="inlineStr">
@@ -4983,7 +4829,7 @@
       </c>
       <c r="H32" s="23" t="inlineStr">
         <is>
-          <t>Home (auto)</t>
+          <t>Away</t>
         </is>
       </c>
       <c r="I32" s="23" t="inlineStr">
@@ -4993,7 +4839,7 @@
       </c>
       <c r="J32" s="23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="K32" s="24" t="inlineStr">
@@ -5004,462 +4850,702 @@
     </row>
     <row r="33">
       <c r="A33" s="23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B33" s="23" t="inlineStr">
         <is>
-          <t>Fordham @ North Dakota State</t>
+          <t>Montana State @ Nevada</t>
         </is>
       </c>
       <c r="C33" s="23" t="inlineStr">
         <is>
-          <t>-41.5</t>
+          <t>--</t>
         </is>
       </c>
       <c r="D33" s="23" t="inlineStr">
         <is>
-          <t>-39.8</t>
+          <t>-17.2</t>
         </is>
       </c>
       <c r="E33" s="23" t="inlineStr">
         <is>
-          <t>-32.6</t>
+          <t>-12.7</t>
         </is>
       </c>
       <c r="F33" s="23" t="inlineStr">
         <is>
-          <t>-19.6</t>
+          <t>+5.3</t>
         </is>
       </c>
       <c r="G33" s="23" t="inlineStr">
         <is>
-          <t>Home (auto)</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="H33" s="23" t="inlineStr">
         <is>
-          <t>Away</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="I33" s="23" t="inlineStr">
         <is>
-          <t>Away</t>
+          <t>n/a</t>
         </is>
       </c>
       <c r="J33" s="23" t="inlineStr">
         <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K33" s="24" t="inlineStr">
-        <is>
-          <t>Ridge</t>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="K33" s="23" t="inlineStr">
+        <is>
+          <t>n/a</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="B34" s="23" t="inlineStr">
+        <is>
+          <t>New Mexico State @ Hawai'i</t>
+        </is>
+      </c>
+      <c r="C34" s="23" t="inlineStr">
+        <is>
+          <t>-9.8</t>
+        </is>
+      </c>
+      <c r="D34" s="23" t="inlineStr">
+        <is>
+          <t>-14.2</t>
+        </is>
+      </c>
+      <c r="E34" s="23" t="inlineStr">
+        <is>
+          <t>-13.2</t>
+        </is>
+      </c>
+      <c r="F34" s="23" t="inlineStr">
+        <is>
+          <t>-7.6</t>
+        </is>
+      </c>
+      <c r="G34" s="23" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="H34" s="23" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="I34" s="23" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="J34" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="K34" s="24" t="inlineStr">
+        <is>
+          <t>Gamma</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="20" t="inlineStr">
+        <is>
+          <t>* Tightest (Live) compares each model's line to TODAY's still-moving market line, not a final closing line -- it will keep changing until kickoff. See the graded Game-by-Game table below for the real, closing-line version of this comparison.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="21" t="inlineStr">
+        <is>
+          <t>2026 Mountain West Games -- Game by Game</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="22" t="inlineStr">
+        <is>
+          <t>Week</t>
+        </is>
+      </c>
+      <c r="B39" s="22" t="inlineStr">
+        <is>
+          <t>Matchup</t>
+        </is>
+      </c>
+      <c r="C39" s="22" t="inlineStr">
+        <is>
+          <t>Final Score</t>
+        </is>
+      </c>
+      <c r="D39" s="22" t="inlineStr">
+        <is>
+          <t>Vegas Spread (Home)</t>
+        </is>
+      </c>
+      <c r="E39" s="22" t="inlineStr">
+        <is>
+          <t>Actual Margin (Home)</t>
+        </is>
+      </c>
+      <c r="F39" s="22" t="inlineStr">
+        <is>
+          <t>Ridge Line</t>
+        </is>
+      </c>
+      <c r="G39" s="22" t="inlineStr">
+        <is>
+          <t>Ridge Edge</t>
+        </is>
+      </c>
+      <c r="H39" s="22" t="inlineStr">
+        <is>
+          <t>Ridge Lean</t>
+        </is>
+      </c>
+      <c r="I39" s="22" t="inlineStr">
+        <is>
+          <t>Ridge Result</t>
+        </is>
+      </c>
+      <c r="J39" s="22" t="inlineStr">
+        <is>
+          <t>XGBoost Line</t>
+        </is>
+      </c>
+      <c r="K39" s="22" t="inlineStr">
+        <is>
+          <t>XGBoost Edge</t>
+        </is>
+      </c>
+      <c r="L39" s="22" t="inlineStr">
+        <is>
+          <t>XGBoost Lean</t>
+        </is>
+      </c>
+      <c r="M39" s="22" t="inlineStr">
+        <is>
+          <t>XGBoost Result</t>
+        </is>
+      </c>
+      <c r="N39" s="22" t="inlineStr">
+        <is>
+          <t>Gamma Line</t>
+        </is>
+      </c>
+      <c r="O39" s="22" t="inlineStr">
+        <is>
+          <t>Gamma Edge</t>
+        </is>
+      </c>
+      <c r="P39" s="22" t="inlineStr">
+        <is>
+          <t>Gamma Lean</t>
+        </is>
+      </c>
+      <c r="Q39" s="22" t="inlineStr">
+        <is>
+          <t>Gamma Result</t>
+        </is>
+      </c>
+      <c r="R39" s="22" t="inlineStr">
+        <is>
+          <t>Ridge/XGBoost Agree?</t>
+        </is>
+      </c>
+      <c r="S39" s="22" t="inlineStr">
+        <is>
+          <t>Gamma Agrees (w/ Ridge)?</t>
+        </is>
+      </c>
+      <c r="T39" s="22" t="inlineStr">
+        <is>
+          <t>Tightest CLV Line</t>
+        </is>
+      </c>
+      <c r="U39" s="22" t="inlineStr">
+        <is>
+          <t>Ridge CLV Pts (Cum.)</t>
+        </is>
+      </c>
+      <c r="V39" s="22" t="inlineStr">
+        <is>
+          <t>XGBoost CLV Pts (Cum.)</t>
+        </is>
+      </c>
+      <c r="W39" s="22" t="inlineStr">
+        <is>
+          <t>Gamma CLV Pts (Cum.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="B34" s="23" t="inlineStr">
-        <is>
-          <t>Northern Illinois @ Iowa</t>
-        </is>
-      </c>
-      <c r="C34" s="23" t="inlineStr">
-        <is>
-          <t>-31.8</t>
-        </is>
-      </c>
-      <c r="D34" s="23" t="inlineStr">
+      <c r="B40" s="23" t="inlineStr">
+        <is>
+          <t>Duquesne @ Air Force</t>
+        </is>
+      </c>
+      <c r="C40" s="23" t="inlineStr">
+        <is>
+          <t>0-34</t>
+        </is>
+      </c>
+      <c r="D40" s="23" t="inlineStr">
+        <is>
+          <t>-30.0</t>
+        </is>
+      </c>
+      <c r="E40" s="23" t="inlineStr">
+        <is>
+          <t>+34.0</t>
+        </is>
+      </c>
+      <c r="F40" s="23" t="inlineStr">
+        <is>
+          <t>-17.0</t>
+        </is>
+      </c>
+      <c r="G40" s="23" t="inlineStr">
+        <is>
+          <t>-13.0</t>
+        </is>
+      </c>
+      <c r="H40" s="23" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="I40" s="25" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="J40" s="23" t="inlineStr">
+        <is>
+          <t>-28.3</t>
+        </is>
+      </c>
+      <c r="K40" s="23" t="inlineStr">
+        <is>
+          <t>-1.7</t>
+        </is>
+      </c>
+      <c r="L40" s="23" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="M40" s="24" t="inlineStr">
+        <is>
+          <t>Win (no real edge)</t>
+        </is>
+      </c>
+      <c r="N40" s="23" t="inlineStr">
+        <is>
+          <t>+2.3</t>
+        </is>
+      </c>
+      <c r="O40" s="23" t="inlineStr">
+        <is>
+          <t>-32.3</t>
+        </is>
+      </c>
+      <c r="P40" s="23" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="Q40" s="25" t="inlineStr">
+        <is>
+          <t>Loss (seed week)</t>
+        </is>
+      </c>
+      <c r="R40" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S40" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T40" s="24" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="U40" s="23" t="inlineStr">
+        <is>
+          <t>-13.0</t>
+        </is>
+      </c>
+      <c r="V40" s="23" t="inlineStr">
+        <is>
+          <t>-1.7</t>
+        </is>
+      </c>
+      <c r="W40" s="23" t="inlineStr">
+        <is>
+          <t>-32.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="B41" s="23" t="inlineStr">
+        <is>
+          <t>Wyoming @ Colorado State</t>
+        </is>
+      </c>
+      <c r="C41" s="23" t="inlineStr">
+        <is>
+          <t>13-35</t>
+        </is>
+      </c>
+      <c r="D41" s="23" t="inlineStr">
+        <is>
+          <t>-2.8</t>
+        </is>
+      </c>
+      <c r="E41" s="23" t="inlineStr">
+        <is>
+          <t>+22.0</t>
+        </is>
+      </c>
+      <c r="F41" s="23" t="inlineStr">
+        <is>
+          <t>-7.8</t>
+        </is>
+      </c>
+      <c r="G41" s="23" t="inlineStr">
+        <is>
+          <t>+5.1</t>
+        </is>
+      </c>
+      <c r="H41" s="23" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="I41" s="24" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="J41" s="23" t="inlineStr">
+        <is>
+          <t>-2.5</t>
+        </is>
+      </c>
+      <c r="K41" s="23" t="inlineStr">
+        <is>
+          <t>-0.2</t>
+        </is>
+      </c>
+      <c r="L41" s="23" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="M41" s="24" t="inlineStr">
+        <is>
+          <t>Win (no real edge)</t>
+        </is>
+      </c>
+      <c r="N41" s="23" t="inlineStr">
+        <is>
+          <t>-6.4</t>
+        </is>
+      </c>
+      <c r="O41" s="23" t="inlineStr">
+        <is>
+          <t>+3.7</t>
+        </is>
+      </c>
+      <c r="P41" s="23" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="Q41" s="24" t="inlineStr">
+        <is>
+          <t>Win (seed week)</t>
+        </is>
+      </c>
+      <c r="R41" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S41" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="T41" s="24" t="inlineStr">
+        <is>
+          <t>XGBoost</t>
+        </is>
+      </c>
+      <c r="U41" s="23" t="inlineStr">
+        <is>
+          <t>-7.9</t>
+        </is>
+      </c>
+      <c r="V41" s="23" t="inlineStr">
+        <is>
+          <t>-1.9</t>
+        </is>
+      </c>
+      <c r="W41" s="23" t="inlineStr">
         <is>
           <t>-28.7</t>
         </is>
       </c>
-      <c r="E34" s="23" t="inlineStr">
-        <is>
-          <t>-25.3</t>
-        </is>
-      </c>
-      <c r="F34" s="23" t="inlineStr">
-        <is>
-          <t>-41.0</t>
-        </is>
-      </c>
-      <c r="G34" s="23" t="inlineStr">
+    </row>
+    <row r="42">
+      <c r="A42" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="B42" s="23" t="inlineStr">
+        <is>
+          <t>San José State @ Eastern Michigan</t>
+        </is>
+      </c>
+      <c r="C42" s="23" t="inlineStr">
+        <is>
+          <t>27-21</t>
+        </is>
+      </c>
+      <c r="D42" s="23" t="inlineStr">
+        <is>
+          <t>-1.5</t>
+        </is>
+      </c>
+      <c r="E42" s="23" t="inlineStr">
+        <is>
+          <t>-6.0</t>
+        </is>
+      </c>
+      <c r="F42" s="23" t="inlineStr">
+        <is>
+          <t>-15.8</t>
+        </is>
+      </c>
+      <c r="G42" s="23" t="inlineStr">
+        <is>
+          <t>+14.3</t>
+        </is>
+      </c>
+      <c r="H42" s="23" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="I42" s="25" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="J42" s="23" t="inlineStr">
+        <is>
+          <t>-10.5</t>
+        </is>
+      </c>
+      <c r="K42" s="23" t="inlineStr">
+        <is>
+          <t>+9.0</t>
+        </is>
+      </c>
+      <c r="L42" s="23" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="M42" s="25" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="N42" s="23" t="inlineStr">
+        <is>
+          <t>+0.5</t>
+        </is>
+      </c>
+      <c r="O42" s="23" t="inlineStr">
+        <is>
+          <t>-2.0</t>
+        </is>
+      </c>
+      <c r="P42" s="23" t="inlineStr">
         <is>
           <t>Away</t>
         </is>
       </c>
-      <c r="H34" s="23" t="inlineStr">
+      <c r="Q42" s="24" t="inlineStr">
+        <is>
+          <t>Win (seed week)</t>
+        </is>
+      </c>
+      <c r="R42" s="23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S42" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="T42" s="24" t="inlineStr">
+        <is>
+          <t>Gamma</t>
+        </is>
+      </c>
+      <c r="U42" s="23" t="inlineStr">
+        <is>
+          <t>+6.4</t>
+        </is>
+      </c>
+      <c r="V42" s="23" t="inlineStr">
+        <is>
+          <t>+7.2</t>
+        </is>
+      </c>
+      <c r="W42" s="23" t="inlineStr">
+        <is>
+          <t>-30.7</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="B43" s="23" t="inlineStr">
+        <is>
+          <t>UNLV @ Hawai'i</t>
+        </is>
+      </c>
+      <c r="C43" s="23" t="inlineStr">
+        <is>
+          <t>21-6</t>
+        </is>
+      </c>
+      <c r="D43" s="23" t="inlineStr">
+        <is>
+          <t>+2.8</t>
+        </is>
+      </c>
+      <c r="E43" s="23" t="inlineStr">
+        <is>
+          <t>-15.0</t>
+        </is>
+      </c>
+      <c r="F43" s="23" t="inlineStr">
+        <is>
+          <t>+2.9</t>
+        </is>
+      </c>
+      <c r="G43" s="23" t="inlineStr">
+        <is>
+          <t>-0.1</t>
+        </is>
+      </c>
+      <c r="H43" s="23" t="inlineStr">
         <is>
           <t>Away</t>
         </is>
       </c>
-      <c r="I34" s="23" t="inlineStr">
+      <c r="I43" s="24" t="inlineStr">
+        <is>
+          <t>Win (no real edge)</t>
+        </is>
+      </c>
+      <c r="J43" s="23" t="inlineStr">
+        <is>
+          <t>-1.8</t>
+        </is>
+      </c>
+      <c r="K43" s="23" t="inlineStr">
+        <is>
+          <t>+4.6</t>
+        </is>
+      </c>
+      <c r="L43" s="23" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="J34" s="23" t="inlineStr">
+      <c r="M43" s="25" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="N43" s="23" t="inlineStr">
+        <is>
+          <t>+4.4</t>
+        </is>
+      </c>
+      <c r="O43" s="23" t="inlineStr">
+        <is>
+          <t>-1.6</t>
+        </is>
+      </c>
+      <c r="P43" s="23" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="Q43" s="24" t="inlineStr">
+        <is>
+          <t>Win (no real edge) (seed week)</t>
+        </is>
+      </c>
+      <c r="R43" s="23" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="S43" s="23" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K34" s="24" t="inlineStr">
+      <c r="T43" s="24" t="inlineStr">
         <is>
           <t>Ridge</t>
         </is>
       </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="B35" s="23" t="inlineStr">
-        <is>
-          <t>Wyoming @ Colorado State</t>
-        </is>
-      </c>
-      <c r="C35" s="23" t="inlineStr">
-        <is>
-          <t>-2.8</t>
-        </is>
-      </c>
-      <c r="D35" s="23" t="inlineStr">
-        <is>
-          <t>-8.3</t>
-        </is>
-      </c>
-      <c r="E35" s="23" t="inlineStr">
-        <is>
-          <t>-4.3</t>
-        </is>
-      </c>
-      <c r="F35" s="23" t="inlineStr">
-        <is>
-          <t>-6.4</t>
-        </is>
-      </c>
-      <c r="G35" s="23" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="H35" s="23" t="inlineStr">
-        <is>
-          <t>Home (auto)</t>
-        </is>
-      </c>
-      <c r="I35" s="23" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="J35" s="23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K35" s="24" t="inlineStr">
-        <is>
-          <t>XGBoost</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="B36" s="23" t="inlineStr">
-        <is>
-          <t>UNLV @ Hawai'i</t>
-        </is>
-      </c>
-      <c r="C36" s="23" t="inlineStr">
-        <is>
-          <t>+2.8</t>
-        </is>
-      </c>
-      <c r="D36" s="23" t="inlineStr">
-        <is>
-          <t>+3.5</t>
-        </is>
-      </c>
-      <c r="E36" s="23" t="inlineStr">
-        <is>
-          <t>-0.7</t>
-        </is>
-      </c>
-      <c r="F36" s="23" t="inlineStr">
-        <is>
-          <t>+4.4</t>
-        </is>
-      </c>
-      <c r="G36" s="23" t="inlineStr">
-        <is>
-          <t>Away (auto)</t>
-        </is>
-      </c>
-      <c r="H36" s="23" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="I36" s="23" t="inlineStr">
-        <is>
-          <t>Away (auto)</t>
-        </is>
-      </c>
-      <c r="J36" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="K36" s="24" t="inlineStr">
-        <is>
-          <t>Ridge</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="B37" s="23" t="inlineStr">
-        <is>
-          <t>Central Michigan @ New Mexico</t>
-        </is>
-      </c>
-      <c r="C37" s="23" t="inlineStr">
-        <is>
-          <t>-11.2</t>
-        </is>
-      </c>
-      <c r="D37" s="23" t="inlineStr">
-        <is>
-          <t>-18.2</t>
-        </is>
-      </c>
-      <c r="E37" s="23" t="inlineStr">
-        <is>
-          <t>-12.3</t>
-        </is>
-      </c>
-      <c r="F37" s="23" t="inlineStr">
-        <is>
-          <t>-15.6</t>
-        </is>
-      </c>
-      <c r="G37" s="23" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="H37" s="23" t="inlineStr">
-        <is>
-          <t>Home (auto)</t>
-        </is>
-      </c>
-      <c r="I37" s="23" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="J37" s="23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K37" s="24" t="inlineStr">
-        <is>
-          <t>XGBoost</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="B38" s="23" t="inlineStr">
-        <is>
-          <t>Western Kentucky @ Nevada</t>
-        </is>
-      </c>
-      <c r="C38" s="23" t="inlineStr">
-        <is>
-          <t>+0.2</t>
-        </is>
-      </c>
-      <c r="D38" s="23" t="inlineStr">
-        <is>
-          <t>+2.6</t>
-        </is>
-      </c>
-      <c r="E38" s="23" t="inlineStr">
-        <is>
-          <t>+4.2</t>
-        </is>
-      </c>
-      <c r="F38" s="23" t="inlineStr">
-        <is>
-          <t>-2.5</t>
-        </is>
-      </c>
-      <c r="G38" s="23" t="inlineStr">
-        <is>
-          <t>Away</t>
-        </is>
-      </c>
-      <c r="H38" s="23" t="inlineStr">
-        <is>
-          <t>Away</t>
-        </is>
-      </c>
-      <c r="I38" s="23" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="J38" s="23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="K38" s="24" t="inlineStr">
-        <is>
-          <t>Ridge</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="20" t="inlineStr">
-        <is>
-          <t>* Tightest (Live) compares each model's line to TODAY's still-moving market line, not a final closing line -- it will keep changing until kickoff. See the graded Game-by-Game table below for the real, closing-line version of this comparison.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="21" t="inlineStr">
-        <is>
-          <t>2026 Mountain West Games -- Game by Game</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="22" t="inlineStr">
-        <is>
-          <t>Week</t>
-        </is>
-      </c>
-      <c r="B43" s="22" t="inlineStr">
-        <is>
-          <t>Matchup</t>
-        </is>
-      </c>
-      <c r="C43" s="22" t="inlineStr">
-        <is>
-          <t>Final Score</t>
-        </is>
-      </c>
-      <c r="D43" s="22" t="inlineStr">
-        <is>
-          <t>Vegas Spread (Home)</t>
-        </is>
-      </c>
-      <c r="E43" s="22" t="inlineStr">
-        <is>
-          <t>Actual Margin (Home)</t>
-        </is>
-      </c>
-      <c r="F43" s="22" t="inlineStr">
-        <is>
-          <t>Ridge Line</t>
-        </is>
-      </c>
-      <c r="G43" s="22" t="inlineStr">
-        <is>
-          <t>Ridge Edge</t>
-        </is>
-      </c>
-      <c r="H43" s="22" t="inlineStr">
-        <is>
-          <t>Ridge Lean</t>
-        </is>
-      </c>
-      <c r="I43" s="22" t="inlineStr">
-        <is>
-          <t>Ridge Result</t>
-        </is>
-      </c>
-      <c r="J43" s="22" t="inlineStr">
-        <is>
-          <t>XGBoost Line</t>
-        </is>
-      </c>
-      <c r="K43" s="22" t="inlineStr">
-        <is>
-          <t>XGBoost Edge</t>
-        </is>
-      </c>
-      <c r="L43" s="22" t="inlineStr">
-        <is>
-          <t>XGBoost Lean</t>
-        </is>
-      </c>
-      <c r="M43" s="22" t="inlineStr">
-        <is>
-          <t>XGBoost Result</t>
-        </is>
-      </c>
-      <c r="N43" s="22" t="inlineStr">
-        <is>
-          <t>Gamma Line</t>
-        </is>
-      </c>
-      <c r="O43" s="22" t="inlineStr">
-        <is>
-          <t>Gamma Edge</t>
-        </is>
-      </c>
-      <c r="P43" s="22" t="inlineStr">
-        <is>
-          <t>Gamma Lean</t>
-        </is>
-      </c>
-      <c r="Q43" s="22" t="inlineStr">
-        <is>
-          <t>Gamma Result</t>
-        </is>
-      </c>
-      <c r="R43" s="22" t="inlineStr">
-        <is>
-          <t>Ridge/XGBoost Agree?</t>
-        </is>
-      </c>
-      <c r="S43" s="22" t="inlineStr">
-        <is>
-          <t>Gamma Agrees (w/ Ridge)?</t>
-        </is>
-      </c>
-      <c r="T43" s="22" t="inlineStr">
-        <is>
-          <t>Tightest CLV Line</t>
-        </is>
-      </c>
-      <c r="U43" s="22" t="inlineStr">
-        <is>
-          <t>Ridge CLV Pts (Cum.)</t>
-        </is>
-      </c>
-      <c r="V43" s="22" t="inlineStr">
-        <is>
-          <t>XGBoost CLV Pts (Cum.)</t>
-        </is>
-      </c>
-      <c r="W43" s="22" t="inlineStr">
-        <is>
-          <t>Gamma CLV Pts (Cum.)</t>
+      <c r="U43" s="23" t="inlineStr">
+        <is>
+          <t>+6.2</t>
+        </is>
+      </c>
+      <c r="V43" s="23" t="inlineStr">
+        <is>
+          <t>+11.8</t>
+        </is>
+      </c>
+      <c r="W43" s="23" t="inlineStr">
+        <is>
+          <t>-32.3</t>
         </is>
       </c>
     </row>
@@ -5469,32 +5555,32 @@
       </c>
       <c r="B44" s="23" t="inlineStr">
         <is>
-          <t>Duquesne @ Air Force</t>
+          <t>Northern Illinois @ Iowa</t>
         </is>
       </c>
       <c r="C44" s="23" t="inlineStr">
         <is>
-          <t>0-34</t>
+          <t>0-40</t>
         </is>
       </c>
       <c r="D44" s="23" t="inlineStr">
         <is>
-          <t>-30.0</t>
+          <t>-31.8</t>
         </is>
       </c>
       <c r="E44" s="23" t="inlineStr">
         <is>
-          <t>+34.0</t>
+          <t>+40.0</t>
         </is>
       </c>
       <c r="F44" s="23" t="inlineStr">
         <is>
-          <t>-17.0</t>
+          <t>-28.3</t>
         </is>
       </c>
       <c r="G44" s="23" t="inlineStr">
         <is>
-          <t>-13.0</t>
+          <t>-3.5</t>
         </is>
       </c>
       <c r="H44" s="23" t="inlineStr">
@@ -5509,72 +5595,72 @@
       </c>
       <c r="J44" s="23" t="inlineStr">
         <is>
-          <t>-28.3</t>
+          <t>-25.4</t>
         </is>
       </c>
       <c r="K44" s="23" t="inlineStr">
         <is>
-          <t>-1.7</t>
+          <t>-6.4</t>
         </is>
       </c>
       <c r="L44" s="23" t="inlineStr">
         <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="M44" s="25" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="N44" s="23" t="inlineStr">
+        <is>
+          <t>-41.0</t>
+        </is>
+      </c>
+      <c r="O44" s="23" t="inlineStr">
+        <is>
+          <t>+9.2</t>
+        </is>
+      </c>
+      <c r="P44" s="23" t="inlineStr">
+        <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="M44" s="24" t="inlineStr">
-        <is>
-          <t>Win (no real edge)</t>
-        </is>
-      </c>
-      <c r="N44" s="23" t="inlineStr">
-        <is>
-          <t>+2.3</t>
-        </is>
-      </c>
-      <c r="O44" s="23" t="inlineStr">
-        <is>
-          <t>-32.3</t>
-        </is>
-      </c>
-      <c r="P44" s="23" t="inlineStr">
-        <is>
-          <t>Away</t>
-        </is>
-      </c>
-      <c r="Q44" s="25" t="inlineStr">
-        <is>
-          <t>Loss (seed week)</t>
+      <c r="Q44" s="24" t="inlineStr">
+        <is>
+          <t>Win (seed week)</t>
         </is>
       </c>
       <c r="R44" s="23" t="inlineStr">
         <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="S44" s="23" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="S44" s="23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
       <c r="T44" s="24" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>Ridge</t>
         </is>
       </c>
       <c r="U44" s="23" t="inlineStr">
         <is>
-          <t>-13.0</t>
+          <t>+2.8</t>
         </is>
       </c>
       <c r="V44" s="23" t="inlineStr">
         <is>
-          <t>-1.7</t>
+          <t>+5.4</t>
         </is>
       </c>
       <c r="W44" s="23" t="inlineStr">
         <is>
-          <t>-32.3</t>
+          <t>-23.1</t>
         </is>
       </c>
     </row>
@@ -5584,79 +5670,79 @@
       </c>
       <c r="B45" s="23" t="inlineStr">
         <is>
-          <t>Wyoming @ Colorado State</t>
+          <t>Western Kentucky @ Nevada</t>
         </is>
       </c>
       <c r="C45" s="23" t="inlineStr">
         <is>
-          <t>13-35</t>
+          <t>14-49</t>
         </is>
       </c>
       <c r="D45" s="23" t="inlineStr">
         <is>
-          <t>-2.8</t>
+          <t>+0.2</t>
         </is>
       </c>
       <c r="E45" s="23" t="inlineStr">
         <is>
-          <t>+22.0</t>
+          <t>+35.0</t>
         </is>
       </c>
       <c r="F45" s="23" t="inlineStr">
         <is>
-          <t>-7.8</t>
+          <t>+3.3</t>
         </is>
       </c>
       <c r="G45" s="23" t="inlineStr">
         <is>
-          <t>+5.1</t>
+          <t>-3.0</t>
         </is>
       </c>
       <c r="H45" s="23" t="inlineStr">
         <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="I45" s="25" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="J45" s="23" t="inlineStr">
+        <is>
+          <t>+7.3</t>
+        </is>
+      </c>
+      <c r="K45" s="23" t="inlineStr">
+        <is>
+          <t>-7.1</t>
+        </is>
+      </c>
+      <c r="L45" s="23" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="M45" s="25" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="N45" s="23" t="inlineStr">
+        <is>
+          <t>-2.5</t>
+        </is>
+      </c>
+      <c r="O45" s="23" t="inlineStr">
+        <is>
+          <t>+2.7</t>
+        </is>
+      </c>
+      <c r="P45" s="23" t="inlineStr">
+        <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="I45" s="24" t="inlineStr">
-        <is>
-          <t>Win</t>
-        </is>
-      </c>
-      <c r="J45" s="23" t="inlineStr">
-        <is>
-          <t>-2.5</t>
-        </is>
-      </c>
-      <c r="K45" s="23" t="inlineStr">
-        <is>
-          <t>-0.2</t>
-        </is>
-      </c>
-      <c r="L45" s="23" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="M45" s="24" t="inlineStr">
-        <is>
-          <t>Win (no real edge)</t>
-        </is>
-      </c>
-      <c r="N45" s="23" t="inlineStr">
-        <is>
-          <t>-6.4</t>
-        </is>
-      </c>
-      <c r="O45" s="23" t="inlineStr">
-        <is>
-          <t>+3.7</t>
-        </is>
-      </c>
-      <c r="P45" s="23" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
       <c r="Q45" s="24" t="inlineStr">
         <is>
           <t>Win (seed week)</t>
@@ -5669,27 +5755,27 @@
       </c>
       <c r="S45" s="23" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="T45" s="24" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>Gamma</t>
         </is>
       </c>
       <c r="U45" s="23" t="inlineStr">
         <is>
-          <t>-7.9</t>
+          <t>-0.3</t>
         </is>
       </c>
       <c r="V45" s="23" t="inlineStr">
         <is>
-          <t>-1.9</t>
+          <t>-1.7</t>
         </is>
       </c>
       <c r="W45" s="23" t="inlineStr">
         <is>
-          <t>-28.7</t>
+          <t>-20.4</t>
         </is>
       </c>
     </row>
@@ -5699,32 +5785,32 @@
       </c>
       <c r="B46" s="23" t="inlineStr">
         <is>
-          <t>San José State @ Eastern Michigan</t>
+          <t>Central Michigan @ New Mexico</t>
         </is>
       </c>
       <c r="C46" s="23" t="inlineStr">
         <is>
-          <t>27-21</t>
+          <t>7-38</t>
         </is>
       </c>
       <c r="D46" s="23" t="inlineStr">
         <is>
-          <t>-1.5</t>
+          <t>-11.2</t>
         </is>
       </c>
       <c r="E46" s="23" t="inlineStr">
         <is>
-          <t>-6.0</t>
+          <t>+31.0</t>
         </is>
       </c>
       <c r="F46" s="23" t="inlineStr">
         <is>
-          <t>-15.8</t>
+          <t>-17.5</t>
         </is>
       </c>
       <c r="G46" s="23" t="inlineStr">
         <is>
-          <t>+14.3</t>
+          <t>+6.2</t>
         </is>
       </c>
       <c r="H46" s="23" t="inlineStr">
@@ -5732,19 +5818,19 @@
           <t>Home</t>
         </is>
       </c>
-      <c r="I46" s="25" t="inlineStr">
-        <is>
-          <t>Loss</t>
+      <c r="I46" s="24" t="inlineStr">
+        <is>
+          <t>Win</t>
         </is>
       </c>
       <c r="J46" s="23" t="inlineStr">
         <is>
-          <t>-10.5</t>
+          <t>-11.6</t>
         </is>
       </c>
       <c r="K46" s="23" t="inlineStr">
         <is>
-          <t>+9.0</t>
+          <t>+0.3</t>
         </is>
       </c>
       <c r="L46" s="23" t="inlineStr">
@@ -5752,24 +5838,24 @@
           <t>Home</t>
         </is>
       </c>
-      <c r="M46" s="25" t="inlineStr">
-        <is>
-          <t>Loss</t>
+      <c r="M46" s="24" t="inlineStr">
+        <is>
+          <t>Win (no real edge)</t>
         </is>
       </c>
       <c r="N46" s="23" t="inlineStr">
         <is>
-          <t>+0.5</t>
+          <t>-15.6</t>
         </is>
       </c>
       <c r="O46" s="23" t="inlineStr">
         <is>
-          <t>-2.0</t>
+          <t>+4.3</t>
         </is>
       </c>
       <c r="P46" s="23" t="inlineStr">
         <is>
-          <t>Away</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="Q46" s="24" t="inlineStr">
@@ -5784,27 +5870,27 @@
       </c>
       <c r="S46" s="23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="T46" s="24" t="inlineStr">
         <is>
-          <t>Gamma</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="U46" s="23" t="inlineStr">
         <is>
-          <t>+6.4</t>
+          <t>+5.9</t>
         </is>
       </c>
       <c r="V46" s="23" t="inlineStr">
         <is>
-          <t>+7.2</t>
+          <t>-1.4</t>
         </is>
       </c>
       <c r="W46" s="23" t="inlineStr">
         <is>
-          <t>-30.7</t>
+          <t>-16.0</t>
         </is>
       </c>
     </row>
@@ -5814,52 +5900,52 @@
       </c>
       <c r="B47" s="23" t="inlineStr">
         <is>
-          <t>UNLV @ Hawai'i</t>
+          <t>Jacksonville State @ North Dakota State</t>
         </is>
       </c>
       <c r="C47" s="23" t="inlineStr">
         <is>
-          <t>21-6</t>
+          <t>7-33</t>
         </is>
       </c>
       <c r="D47" s="23" t="inlineStr">
         <is>
-          <t>+2.8</t>
+          <t>-6.8</t>
         </is>
       </c>
       <c r="E47" s="23" t="inlineStr">
         <is>
-          <t>-15.0</t>
+          <t>+26.0</t>
         </is>
       </c>
       <c r="F47" s="23" t="inlineStr">
         <is>
-          <t>+2.9</t>
+          <t>-18.4</t>
         </is>
       </c>
       <c r="G47" s="23" t="inlineStr">
         <is>
-          <t>-0.1</t>
+          <t>+11.6</t>
         </is>
       </c>
       <c r="H47" s="23" t="inlineStr">
         <is>
-          <t>Away</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="I47" s="24" t="inlineStr">
         <is>
-          <t>Win (no real edge)</t>
+          <t>Win</t>
         </is>
       </c>
       <c r="J47" s="23" t="inlineStr">
         <is>
-          <t>-1.8</t>
+          <t>-14.4</t>
         </is>
       </c>
       <c r="K47" s="23" t="inlineStr">
         <is>
-          <t>+4.6</t>
+          <t>+7.7</t>
         </is>
       </c>
       <c r="L47" s="23" t="inlineStr">
@@ -5867,34 +5953,34 @@
           <t>Home</t>
         </is>
       </c>
-      <c r="M47" s="25" t="inlineStr">
-        <is>
-          <t>Loss</t>
+      <c r="M47" s="24" t="inlineStr">
+        <is>
+          <t>Win</t>
         </is>
       </c>
       <c r="N47" s="23" t="inlineStr">
         <is>
-          <t>+4.4</t>
+          <t>-25.5</t>
         </is>
       </c>
       <c r="O47" s="23" t="inlineStr">
         <is>
-          <t>-1.6</t>
+          <t>+18.7</t>
         </is>
       </c>
       <c r="P47" s="23" t="inlineStr">
         <is>
-          <t>Away</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="Q47" s="24" t="inlineStr">
         <is>
-          <t>Win (no real edge) (seed week)</t>
+          <t>Win (seed week)</t>
         </is>
       </c>
       <c r="R47" s="23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="S47" s="23" t="inlineStr">
@@ -5904,22 +5990,22 @@
       </c>
       <c r="T47" s="24" t="inlineStr">
         <is>
-          <t>Ridge</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="U47" s="23" t="inlineStr">
         <is>
-          <t>+6.2</t>
+          <t>+17.6</t>
         </is>
       </c>
       <c r="V47" s="23" t="inlineStr">
         <is>
-          <t>+11.8</t>
+          <t>+6.3</t>
         </is>
       </c>
       <c r="W47" s="23" t="inlineStr">
         <is>
-          <t>-32.3</t>
+          <t>+2.7</t>
         </is>
       </c>
     </row>
@@ -5929,79 +6015,79 @@
       </c>
       <c r="B48" s="23" t="inlineStr">
         <is>
-          <t>Northern Illinois @ Iowa</t>
+          <t>Fordham @ North Dakota State</t>
         </is>
       </c>
       <c r="C48" s="23" t="inlineStr">
         <is>
-          <t>0-40</t>
+          <t>0-38</t>
         </is>
       </c>
       <c r="D48" s="23" t="inlineStr">
         <is>
-          <t>-31.8</t>
+          <t>-41.5</t>
         </is>
       </c>
       <c r="E48" s="23" t="inlineStr">
         <is>
-          <t>+40.0</t>
+          <t>+38.0</t>
         </is>
       </c>
       <c r="F48" s="23" t="inlineStr">
         <is>
-          <t>-28.3</t>
+          <t>-40.9</t>
         </is>
       </c>
       <c r="G48" s="23" t="inlineStr">
         <is>
-          <t>-3.5</t>
+          <t>-0.6</t>
         </is>
       </c>
       <c r="H48" s="23" t="inlineStr">
         <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="I48" s="25" t="inlineStr">
+        <is>
+          <t>Loss (no real edge)</t>
+        </is>
+      </c>
+      <c r="J48" s="23" t="inlineStr">
+        <is>
+          <t>-35.0</t>
+        </is>
+      </c>
+      <c r="K48" s="23" t="inlineStr">
+        <is>
+          <t>-6.5</t>
+        </is>
+      </c>
+      <c r="L48" s="23" t="inlineStr">
+        <is>
           <t>Away</t>
         </is>
       </c>
-      <c r="I48" s="25" t="inlineStr">
-        <is>
-          <t>Loss</t>
-        </is>
-      </c>
-      <c r="J48" s="23" t="inlineStr">
-        <is>
-          <t>-25.4</t>
-        </is>
-      </c>
-      <c r="K48" s="23" t="inlineStr">
-        <is>
-          <t>-6.4</t>
-        </is>
-      </c>
-      <c r="L48" s="23" t="inlineStr">
+      <c r="M48" s="24" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="N48" s="23" t="inlineStr">
+        <is>
+          <t>-19.6</t>
+        </is>
+      </c>
+      <c r="O48" s="23" t="inlineStr">
+        <is>
+          <t>-21.9</t>
+        </is>
+      </c>
+      <c r="P48" s="23" t="inlineStr">
         <is>
           <t>Away</t>
         </is>
       </c>
-      <c r="M48" s="25" t="inlineStr">
-        <is>
-          <t>Loss</t>
-        </is>
-      </c>
-      <c r="N48" s="23" t="inlineStr">
-        <is>
-          <t>-41.0</t>
-        </is>
-      </c>
-      <c r="O48" s="23" t="inlineStr">
-        <is>
-          <t>+9.2</t>
-        </is>
-      </c>
-      <c r="P48" s="23" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
       <c r="Q48" s="24" t="inlineStr">
         <is>
           <t>Win (seed week)</t>
@@ -6009,7 +6095,7 @@
       </c>
       <c r="R48" s="23" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="S48" s="23" t="inlineStr">
@@ -6024,17 +6110,17 @@
       </c>
       <c r="U48" s="23" t="inlineStr">
         <is>
-          <t>+2.8</t>
+          <t>+16.9</t>
         </is>
       </c>
       <c r="V48" s="23" t="inlineStr">
         <is>
-          <t>+5.4</t>
+          <t>-0.2</t>
         </is>
       </c>
       <c r="W48" s="23" t="inlineStr">
         <is>
-          <t>-23.1</t>
+          <t>-19.2</t>
         </is>
       </c>
     </row>
@@ -6044,32 +6130,32 @@
       </c>
       <c r="B49" s="23" t="inlineStr">
         <is>
-          <t>Western Kentucky @ Nevada</t>
+          <t>UTEP @ Oklahoma</t>
         </is>
       </c>
       <c r="C49" s="23" t="inlineStr">
         <is>
-          <t>14-49</t>
+          <t>0-51</t>
         </is>
       </c>
       <c r="D49" s="23" t="inlineStr">
         <is>
-          <t>+0.2</t>
+          <t>-40.8</t>
         </is>
       </c>
       <c r="E49" s="23" t="inlineStr">
         <is>
-          <t>+35.0</t>
+          <t>+51.0</t>
         </is>
       </c>
       <c r="F49" s="23" t="inlineStr">
         <is>
-          <t>+3.3</t>
+          <t>-34.8</t>
         </is>
       </c>
       <c r="G49" s="23" t="inlineStr">
         <is>
-          <t>-3.0</t>
+          <t>-5.9</t>
         </is>
       </c>
       <c r="H49" s="23" t="inlineStr">
@@ -6084,12 +6170,12 @@
       </c>
       <c r="J49" s="23" t="inlineStr">
         <is>
-          <t>+7.3</t>
+          <t>-32.8</t>
         </is>
       </c>
       <c r="K49" s="23" t="inlineStr">
         <is>
-          <t>-7.1</t>
+          <t>-8.0</t>
         </is>
       </c>
       <c r="L49" s="23" t="inlineStr">
@@ -6104,12 +6190,12 @@
       </c>
       <c r="N49" s="23" t="inlineStr">
         <is>
-          <t>-2.5</t>
+          <t>-44.4</t>
         </is>
       </c>
       <c r="O49" s="23" t="inlineStr">
         <is>
-          <t>+2.7</t>
+          <t>+3.6</t>
         </is>
       </c>
       <c r="P49" s="23" t="inlineStr">
@@ -6139,17 +6225,17 @@
       </c>
       <c r="U49" s="23" t="inlineStr">
         <is>
-          <t>-0.3</t>
+          <t>+11.0</t>
         </is>
       </c>
       <c r="V49" s="23" t="inlineStr">
         <is>
-          <t>-1.7</t>
+          <t>-8.2</t>
         </is>
       </c>
       <c r="W49" s="23" t="inlineStr">
         <is>
-          <t>-20.4</t>
+          <t>-15.6</t>
         </is>
       </c>
     </row>
@@ -6159,79 +6245,79 @@
       </c>
       <c r="B50" s="23" t="inlineStr">
         <is>
-          <t>Central Michigan @ New Mexico</t>
+          <t>Hawai'i @ Stanford</t>
         </is>
       </c>
       <c r="C50" s="23" t="inlineStr">
         <is>
-          <t>7-38</t>
+          <t>27-37</t>
         </is>
       </c>
       <c r="D50" s="23" t="inlineStr">
         <is>
+          <t>-4.8</t>
+        </is>
+      </c>
+      <c r="E50" s="23" t="inlineStr">
+        <is>
+          <t>+10.0</t>
+        </is>
+      </c>
+      <c r="F50" s="23" t="inlineStr">
+        <is>
+          <t>-1.5</t>
+        </is>
+      </c>
+      <c r="G50" s="23" t="inlineStr">
+        <is>
+          <t>-3.3</t>
+        </is>
+      </c>
+      <c r="H50" s="23" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="I50" s="25" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="J50" s="23" t="inlineStr">
+        <is>
+          <t>+1.1</t>
+        </is>
+      </c>
+      <c r="K50" s="23" t="inlineStr">
+        <is>
+          <t>-5.8</t>
+        </is>
+      </c>
+      <c r="L50" s="23" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="M50" s="25" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="N50" s="23" t="inlineStr">
+        <is>
           <t>-11.2</t>
         </is>
       </c>
-      <c r="E50" s="23" t="inlineStr">
-        <is>
-          <t>+31.0</t>
-        </is>
-      </c>
-      <c r="F50" s="23" t="inlineStr">
-        <is>
-          <t>-17.5</t>
-        </is>
-      </c>
-      <c r="G50" s="23" t="inlineStr">
-        <is>
-          <t>+6.2</t>
-        </is>
-      </c>
-      <c r="H50" s="23" t="inlineStr">
+      <c r="O50" s="23" t="inlineStr">
+        <is>
+          <t>+6.4</t>
+        </is>
+      </c>
+      <c r="P50" s="23" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="I50" s="24" t="inlineStr">
-        <is>
-          <t>Win</t>
-        </is>
-      </c>
-      <c r="J50" s="23" t="inlineStr">
-        <is>
-          <t>-11.6</t>
-        </is>
-      </c>
-      <c r="K50" s="23" t="inlineStr">
-        <is>
-          <t>+0.3</t>
-        </is>
-      </c>
-      <c r="L50" s="23" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="M50" s="24" t="inlineStr">
-        <is>
-          <t>Win (no real edge)</t>
-        </is>
-      </c>
-      <c r="N50" s="23" t="inlineStr">
-        <is>
-          <t>-15.6</t>
-        </is>
-      </c>
-      <c r="O50" s="23" t="inlineStr">
-        <is>
-          <t>+4.3</t>
-        </is>
-      </c>
-      <c r="P50" s="23" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
       <c r="Q50" s="24" t="inlineStr">
         <is>
           <t>Win (seed week)</t>
@@ -6244,27 +6330,27 @@
       </c>
       <c r="S50" s="23" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="T50" s="24" t="inlineStr">
         <is>
-          <t>XGBoost</t>
+          <t>Ridge</t>
         </is>
       </c>
       <c r="U50" s="23" t="inlineStr">
         <is>
-          <t>+5.9</t>
+          <t>+7.7</t>
         </is>
       </c>
       <c r="V50" s="23" t="inlineStr">
         <is>
-          <t>-1.4</t>
+          <t>-14.0</t>
         </is>
       </c>
       <c r="W50" s="23" t="inlineStr">
         <is>
-          <t>-16.0</t>
+          <t>-9.2</t>
         </is>
       </c>
     </row>
@@ -6274,32 +6360,32 @@
       </c>
       <c r="B51" s="23" t="inlineStr">
         <is>
-          <t>Jacksonville State @ North Dakota State</t>
+          <t>Memphis @ UNLV</t>
         </is>
       </c>
       <c r="C51" s="23" t="inlineStr">
         <is>
-          <t>7-33</t>
+          <t>27-21</t>
         </is>
       </c>
       <c r="D51" s="23" t="inlineStr">
         <is>
-          <t>-6.8</t>
+          <t>-4.8</t>
         </is>
       </c>
       <c r="E51" s="23" t="inlineStr">
         <is>
-          <t>+26.0</t>
+          <t>-6.0</t>
         </is>
       </c>
       <c r="F51" s="23" t="inlineStr">
         <is>
-          <t>-18.4</t>
+          <t>-10.9</t>
         </is>
       </c>
       <c r="G51" s="23" t="inlineStr">
         <is>
-          <t>+11.6</t>
+          <t>+6.2</t>
         </is>
       </c>
       <c r="H51" s="23" t="inlineStr">
@@ -6307,19 +6393,19 @@
           <t>Home</t>
         </is>
       </c>
-      <c r="I51" s="24" t="inlineStr">
-        <is>
-          <t>Win</t>
+      <c r="I51" s="25" t="inlineStr">
+        <is>
+          <t>Loss</t>
         </is>
       </c>
       <c r="J51" s="23" t="inlineStr">
         <is>
-          <t>-14.4</t>
+          <t>-7.4</t>
         </is>
       </c>
       <c r="K51" s="23" t="inlineStr">
         <is>
-          <t>+7.7</t>
+          <t>+2.6</t>
         </is>
       </c>
       <c r="L51" s="23" t="inlineStr">
@@ -6327,24 +6413,24 @@
           <t>Home</t>
         </is>
       </c>
-      <c r="M51" s="24" t="inlineStr">
-        <is>
-          <t>Win</t>
+      <c r="M51" s="25" t="inlineStr">
+        <is>
+          <t>Loss</t>
         </is>
       </c>
       <c r="N51" s="23" t="inlineStr">
         <is>
-          <t>-25.5</t>
+          <t>+1.6</t>
         </is>
       </c>
       <c r="O51" s="23" t="inlineStr">
         <is>
-          <t>+18.7</t>
+          <t>-6.3</t>
         </is>
       </c>
       <c r="P51" s="23" t="inlineStr">
         <is>
-          <t>Home</t>
+          <t>Away</t>
         </is>
       </c>
       <c r="Q51" s="24" t="inlineStr">
@@ -6359,7 +6445,7 @@
       </c>
       <c r="S51" s="23" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="T51" s="24" t="inlineStr">
@@ -6369,17 +6455,17 @@
       </c>
       <c r="U51" s="23" t="inlineStr">
         <is>
-          <t>+17.6</t>
+          <t>+13.9</t>
         </is>
       </c>
       <c r="V51" s="23" t="inlineStr">
         <is>
-          <t>+6.3</t>
+          <t>-11.4</t>
         </is>
       </c>
       <c r="W51" s="23" t="inlineStr">
         <is>
-          <t>+2.7</t>
+          <t>-15.6</t>
         </is>
       </c>
     </row>
@@ -6389,79 +6475,79 @@
       </c>
       <c r="B52" s="23" t="inlineStr">
         <is>
-          <t>Fordham @ North Dakota State</t>
+          <t>San José State @ USC</t>
         </is>
       </c>
       <c r="C52" s="23" t="inlineStr">
         <is>
-          <t>0-38</t>
+          <t>26-42</t>
         </is>
       </c>
       <c r="D52" s="23" t="inlineStr">
         <is>
-          <t>-41.5</t>
+          <t>-37.2</t>
         </is>
       </c>
       <c r="E52" s="23" t="inlineStr">
         <is>
-          <t>+38.0</t>
+          <t>+16.0</t>
         </is>
       </c>
       <c r="F52" s="23" t="inlineStr">
         <is>
-          <t>-40.9</t>
+          <t>-34.6</t>
         </is>
       </c>
       <c r="G52" s="23" t="inlineStr">
         <is>
-          <t>-0.6</t>
+          <t>-2.7</t>
         </is>
       </c>
       <c r="H52" s="23" t="inlineStr">
         <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="I52" s="24" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="J52" s="23" t="inlineStr">
+        <is>
+          <t>-35.3</t>
+        </is>
+      </c>
+      <c r="K52" s="23" t="inlineStr">
+        <is>
+          <t>-2.0</t>
+        </is>
+      </c>
+      <c r="L52" s="23" t="inlineStr">
+        <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="I52" s="25" t="inlineStr">
+      <c r="M52" s="25" t="inlineStr">
         <is>
           <t>Loss (no real edge)</t>
         </is>
       </c>
-      <c r="J52" s="23" t="inlineStr">
-        <is>
-          <t>-35.0</t>
-        </is>
-      </c>
-      <c r="K52" s="23" t="inlineStr">
-        <is>
-          <t>-6.5</t>
-        </is>
-      </c>
-      <c r="L52" s="23" t="inlineStr">
+      <c r="N52" s="23" t="inlineStr">
+        <is>
+          <t>-16.1</t>
+        </is>
+      </c>
+      <c r="O52" s="23" t="inlineStr">
+        <is>
+          <t>-21.1</t>
+        </is>
+      </c>
+      <c r="P52" s="23" t="inlineStr">
         <is>
           <t>Away</t>
         </is>
       </c>
-      <c r="M52" s="24" t="inlineStr">
-        <is>
-          <t>Win</t>
-        </is>
-      </c>
-      <c r="N52" s="23" t="inlineStr">
-        <is>
-          <t>-19.6</t>
-        </is>
-      </c>
-      <c r="O52" s="23" t="inlineStr">
-        <is>
-          <t>-21.9</t>
-        </is>
-      </c>
-      <c r="P52" s="23" t="inlineStr">
-        <is>
-          <t>Away</t>
-        </is>
-      </c>
       <c r="Q52" s="24" t="inlineStr">
         <is>
           <t>Win (seed week)</t>
@@ -6474,485 +6560,25 @@
       </c>
       <c r="S52" s="23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="T52" s="24" t="inlineStr">
         <is>
-          <t>Ridge</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="U52" s="23" t="inlineStr">
         <is>
-          <t>+16.9</t>
+          <t>+11.2</t>
         </is>
       </c>
       <c r="V52" s="23" t="inlineStr">
         <is>
-          <t>-0.2</t>
+          <t>-13.3</t>
         </is>
       </c>
       <c r="W52" s="23" t="inlineStr">
-        <is>
-          <t>-19.2</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="B53" s="23" t="inlineStr">
-        <is>
-          <t>UTEP @ Oklahoma</t>
-        </is>
-      </c>
-      <c r="C53" s="23" t="inlineStr">
-        <is>
-          <t>0-51</t>
-        </is>
-      </c>
-      <c r="D53" s="23" t="inlineStr">
-        <is>
-          <t>-40.8</t>
-        </is>
-      </c>
-      <c r="E53" s="23" t="inlineStr">
-        <is>
-          <t>+51.0</t>
-        </is>
-      </c>
-      <c r="F53" s="23" t="inlineStr">
-        <is>
-          <t>-34.8</t>
-        </is>
-      </c>
-      <c r="G53" s="23" t="inlineStr">
-        <is>
-          <t>-5.9</t>
-        </is>
-      </c>
-      <c r="H53" s="23" t="inlineStr">
-        <is>
-          <t>Away</t>
-        </is>
-      </c>
-      <c r="I53" s="25" t="inlineStr">
-        <is>
-          <t>Loss</t>
-        </is>
-      </c>
-      <c r="J53" s="23" t="inlineStr">
-        <is>
-          <t>-32.8</t>
-        </is>
-      </c>
-      <c r="K53" s="23" t="inlineStr">
-        <is>
-          <t>-8.0</t>
-        </is>
-      </c>
-      <c r="L53" s="23" t="inlineStr">
-        <is>
-          <t>Away</t>
-        </is>
-      </c>
-      <c r="M53" s="25" t="inlineStr">
-        <is>
-          <t>Loss</t>
-        </is>
-      </c>
-      <c r="N53" s="23" t="inlineStr">
-        <is>
-          <t>-44.4</t>
-        </is>
-      </c>
-      <c r="O53" s="23" t="inlineStr">
-        <is>
-          <t>+3.6</t>
-        </is>
-      </c>
-      <c r="P53" s="23" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="Q53" s="24" t="inlineStr">
-        <is>
-          <t>Win (seed week)</t>
-        </is>
-      </c>
-      <c r="R53" s="23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="S53" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="T53" s="24" t="inlineStr">
-        <is>
-          <t>Gamma</t>
-        </is>
-      </c>
-      <c r="U53" s="23" t="inlineStr">
-        <is>
-          <t>+11.0</t>
-        </is>
-      </c>
-      <c r="V53" s="23" t="inlineStr">
-        <is>
-          <t>-8.2</t>
-        </is>
-      </c>
-      <c r="W53" s="23" t="inlineStr">
-        <is>
-          <t>-15.6</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="B54" s="23" t="inlineStr">
-        <is>
-          <t>Hawai'i @ Stanford</t>
-        </is>
-      </c>
-      <c r="C54" s="23" t="inlineStr">
-        <is>
-          <t>27-37</t>
-        </is>
-      </c>
-      <c r="D54" s="23" t="inlineStr">
-        <is>
-          <t>-4.8</t>
-        </is>
-      </c>
-      <c r="E54" s="23" t="inlineStr">
-        <is>
-          <t>+10.0</t>
-        </is>
-      </c>
-      <c r="F54" s="23" t="inlineStr">
-        <is>
-          <t>-1.5</t>
-        </is>
-      </c>
-      <c r="G54" s="23" t="inlineStr">
-        <is>
-          <t>-3.3</t>
-        </is>
-      </c>
-      <c r="H54" s="23" t="inlineStr">
-        <is>
-          <t>Away</t>
-        </is>
-      </c>
-      <c r="I54" s="25" t="inlineStr">
-        <is>
-          <t>Loss</t>
-        </is>
-      </c>
-      <c r="J54" s="23" t="inlineStr">
-        <is>
-          <t>+1.1</t>
-        </is>
-      </c>
-      <c r="K54" s="23" t="inlineStr">
-        <is>
-          <t>-5.8</t>
-        </is>
-      </c>
-      <c r="L54" s="23" t="inlineStr">
-        <is>
-          <t>Away</t>
-        </is>
-      </c>
-      <c r="M54" s="25" t="inlineStr">
-        <is>
-          <t>Loss</t>
-        </is>
-      </c>
-      <c r="N54" s="23" t="inlineStr">
-        <is>
-          <t>-11.2</t>
-        </is>
-      </c>
-      <c r="O54" s="23" t="inlineStr">
-        <is>
-          <t>+6.4</t>
-        </is>
-      </c>
-      <c r="P54" s="23" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="Q54" s="24" t="inlineStr">
-        <is>
-          <t>Win (seed week)</t>
-        </is>
-      </c>
-      <c r="R54" s="23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="S54" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="T54" s="24" t="inlineStr">
-        <is>
-          <t>Ridge</t>
-        </is>
-      </c>
-      <c r="U54" s="23" t="inlineStr">
-        <is>
-          <t>+7.7</t>
-        </is>
-      </c>
-      <c r="V54" s="23" t="inlineStr">
-        <is>
-          <t>-14.0</t>
-        </is>
-      </c>
-      <c r="W54" s="23" t="inlineStr">
-        <is>
-          <t>-9.2</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="B55" s="23" t="inlineStr">
-        <is>
-          <t>Memphis @ UNLV</t>
-        </is>
-      </c>
-      <c r="C55" s="23" t="inlineStr">
-        <is>
-          <t>27-21</t>
-        </is>
-      </c>
-      <c r="D55" s="23" t="inlineStr">
-        <is>
-          <t>-4.8</t>
-        </is>
-      </c>
-      <c r="E55" s="23" t="inlineStr">
-        <is>
-          <t>-6.0</t>
-        </is>
-      </c>
-      <c r="F55" s="23" t="inlineStr">
-        <is>
-          <t>-10.9</t>
-        </is>
-      </c>
-      <c r="G55" s="23" t="inlineStr">
-        <is>
-          <t>+6.2</t>
-        </is>
-      </c>
-      <c r="H55" s="23" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="I55" s="25" t="inlineStr">
-        <is>
-          <t>Loss</t>
-        </is>
-      </c>
-      <c r="J55" s="23" t="inlineStr">
-        <is>
-          <t>-7.4</t>
-        </is>
-      </c>
-      <c r="K55" s="23" t="inlineStr">
-        <is>
-          <t>+2.6</t>
-        </is>
-      </c>
-      <c r="L55" s="23" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="M55" s="25" t="inlineStr">
-        <is>
-          <t>Loss</t>
-        </is>
-      </c>
-      <c r="N55" s="23" t="inlineStr">
-        <is>
-          <t>+1.6</t>
-        </is>
-      </c>
-      <c r="O55" s="23" t="inlineStr">
-        <is>
-          <t>-6.3</t>
-        </is>
-      </c>
-      <c r="P55" s="23" t="inlineStr">
-        <is>
-          <t>Away</t>
-        </is>
-      </c>
-      <c r="Q55" s="24" t="inlineStr">
-        <is>
-          <t>Win (seed week)</t>
-        </is>
-      </c>
-      <c r="R55" s="23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="S55" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="T55" s="24" t="inlineStr">
-        <is>
-          <t>XGBoost</t>
-        </is>
-      </c>
-      <c r="U55" s="23" t="inlineStr">
-        <is>
-          <t>+13.9</t>
-        </is>
-      </c>
-      <c r="V55" s="23" t="inlineStr">
-        <is>
-          <t>-11.4</t>
-        </is>
-      </c>
-      <c r="W55" s="23" t="inlineStr">
-        <is>
-          <t>-15.6</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="B56" s="23" t="inlineStr">
-        <is>
-          <t>San José State @ USC</t>
-        </is>
-      </c>
-      <c r="C56" s="23" t="inlineStr">
-        <is>
-          <t>26-42</t>
-        </is>
-      </c>
-      <c r="D56" s="23" t="inlineStr">
-        <is>
-          <t>-37.2</t>
-        </is>
-      </c>
-      <c r="E56" s="23" t="inlineStr">
-        <is>
-          <t>+16.0</t>
-        </is>
-      </c>
-      <c r="F56" s="23" t="inlineStr">
-        <is>
-          <t>-34.6</t>
-        </is>
-      </c>
-      <c r="G56" s="23" t="inlineStr">
-        <is>
-          <t>-2.7</t>
-        </is>
-      </c>
-      <c r="H56" s="23" t="inlineStr">
-        <is>
-          <t>Away</t>
-        </is>
-      </c>
-      <c r="I56" s="24" t="inlineStr">
-        <is>
-          <t>Win</t>
-        </is>
-      </c>
-      <c r="J56" s="23" t="inlineStr">
-        <is>
-          <t>-35.3</t>
-        </is>
-      </c>
-      <c r="K56" s="23" t="inlineStr">
-        <is>
-          <t>-2.0</t>
-        </is>
-      </c>
-      <c r="L56" s="23" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="M56" s="25" t="inlineStr">
-        <is>
-          <t>Loss (no real edge)</t>
-        </is>
-      </c>
-      <c r="N56" s="23" t="inlineStr">
-        <is>
-          <t>-16.1</t>
-        </is>
-      </c>
-      <c r="O56" s="23" t="inlineStr">
-        <is>
-          <t>-21.1</t>
-        </is>
-      </c>
-      <c r="P56" s="23" t="inlineStr">
-        <is>
-          <t>Away</t>
-        </is>
-      </c>
-      <c r="Q56" s="24" t="inlineStr">
-        <is>
-          <t>Win (seed week)</t>
-        </is>
-      </c>
-      <c r="R56" s="23" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="S56" s="23" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="T56" s="24" t="inlineStr">
-        <is>
-          <t>XGBoost</t>
-        </is>
-      </c>
-      <c r="U56" s="23" t="inlineStr">
-        <is>
-          <t>+11.2</t>
-        </is>
-      </c>
-      <c r="V56" s="23" t="inlineStr">
-        <is>
-          <t>-13.3</t>
-        </is>
-      </c>
-      <c r="W56" s="23" t="inlineStr">
         <is>
           <t>-36.7</t>
         </is>

</xml_diff>